<commit_message>
start adding market participation constraints
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\OneDrive\Desktop\ongoing_projects\MVS\dev\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91AC85EA-7180-4DA1-B764-A979000B966B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51209128-CC5D-430A-8937-22E0CB54AB0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-9950" yWindow="-21710" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -191,7 +191,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -914,6 +914,7 @@
   <cols>
     <col min="1" max="1" width="29.33203125" customWidth="1"/>
     <col min="4" max="4" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.77734375" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="9.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1165,7 +1166,7 @@
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="1"/>
+      <c r="E12" s="3"/>
       <c r="H12" s="1"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
@@ -1175,6 +1176,9 @@
       <c r="D13" s="3">
         <v>-566684168.67891097</v>
       </c>
+      <c r="E13" s="3">
+        <v>-566684168.67891097</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -1183,6 +1187,9 @@
       <c r="D14" s="3">
         <v>6.1319999694824201</v>
       </c>
+      <c r="E14" s="3">
+        <v>2.5789999961853001</v>
+      </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
@@ -1191,6 +1198,9 @@
       <c r="D15" s="3">
         <v>0</v>
       </c>
+      <c r="E15" s="3">
+        <v>9.2925621330612702E-5</v>
+      </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
@@ -1199,230 +1209,309 @@
       <c r="D16" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E16" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D17" s="3"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>2</v>
       </c>
       <c r="D18" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E18" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>0</v>
       </c>
       <c r="D19" s="3">
         <v>80</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E19" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>1</v>
       </c>
       <c r="D20" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E20" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>29</v>
       </c>
       <c r="D21" s="3">
         <v>80</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E21" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>30</v>
       </c>
       <c r="D22" s="3">
         <v>58.084000000000003</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E22" s="3">
+        <v>58.084000000000003</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D23" s="3"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E23" s="3"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>2</v>
       </c>
       <c r="D24" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E24" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>0</v>
       </c>
       <c r="D25" s="3">
         <v>80</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E25" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>1</v>
       </c>
       <c r="D26" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E26" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="3"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E27" s="3"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>2</v>
       </c>
       <c r="D28" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E28" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>0</v>
       </c>
       <c r="D29" s="3">
         <v>93383545.771093696</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E29" s="3">
+        <v>93383545.771093696</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>1</v>
       </c>
       <c r="D30" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E30" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D31" s="3"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E31" s="3"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>2</v>
       </c>
       <c r="D32" s="3">
         <v>10839.670693578801</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E32" s="3">
+        <v>10839.670693578801</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>0</v>
       </c>
       <c r="D33" s="3">
         <v>820924.35254566895</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E33" s="3">
+        <v>755352.36146108399</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>1</v>
       </c>
       <c r="D34" s="3">
         <v>8697.9159292100703</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E34" s="3">
+        <v>8697.9159292100794</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D35" s="3"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E35" s="3"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>0</v>
       </c>
       <c r="D36" s="3">
         <v>65571.991084584399</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E36" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="3">
         <v>764613.58238300995</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E37" s="3">
+        <v>764613.58238300995</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>1</v>
       </c>
       <c r="D38" s="3">
         <v>10276.3657008625</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E38" s="3">
+        <v>10276.3657008625</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D39" s="3"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E39" s="3"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>2</v>
       </c>
       <c r="D40" s="3">
         <v>1636903.5360916599</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E40" s="3">
+        <v>1636903.5360916599</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>0</v>
       </c>
       <c r="D41" s="3">
         <v>15934518.027864</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E41" s="3">
+        <v>14194345.611482101</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>1</v>
       </c>
       <c r="D42" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E42" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>28</v>
       </c>
       <c r="D43" s="3"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E43" s="3"/>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>0</v>
       </c>
       <c r="D44" s="3">
         <v>1740172.41638191</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E44" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>24</v>
       </c>
       <c r="D45" s="3">
         <v>675898963.597579</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E45" s="3">
+        <v>675898963.597579</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>1</v>
       </c>
       <c r="D46" s="3">
+        <v>0</v>
+      </c>
+      <c r="E46" s="3">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
increase value of lost load to trigger storage deployment
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\OneDrive\Desktop\ongoing_projects\MVS\dev\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51209128-CC5D-430A-8937-22E0CB54AB0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38ED15E6-E822-45A9-AD24-8EC5C03D45CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-9950" yWindow="-21710" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-9030" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Experiments" sheetId="1" r:id="rId1"/>
-    <sheet name="20250424" sheetId="2" r:id="rId2"/>
+    <sheet name="20250425" sheetId="3" r:id="rId2"/>
+    <sheet name="20250424" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="39">
   <si>
     <t>Grid</t>
   </si>
@@ -125,14 +126,33 @@
   </si>
   <si>
     <t>Computing time (s)</t>
+  </si>
+  <si>
+    <t>Market parameters</t>
+  </si>
+  <si>
+    <t>Discount rate</t>
+  </si>
+  <si>
+    <t>Unmet Load</t>
+  </si>
+  <si>
+    <t>Number of peak load days in 2050</t>
+  </si>
+  <si>
+    <t>Probability of contingency on peak load days</t>
+  </si>
+  <si>
+    <t>Consumer value of electricity</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -187,11 +207,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -474,28 +496,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J46"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.33203125" customWidth="1"/>
-    <col min="7" max="8" width="9.33203125" customWidth="1"/>
+    <col min="1" max="1" width="29.28515625" customWidth="1"/>
+    <col min="7" max="8" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -527,7 +549,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -559,7 +581,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -591,12 +613,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -628,7 +650,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -660,7 +682,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -692,7 +714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -724,179 +746,179 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E12" s="1"/>
       <c r="H12" s="1"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>1</v>
       </c>
@@ -908,220 +930,1076 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4317E227-4F2F-4766-80E7-4A0C11DC1BA8}">
-  <dimension ref="A1:J46"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00CD46BB-A2D1-4791-8AAC-69869F785713}">
+  <dimension ref="A1:L52"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.33203125" customWidth="1"/>
-    <col min="4" max="4" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="9.33203125" customWidth="1"/>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="4" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.28515625" customWidth="1"/>
+    <col min="11" max="12" width="19.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="K5" s="4">
+        <v>10000</v>
+      </c>
+      <c r="L5" s="4">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>36</v>
+      </c>
+      <c r="K6">
+        <v>40</v>
+      </c>
+      <c r="L6">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>37</v>
+      </c>
+      <c r="K7">
+        <v>0.2</v>
+      </c>
+      <c r="L7">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9">
+        <v>1</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+      <c r="J10">
+        <v>1</v>
+      </c>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>1</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>1</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>1</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>1</v>
+      </c>
+      <c r="J14">
+        <v>1</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>1</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17" s="3"/>
+      <c r="H17" s="1"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="4">
+        <v>-1816246557.4803801</v>
+      </c>
+      <c r="E18" s="4">
+        <v>-1816151942.22171</v>
+      </c>
+      <c r="K18" s="3">
+        <v>-34203470096.309399</v>
+      </c>
+      <c r="L18" s="3">
+        <v>-34205493917.001499</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="4">
+        <v>3.3900001049041699</v>
+      </c>
+      <c r="E19" s="4">
+        <v>3.0910000801086399</v>
+      </c>
+      <c r="K19" s="3">
+        <v>7.3829998970031703</v>
+      </c>
+      <c r="L19" s="3">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>17</v>
+      </c>
+      <c r="D20" s="4">
+        <v>0</v>
+      </c>
+      <c r="E20" s="4">
+        <v>9.8172251951082401E-5</v>
+      </c>
+      <c r="K20" s="3">
+        <v>6.74029824543434E-5</v>
+      </c>
+      <c r="L20" s="3">
+        <v>9.0114622647770906E-5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" s="4">
+        <v>0</v>
+      </c>
+      <c r="E21" s="4">
+        <v>0</v>
+      </c>
+      <c r="K21" s="3">
+        <v>0</v>
+      </c>
+      <c r="L21" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>2</v>
+      </c>
+      <c r="D23" s="4">
+        <v>0</v>
+      </c>
+      <c r="E23" s="4">
+        <v>0</v>
+      </c>
+      <c r="K23" s="3">
+        <v>0</v>
+      </c>
+      <c r="L23" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>0</v>
+      </c>
+      <c r="D24" s="4">
+        <v>120</v>
+      </c>
+      <c r="E24" s="4">
+        <v>120</v>
+      </c>
+      <c r="K24" s="3">
+        <v>120</v>
+      </c>
+      <c r="L24" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>1</v>
+      </c>
+      <c r="D25" s="4">
+        <v>0</v>
+      </c>
+      <c r="E25" s="4">
+        <v>0</v>
+      </c>
+      <c r="K25" s="3">
+        <v>15.103999999999999</v>
+      </c>
+      <c r="L25" s="3">
+        <v>17.785999999999898</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>29</v>
+      </c>
+      <c r="D26" s="4">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="E26" s="4">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="K26" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="L26" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>30</v>
+      </c>
+      <c r="D27" s="4">
+        <v>18.084</v>
+      </c>
+      <c r="E27" s="4">
+        <v>18.084</v>
+      </c>
+      <c r="K27" s="3">
+        <v>2.98</v>
+      </c>
+      <c r="L27" s="3">
+        <v>0.29800000000000099</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>2</v>
+      </c>
+      <c r="D29" s="4">
+        <v>0</v>
+      </c>
+      <c r="E29" s="4">
+        <v>0</v>
+      </c>
+      <c r="K29" s="3">
+        <v>0</v>
+      </c>
+      <c r="L29" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>0</v>
+      </c>
+      <c r="D30" s="4">
+        <v>120</v>
+      </c>
+      <c r="E30" s="4">
+        <v>120</v>
+      </c>
+      <c r="K30" s="3">
+        <v>120</v>
+      </c>
+      <c r="L30" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>1</v>
+      </c>
+      <c r="D31" s="4">
+        <v>0</v>
+      </c>
+      <c r="E31" s="4">
+        <v>0</v>
+      </c>
+      <c r="K31" s="3">
+        <v>15.103999999999999</v>
+      </c>
+      <c r="L31" s="3">
+        <v>17.785999999999898</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="K32" s="3"/>
+      <c r="L32" s="3"/>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>2</v>
+      </c>
+      <c r="D33" s="4">
+        <v>0</v>
+      </c>
+      <c r="E33" s="4">
+        <v>0</v>
+      </c>
+      <c r="K33" s="3">
+        <v>0</v>
+      </c>
+      <c r="L33" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>0</v>
+      </c>
+      <c r="D34" s="4">
+        <v>174732082.43857899</v>
+      </c>
+      <c r="E34" s="4">
+        <v>168491650.922916</v>
+      </c>
+      <c r="K34" s="3">
+        <v>262098123.65786901</v>
+      </c>
+      <c r="L34" s="3">
+        <v>268338555.17353299</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>1</v>
+      </c>
+      <c r="D35" s="4">
+        <v>0</v>
+      </c>
+      <c r="E35" s="4">
+        <v>0</v>
+      </c>
+      <c r="K35" s="3">
+        <v>41539681.597128302</v>
+      </c>
+      <c r="L35" s="3">
+        <v>42147012.109867401</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
+      <c r="K36" s="3"/>
+      <c r="L36" s="3"/>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>2</v>
+      </c>
+      <c r="D37" s="4">
+        <v>5567.7598935788701</v>
+      </c>
+      <c r="E37" s="4">
+        <v>5567.7598935788701</v>
+      </c>
+      <c r="K37" s="3">
+        <v>1728.1617106413701</v>
+      </c>
+      <c r="L37" s="3">
+        <v>843.13385541081698</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>0</v>
+      </c>
+      <c r="D38" s="4">
+        <v>978304.363808266</v>
+      </c>
+      <c r="E38" s="4">
+        <v>808132.80189079896</v>
+      </c>
+      <c r="K38" s="3">
+        <v>2110776.2209756798</v>
+      </c>
+      <c r="L38" s="3">
+        <v>1395944.4604960401</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>1</v>
+      </c>
+      <c r="D39" s="4">
+        <v>9311.3535690200606</v>
+      </c>
+      <c r="E39" s="4">
+        <v>9311.3535690200606</v>
+      </c>
+      <c r="K39" s="3">
+        <v>70388.471206651404</v>
+      </c>
+      <c r="L39" s="3">
+        <v>72794.0703632644</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+      <c r="K40" s="3"/>
+      <c r="L40" s="3"/>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>0</v>
+      </c>
+      <c r="D41" s="4">
+        <v>167570.938196884</v>
+      </c>
+      <c r="E41" s="4">
+        <v>0</v>
+      </c>
+      <c r="K41" s="3">
+        <v>716497.26674218394</v>
+      </c>
+      <c r="L41" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>24</v>
+      </c>
+      <c r="D42" s="4">
+        <v>814611.41245651699</v>
+      </c>
+      <c r="E42" s="4">
+        <v>812010.78873593605</v>
+      </c>
+      <c r="K42" s="3">
+        <v>1383233.4047232701</v>
+      </c>
+      <c r="L42" s="3">
+        <v>1383577.3282741799</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>35</v>
+      </c>
+      <c r="D43" s="4">
+        <v>9497.9028860672006</v>
+      </c>
+      <c r="E43" s="4">
+        <v>12098.5266066486</v>
+      </c>
+      <c r="K43" s="3">
+        <v>608.27249077396004</v>
+      </c>
+      <c r="L43" s="3">
+        <v>264.34893985823402</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>1</v>
+      </c>
+      <c r="D44" s="4">
+        <v>11001.1266174622</v>
+      </c>
+      <c r="E44" s="4">
+        <v>11001.1266174622</v>
+      </c>
+      <c r="K44" s="3">
+        <v>83162.182427518201</v>
+      </c>
+      <c r="L44" s="3">
+        <v>86004.336440529805</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="K45" s="3"/>
+      <c r="L45" s="3"/>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>2</v>
+      </c>
+      <c r="D46" s="4">
+        <v>1699829.82219933</v>
+      </c>
+      <c r="E46" s="4">
+        <v>1699829.82219933</v>
+      </c>
+      <c r="K46" s="3">
+        <v>527605.51271599403</v>
+      </c>
+      <c r="L46" s="3">
+        <v>257407.664649126</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>0</v>
+      </c>
+      <c r="D47" s="4">
+        <v>52575087.091096699</v>
+      </c>
+      <c r="E47" s="4">
+        <v>43683548.873010099</v>
+      </c>
+      <c r="K47" s="3">
+        <v>111647367.375127</v>
+      </c>
+      <c r="L47" s="3">
+        <v>73196314.905121207</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>1</v>
+      </c>
+      <c r="D48" s="4">
+        <v>0</v>
+      </c>
+      <c r="E48" s="4">
+        <v>0</v>
+      </c>
+      <c r="K48" s="3">
+        <v>0</v>
+      </c>
+      <c r="L48" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4"/>
+      <c r="K49" s="3"/>
+      <c r="L49" s="3"/>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>0</v>
+      </c>
+      <c r="D50" s="4">
+        <v>8725025.6909637991</v>
+      </c>
+      <c r="E50" s="4">
+        <v>0</v>
+      </c>
+      <c r="K50" s="3">
+        <v>38447756.3704492</v>
+      </c>
+      <c r="L50" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>24</v>
+      </c>
+      <c r="D51" s="4">
+        <v>2036528531.1412899</v>
+      </c>
+      <c r="E51" s="4">
+        <v>2030026971.8398399</v>
+      </c>
+      <c r="K51" s="3">
+        <v>34580835118.081802</v>
+      </c>
+      <c r="L51" s="3">
+        <v>34589433206.854698</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>1</v>
+      </c>
+      <c r="D52" s="4">
+        <v>0</v>
+      </c>
+      <c r="E52" s="4">
+        <v>0</v>
+      </c>
+      <c r="K52" s="3">
+        <v>0</v>
+      </c>
+      <c r="L52" s="3">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4317E227-4F2F-4766-80E7-4A0C11DC1BA8}">
+  <dimension ref="A1:J48"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="29.28515625" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>6.8500000000000005E-2</v>
       </c>
       <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="J5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6.8500000000000005E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>2</v>
       </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6">
-        <v>0</v>
-      </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>8</v>
-      </c>
-      <c r="B8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>1</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-      <c r="J8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9">
-        <v>1</v>
-      </c>
-      <c r="G9">
-        <v>1</v>
-      </c>
-      <c r="H9">
-        <v>0</v>
-      </c>
-      <c r="I9">
-        <v>1</v>
-      </c>
-      <c r="J9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>4</v>
       </c>
       <c r="B10" t="s">
         <v>18</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10">
         <v>0</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10">
         <v>0</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -1130,122 +2008,164 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B11" t="s">
         <v>18</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
+      <c r="J11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
         <v>18</v>
       </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11">
-        <v>0</v>
-      </c>
-      <c r="G11">
-        <v>1</v>
-      </c>
-      <c r="H11">
-        <v>0</v>
-      </c>
-      <c r="I11">
-        <v>0</v>
-      </c>
-      <c r="J11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="3"/>
-      <c r="H12" s="1"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="E14" s="3"/>
+      <c r="H14" s="1"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D15" s="3">
         <v>-566684168.67891097</v>
       </c>
-      <c r="E13" s="3">
+      <c r="E15" s="3">
         <v>-566684168.67891097</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D16" s="3">
         <v>6.1319999694824201</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E16" s="3">
         <v>2.5789999961853001</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>17</v>
       </c>
-      <c r="D15" s="3">
-        <v>0</v>
-      </c>
-      <c r="E15" s="3">
+      <c r="D17" s="3">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3">
         <v>9.2925621330612702E-5</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="3">
-        <v>0</v>
-      </c>
-      <c r="E16" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+      <c r="D18" s="3">
+        <v>0</v>
+      </c>
+      <c r="E18" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>2</v>
       </c>
-      <c r="D18" s="3">
-        <v>0</v>
-      </c>
-      <c r="E18" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>0</v>
-      </c>
-      <c r="D19" s="3">
-        <v>80</v>
-      </c>
-      <c r="E19" s="3">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>1</v>
-      </c>
       <c r="D20" s="3">
         <v>0</v>
       </c>
@@ -1253,9 +2173,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="D21" s="3">
         <v>80</v>
@@ -1264,254 +2184,276 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>1</v>
+      </c>
+      <c r="D22" s="3">
+        <v>0</v>
+      </c>
+      <c r="E22" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>29</v>
+      </c>
+      <c r="D23" s="3">
+        <v>80</v>
+      </c>
+      <c r="E23" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>30</v>
       </c>
-      <c r="D22" s="3">
+      <c r="D24" s="3">
         <v>58.084000000000003</v>
       </c>
-      <c r="E22" s="3">
+      <c r="E24" s="3">
         <v>58.084000000000003</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>2</v>
       </c>
-      <c r="D24" s="3">
-        <v>0</v>
-      </c>
-      <c r="E24" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>0</v>
-      </c>
-      <c r="D25" s="3">
+      <c r="D26" s="3">
+        <v>0</v>
+      </c>
+      <c r="E26" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>0</v>
+      </c>
+      <c r="D27" s="3">
         <v>80</v>
       </c>
-      <c r="E25" s="3">
+      <c r="E27" s="3">
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>1</v>
-      </c>
-      <c r="D26" s="3">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>1</v>
+      </c>
+      <c r="D28" s="3">
+        <v>0</v>
+      </c>
+      <c r="E28" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>2</v>
       </c>
-      <c r="D28" s="3">
-        <v>0</v>
-      </c>
-      <c r="E28" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>0</v>
-      </c>
-      <c r="D29" s="3">
+      <c r="D30" s="3">
+        <v>0</v>
+      </c>
+      <c r="E30" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>0</v>
+      </c>
+      <c r="D31" s="3">
         <v>93383545.771093696</v>
       </c>
-      <c r="E29" s="3">
+      <c r="E31" s="3">
         <v>93383545.771093696</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>1</v>
-      </c>
-      <c r="D30" s="3">
-        <v>0</v>
-      </c>
-      <c r="E30" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" s="2" t="s">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>1</v>
+      </c>
+      <c r="D32" s="3">
+        <v>0</v>
+      </c>
+      <c r="E32" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>2</v>
       </c>
-      <c r="D32" s="3">
+      <c r="D34" s="3">
         <v>10839.670693578801</v>
       </c>
-      <c r="E32" s="3">
+      <c r="E34" s="3">
         <v>10839.670693578801</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>0</v>
-      </c>
-      <c r="D33" s="3">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>0</v>
+      </c>
+      <c r="D35" s="3">
         <v>820924.35254566895</v>
       </c>
-      <c r="E33" s="3">
+      <c r="E35" s="3">
         <v>755352.36146108399</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>1</v>
-      </c>
-      <c r="D34" s="3">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>1</v>
+      </c>
+      <c r="D36" s="3">
         <v>8697.9159292100703</v>
       </c>
-      <c r="E34" s="3">
+      <c r="E36" s="3">
         <v>8697.9159292100794</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A35" s="2" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>0</v>
-      </c>
-      <c r="D36" s="3">
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>0</v>
+      </c>
+      <c r="D38" s="3">
         <v>65571.991084584399</v>
       </c>
-      <c r="E36" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
+      <c r="E38" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>24</v>
       </c>
-      <c r="D37" s="3">
+      <c r="D39" s="3">
         <v>764613.58238300995</v>
       </c>
-      <c r="E37" s="3">
+      <c r="E39" s="3">
         <v>764613.58238300995</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>1</v>
-      </c>
-      <c r="D38" s="3">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>1</v>
+      </c>
+      <c r="D40" s="3">
         <v>10276.3657008625</v>
       </c>
-      <c r="E38" s="3">
+      <c r="E40" s="3">
         <v>10276.3657008625</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A39" s="2" t="s">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D39" s="3"/>
-      <c r="E39" s="3"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
+      <c r="D41" s="3"/>
+      <c r="E41" s="3"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>2</v>
       </c>
-      <c r="D40" s="3">
+      <c r="D42" s="3">
         <v>1636903.5360916599</v>
       </c>
-      <c r="E40" s="3">
+      <c r="E42" s="3">
         <v>1636903.5360916599</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>0</v>
-      </c>
-      <c r="D41" s="3">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>0</v>
+      </c>
+      <c r="D43" s="3">
         <v>15934518.027864</v>
       </c>
-      <c r="E41" s="3">
+      <c r="E43" s="3">
         <v>14194345.611482101</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>1</v>
-      </c>
-      <c r="D42" s="3">
-        <v>0</v>
-      </c>
-      <c r="E42" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A43" s="2" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>1</v>
+      </c>
+      <c r="D44" s="3">
+        <v>0</v>
+      </c>
+      <c r="E44" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D43" s="3"/>
-      <c r="E43" s="3"/>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>0</v>
-      </c>
-      <c r="D44" s="3">
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>0</v>
+      </c>
+      <c r="D46" s="3">
         <v>1740172.41638191</v>
       </c>
-      <c r="E44" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
+      <c r="E46" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>24</v>
       </c>
-      <c r="D45" s="3">
+      <c r="D47" s="3">
         <v>675898963.597579</v>
       </c>
-      <c r="E45" s="3">
+      <c r="E47" s="3">
         <v>675898963.597579</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>1</v>
-      </c>
-      <c r="D46" s="3">
-        <v>0</v>
-      </c>
-      <c r="E46" s="3">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>1</v>
+      </c>
+      <c r="D48" s="3">
+        <v>0</v>
+      </c>
+      <c r="E48" s="3">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add peak_shaving market participation
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\OneDrive\Desktop\ongoing_projects\MVS\dev\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38ED15E6-E822-45A9-AD24-8EC5C03D45CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A17C546D-62BD-448F-8F48-ECC130F86A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-9030" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -207,13 +207,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -931,31 +930,31 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00CD46BB-A2D1-4791-8AAC-69869F785713}">
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:M52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="4" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="9.28515625" customWidth="1"/>
-    <col min="11" max="12" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="19.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -971,9 +970,12 @@
       <c r="L4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="M4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>38</v>
       </c>
       <c r="K5" s="4">
@@ -982,8 +984,11 @@
       <c r="L5" s="4">
         <v>10000</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M5" s="4">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>36</v>
       </c>
@@ -993,8 +998,11 @@
       <c r="L6">
         <v>40</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M6">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>37</v>
       </c>
@@ -1004,13 +1012,16 @@
       <c r="L7">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M7">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -1047,8 +1058,11 @@
       <c r="L9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -1085,8 +1099,11 @@
       <c r="L10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -1123,13 +1140,16 @@
       <c r="L11">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -1166,8 +1186,11 @@
       <c r="L13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1204,8 +1227,11 @@
       <c r="L14">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -1242,8 +1268,11 @@
       <c r="L15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -1280,15 +1309,18 @@
       <c r="L16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E17" s="3"/>
       <c r="H17" s="1"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>10</v>
       </c>
@@ -1299,13 +1331,16 @@
         <v>-1816151942.22171</v>
       </c>
       <c r="K18" s="3">
-        <v>-34203470096.309399</v>
+        <v>-13464876360.058001</v>
       </c>
       <c r="L18" s="3">
-        <v>-34205493917.001499</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+        <v>-13464792750.8997</v>
+      </c>
+      <c r="M18" s="3">
+        <v>-13456893997.0168</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -1316,13 +1351,16 @@
         <v>3.0910000801086399</v>
       </c>
       <c r="K19" s="3">
-        <v>7.3829998970031703</v>
+        <v>7.2590000629425004</v>
       </c>
       <c r="L19" s="3">
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+        <v>8.6590001583099294</v>
+      </c>
+      <c r="M19" s="3">
+        <v>34.491999864578197</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -1333,13 +1371,16 @@
         <v>9.8172251951082401E-5</v>
       </c>
       <c r="K20" s="3">
-        <v>6.74029824543434E-5</v>
+        <v>2.4509630770603201E-5</v>
       </c>
       <c r="L20" s="3">
-        <v>9.0114622647770906E-5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+        <v>1.94134036118058E-5</v>
+      </c>
+      <c r="M20" s="3">
+        <v>8.0815127926575099E-5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -1355,8 +1396,11 @@
       <c r="L21" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M21" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>11</v>
       </c>
@@ -1364,8 +1408,9 @@
       <c r="E22" s="4"/>
       <c r="K22" s="3"/>
       <c r="L22" s="3"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M22" s="3"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>2</v>
       </c>
@@ -1381,8 +1426,11 @@
       <c r="L23" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M23" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -1398,8 +1446,11 @@
       <c r="L24" s="3">
         <v>120</v>
       </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M24" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>1</v>
       </c>
@@ -1410,13 +1461,16 @@
         <v>0</v>
       </c>
       <c r="K25" s="3">
-        <v>15.103999999999999</v>
+        <v>15.427141887889199</v>
       </c>
       <c r="L25" s="3">
-        <v>17.785999999999898</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+        <v>15.4271418878891</v>
+      </c>
+      <c r="M25" s="3">
+        <v>15.427141887890601</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>29</v>
       </c>
@@ -1432,8 +1486,11 @@
       <c r="L26" s="3">
         <v>98.084000000000003</v>
       </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M26" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>30</v>
       </c>
@@ -1444,13 +1501,16 @@
         <v>18.084</v>
       </c>
       <c r="K27" s="3">
-        <v>2.98</v>
+        <v>2.6568581121100401</v>
       </c>
       <c r="L27" s="3">
-        <v>0.29800000000000099</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+        <v>2.6568581121102</v>
+      </c>
+      <c r="M27" s="3">
+        <v>2.65685811210931</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>15</v>
       </c>
@@ -1458,8 +1518,9 @@
       <c r="E28" s="4"/>
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M28" s="3"/>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>2</v>
       </c>
@@ -1475,8 +1536,11 @@
       <c r="L29" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M29" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>0</v>
       </c>
@@ -1492,8 +1556,11 @@
       <c r="L30" s="3">
         <v>120</v>
       </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M30" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>1</v>
       </c>
@@ -1504,13 +1571,16 @@
         <v>0</v>
       </c>
       <c r="K31" s="3">
-        <v>15.103999999999999</v>
+        <v>15.427141887889199</v>
       </c>
       <c r="L31" s="3">
-        <v>17.785999999999898</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+        <v>15.4271418878891</v>
+      </c>
+      <c r="M31" s="3">
+        <v>15.427141887890601</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>16</v>
       </c>
@@ -1518,8 +1588,9 @@
       <c r="E32" s="4"/>
       <c r="K32" s="3"/>
       <c r="L32" s="3"/>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M32" s="3"/>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -1535,8 +1606,11 @@
       <c r="L33" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M33" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>0</v>
       </c>
@@ -1547,13 +1621,16 @@
         <v>168491650.922916</v>
       </c>
       <c r="K34" s="3">
-        <v>262098123.65786901</v>
+        <v>243376829.110879</v>
       </c>
       <c r="L34" s="3">
-        <v>268338555.17353299</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+        <v>243376829.110879</v>
+      </c>
+      <c r="M34" s="3">
+        <v>249617260.626542</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>1</v>
       </c>
@@ -1564,13 +1641,16 @@
         <v>0</v>
       </c>
       <c r="K35" s="3">
-        <v>41539681.597128302</v>
+        <v>30455887.5617279</v>
       </c>
       <c r="L35" s="3">
-        <v>42147012.109867401</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+        <v>30544228.586333599</v>
+      </c>
+      <c r="M35" s="3">
+        <v>30544228.586336799</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>23</v>
       </c>
@@ -1578,8 +1658,9 @@
       <c r="E36" s="4"/>
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M36" s="3"/>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>2</v>
       </c>
@@ -1590,13 +1671,16 @@
         <v>5567.7598935788701</v>
       </c>
       <c r="K37" s="3">
-        <v>1728.1617106413701</v>
+        <v>4826.3183783554796</v>
       </c>
       <c r="L37" s="3">
-        <v>843.13385541081698</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+        <v>4826.3183783554896</v>
+      </c>
+      <c r="M37" s="3">
+        <v>3421.3094646414202</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>0</v>
       </c>
@@ -1607,13 +1691,16 @@
         <v>808132.80189079896</v>
       </c>
       <c r="K38" s="3">
-        <v>2110776.2209756798</v>
+        <v>2051061.57238617</v>
       </c>
       <c r="L38" s="3">
-        <v>1395944.4604960401</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+        <v>1386880.28540422</v>
+      </c>
+      <c r="M38" s="3">
+        <v>1772151.2791056901</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>1</v>
       </c>
@@ -1624,13 +1711,16 @@
         <v>9311.3535690200606</v>
       </c>
       <c r="K39" s="3">
-        <v>70388.471206651404</v>
+        <v>57042.475334709103</v>
       </c>
       <c r="L39" s="3">
-        <v>72794.0703632644</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+        <v>57044.315022773</v>
+      </c>
+      <c r="M39" s="3">
+        <v>7524.5956312832805</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>22</v>
       </c>
@@ -1638,8 +1728,9 @@
       <c r="E40" s="4"/>
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M40" s="3"/>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>0</v>
       </c>
@@ -1650,13 +1741,16 @@
         <v>0</v>
       </c>
       <c r="K41" s="3">
-        <v>716497.26674218394</v>
+        <v>664182.13855842699</v>
       </c>
       <c r="L41" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M41" s="3">
+        <v>392888.13096246601</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>24</v>
       </c>
@@ -1667,13 +1761,16 @@
         <v>812010.78873593605</v>
       </c>
       <c r="K42" s="3">
-        <v>1383233.4047232701</v>
+        <v>1381353.9986481899</v>
       </c>
       <c r="L42" s="3">
-        <v>1383577.3282741799</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+        <v>1381354.5163682399</v>
+      </c>
+      <c r="M42" s="3">
+        <v>1381318.93552733</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>35</v>
       </c>
@@ -1684,13 +1781,16 @@
         <v>12098.5266066486</v>
       </c>
       <c r="K43" s="3">
-        <v>608.27249077396004</v>
+        <v>2487.6785658501699</v>
       </c>
       <c r="L43" s="3">
-        <v>264.34893985823402</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+        <v>2487.16084580499</v>
+      </c>
+      <c r="M43" s="3">
+        <v>2522.7416867100901</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -1701,13 +1801,16 @@
         <v>11001.1266174622</v>
       </c>
       <c r="K44" s="3">
-        <v>83162.182427518201</v>
+        <v>67394.228892614701</v>
       </c>
       <c r="L44" s="3">
-        <v>86004.336440529805</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+        <v>67396.402437113706</v>
+      </c>
+      <c r="M44" s="3">
+        <v>8890.1177118186097</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>27</v>
       </c>
@@ -1715,8 +1818,9 @@
       <c r="E45" s="4"/>
       <c r="K45" s="3"/>
       <c r="L45" s="3"/>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M45" s="3"/>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>2</v>
       </c>
@@ -1727,13 +1831,16 @@
         <v>1699829.82219933</v>
       </c>
       <c r="K46" s="3">
-        <v>527605.51271599403</v>
+        <v>1473468.6961660599</v>
       </c>
       <c r="L46" s="3">
-        <v>257407.664649126</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+        <v>1473468.6961660599</v>
+      </c>
+      <c r="M46" s="3">
+        <v>1044521.3102090301</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>0</v>
       </c>
@@ -1744,13 +1851,16 @@
         <v>43683548.873010099</v>
       </c>
       <c r="K47" s="3">
-        <v>111647367.375127</v>
+        <v>107871853.336619</v>
       </c>
       <c r="L47" s="3">
-        <v>73196314.905121207</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+        <v>73357886.389309898</v>
+      </c>
+      <c r="M47" s="3">
+        <v>96512651.699123099</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>1</v>
       </c>
@@ -1766,8 +1876,11 @@
       <c r="L48" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M48" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>28</v>
       </c>
@@ -1775,8 +1888,9 @@
       <c r="E49" s="4"/>
       <c r="K49" s="3"/>
       <c r="L49" s="3"/>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M49" s="3"/>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>0</v>
       </c>
@@ -1787,13 +1901,16 @@
         <v>0</v>
       </c>
       <c r="K50" s="3">
-        <v>38447756.3704492</v>
+        <v>34514412.281520903</v>
       </c>
       <c r="L50" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M50" s="3">
+        <v>21423303.9657369</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>24</v>
       </c>
@@ -1804,13 +1921,16 @@
         <v>2030026971.8398399</v>
       </c>
       <c r="K51" s="3">
-        <v>34580835118.081802</v>
+        <v>13813539986.481899</v>
       </c>
       <c r="L51" s="3">
-        <v>34589433206.854698</v>
-      </c>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+        <v>13813545163.6824</v>
+      </c>
+      <c r="M51" s="3">
+        <v>13813189355.2733</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>1</v>
       </c>
@@ -1824,6 +1944,9 @@
         <v>0</v>
       </c>
       <c r="L52" s="3">
+        <v>0</v>
+      </c>
+      <c r="M52" s="3">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
analyze impact of battery warranty and days with/without storage activity
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\OneDrive\Desktop\ongoing_projects\MVS\dev\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\Desktop\ongoing_projects\MVS\dev\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0990F3E1-3313-47D7-A46A-955D0E900B78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7876657-09CB-4059-89FA-04F7BCACAE98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-9030" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Experiments" sheetId="1" r:id="rId1"/>
     <sheet name="20250425" sheetId="3" r:id="rId2"/>
     <sheet name="20250424" sheetId="2" r:id="rId3"/>
     <sheet name="20250505_Ops" sheetId="4" r:id="rId4"/>
+    <sheet name="250601_ops" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
     <author>tc={3596D6DD-00D5-48B9-98E5-2DE582B601C8}</author>
   </authors>
   <commentList>
-    <comment ref="G39" authorId="0" shapeId="0" xr:uid="{3596D6DD-00D5-48B9-98E5-2DE582B601C8}">
+    <comment ref="G40" authorId="0" shapeId="0" xr:uid="{3596D6DD-00D5-48B9-98E5-2DE582B601C8}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -57,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="62">
   <si>
     <t>Grid</t>
   </si>
@@ -204,6 +205,45 @@
   </si>
   <si>
     <t>Objective (Cost)</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Peak</t>
+  </si>
+  <si>
+    <t>Time Horizon</t>
+  </si>
+  <si>
+    <t>Value of lost load ($/MWh)</t>
+  </si>
+  <si>
+    <t>Running peak load for 2025!</t>
+  </si>
+  <si>
+    <t>Operating cost ($)</t>
+  </si>
+  <si>
+    <t>Maximum battery supply (MWh/yr)</t>
+  </si>
+  <si>
+    <t>Days with storage supply (-)</t>
+  </si>
+  <si>
+    <t>Time Horizon (h)</t>
+  </si>
+  <si>
+    <t>Days with insufficient grid capacity (-)</t>
+  </si>
+  <si>
+    <t>Days with storage demand (-)</t>
+  </si>
+  <si>
+    <t>(perfect foresight)</t>
+  </si>
+  <si>
+    <t>Contingencies</t>
   </si>
 </sst>
 </file>
@@ -214,7 +254,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -245,12 +285,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -273,13 +307,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -567,7 +605,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="G39" dT="2025-05-05T20:36:53.40" personId="{ECC6709C-9A20-4DC5-ADE3-5C36CDEEBD3D}" id="{3596D6DD-00D5-48B9-98E5-2DE582B601C8}">
+  <threadedComment ref="G40" dT="2025-05-05T20:36:53.40" personId="{ECC6709C-9A20-4DC5-ADE3-5C36CDEEBD3D}" id="{3596D6DD-00D5-48B9-98E5-2DE582B601C8}">
     <text>Higher load shed because we cannot use backup generation to load storage anymore.</text>
   </threadedComment>
 </ThreadedComments>
@@ -2669,337 +2707,442 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CDE5EF9-418E-4572-AF84-E6DEF6E71829}">
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:M49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.28515625" customWidth="1"/>
+    <col min="8" max="8" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="13" width="19.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" s="6">
+        <v>45810</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H3" s="4">
+        <v>2500</v>
+      </c>
+      <c r="I3" s="4">
+        <v>2500</v>
+      </c>
+      <c r="J3" s="4">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="3"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B6" s="3">
         <v>12.92135</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C6" s="3">
         <v>12.92135</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D6" s="3">
         <v>12.92135</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E6" s="3">
         <v>12.92135</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F6" s="3">
         <v>12.92135</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G6" s="3">
         <v>12.92135</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="3">
+      <c r="H6" s="3">
+        <v>12.920999999999999</v>
+      </c>
+      <c r="I6" s="3">
+        <v>12.920999999999999</v>
+      </c>
+      <c r="J6">
+        <v>12.920999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="3">
         <v>74</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C7" s="3">
         <v>74</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D7" s="3">
         <v>74</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E7" s="3">
         <v>36</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F7" s="3">
         <v>36</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G7" s="3">
         <v>36</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="3">
+      <c r="H7" s="3">
+        <v>36</v>
+      </c>
+      <c r="I7" s="3">
+        <v>36</v>
+      </c>
+      <c r="J7" s="8">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="3">
         <v>6</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C8" s="3">
         <v>6</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D8" s="3">
         <v>6</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E8" s="3">
         <v>6</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F8" s="3">
         <v>6</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G8" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="H8" s="3">
+        <v>6</v>
+      </c>
+      <c r="I8" s="3">
+        <v>6</v>
+      </c>
+      <c r="J8" s="8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="3">
-        <v>1</v>
-      </c>
-      <c r="C9" s="3">
-        <v>0</v>
-      </c>
-      <c r="D9" s="3">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3">
-        <v>1</v>
-      </c>
-      <c r="F9" s="3">
-        <v>0</v>
-      </c>
-      <c r="G9" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B10" s="3">
+        <v>1</v>
+      </c>
+      <c r="C10" s="3">
+        <v>0</v>
+      </c>
+      <c r="D10" s="3">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3">
+        <v>1</v>
+      </c>
+      <c r="F10" s="3">
+        <v>0</v>
+      </c>
+      <c r="G10" s="3">
+        <v>0</v>
+      </c>
+      <c r="H10" s="3">
+        <v>0</v>
+      </c>
+      <c r="I10" s="3">
+        <v>0</v>
+      </c>
+      <c r="J10" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="3">
-        <v>0</v>
-      </c>
-      <c r="C10" s="3">
-        <v>1</v>
-      </c>
-      <c r="D10" s="3">
-        <v>0</v>
-      </c>
-      <c r="E10" s="3">
-        <v>0</v>
-      </c>
-      <c r="F10" s="3">
-        <v>1</v>
-      </c>
-      <c r="G10" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="B11" s="3">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3">
+        <v>1</v>
+      </c>
+      <c r="D11" s="3">
+        <v>0</v>
+      </c>
+      <c r="E11" s="3">
+        <v>0</v>
+      </c>
+      <c r="F11" s="3">
+        <v>1</v>
+      </c>
+      <c r="G11" s="3">
+        <v>0</v>
+      </c>
+      <c r="H11" s="3">
+        <v>1</v>
+      </c>
+      <c r="I11" s="3">
+        <v>1</v>
+      </c>
+      <c r="J11" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="3">
-        <v>0</v>
-      </c>
-      <c r="C11" s="3">
-        <v>0</v>
-      </c>
-      <c r="D11" s="3">
-        <v>0</v>
-      </c>
-      <c r="E11" s="3">
-        <v>0</v>
-      </c>
-      <c r="F11" s="3">
-        <v>0</v>
-      </c>
-      <c r="G11" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="B12" s="3">
+        <v>0</v>
+      </c>
+      <c r="C12" s="3">
+        <v>0</v>
+      </c>
+      <c r="D12" s="3">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3">
+        <v>0</v>
+      </c>
+      <c r="F12" s="3">
+        <v>0</v>
+      </c>
+      <c r="G12" s="3">
+        <v>0</v>
+      </c>
+      <c r="H12" s="3">
+        <v>0</v>
+      </c>
+      <c r="I12" s="3">
+        <v>0</v>
+      </c>
+      <c r="J12" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="3">
-        <v>0</v>
-      </c>
-      <c r="C12" s="3">
-        <v>0</v>
-      </c>
-      <c r="D12" s="3">
-        <v>1</v>
-      </c>
-      <c r="E12" s="3">
-        <v>0</v>
-      </c>
-      <c r="F12" s="3">
-        <v>0</v>
-      </c>
-      <c r="G12" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="B13" s="3">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3">
+        <v>0</v>
+      </c>
+      <c r="D13" s="3">
+        <v>1</v>
+      </c>
+      <c r="E13" s="3">
+        <v>0</v>
+      </c>
+      <c r="F13" s="3">
+        <v>0</v>
+      </c>
+      <c r="G13" s="3">
+        <v>1</v>
+      </c>
+      <c r="H13" s="3">
+        <v>0</v>
+      </c>
+      <c r="I13" s="3">
+        <v>0</v>
+      </c>
+      <c r="J13" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="3">
-        <v>1</v>
-      </c>
-      <c r="C14" s="3">
-        <v>1</v>
-      </c>
-      <c r="D14" s="3">
-        <v>1</v>
-      </c>
-      <c r="E14" s="3">
-        <v>1</v>
-      </c>
-      <c r="F14" s="3">
-        <v>1</v>
-      </c>
-      <c r="G14" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="B15" s="3">
+        <v>1</v>
+      </c>
+      <c r="C15" s="3">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3">
+        <v>1</v>
+      </c>
+      <c r="E15" s="3">
+        <v>1</v>
+      </c>
+      <c r="F15" s="3">
+        <v>1</v>
+      </c>
+      <c r="G15" s="3">
+        <v>1</v>
+      </c>
+      <c r="H15" s="3">
+        <v>1</v>
+      </c>
+      <c r="I15" s="3">
+        <v>1</v>
+      </c>
+      <c r="J15" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="3">
-        <v>0</v>
-      </c>
-      <c r="C16" s="3">
-        <v>0</v>
-      </c>
-      <c r="D16" s="3">
-        <v>0</v>
-      </c>
-      <c r="E16" s="3">
-        <v>0</v>
-      </c>
-      <c r="F16" s="3">
-        <v>0</v>
-      </c>
-      <c r="G16" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="B17" s="3">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3">
+        <v>0</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3">
+        <v>0</v>
+      </c>
+      <c r="F17" s="3">
+        <v>0</v>
+      </c>
+      <c r="G17" s="3">
+        <v>0</v>
+      </c>
+      <c r="H17" s="3">
+        <v>0</v>
+      </c>
+      <c r="I17" s="3">
+        <v>0</v>
+      </c>
+      <c r="J17" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="1"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>48</v>
-      </c>
-      <c r="B18" s="3">
-        <v>-11748713.5580501</v>
-      </c>
-      <c r="C18" s="3">
-        <v>-11748713.5580501</v>
-      </c>
-      <c r="D18" s="3">
-        <v>-11747043.401719</v>
-      </c>
-      <c r="E18" s="3">
-        <v>-11124177.386580201</v>
-      </c>
-      <c r="F18" s="3">
-        <v>-11124177.386580201</v>
-      </c>
-      <c r="G18" s="3">
-        <v>-10722897.898614399</v>
-      </c>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
-      <c r="M18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="B19" s="3">
-        <v>4.9998760223388602E-3</v>
+        <v>-11748713.5580501</v>
       </c>
       <c r="C19" s="3">
-        <v>7.0002079010009696E-3</v>
+        <v>-11748713.5580501</v>
       </c>
       <c r="D19" s="3">
-        <v>5.0001144409179601E-3</v>
+        <v>-11747043.401719</v>
       </c>
       <c r="E19" s="3">
-        <v>3.9999485015869097E-3</v>
+        <v>-11124177.386580201</v>
       </c>
       <c r="F19" s="3">
-        <v>0</v>
+        <v>-11124177.386580201</v>
       </c>
       <c r="G19" s="3">
-        <v>2.6999950408935498E-2</v>
+        <v>-10722897.898614399</v>
+      </c>
+      <c r="H19" s="3">
+        <v>-503511503.88285297</v>
+      </c>
+      <c r="I19" s="3">
+        <v>-2573028.8945680601</v>
+      </c>
+      <c r="J19" s="3">
+        <v>-10626251.394568</v>
       </c>
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
@@ -3007,25 +3150,34 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="B20" s="3">
-        <v>0</v>
+        <v>4.9998760223388602E-3</v>
       </c>
       <c r="C20" s="3">
-        <v>0</v>
+        <v>7.0002079010009696E-3</v>
       </c>
       <c r="D20" s="3">
-        <v>0</v>
+        <v>5.0001144409179601E-3</v>
       </c>
       <c r="E20" s="3">
-        <v>0</v>
+        <v>3.9999485015869097E-3</v>
       </c>
       <c r="F20" s="3">
         <v>0</v>
       </c>
       <c r="G20" s="3">
-        <v>1.7370725403173299E-16</v>
+        <v>2.6999950408935498E-2</v>
+      </c>
+      <c r="H20" s="3">
+        <v>0.53500008583068803</v>
+      </c>
+      <c r="I20" s="3">
+        <v>7.9998970031738195E-3</v>
+      </c>
+      <c r="J20" s="3">
+        <v>2.000093460083E-3</v>
       </c>
       <c r="K20" s="3"/>
       <c r="L20" s="3"/>
@@ -3033,7 +3185,7 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="B21" s="3">
         <v>0</v>
@@ -3051,6 +3203,15 @@
         <v>0</v>
       </c>
       <c r="G21" s="3">
+        <v>1.7370725403173299E-16</v>
+      </c>
+      <c r="H21" s="3">
+        <v>0</v>
+      </c>
+      <c r="I21" s="3">
+        <v>0</v>
+      </c>
+      <c r="J21" s="3">
         <v>0</v>
       </c>
       <c r="K21" s="3"/>
@@ -3059,13 +3220,13 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="B22" s="3">
-        <v>0.27173913043478198</v>
+        <v>0</v>
       </c>
       <c r="C22" s="3">
-        <v>0.27173913043478198</v>
+        <v>0</v>
       </c>
       <c r="D22" s="3">
         <v>0</v>
@@ -3077,6 +3238,15 @@
         <v>0</v>
       </c>
       <c r="G22" s="3">
+        <v>0</v>
+      </c>
+      <c r="H22" s="3">
+        <v>0</v>
+      </c>
+      <c r="I22" s="3">
+        <v>0</v>
+      </c>
+      <c r="J22" s="3">
         <v>0</v>
       </c>
       <c r="K22" s="3"/>
@@ -3084,66 +3254,87 @@
       <c r="M22" s="3"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
+      <c r="A23" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" s="3">
+        <v>0.27173913043478198</v>
+      </c>
+      <c r="C23" s="3">
+        <v>0.27173913043478198</v>
+      </c>
+      <c r="D23" s="3">
+        <v>0</v>
+      </c>
+      <c r="E23" s="3">
+        <v>0</v>
+      </c>
+      <c r="F23" s="3">
+        <v>0</v>
+      </c>
+      <c r="G23" s="3">
+        <v>0</v>
+      </c>
+      <c r="H23" s="3">
+        <v>0.27173913043478198</v>
+      </c>
+      <c r="I23" s="3">
+        <v>0</v>
+      </c>
+      <c r="J23" s="3">
+        <v>0</v>
+      </c>
       <c r="K23" s="3"/>
       <c r="L23" s="3"/>
       <c r="M23" s="3"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>2</v>
-      </c>
-      <c r="B24" s="3">
-        <v>0</v>
-      </c>
-      <c r="C24" s="3">
-        <v>0</v>
-      </c>
-      <c r="D24" s="3">
-        <v>0</v>
-      </c>
-      <c r="E24" s="3">
-        <v>12.92135</v>
-      </c>
-      <c r="F24" s="3">
-        <v>12.92135</v>
-      </c>
-      <c r="G24" s="3">
-        <v>12.92135</v>
-      </c>
+      <c r="A24" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
       <c r="K24" s="3"/>
       <c r="L24" s="3"/>
       <c r="M24" s="3"/>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B25" s="3">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="C25" s="3">
-        <v>59.025551892380903</v>
+        <v>0</v>
       </c>
       <c r="D25" s="3">
-        <v>62.454999999999998</v>
+        <v>0</v>
       </c>
       <c r="E25" s="3">
-        <v>36</v>
+        <v>12.92135</v>
       </c>
       <c r="F25" s="3">
-        <v>36</v>
+        <v>12.92135</v>
       </c>
       <c r="G25" s="3">
-        <v>36</v>
+        <v>12.92135</v>
+      </c>
+      <c r="H25" s="3">
+        <v>12.920999999999999</v>
+      </c>
+      <c r="I25" s="3">
+        <v>12.920999999999999</v>
+      </c>
+      <c r="J25" s="3">
+        <v>12.920999999999999</v>
       </c>
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
@@ -3151,91 +3342,121 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B26" s="3">
-        <v>6</v>
+        <v>74</v>
       </c>
       <c r="C26" s="3">
-        <v>6</v>
+        <v>59.025551892380903</v>
       </c>
       <c r="D26" s="3">
-        <v>0</v>
+        <v>62.454999999999998</v>
       </c>
       <c r="E26" s="3">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="F26" s="3">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="G26" s="3">
-        <v>2.3815138030285001</v>
+        <v>36</v>
+      </c>
+      <c r="H26" s="3">
+        <v>36</v>
+      </c>
+      <c r="I26" s="3">
+        <v>36</v>
+      </c>
+      <c r="J26" s="3">
+        <v>36</v>
       </c>
       <c r="K26" s="3"/>
       <c r="L26" s="3"/>
       <c r="M26" s="3"/>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
+      <c r="A27" t="s">
+        <v>1</v>
+      </c>
+      <c r="B27" s="3">
+        <v>6</v>
+      </c>
+      <c r="C27" s="3">
+        <v>6</v>
+      </c>
+      <c r="D27" s="3">
+        <v>0</v>
+      </c>
+      <c r="E27" s="3">
+        <v>6</v>
+      </c>
+      <c r="F27" s="3">
+        <v>6</v>
+      </c>
+      <c r="G27" s="3">
+        <v>2.3815138030285001</v>
+      </c>
+      <c r="H27" s="3">
+        <v>6</v>
+      </c>
+      <c r="I27" s="3">
+        <v>6</v>
+      </c>
+      <c r="J27" s="3">
+        <v>6</v>
+      </c>
       <c r="K27" s="3"/>
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>0</v>
-      </c>
-      <c r="B28" s="3">
-        <v>38.363688734486203</v>
-      </c>
-      <c r="C28" s="3">
-        <v>0</v>
-      </c>
-      <c r="D28" s="3">
-        <v>0</v>
-      </c>
-      <c r="E28" s="3">
-        <v>0</v>
-      </c>
-      <c r="F28" s="3">
-        <v>0</v>
-      </c>
-      <c r="G28" s="3">
-        <v>0</v>
-      </c>
+      <c r="A28" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
       <c r="M28" s="3"/>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="B29" s="3">
-        <v>62.454999999999998</v>
+        <v>38.363688734486203</v>
       </c>
       <c r="C29" s="3">
-        <v>62.454999999999998</v>
+        <v>0</v>
       </c>
       <c r="D29" s="3">
-        <v>62.454999999999998</v>
+        <v>0</v>
       </c>
       <c r="E29" s="3">
-        <v>54.921349999999997</v>
+        <v>0</v>
       </c>
       <c r="F29" s="3">
-        <v>54.921349999999997</v>
+        <v>0</v>
       </c>
       <c r="G29" s="3">
-        <v>51.302863803028501</v>
+        <v>0</v>
+      </c>
+      <c r="H29" s="3">
+        <v>0</v>
+      </c>
+      <c r="I29" s="3">
+        <v>0</v>
+      </c>
+      <c r="J29" s="3">
+        <v>0</v>
       </c>
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
@@ -3243,91 +3464,121 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="B30" s="3">
-        <v>6</v>
+        <v>62.454999999999998</v>
       </c>
       <c r="C30" s="3">
-        <v>6</v>
+        <v>62.454999999999998</v>
       </c>
       <c r="D30" s="3">
-        <v>0</v>
+        <v>62.454999999999998</v>
       </c>
       <c r="E30" s="3">
-        <v>6</v>
+        <v>54.921349999999997</v>
       </c>
       <c r="F30" s="3">
-        <v>6</v>
+        <v>54.921349999999997</v>
       </c>
       <c r="G30" s="3">
-        <v>0.93789926080202601</v>
+        <v>51.302863803028501</v>
+      </c>
+      <c r="H30" s="3">
+        <v>54.920999999999999</v>
+      </c>
+      <c r="I30" s="3">
+        <v>54.920999999999999</v>
+      </c>
+      <c r="J30" s="3">
+        <v>54.920999999999999</v>
       </c>
       <c r="K30" s="3"/>
       <c r="L30" s="3"/>
       <c r="M30" s="3"/>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A31" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
-      <c r="G31" s="3"/>
+      <c r="A31" t="s">
+        <v>1</v>
+      </c>
+      <c r="B31" s="3">
+        <v>6</v>
+      </c>
+      <c r="C31" s="3">
+        <v>6</v>
+      </c>
+      <c r="D31" s="3">
+        <v>0</v>
+      </c>
+      <c r="E31" s="3">
+        <v>6</v>
+      </c>
+      <c r="F31" s="3">
+        <v>6</v>
+      </c>
+      <c r="G31" s="3">
+        <v>0.93789926080202601</v>
+      </c>
+      <c r="H31" s="3">
+        <v>6</v>
+      </c>
+      <c r="I31" s="3">
+        <v>6</v>
+      </c>
+      <c r="J31" s="3">
+        <v>6</v>
+      </c>
       <c r="K31" s="3"/>
       <c r="L31" s="3"/>
       <c r="M31" s="3"/>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>2</v>
-      </c>
-      <c r="B32" s="3">
-        <v>0</v>
-      </c>
-      <c r="C32" s="3">
-        <v>0</v>
-      </c>
-      <c r="D32" s="3">
-        <v>0</v>
-      </c>
-      <c r="E32" s="3">
-        <v>269.15315180360801</v>
-      </c>
-      <c r="F32" s="3">
-        <v>269.15315180360801</v>
-      </c>
-      <c r="G32" s="3">
-        <v>219.96891611468601</v>
-      </c>
+      <c r="A32" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="3"/>
       <c r="K32" s="3"/>
       <c r="L32" s="3"/>
       <c r="M32" s="3"/>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B33" s="3">
-        <v>1448.3702360141299</v>
+        <v>0</v>
       </c>
       <c r="C33" s="3">
-        <v>1190.09916106232</v>
+        <v>0</v>
       </c>
       <c r="D33" s="3">
-        <v>1181.1636480188399</v>
+        <v>0</v>
       </c>
       <c r="E33" s="3">
-        <v>864</v>
+        <v>269.15315180360801</v>
       </c>
       <c r="F33" s="3">
-        <v>864</v>
+        <v>269.15315180360801</v>
       </c>
       <c r="G33" s="3">
-        <v>864</v>
+        <v>219.96891611468601</v>
+      </c>
+      <c r="H33" s="3">
+        <v>3098.5730090737102</v>
+      </c>
+      <c r="I33" s="3">
+        <v>216.39643667296701</v>
+      </c>
+      <c r="J33" s="3">
+        <v>216.39643667296701</v>
       </c>
       <c r="K33" s="3"/>
       <c r="L33" s="3"/>
@@ -3335,91 +3586,121 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B34" s="3">
-        <v>49.238399999999999</v>
+        <v>1448.3702360141299</v>
       </c>
       <c r="C34" s="3">
-        <v>49.238399999999999</v>
+        <v>1190.09916106232</v>
       </c>
       <c r="D34" s="3">
-        <v>0</v>
+        <v>1181.1636480188399</v>
       </c>
       <c r="E34" s="3">
-        <v>44.011050890132303</v>
+        <v>864</v>
       </c>
       <c r="F34" s="3">
-        <v>44.011050890132303</v>
+        <v>864</v>
       </c>
       <c r="G34" s="3">
-        <v>2.3815138030285001</v>
+        <v>864</v>
+      </c>
+      <c r="H34" s="3">
+        <v>204910.501150094</v>
+      </c>
+      <c r="I34" s="3">
+        <v>864</v>
+      </c>
+      <c r="J34" s="3">
+        <v>864</v>
       </c>
       <c r="K34" s="3"/>
       <c r="L34" s="3"/>
       <c r="M34" s="3"/>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
-      <c r="F35" s="3"/>
-      <c r="G35" s="3"/>
+      <c r="A35" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35" s="3">
+        <v>49.238399999999999</v>
+      </c>
+      <c r="C35" s="3">
+        <v>49.238399999999999</v>
+      </c>
+      <c r="D35" s="3">
+        <v>0</v>
+      </c>
+      <c r="E35" s="3">
+        <v>44.011050890132303</v>
+      </c>
+      <c r="F35" s="3">
+        <v>44.011050890132303</v>
+      </c>
+      <c r="G35" s="3">
+        <v>2.3815138030285001</v>
+      </c>
+      <c r="H35" s="3">
+        <v>16205.8221999999</v>
+      </c>
+      <c r="I35" s="3">
+        <v>36.552999999999997</v>
+      </c>
+      <c r="J35" s="3">
+        <v>36.552999999999997</v>
+      </c>
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
       <c r="M35" s="3"/>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>0</v>
-      </c>
-      <c r="B36" s="3">
-        <v>258.27107495181002</v>
-      </c>
-      <c r="C36" s="3">
-        <v>0</v>
-      </c>
-      <c r="D36" s="3">
-        <v>0</v>
-      </c>
-      <c r="E36" s="3">
-        <v>0</v>
-      </c>
-      <c r="F36" s="3">
-        <v>0</v>
-      </c>
-      <c r="G36" s="3">
-        <v>0</v>
-      </c>
+      <c r="A36" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
+      <c r="J36" s="3"/>
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
       <c r="M36" s="3"/>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="B37" s="3">
-        <v>1181.1636480188399</v>
+        <v>258.27107495181002</v>
       </c>
       <c r="C37" s="3">
-        <v>1181.1636480188399</v>
+        <v>0</v>
       </c>
       <c r="D37" s="3">
-        <v>1181.1636480188399</v>
+        <v>0</v>
       </c>
       <c r="E37" s="3">
-        <v>1125.1662692224099</v>
+        <v>0</v>
       </c>
       <c r="F37" s="3">
-        <v>1125.1662692224099</v>
+        <v>0</v>
       </c>
       <c r="G37" s="3">
-        <v>1083.5367321353001</v>
+        <v>0</v>
+      </c>
+      <c r="H37" s="3">
+        <v>0</v>
+      </c>
+      <c r="I37" s="3">
+        <v>0</v>
+      </c>
+      <c r="J37" s="3">
+        <v>0</v>
       </c>
       <c r="K37" s="3"/>
       <c r="L37" s="3"/>
@@ -3427,119 +3708,156 @@
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="B38" s="3">
-        <v>58.173913043478201</v>
+        <v>1181.1636480188399</v>
       </c>
       <c r="C38" s="3">
-        <v>58.173913043478201</v>
+        <v>1181.1636480188399</v>
       </c>
       <c r="D38" s="3">
-        <v>0</v>
+        <v>1181.1636480188399</v>
       </c>
       <c r="E38" s="3">
-        <v>51.997933471328302</v>
+        <v>1125.1662692224099</v>
       </c>
       <c r="F38" s="3">
-        <v>51.997933471328302</v>
+        <v>1125.1662692224099</v>
       </c>
       <c r="G38" s="3">
-        <v>2.8136977824060798</v>
-      </c>
-      <c r="H38" s="3"/>
+        <v>1083.5367321353001</v>
+      </c>
+      <c r="H38" s="3">
+        <v>205068.13099999999</v>
+      </c>
+      <c r="I38" s="3">
+        <v>1073.7629999999999</v>
+      </c>
+      <c r="J38" s="3">
+        <v>1073.7629999999999</v>
+      </c>
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
       <c r="M38" s="3"/>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="B39" s="3">
-        <v>0</v>
+        <v>58.173913043478201</v>
       </c>
       <c r="C39" s="3">
-        <v>0</v>
+        <v>58.173913043478201</v>
       </c>
       <c r="D39" s="3">
         <v>0</v>
       </c>
       <c r="E39" s="3">
-        <v>55.997378796433999</v>
+        <v>51.997933471328302</v>
       </c>
       <c r="F39" s="3">
-        <v>55.997378796433999</v>
+        <v>51.997933471328302</v>
       </c>
       <c r="G39" s="3">
-        <v>97.626915883537805</v>
-      </c>
-      <c r="H39" s="5"/>
+        <v>2.8136977824060798</v>
+      </c>
+      <c r="H39" s="3">
+        <v>19146.765359168199</v>
+      </c>
+      <c r="I39" s="3">
+        <v>43.186436672967801</v>
+      </c>
+      <c r="J39" s="3">
+        <v>43.186436672967801</v>
+      </c>
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
       <c r="M39" s="3"/>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
-      <c r="D40" s="3"/>
-      <c r="E40" s="3"/>
-      <c r="F40" s="3"/>
-      <c r="G40" s="3"/>
+      <c r="A40" t="s">
+        <v>35</v>
+      </c>
+      <c r="B40" s="3">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3">
+        <v>0</v>
+      </c>
+      <c r="D40" s="3">
+        <v>0</v>
+      </c>
+      <c r="E40" s="3">
+        <v>55.997378796433999</v>
+      </c>
+      <c r="F40" s="3">
+        <v>55.997378796433999</v>
+      </c>
+      <c r="G40" s="3">
+        <v>97.626915883537805</v>
+      </c>
+      <c r="H40" s="3">
+        <v>8.8689999999999998</v>
+      </c>
+      <c r="I40" s="3">
+        <v>4.2370000000000001</v>
+      </c>
+      <c r="J40" s="3">
+        <v>4.2370000000000001</v>
+      </c>
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
       <c r="M40" s="3"/>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>2</v>
-      </c>
-      <c r="B41" s="3">
-        <v>0</v>
-      </c>
-      <c r="C41" s="3">
-        <v>0</v>
-      </c>
-      <c r="D41" s="3">
-        <v>0</v>
-      </c>
-      <c r="E41" s="3">
-        <v>82172.105643843504</v>
-      </c>
-      <c r="F41" s="3">
-        <v>82172.105643843504</v>
-      </c>
-      <c r="G41" s="3">
-        <v>67156.222738668395</v>
-      </c>
+      <c r="A41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B41" s="3"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="3"/>
+      <c r="E41" s="3"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="3"/>
+      <c r="I41" s="3"/>
+      <c r="J41" s="3"/>
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
       <c r="M41" s="3"/>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B42" s="3">
-        <v>78665.906333971507</v>
+        <v>0</v>
       </c>
       <c r="C42" s="3">
-        <v>62922.922138276503</v>
+        <v>0</v>
       </c>
       <c r="D42" s="3">
-        <v>64593.078469406901</v>
+        <v>0</v>
       </c>
       <c r="E42" s="3">
-        <v>45313.2</v>
+        <v>82172.105643843504</v>
       </c>
       <c r="F42" s="3">
-        <v>45313.2</v>
+        <v>82172.105643843504</v>
       </c>
       <c r="G42" s="3">
-        <v>45313.2</v>
+        <v>67156.222738668395</v>
+      </c>
+      <c r="H42" s="3">
+        <v>945990.291923285</v>
+      </c>
+      <c r="I42" s="3">
+        <v>66065.549431934996</v>
+      </c>
+      <c r="J42" s="3">
+        <v>66065.549431934996</v>
       </c>
       <c r="K42" s="3"/>
       <c r="L42" s="3"/>
@@ -3547,113 +3865,1103 @@
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B43" s="3">
-        <v>0</v>
+        <v>78665.906333971507</v>
       </c>
       <c r="C43" s="3">
-        <v>0</v>
+        <v>62922.922138276503</v>
       </c>
       <c r="D43" s="3">
-        <v>0</v>
+        <v>64593.078469406901</v>
       </c>
       <c r="E43" s="3">
-        <v>0</v>
+        <v>45313.2</v>
       </c>
       <c r="F43" s="3">
-        <v>0</v>
+        <v>45313.2</v>
       </c>
       <c r="G43" s="3">
-        <v>0</v>
-      </c>
+        <v>45313.2</v>
+      </c>
+      <c r="H43" s="3">
+        <v>8212833.3252236303</v>
+      </c>
+      <c r="I43" s="3">
+        <v>45313.055999999997</v>
+      </c>
+      <c r="J43" s="3">
+        <v>45313.055999999997</v>
+      </c>
+      <c r="K43" s="3"/>
+      <c r="L43" s="3"/>
+      <c r="M43" s="3"/>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A44" s="2" t="s">
+      <c r="A44" t="s">
+        <v>1</v>
+      </c>
+      <c r="B44" s="3">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3">
+        <v>0</v>
+      </c>
+      <c r="D44" s="3">
+        <v>0</v>
+      </c>
+      <c r="E44" s="3">
+        <v>0</v>
+      </c>
+      <c r="F44" s="3">
+        <v>0</v>
+      </c>
+      <c r="G44" s="3">
+        <v>0</v>
+      </c>
+      <c r="H44" s="3">
+        <v>0</v>
+      </c>
+      <c r="I44" s="3">
+        <v>0</v>
+      </c>
+      <c r="J44" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B44" s="3"/>
-      <c r="C44" s="3"/>
-      <c r="D44" s="3"/>
-      <c r="E44" s="3"/>
-      <c r="F44" s="3"/>
-      <c r="G44" s="3"/>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>0</v>
-      </c>
-      <c r="B45" s="3">
-        <v>15742.984195695</v>
-      </c>
-      <c r="C45" s="3">
-        <v>0</v>
-      </c>
-      <c r="D45" s="3">
-        <v>0</v>
-      </c>
-      <c r="E45" s="3">
-        <v>0</v>
-      </c>
-      <c r="F45" s="3">
-        <v>0</v>
-      </c>
-      <c r="G45" s="3">
-        <v>0</v>
-      </c>
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="B46" s="3">
-        <v>11811636.4801884</v>
+        <v>15742.984195695</v>
       </c>
       <c r="C46" s="3">
-        <v>11811636.4801884</v>
+        <v>0</v>
       </c>
       <c r="D46" s="3">
-        <v>11811636.4801884</v>
+        <v>0</v>
       </c>
       <c r="E46" s="3">
-        <v>11251662.6922241</v>
+        <v>0</v>
       </c>
       <c r="F46" s="3">
-        <v>11251662.6922241</v>
+        <v>0</v>
       </c>
       <c r="G46" s="3">
-        <v>10835367.321353</v>
+        <v>0</v>
+      </c>
+      <c r="H46" s="3">
+        <v>0</v>
+      </c>
+      <c r="I46" s="3">
+        <v>0</v>
+      </c>
+      <c r="J46" s="3">
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="B47" s="3">
-        <v>0</v>
+        <v>11811636.4801884</v>
       </c>
       <c r="C47" s="3">
-        <v>0</v>
+        <v>11811636.4801884</v>
       </c>
       <c r="D47" s="3">
-        <v>0</v>
+        <v>11811636.4801884</v>
       </c>
       <c r="E47" s="3">
-        <v>0</v>
+        <v>11251662.6922241</v>
       </c>
       <c r="F47" s="3">
-        <v>0</v>
+        <v>11251662.6922241</v>
       </c>
       <c r="G47" s="3">
-        <v>0</v>
+        <v>10835367.321353</v>
+      </c>
+      <c r="H47" s="3">
+        <v>512670327.5</v>
+      </c>
+      <c r="I47" s="3">
+        <v>2684407.5</v>
+      </c>
+      <c r="J47" s="3">
+        <v>10737630</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="D48" s="3"/>
+      <c r="A48" t="s">
+        <v>1</v>
+      </c>
+      <c r="B48" s="3">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3">
+        <v>0</v>
+      </c>
+      <c r="D48" s="3">
+        <v>0</v>
+      </c>
+      <c r="E48" s="3">
+        <v>0</v>
+      </c>
+      <c r="F48" s="3">
+        <v>0</v>
+      </c>
+      <c r="G48" s="3">
+        <v>0</v>
+      </c>
+      <c r="H48" s="3">
+        <v>0</v>
+      </c>
+      <c r="I48" s="3">
+        <v>0</v>
+      </c>
+      <c r="J48" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D49" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4F0EF5-9E64-45A3-AF76-8FD0E53934FE}">
+  <dimension ref="A1:G53"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" customWidth="1"/>
+    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="16" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" s="4">
+        <v>6624</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="4">
+        <v>10000</v>
+      </c>
+      <c r="C4" s="4">
+        <v>2500</v>
+      </c>
+      <c r="D4" s="4">
+        <v>2500</v>
+      </c>
+      <c r="E4" s="4">
+        <v>2500</v>
+      </c>
+      <c r="F4" s="4">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="4">
+        <v>24</v>
+      </c>
+      <c r="C5" s="4">
+        <v>24</v>
+      </c>
+      <c r="D5" s="4">
+        <v>8783</v>
+      </c>
+      <c r="E5" s="4">
+        <v>8783</v>
+      </c>
+      <c r="F5" s="4">
+        <v>8783</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4">
+        <v>66</v>
+      </c>
+      <c r="E6" s="4">
+        <v>66</v>
+      </c>
+      <c r="F6" s="9">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="4">
+        <v>12.920999999999999</v>
+      </c>
+      <c r="C8" s="4">
+        <v>12.920999999999999</v>
+      </c>
+      <c r="D8" s="4">
+        <v>12.920999999999999</v>
+      </c>
+      <c r="E8" s="4">
+        <v>12.920999999999999</v>
+      </c>
+      <c r="F8" s="4">
+        <v>12.920999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" s="4">
+        <v>36</v>
+      </c>
+      <c r="C9" s="4">
+        <v>36</v>
+      </c>
+      <c r="D9" s="4">
+        <v>36</v>
+      </c>
+      <c r="E9" s="4">
+        <v>36</v>
+      </c>
+      <c r="F9" s="4">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="4">
+        <v>6</v>
+      </c>
+      <c r="C10" s="4">
+        <v>6</v>
+      </c>
+      <c r="D10" s="4">
+        <v>6</v>
+      </c>
+      <c r="E10" s="4">
+        <v>6</v>
+      </c>
+      <c r="F10" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="4">
+        <v>0</v>
+      </c>
+      <c r="C12" s="4">
+        <v>0</v>
+      </c>
+      <c r="D12" s="4">
+        <v>0</v>
+      </c>
+      <c r="E12" s="4">
+        <v>0</v>
+      </c>
+      <c r="F12" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="4">
+        <v>1</v>
+      </c>
+      <c r="C13" s="4">
+        <v>1</v>
+      </c>
+      <c r="D13" s="4">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4">
+        <v>1</v>
+      </c>
+      <c r="F13" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" s="4">
+        <v>0</v>
+      </c>
+      <c r="C14" s="4">
+        <v>0</v>
+      </c>
+      <c r="D14" s="4">
+        <v>0</v>
+      </c>
+      <c r="E14" s="4">
+        <v>0</v>
+      </c>
+      <c r="F14" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" s="4">
+        <v>0</v>
+      </c>
+      <c r="C15" s="4">
+        <v>0</v>
+      </c>
+      <c r="D15" s="4">
+        <v>0</v>
+      </c>
+      <c r="E15" s="4">
+        <v>0</v>
+      </c>
+      <c r="F15" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="4">
+        <v>1</v>
+      </c>
+      <c r="C17" s="4">
+        <v>1</v>
+      </c>
+      <c r="D17" s="4">
+        <v>1</v>
+      </c>
+      <c r="E17" s="4">
+        <v>1</v>
+      </c>
+      <c r="F17" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="4">
+        <v>0</v>
+      </c>
+      <c r="C19" s="4">
+        <v>0</v>
+      </c>
+      <c r="D19" s="4">
+        <v>0</v>
+      </c>
+      <c r="E19" s="4">
+        <v>0</v>
+      </c>
+      <c r="F19" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" s="4">
+        <v>-10626251.394568</v>
+      </c>
+      <c r="C21" s="4">
+        <v>-2573028.8945680601</v>
+      </c>
+      <c r="D21" s="4">
+        <v>-503511503.88285297</v>
+      </c>
+      <c r="E21" s="4">
+        <v>-503428701.306997</v>
+      </c>
+      <c r="F21" s="4">
+        <v>-503145897.59350002</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>54</v>
+      </c>
+      <c r="B22" s="4">
+        <v>153748.605431934</v>
+      </c>
+      <c r="C22" s="4">
+        <v>121971.105431934</v>
+      </c>
+      <c r="D22" s="9">
+        <v>9180996.1171469297</v>
+      </c>
+      <c r="E22" s="9">
+        <v>9263798.6930023599</v>
+      </c>
+      <c r="F22" s="9">
+        <v>9546602.4064993802</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="4">
+        <v>4.0001869201660104E-3</v>
+      </c>
+      <c r="C23" s="4">
+        <v>0</v>
+      </c>
+      <c r="D23" s="4">
+        <v>0.480999946594238</v>
+      </c>
+      <c r="E23" s="4">
+        <v>0.56500005722045898</v>
+      </c>
+      <c r="F23" s="4">
+        <v>0.26200008392333901</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" s="4">
+        <v>0</v>
+      </c>
+      <c r="C24" s="4">
+        <v>0</v>
+      </c>
+      <c r="D24" s="4">
+        <v>0</v>
+      </c>
+      <c r="E24" s="4">
+        <v>0</v>
+      </c>
+      <c r="F24" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" s="4">
+        <v>0</v>
+      </c>
+      <c r="C25" s="4">
+        <v>0</v>
+      </c>
+      <c r="D25" s="4">
+        <v>0</v>
+      </c>
+      <c r="E25" s="4">
+        <v>0</v>
+      </c>
+      <c r="F25" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26" s="4">
+        <v>0</v>
+      </c>
+      <c r="C26" s="4">
+        <v>0</v>
+      </c>
+      <c r="D26" s="4">
+        <v>0.27173913043478198</v>
+      </c>
+      <c r="E26" s="4">
+        <v>0.89913043478260801</v>
+      </c>
+      <c r="F26" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>56</v>
+      </c>
+      <c r="D27" s="1">
+        <v>366</v>
+      </c>
+      <c r="E27" s="1">
+        <v>301</v>
+      </c>
+      <c r="F27" s="9">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>59</v>
+      </c>
+      <c r="D28" s="1">
+        <v>366</v>
+      </c>
+      <c r="E28" s="1">
+        <v>306</v>
+      </c>
+      <c r="F28" s="9">
+        <v>76</v>
+      </c>
+      <c r="G28" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>2</v>
+      </c>
+      <c r="B30" s="4">
+        <v>12.920999999999999</v>
+      </c>
+      <c r="C30" s="4">
+        <v>12.920999999999999</v>
+      </c>
+      <c r="D30" s="4">
+        <v>12.920999999999999</v>
+      </c>
+      <c r="E30" s="4">
+        <v>12.920999999999999</v>
+      </c>
+      <c r="F30" s="4">
+        <v>12.920999999999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>0</v>
+      </c>
+      <c r="B31" s="4">
+        <v>36</v>
+      </c>
+      <c r="C31" s="4">
+        <v>36</v>
+      </c>
+      <c r="D31" s="4">
+        <v>36</v>
+      </c>
+      <c r="E31" s="4">
+        <v>36</v>
+      </c>
+      <c r="F31" s="4">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>1</v>
+      </c>
+      <c r="B32" s="4">
+        <v>6</v>
+      </c>
+      <c r="C32" s="4">
+        <v>6</v>
+      </c>
+      <c r="D32" s="4">
+        <v>6</v>
+      </c>
+      <c r="E32" s="4">
+        <v>6</v>
+      </c>
+      <c r="F32" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>0</v>
+      </c>
+      <c r="B34" s="4">
+        <v>0</v>
+      </c>
+      <c r="C34" s="4">
+        <v>0</v>
+      </c>
+      <c r="D34" s="4">
+        <v>0</v>
+      </c>
+      <c r="E34" s="4">
+        <v>0</v>
+      </c>
+      <c r="F34" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>24</v>
+      </c>
+      <c r="B35" s="4">
+        <v>54.920999999999999</v>
+      </c>
+      <c r="C35" s="4">
+        <v>54.920999999999999</v>
+      </c>
+      <c r="D35" s="4">
+        <v>54.920999999999999</v>
+      </c>
+      <c r="E35" s="4">
+        <v>54.920999999999999</v>
+      </c>
+      <c r="F35" s="4">
+        <v>54.920999999999999</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>1</v>
+      </c>
+      <c r="B36" s="4">
+        <v>6</v>
+      </c>
+      <c r="C36" s="4">
+        <v>6</v>
+      </c>
+      <c r="D36" s="4">
+        <v>6</v>
+      </c>
+      <c r="E36" s="4">
+        <v>6</v>
+      </c>
+      <c r="F36" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>2</v>
+      </c>
+      <c r="B38" s="4">
+        <v>216.39643667296701</v>
+      </c>
+      <c r="C38" s="4">
+        <v>216.39643667296701</v>
+      </c>
+      <c r="D38" s="4">
+        <v>3098.5730090737102</v>
+      </c>
+      <c r="E38" s="4">
+        <v>3098.5730090737102</v>
+      </c>
+      <c r="F38" s="4">
+        <v>3000.0191999999902</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>0</v>
+      </c>
+      <c r="B39" s="4">
+        <v>864</v>
+      </c>
+      <c r="C39" s="4">
+        <v>864</v>
+      </c>
+      <c r="D39" s="4">
+        <v>204910.501150094</v>
+      </c>
+      <c r="E39" s="4">
+        <v>203171.64494744799</v>
+      </c>
+      <c r="F39" s="4">
+        <v>202367.83931946999</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>1</v>
+      </c>
+      <c r="B40" s="4">
+        <v>36.552999999999997</v>
+      </c>
+      <c r="C40" s="4">
+        <v>36.552999999999997</v>
+      </c>
+      <c r="D40" s="9">
+        <v>16205.8221999999</v>
+      </c>
+      <c r="E40" s="9">
+        <v>6623.99999999989</v>
+      </c>
+      <c r="F40" s="9">
+        <v>1685.0463999999899</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>0</v>
+      </c>
+      <c r="B42" s="4">
+        <v>0</v>
+      </c>
+      <c r="C42" s="4">
+        <v>0</v>
+      </c>
+      <c r="D42" s="4">
+        <v>0</v>
+      </c>
+      <c r="E42" s="4">
+        <v>0</v>
+      </c>
+      <c r="F42" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>24</v>
+      </c>
+      <c r="B43" s="4">
+        <v>1073.7629999999999</v>
+      </c>
+      <c r="C43" s="4">
+        <v>1073.7629999999999</v>
+      </c>
+      <c r="D43" s="4">
+        <v>205068.13099999999</v>
+      </c>
+      <c r="E43" s="4">
+        <v>205068.13099999999</v>
+      </c>
+      <c r="F43" s="4">
+        <v>205050.0656</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>1</v>
+      </c>
+      <c r="B44" s="4">
+        <v>43.186436672967801</v>
+      </c>
+      <c r="C44" s="4">
+        <v>43.186436672967801</v>
+      </c>
+      <c r="D44" s="4">
+        <v>19146.765359168199</v>
+      </c>
+      <c r="E44" s="4">
+        <v>7826.0869565215899</v>
+      </c>
+      <c r="F44" s="4">
+        <v>2002.83931947069</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>35</v>
+      </c>
+      <c r="B45" s="4">
+        <v>4.2370000000000001</v>
+      </c>
+      <c r="C45" s="4">
+        <v>4.2370000000000001</v>
+      </c>
+      <c r="D45" s="4">
+        <v>8.8689999999999998</v>
+      </c>
+      <c r="E45" s="4">
+        <v>8.8689999999999998</v>
+      </c>
+      <c r="F45" s="4">
+        <v>26.9344</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B46" s="4"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>2</v>
+      </c>
+      <c r="B47" s="4">
+        <v>66065.549431934996</v>
+      </c>
+      <c r="C47" s="4">
+        <v>66065.549431934996</v>
+      </c>
+      <c r="D47" s="4">
+        <v>945990.291923285</v>
+      </c>
+      <c r="E47" s="4">
+        <v>945990.291923285</v>
+      </c>
+      <c r="F47" s="4">
+        <v>915901.94275649404</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>0</v>
+      </c>
+      <c r="B48" s="4">
+        <v>45313.055999999997</v>
+      </c>
+      <c r="C48" s="4">
+        <v>45313.055999999997</v>
+      </c>
+      <c r="D48" s="4">
+        <v>8212833.3252236303</v>
+      </c>
+      <c r="E48" s="4">
+        <v>8295635.9010790698</v>
+      </c>
+      <c r="F48" s="4">
+        <v>8563364.4637428895</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>1</v>
+      </c>
+      <c r="B49" s="4">
+        <v>0</v>
+      </c>
+      <c r="C49" s="4">
+        <v>0</v>
+      </c>
+      <c r="D49" s="4">
+        <v>0</v>
+      </c>
+      <c r="E49" s="4">
+        <v>0</v>
+      </c>
+      <c r="F49" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>0</v>
+      </c>
+      <c r="B51" s="4">
+        <v>0</v>
+      </c>
+      <c r="C51" s="4">
+        <v>0</v>
+      </c>
+      <c r="D51" s="4">
+        <v>0</v>
+      </c>
+      <c r="E51" s="4">
+        <v>0</v>
+      </c>
+      <c r="F51" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>24</v>
+      </c>
+      <c r="B52" s="4">
+        <v>10737630</v>
+      </c>
+      <c r="C52" s="4">
+        <v>2684407.5</v>
+      </c>
+      <c r="D52" s="4">
+        <v>512670327.5</v>
+      </c>
+      <c r="E52" s="4">
+        <v>512670327.5</v>
+      </c>
+      <c r="F52" s="4">
+        <v>512625164</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>1</v>
+      </c>
+      <c r="B53" s="4">
+        <v>0</v>
+      </c>
+      <c r="C53" s="4">
+        <v>0</v>
+      </c>
+      <c r="D53" s="4">
+        <v>0</v>
+      </c>
+      <c r="E53" s="4">
+        <v>0</v>
+      </c>
+      <c r="F53" s="4">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
update planning results and todo
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\Desktop\ongoing_projects\MVS\dev\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7876657-09CB-4059-89FA-04F7BCACAE98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E3FFFD-BAA2-43F0-A054-F6740B8FA97C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28815" yWindow="-8910" windowWidth="14310" windowHeight="15585" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Experiments" sheetId="1" r:id="rId1"/>
-    <sheet name="20250425" sheetId="3" r:id="rId2"/>
-    <sheet name="20250424" sheetId="2" r:id="rId3"/>
-    <sheet name="20250505_Ops" sheetId="4" r:id="rId4"/>
-    <sheet name="250601_ops" sheetId="5" r:id="rId5"/>
+    <sheet name="250616_plan" sheetId="6" r:id="rId2"/>
+    <sheet name="20250425" sheetId="3" r:id="rId3"/>
+    <sheet name="20250424" sheetId="2" r:id="rId4"/>
+    <sheet name="20250505_Ops" sheetId="4" r:id="rId5"/>
+    <sheet name="250601_ops" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -58,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="90">
   <si>
     <t>Grid</t>
   </si>
@@ -244,6 +245,90 @@
   </si>
   <si>
     <t>Contingencies</t>
+  </si>
+  <si>
+    <t>Maximum battery supply (cycles/yr)</t>
+  </si>
+  <si>
+    <t>Mean value of lost load in 2025 ($/MWh)</t>
+  </si>
+  <si>
+    <t>Available resources</t>
+  </si>
+  <si>
+    <t>Discount rate (-)</t>
+  </si>
+  <si>
+    <t>Solve time (s)</t>
+  </si>
+  <si>
+    <t>Objective (Surplus in $)</t>
+  </si>
+  <si>
+    <t>Max. storage supply  cycles base case (-)</t>
+  </si>
+  <si>
+    <t>Max. storage supply  cycles contingency (-)</t>
+  </si>
+  <si>
+    <t>Avg. storage supply  cycles base case (-)</t>
+  </si>
+  <si>
+    <t>Avg. storage supply  cycles contingency (-)</t>
+  </si>
+  <si>
+    <t>Total operating cost -- base case ($)</t>
+  </si>
+  <si>
+    <t>Total operating cost -- contingency ($)</t>
+  </si>
+  <si>
+    <t>Total cost of lost load -- contingency ($)</t>
+  </si>
+  <si>
+    <t>Total cost of lost load -- base case ($)</t>
+  </si>
+  <si>
+    <t>Total depreceated capital cost ($)</t>
+  </si>
+  <si>
+    <t>Terminal capacity (MW)</t>
+  </si>
+  <si>
+    <t>Total investment (M$)</t>
+  </si>
+  <si>
+    <t>Unmet load</t>
+  </si>
+  <si>
+    <t>--- Base case operations</t>
+  </si>
+  <si>
+    <t>--- Contingency operations</t>
+  </si>
+  <si>
+    <t>["b", "g", "s"]</t>
+  </si>
+  <si>
+    <t>peak_shaving</t>
+  </si>
+  <si>
+    <t>Max optimality gap (%)</t>
+  </si>
+  <si>
+    <t>Mean contingency probability (%)</t>
+  </si>
+  <si>
+    <t>Mean base case probability (%)</t>
+  </si>
+  <si>
+    <t>Complementarity violations (-)</t>
+  </si>
+  <si>
+    <t>NaN</t>
+  </si>
+  <si>
+    <t>full</t>
   </si>
 </sst>
 </file>
@@ -254,7 +339,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -285,13 +370,37 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -303,11 +412,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -315,12 +426,19 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="5" fillId="3" borderId="0" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="43" fontId="4" fillId="2" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="4">
+    <cellStyle name="Bad" xfId="3" builtinId="27"/>
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Good" xfId="2" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1048,6 +1166,1610 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEB77188-4C54-4D05-A0BB-AB8E292CE16E}">
+  <dimension ref="A1:F90"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="6" width="18" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" s="3">
+        <v>150</v>
+      </c>
+      <c r="C3" s="3">
+        <v>0</v>
+      </c>
+      <c r="D3" s="3">
+        <v>366</v>
+      </c>
+      <c r="E3" s="3">
+        <v>150</v>
+      </c>
+      <c r="F3" s="3">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" s="3">
+        <v>2500</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2500</v>
+      </c>
+      <c r="D4" s="3">
+        <v>2500</v>
+      </c>
+      <c r="E4" s="3">
+        <v>2500</v>
+      </c>
+      <c r="F4" s="3">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="3">
+        <v>8783</v>
+      </c>
+      <c r="C5" s="3">
+        <v>8783</v>
+      </c>
+      <c r="D5" s="3">
+        <v>8783</v>
+      </c>
+      <c r="E5" s="3">
+        <v>8783</v>
+      </c>
+      <c r="F5" s="3">
+        <v>8783</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="C6" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="E6" s="3">
+        <v>20</v>
+      </c>
+      <c r="F6" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" s="3">
+        <v>1</v>
+      </c>
+      <c r="C7" s="3">
+        <v>1</v>
+      </c>
+      <c r="D7" s="3">
+        <v>1</v>
+      </c>
+      <c r="E7" s="3">
+        <v>100</v>
+      </c>
+      <c r="F7" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" s="3">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3">
+        <v>0</v>
+      </c>
+      <c r="D10" s="3">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3">
+        <v>0</v>
+      </c>
+      <c r="F10" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" s="3">
+        <v>19914533339.040901</v>
+      </c>
+      <c r="C12" s="3">
+        <v>19809841481.080101</v>
+      </c>
+      <c r="D12" s="3">
+        <v>19914698719.838902</v>
+      </c>
+      <c r="E12" s="3">
+        <v>21802857320.342499</v>
+      </c>
+      <c r="F12" s="3">
+        <v>21810624237.791698</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" s="3">
+        <v>15341.212288856501</v>
+      </c>
+      <c r="C13" s="3">
+        <v>700.15005302429199</v>
+      </c>
+      <c r="D13" s="3">
+        <v>30195.948692083301</v>
+      </c>
+      <c r="E13" s="3">
+        <v>6552.0655179023697</v>
+      </c>
+      <c r="F13" s="3">
+        <v>9986.4023299217206</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B14" s="3">
+        <v>5.0159819466078997E-5</v>
+      </c>
+      <c r="C14" s="3">
+        <v>9.89790503088415E-5</v>
+      </c>
+      <c r="D14" s="3">
+        <v>5.75063834460946E-5</v>
+      </c>
+      <c r="E14" s="3">
+        <v>5.1153643556451998E-3</v>
+      </c>
+      <c r="F14" s="3">
+        <v>6.7193071307100902E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>87</v>
+      </c>
+      <c r="B15" s="3">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3">
+        <v>0</v>
+      </c>
+      <c r="D15" s="3">
+        <v>0</v>
+      </c>
+      <c r="E15" s="3">
+        <v>0</v>
+      </c>
+      <c r="F15" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" s="3">
+        <v>60.420364466636798</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D16" s="3">
+        <v>60.453825953486898</v>
+      </c>
+      <c r="E16" s="3">
+        <v>136.32216282309801</v>
+      </c>
+      <c r="F16" s="3">
+        <v>249.106177578238</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>68</v>
+      </c>
+      <c r="B17" s="3">
+        <v>117.511996639882</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D17" s="3">
+        <v>121.52741218059001</v>
+      </c>
+      <c r="E17" s="3">
+        <v>150.00000000000301</v>
+      </c>
+      <c r="F17" s="3">
+        <v>366.000000000017</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" s="3">
+        <v>75.955726389845793</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D18" s="3">
+        <v>77.744130515221698</v>
+      </c>
+      <c r="E18" s="3">
+        <v>127.609476445046</v>
+      </c>
+      <c r="F18" s="3">
+        <v>212.36105235593601</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>69</v>
+      </c>
+      <c r="B19" s="3">
+        <v>149.99999999999699</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D19" s="3">
+        <v>152.83528225048701</v>
+      </c>
+      <c r="E19" s="3">
+        <v>150</v>
+      </c>
+      <c r="F19" s="3">
+        <v>366.00000000001398</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>72</v>
+      </c>
+      <c r="B20" s="3">
+        <v>2276815636.0092702</v>
+      </c>
+      <c r="C20" s="3">
+        <v>2256215991.8481898</v>
+      </c>
+      <c r="D20" s="3">
+        <v>2277144130.8397799</v>
+      </c>
+      <c r="E20" s="3">
+        <v>695164386.753407</v>
+      </c>
+      <c r="F20" s="3">
+        <v>688058509.35971904</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>73</v>
+      </c>
+      <c r="B21" s="3">
+        <v>2314736549.2487898</v>
+      </c>
+      <c r="C21" s="3">
+        <v>2281123150.7440901</v>
+      </c>
+      <c r="D21" s="3">
+        <v>2313654764.43961</v>
+      </c>
+      <c r="E21" s="3">
+        <v>1558489537.16799</v>
+      </c>
+      <c r="F21" s="3">
+        <v>1546565315.5455699</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>75</v>
+      </c>
+      <c r="B22" s="3">
+        <v>16882345.0438595</v>
+      </c>
+      <c r="C22" s="3">
+        <v>41060829.7149124</v>
+      </c>
+      <c r="D22" s="3">
+        <v>15874476.1923769</v>
+      </c>
+      <c r="E22" s="3">
+        <v>2344171.40350876</v>
+      </c>
+      <c r="F22" s="3">
+        <v>2520216.1403508801</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>74</v>
+      </c>
+      <c r="B23" s="3">
+        <v>53005356.477268197</v>
+      </c>
+      <c r="C23" s="3">
+        <v>143139719.29824501</v>
+      </c>
+      <c r="D23" s="3">
+        <v>62065398.029189803</v>
+      </c>
+      <c r="E23" s="3">
+        <v>50075728.700554296</v>
+      </c>
+      <c r="F23" s="3">
+        <v>66086422.465755902</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>76</v>
+      </c>
+      <c r="B24" s="3">
+        <v>375804542.65472698</v>
+      </c>
+      <c r="C24" s="3">
+        <v>465613367.24283397</v>
+      </c>
+      <c r="D24" s="3">
+        <v>374722884.53010398</v>
+      </c>
+      <c r="E24" s="3">
+        <v>235505312.222462</v>
+      </c>
+      <c r="F24" s="3">
+        <v>233850933.002204</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>2</v>
+      </c>
+      <c r="B26" s="3">
+        <v>53.3439298245614</v>
+      </c>
+      <c r="C26" s="3">
+        <v>84.317824561403498</v>
+      </c>
+      <c r="D26" s="3">
+        <v>53.3439298245614</v>
+      </c>
+      <c r="E26" s="3">
+        <v>53.3439298245614</v>
+      </c>
+      <c r="F26" s="3">
+        <v>54.917894736842101</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>0</v>
+      </c>
+      <c r="B27" s="11">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3">
+        <v>0</v>
+      </c>
+      <c r="D27" s="3">
+        <v>0</v>
+      </c>
+      <c r="E27" s="3">
+        <v>0</v>
+      </c>
+      <c r="F27" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>1</v>
+      </c>
+      <c r="B28" s="3">
+        <v>32.769017543859597</v>
+      </c>
+      <c r="C28" s="3">
+        <v>0</v>
+      </c>
+      <c r="D28" s="3">
+        <v>32.694666666666599</v>
+      </c>
+      <c r="E28" s="3">
+        <v>34.4154385964912</v>
+      </c>
+      <c r="F28" s="3">
+        <v>33.104912280701697</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>2</v>
+      </c>
+      <c r="B30" s="3">
+        <v>73.744847937405396</v>
+      </c>
+      <c r="C30" s="3">
+        <v>128.32412368421001</v>
+      </c>
+      <c r="D30" s="3">
+        <v>74.336303590696502</v>
+      </c>
+      <c r="E30" s="3">
+        <v>53.3439298245614</v>
+      </c>
+      <c r="F30" s="3">
+        <v>54.917894736842101</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>0</v>
+      </c>
+      <c r="B31" s="11">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3">
+        <v>0</v>
+      </c>
+      <c r="D31" s="3">
+        <v>0</v>
+      </c>
+      <c r="E31" s="3">
+        <v>0</v>
+      </c>
+      <c r="F31" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>1</v>
+      </c>
+      <c r="B32" s="3">
+        <v>52.207959957331397</v>
+      </c>
+      <c r="C32" s="3">
+        <v>0</v>
+      </c>
+      <c r="D32" s="3">
+        <v>52.213951928716703</v>
+      </c>
+      <c r="E32" s="3">
+        <v>34.4154385964912</v>
+      </c>
+      <c r="F32" s="3">
+        <v>33.104912280701697</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>2</v>
+      </c>
+      <c r="B34" s="3">
+        <v>257202585.734635</v>
+      </c>
+      <c r="C34" s="3">
+        <v>465613367.24283397</v>
+      </c>
+      <c r="D34" s="3">
+        <v>256538397.61669999</v>
+      </c>
+      <c r="E34" s="3">
+        <v>158079603.55687699</v>
+      </c>
+      <c r="F34" s="3">
+        <v>158108334.629866</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>0</v>
+      </c>
+      <c r="B35" s="11">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3">
+        <v>0</v>
+      </c>
+      <c r="D35" s="3">
+        <v>0</v>
+      </c>
+      <c r="E35" s="3">
+        <v>0</v>
+      </c>
+      <c r="F35" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>1</v>
+      </c>
+      <c r="B36" s="3">
+        <v>118601956.920092</v>
+      </c>
+      <c r="C36" s="3">
+        <v>0</v>
+      </c>
+      <c r="D36" s="3">
+        <v>118184486.913404</v>
+      </c>
+      <c r="E36" s="3">
+        <v>77425708.665584803</v>
+      </c>
+      <c r="F36" s="14">
+        <v>75742598.372338593</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>2</v>
+      </c>
+      <c r="B39" s="3">
+        <v>53.3439298245614</v>
+      </c>
+      <c r="C39" s="3">
+        <v>84.317824561403498</v>
+      </c>
+      <c r="D39" s="3">
+        <v>54.168491228070103</v>
+      </c>
+      <c r="E39" s="3">
+        <v>53.3439298245614</v>
+      </c>
+      <c r="F39" s="3">
+        <v>54.917894736842101</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>0</v>
+      </c>
+      <c r="B40" s="11">
+        <v>38</v>
+      </c>
+      <c r="C40" s="3">
+        <v>38</v>
+      </c>
+      <c r="D40" s="3">
+        <v>38</v>
+      </c>
+      <c r="E40" s="3">
+        <v>74</v>
+      </c>
+      <c r="F40" s="13">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>1</v>
+      </c>
+      <c r="B41" s="3">
+        <v>32.769017543859597</v>
+      </c>
+      <c r="C41" s="3">
+        <v>0</v>
+      </c>
+      <c r="D41" s="3">
+        <v>34.694666666666599</v>
+      </c>
+      <c r="E41" s="3">
+        <v>34.4154385964912</v>
+      </c>
+      <c r="F41" s="3">
+        <v>33.104912280701697</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>79</v>
+      </c>
+      <c r="B42" s="3">
+        <v>13.0106842105263</v>
+      </c>
+      <c r="C42" s="3">
+        <v>19.725350877193002</v>
+      </c>
+      <c r="D42" s="3">
+        <v>12.68270432582</v>
+      </c>
+      <c r="E42" s="3">
+        <v>12.026631578947301</v>
+      </c>
+      <c r="F42" s="3">
+        <v>12.721192982456101</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B43" s="3"/>
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>0</v>
+      </c>
+      <c r="B44" s="11">
+        <v>32.533356835617603</v>
+      </c>
+      <c r="C44" s="3">
+        <v>34.577473684210503</v>
+      </c>
+      <c r="D44" s="3">
+        <v>31.9702956741795</v>
+      </c>
+      <c r="E44" s="3">
+        <v>38</v>
+      </c>
+      <c r="F44" s="3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>24</v>
+      </c>
+      <c r="B45" s="3">
+        <v>95.02</v>
+      </c>
+      <c r="C45" s="3">
+        <v>95.02</v>
+      </c>
+      <c r="D45" s="3">
+        <v>95.02</v>
+      </c>
+      <c r="E45" s="3">
+        <v>95.02</v>
+      </c>
+      <c r="F45" s="13">
+        <v>95.02</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>1</v>
+      </c>
+      <c r="B46" s="3">
+        <v>32.694666666666599</v>
+      </c>
+      <c r="C46" s="3">
+        <v>0</v>
+      </c>
+      <c r="D46" s="3">
+        <v>32.694666666666599</v>
+      </c>
+      <c r="E46" s="3">
+        <v>34.4154385964912</v>
+      </c>
+      <c r="F46" s="3">
+        <v>33.104912280701697</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B47" s="3"/>
+      <c r="C47" s="3"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>2</v>
+      </c>
+      <c r="B48" s="3">
+        <v>7403403.0786220701</v>
+      </c>
+      <c r="C48" s="3">
+        <v>7335264.4874104904</v>
+      </c>
+      <c r="D48" s="3">
+        <v>7404304.3690989399</v>
+      </c>
+      <c r="E48" s="3">
+        <v>1509732.8352443599</v>
+      </c>
+      <c r="F48" s="3">
+        <v>1510482.5054732601</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>0</v>
+      </c>
+      <c r="B49" s="3">
+        <v>337164.63573730801</v>
+      </c>
+      <c r="C49" s="3">
+        <v>336761.958438578</v>
+      </c>
+      <c r="D49" s="3">
+        <v>336872.86486429803</v>
+      </c>
+      <c r="E49" s="3">
+        <v>6278182.9098127401</v>
+      </c>
+      <c r="F49" s="13">
+        <v>6336354.5687585501</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>1</v>
+      </c>
+      <c r="B50" s="12">
+        <v>324696.16976015997</v>
+      </c>
+      <c r="C50" s="3">
+        <v>0</v>
+      </c>
+      <c r="D50" s="3">
+        <v>327715.63633730198</v>
+      </c>
+      <c r="E50" s="3">
+        <v>559330.96795197902</v>
+      </c>
+      <c r="F50" s="3">
+        <v>881256.44645368401</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>35</v>
+      </c>
+      <c r="B51" s="3">
+        <v>6752.93801754385</v>
+      </c>
+      <c r="C51" s="3">
+        <v>16424.331885964901</v>
+      </c>
+      <c r="D51" s="3">
+        <v>6349.7904769507604</v>
+      </c>
+      <c r="E51" s="3">
+        <v>937.66856140350899</v>
+      </c>
+      <c r="F51" s="3">
+        <v>1008.08645614035</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B52" s="3"/>
+      <c r="C52" s="3"/>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>0</v>
+      </c>
+      <c r="B53" s="3">
+        <v>2535.1691318804301</v>
+      </c>
+      <c r="C53" s="3">
+        <v>2589.3631017543798</v>
+      </c>
+      <c r="D53" s="3">
+        <v>2193.5850658356599</v>
+      </c>
+      <c r="E53" s="3">
+        <v>1487.7023433096799</v>
+      </c>
+      <c r="F53" s="3">
+        <v>2058.1905548631398</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>24</v>
+      </c>
+      <c r="B54" s="3">
+        <v>7679108.4766157903</v>
+      </c>
+      <c r="C54" s="3">
+        <v>7669437.0827471996</v>
+      </c>
+      <c r="D54" s="3">
+        <v>7679511.6241560802</v>
+      </c>
+      <c r="E54" s="3">
+        <v>7684923.7460718304</v>
+      </c>
+      <c r="F54" s="3">
+        <v>7684853.3281770796</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>1</v>
+      </c>
+      <c r="B55" s="12">
+        <v>383620.23837449402</v>
+      </c>
+      <c r="C55" s="3">
+        <v>0</v>
+      </c>
+      <c r="D55" s="3">
+        <v>387187.66107901599</v>
+      </c>
+      <c r="E55" s="3">
+        <v>660835.264593623</v>
+      </c>
+      <c r="F55" s="3">
+        <v>1041182.00195373</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B56" s="3"/>
+      <c r="C56" s="3"/>
+      <c r="D56" s="3"/>
+      <c r="E56" s="3"/>
+      <c r="F56" s="3"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>2</v>
+      </c>
+      <c r="B57" s="3">
+        <v>2260249288.6444201</v>
+      </c>
+      <c r="C57" s="3">
+        <v>2239446665.75877</v>
+      </c>
+      <c r="D57" s="3">
+        <v>2260524451.4497299</v>
+      </c>
+      <c r="E57" s="3">
+        <v>460919462.39662403</v>
+      </c>
+      <c r="F57" s="3">
+        <v>461148335.73813999</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>0</v>
+      </c>
+      <c r="B58" s="3">
+        <v>18371882.370204199</v>
+      </c>
+      <c r="C58" s="3">
+        <v>18146873.031422999</v>
+      </c>
+      <c r="D58" s="3">
+        <v>18289531.5125539</v>
+      </c>
+      <c r="E58" s="3">
+        <v>234763710.57674</v>
+      </c>
+      <c r="F58" s="3">
+        <v>227413103.07681701</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>1</v>
+      </c>
+      <c r="B59" s="3">
+        <v>0</v>
+      </c>
+      <c r="C59" s="3">
+        <v>0</v>
+      </c>
+      <c r="D59" s="3">
+        <v>0</v>
+      </c>
+      <c r="E59" s="3">
+        <v>0</v>
+      </c>
+      <c r="F59" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B60" s="3"/>
+      <c r="C60" s="3"/>
+      <c r="D60" s="3"/>
+      <c r="E60" s="3"/>
+      <c r="F60" s="3"/>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>0</v>
+      </c>
+      <c r="B61" s="3">
+        <v>1805535.0043492101</v>
+      </c>
+      <c r="C61" s="3">
+        <v>1377546.9412949099</v>
+      </c>
+      <c r="D61" s="3">
+        <v>1669852.12173551</v>
+      </c>
+      <c r="E61" s="3">
+        <v>518786.21999804798</v>
+      </c>
+      <c r="F61" s="3">
+        <v>502929.45532035403</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>24</v>
+      </c>
+      <c r="B62" s="3">
+        <v>19197771191.536098</v>
+      </c>
+      <c r="C62" s="3">
+        <v>19173592706.863701</v>
+      </c>
+      <c r="D62" s="3">
+        <v>19198779060.3866</v>
+      </c>
+      <c r="E62" s="3">
+        <v>19212309365.176102</v>
+      </c>
+      <c r="F62" s="3">
+        <v>19212133320.439201</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>1</v>
+      </c>
+      <c r="B63" s="3">
+        <v>0</v>
+      </c>
+      <c r="C63" s="3">
+        <v>0</v>
+      </c>
+      <c r="D63" s="3">
+        <v>0</v>
+      </c>
+      <c r="E63" s="3">
+        <v>0</v>
+      </c>
+      <c r="F63" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B64" s="3"/>
+      <c r="C64" s="3"/>
+      <c r="D64" s="3"/>
+      <c r="E64" s="3"/>
+      <c r="F64" s="3"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B65" s="3"/>
+      <c r="C65" s="3"/>
+      <c r="D65" s="3"/>
+      <c r="E65" s="3"/>
+      <c r="F65" s="3"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>2</v>
+      </c>
+      <c r="B66" s="3">
+        <v>53.3439298245614</v>
+      </c>
+      <c r="C66" s="3">
+        <v>84.317824561403498</v>
+      </c>
+      <c r="D66" s="3">
+        <v>54.168491228070103</v>
+      </c>
+      <c r="E66" s="3">
+        <v>53.3439298245614</v>
+      </c>
+      <c r="F66" s="3">
+        <v>54.917894736842101</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B67" s="12">
+        <v>36</v>
+      </c>
+      <c r="C67" s="3">
+        <v>36</v>
+      </c>
+      <c r="D67" s="3">
+        <v>36</v>
+      </c>
+      <c r="E67" s="3">
+        <v>36</v>
+      </c>
+      <c r="F67" s="3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>1</v>
+      </c>
+      <c r="B68" s="3">
+        <v>32.769017543859597</v>
+      </c>
+      <c r="C68" s="3">
+        <v>0</v>
+      </c>
+      <c r="D68" s="3">
+        <v>34.694666666666599</v>
+      </c>
+      <c r="E68" s="3">
+        <v>34.4154385964912</v>
+      </c>
+      <c r="F68" s="3">
+        <v>33.104912280701697</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>79</v>
+      </c>
+      <c r="B69" s="3">
+        <v>26.4866431643824</v>
+      </c>
+      <c r="C69" s="3">
+        <v>34.1799122807017</v>
+      </c>
+      <c r="D69" s="3">
+        <v>26.349473684210501</v>
+      </c>
+      <c r="E69" s="3">
+        <v>23.117388576681101</v>
+      </c>
+      <c r="F69" s="3">
+        <v>24.891352674537298</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B70" s="3"/>
+      <c r="C70" s="3"/>
+      <c r="D70" s="3"/>
+      <c r="E70" s="3"/>
+      <c r="F70" s="3"/>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>0</v>
+      </c>
+      <c r="B71" s="3">
+        <v>31.918315789471698</v>
+      </c>
+      <c r="C71" s="3">
+        <v>34.577473684210503</v>
+      </c>
+      <c r="D71" s="3">
+        <v>31.9702956741802</v>
+      </c>
+      <c r="E71" s="3">
+        <v>23.7619649122806</v>
+      </c>
+      <c r="F71" s="3">
+        <v>20.737122807017499</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>24</v>
+      </c>
+      <c r="B72" s="3">
+        <v>86.112947368421004</v>
+      </c>
+      <c r="C72" s="3">
+        <v>84.317824561403498</v>
+      </c>
+      <c r="D72" s="3">
+        <v>86.863157894736801</v>
+      </c>
+      <c r="E72" s="3">
+        <v>87.759368421052599</v>
+      </c>
+      <c r="F72" s="3">
+        <v>88.022807017543798</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>1</v>
+      </c>
+      <c r="B73" s="3">
+        <v>32.769017543859597</v>
+      </c>
+      <c r="C73" s="3">
+        <v>0</v>
+      </c>
+      <c r="D73" s="3">
+        <v>32.694666666666599</v>
+      </c>
+      <c r="E73" s="3">
+        <v>34.4154385964912</v>
+      </c>
+      <c r="F73" s="3">
+        <v>32.547859649122799</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B74" s="3"/>
+      <c r="C74" s="3"/>
+      <c r="D74" s="3"/>
+      <c r="E74" s="3"/>
+      <c r="F74" s="3"/>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>2</v>
+      </c>
+      <c r="B75" s="3">
+        <v>7551914.9355758801</v>
+      </c>
+      <c r="C75" s="3">
+        <v>7441851.4173080102</v>
+      </c>
+      <c r="D75" s="3">
+        <v>7548317.40107805</v>
+      </c>
+      <c r="E75" s="3">
+        <v>4709370.5991895003</v>
+      </c>
+      <c r="F75" s="3">
+        <v>4695316.8599934299</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>0</v>
+      </c>
+      <c r="B76" s="3">
+        <v>189951.98703510599</v>
+      </c>
+      <c r="C76" s="3">
+        <v>189757.69019297301</v>
+      </c>
+      <c r="D76" s="3">
+        <v>189951.03815598899</v>
+      </c>
+      <c r="E76" s="3">
+        <v>3049066.5912629198</v>
+      </c>
+      <c r="F76" s="3">
+        <v>3092471.8310868102</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>1</v>
+      </c>
+      <c r="B77" s="3">
+        <v>411819.21304413403</v>
+      </c>
+      <c r="C77" s="3">
+        <v>0</v>
+      </c>
+      <c r="D77" s="3">
+        <v>412166.738262809</v>
+      </c>
+      <c r="E77" s="3">
+        <v>507733.34651742602</v>
+      </c>
+      <c r="F77" s="3">
+        <v>704228.27824355895</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>35</v>
+      </c>
+      <c r="B78" s="3">
+        <v>21202.142590907199</v>
+      </c>
+      <c r="C78" s="3">
+        <v>57255.887719298596</v>
+      </c>
+      <c r="D78" s="3">
+        <v>24826.1592116758</v>
+      </c>
+      <c r="E78" s="3">
+        <v>20030.2914802216</v>
+      </c>
+      <c r="F78" s="3">
+        <v>26434.568986302202</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B79" s="3"/>
+      <c r="C79" s="3"/>
+      <c r="D79" s="3"/>
+      <c r="E79" s="3"/>
+      <c r="F79" s="3"/>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>0</v>
+      </c>
+      <c r="B80" s="3">
+        <v>2472.9729662621198</v>
+      </c>
+      <c r="C80" s="3">
+        <v>3003.5805877192902</v>
+      </c>
+      <c r="D80" s="3">
+        <v>2435.4392505638398</v>
+      </c>
+      <c r="E80" s="3">
+        <v>465.42218602278001</v>
+      </c>
+      <c r="F80" s="3">
+        <v>562.38473322931497</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>24</v>
+      </c>
+      <c r="B81" s="3">
+        <v>7664659.2720423704</v>
+      </c>
+      <c r="C81" s="3">
+        <v>7628605.5269133803</v>
+      </c>
+      <c r="D81" s="3">
+        <v>7661035.2554214699</v>
+      </c>
+      <c r="E81" s="3">
+        <v>7665831.1231528902</v>
+      </c>
+      <c r="F81" s="3">
+        <v>7659426.8456469998</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>1</v>
+      </c>
+      <c r="B82" s="3">
+        <v>486553.890647683</v>
+      </c>
+      <c r="C82" s="3">
+        <v>0</v>
+      </c>
+      <c r="D82" s="3">
+        <v>486964.48282476899</v>
+      </c>
+      <c r="E82" s="3">
+        <v>599873.99163205398</v>
+      </c>
+      <c r="F82" s="3">
+        <v>832027.73894551501</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B83" s="3"/>
+      <c r="C83" s="3"/>
+      <c r="D83" s="3"/>
+      <c r="E83" s="3"/>
+      <c r="F83" s="3"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>2</v>
+      </c>
+      <c r="B84" s="3">
+        <v>2305589764.5666699</v>
+      </c>
+      <c r="C84" s="3">
+        <v>2271987516.2199101</v>
+      </c>
+      <c r="D84" s="3">
+        <v>2304491441.9846501</v>
+      </c>
+      <c r="E84" s="3">
+        <v>1437764691.9583001</v>
+      </c>
+      <c r="F84" s="3">
+        <v>1433474103.7413399</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>0</v>
+      </c>
+      <c r="B85" s="3">
+        <v>11084614.929826399</v>
+      </c>
+      <c r="C85" s="3">
+        <v>10906171.4334148</v>
+      </c>
+      <c r="D85" s="3">
+        <v>11086811.791450201</v>
+      </c>
+      <c r="E85" s="3">
+        <v>120960970.15776899</v>
+      </c>
+      <c r="F85" s="3">
+        <v>113312298.149334</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>1</v>
+      </c>
+      <c r="B86" s="3">
+        <v>0</v>
+      </c>
+      <c r="C86" s="3">
+        <v>0</v>
+      </c>
+      <c r="D86" s="3">
+        <v>0</v>
+      </c>
+      <c r="E86" s="3">
+        <v>0</v>
+      </c>
+      <c r="F86" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B87" s="3"/>
+      <c r="C87" s="3"/>
+      <c r="D87" s="3"/>
+      <c r="E87" s="3"/>
+      <c r="F87" s="3"/>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B88" s="3">
+        <v>1937830.24850617</v>
+      </c>
+      <c r="C88" s="3">
+        <v>1770536.9079175801</v>
+      </c>
+      <c r="D88" s="3">
+        <v>1923489.33599052</v>
+      </c>
+      <c r="E88" s="3">
+        <v>236124.94824217999</v>
+      </c>
+      <c r="F88" s="3">
+        <v>221086.345003836</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>24</v>
+      </c>
+      <c r="B89" s="3">
+        <v>19161648180.101898</v>
+      </c>
+      <c r="C89" s="3">
+        <v>19071513817.2785</v>
+      </c>
+      <c r="D89" s="3">
+        <v>19152588138.550098</v>
+      </c>
+      <c r="E89" s="3">
+        <v>19164577807.8797</v>
+      </c>
+      <c r="F89" s="3">
+        <v>19148567114.1133</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>1</v>
+      </c>
+      <c r="B90" s="3">
+        <v>0</v>
+      </c>
+      <c r="C90" s="3">
+        <v>0</v>
+      </c>
+      <c r="D90" s="3">
+        <v>0</v>
+      </c>
+      <c r="E90" s="3">
+        <v>0</v>
+      </c>
+      <c r="F90" s="3">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00CD46BB-A2D1-4791-8AAC-69869F785713}">
   <dimension ref="A1:M52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2075,7 +3797,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4317E227-4F2F-4766-80E7-4A0C11DC1BA8}">
   <dimension ref="A1:J48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2705,7 +4427,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CDE5EF9-418E-4572-AF84-E6DEF6E71829}">
   <dimension ref="A1:M49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2734,7 +4456,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" t="s">
         <v>52</v>
       </c>
       <c r="E3" t="s">
@@ -2751,7 +4473,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" t="s">
         <v>51</v>
       </c>
       <c r="H4" t="s">
@@ -2830,7 +4552,7 @@
       <c r="I7" s="3">
         <v>36</v>
       </c>
-      <c r="J7" s="8">
+      <c r="J7" s="7">
         <v>36</v>
       </c>
     </row>
@@ -2862,7 +4584,7 @@
       <c r="I8" s="3">
         <v>6</v>
       </c>
-      <c r="J8" s="8">
+      <c r="J8" s="7">
         <v>6</v>
       </c>
     </row>
@@ -4050,7 +5772,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4F0EF5-9E64-45A3-AF76-8FD0E53934FE}">
   <dimension ref="A1:G53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4076,7 +5798,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" t="s">
         <v>55</v>
       </c>
       <c r="E3" s="4">
@@ -4084,7 +5806,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" t="s">
         <v>52</v>
       </c>
       <c r="B4" s="4">
@@ -4104,7 +5826,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" t="s">
         <v>57</v>
       </c>
       <c r="B5" s="4">
@@ -4124,7 +5846,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" t="s">
         <v>58</v>
       </c>
       <c r="B6" s="4"/>
@@ -4135,7 +5857,7 @@
       <c r="E6" s="4">
         <v>66</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="8">
         <v>66</v>
       </c>
     </row>
@@ -4399,13 +6121,13 @@
       <c r="C22" s="4">
         <v>121971.105431934</v>
       </c>
-      <c r="D22" s="9">
+      <c r="D22" s="8">
         <v>9180996.1171469297</v>
       </c>
-      <c r="E22" s="9">
+      <c r="E22" s="8">
         <v>9263798.6930023599</v>
       </c>
-      <c r="F22" s="9">
+      <c r="F22" s="8">
         <v>9546602.4064993802</v>
       </c>
     </row>
@@ -4499,7 +6221,7 @@
       <c r="E27" s="1">
         <v>301</v>
       </c>
-      <c r="F27" s="9">
+      <c r="F27" s="8">
         <v>66</v>
       </c>
     </row>
@@ -4513,7 +6235,7 @@
       <c r="E28" s="1">
         <v>306</v>
       </c>
-      <c r="F28" s="9">
+      <c r="F28" s="8">
         <v>76</v>
       </c>
       <c r="G28" t="s">
@@ -4720,13 +6442,13 @@
       <c r="C40" s="4">
         <v>36.552999999999997</v>
       </c>
-      <c r="D40" s="9">
+      <c r="D40" s="8">
         <v>16205.8221999999</v>
       </c>
-      <c r="E40" s="9">
+      <c r="E40" s="8">
         <v>6623.99999999989</v>
       </c>
-      <c r="F40" s="9">
+      <c r="F40" s="8">
         <v>1685.0463999999899</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update todos and results
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\Desktop\ongoing_projects\MVS\dev\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E3FFFD-BAA2-43F0-A054-F6740B8FA97C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED03EADD-B819-4D93-9AC8-393788651A76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28815" yWindow="-8910" windowWidth="14310" windowHeight="15585" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-16950" yWindow="-8910" windowWidth="17055" windowHeight="15585" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Experiments" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="91">
   <si>
     <t>Grid</t>
   </si>
@@ -329,6 +329,9 @@
   </si>
   <si>
     <t>full</t>
+  </si>
+  <si>
+    <t>updated sum in market constraint</t>
   </si>
 </sst>
 </file>
@@ -418,7 +421,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -428,7 +431,6 @@
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="43" fontId="5" fillId="3" borderId="0" xfId="3" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="4" fillId="2" borderId="0" xfId="2" applyNumberFormat="1"/>
@@ -1167,24 +1169,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEB77188-4C54-4D05-A0BB-AB8E292CE16E}">
-  <dimension ref="A1:F90"/>
+  <dimension ref="A1:I90"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="6" width="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="9" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1">
+        <v>250617</v>
+      </c>
+      <c r="I1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>62</v>
       </c>
@@ -1203,8 +1211,17 @@
       <c r="F3" s="3">
         <v>366</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="3">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3">
+        <v>0</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>63</v>
       </c>
@@ -1223,8 +1240,17 @@
       <c r="F4" s="3">
         <v>2500</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="3">
+        <v>2500</v>
+      </c>
+      <c r="H4" s="3">
+        <v>2500</v>
+      </c>
+      <c r="I4" s="3">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>57</v>
       </c>
@@ -1243,8 +1269,17 @@
       <c r="F5" s="3">
         <v>8783</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="3">
+        <v>8783</v>
+      </c>
+      <c r="H5" s="3">
+        <v>8783</v>
+      </c>
+      <c r="I5" s="3">
+        <v>8783</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>85</v>
       </c>
@@ -1263,8 +1298,17 @@
       <c r="F6" s="3">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="3">
+        <v>20</v>
+      </c>
+      <c r="H6" s="3">
+        <v>20</v>
+      </c>
+      <c r="I6" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>86</v>
       </c>
@@ -1283,9 +1327,18 @@
       <c r="F7" s="3">
         <v>100</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
+      <c r="G7" s="3">
+        <v>80</v>
+      </c>
+      <c r="H7" s="3">
+        <v>80</v>
+      </c>
+      <c r="I7" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>64</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -1303,9 +1356,18 @@
       <c r="F8" s="3" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
+      <c r="G8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="3" t="s">
@@ -1323,9 +1385,18 @@
       <c r="F9" s="3" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
+      <c r="G9" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>65</v>
       </c>
       <c r="B10" s="3">
@@ -1343,8 +1414,17 @@
       <c r="F10" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="3">
+        <v>0</v>
+      </c>
+      <c r="H10" s="3">
+        <v>0</v>
+      </c>
+      <c r="I10" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -1353,8 +1433,11 @@
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>67</v>
       </c>
@@ -1373,8 +1456,17 @@
       <c r="F12" s="3">
         <v>21810624237.791698</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="3">
+        <v>17975494486.410198</v>
+      </c>
+      <c r="H12" s="3">
+        <v>16426865420.537399</v>
+      </c>
+      <c r="I12" s="3">
+        <v>17974426085.787498</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>66</v>
       </c>
@@ -1393,19 +1485,28 @@
       <c r="F13" s="3">
         <v>9986.4023299217206</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="3">
+        <v>355.74099993705698</v>
+      </c>
+      <c r="H13" s="3">
+        <v>2013.36700010299</v>
+      </c>
+      <c r="I13" s="3">
+        <v>639.23342490196205</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>84</v>
       </c>
       <c r="B14" s="3">
-        <v>5.0159819466078997E-5</v>
+        <v>5.0159819466078998E-3</v>
       </c>
       <c r="C14" s="3">
-        <v>9.89790503088415E-5</v>
+        <v>9.8979050308841496E-3</v>
       </c>
       <c r="D14" s="3">
-        <v>5.75063834460946E-5</v>
+        <v>5.7506383446094596E-3</v>
       </c>
       <c r="E14" s="3">
         <v>5.1153643556451998E-3</v>
@@ -1413,8 +1514,17 @@
       <c r="F14" s="3">
         <v>6.7193071307100902E-3</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="3">
+        <v>7.0103128127448901E-4</v>
+      </c>
+      <c r="H14" s="3">
+        <v>3.0872638561538399E-3</v>
+      </c>
+      <c r="I14" s="3">
+        <v>7.9187216723792002E-4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>87</v>
       </c>
@@ -1433,8 +1543,17 @@
       <c r="F15" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="3">
+        <v>0</v>
+      </c>
+      <c r="H15" s="3">
+        <v>0</v>
+      </c>
+      <c r="I15" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>70</v>
       </c>
@@ -1453,8 +1572,17 @@
       <c r="F16" s="3">
         <v>249.106177578238</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>68</v>
       </c>
@@ -1473,8 +1601,17 @@
       <c r="F17" s="3">
         <v>366.000000000017</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>71</v>
       </c>
@@ -1493,8 +1630,17 @@
       <c r="F18" s="3">
         <v>212.36105235593601</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>69</v>
       </c>
@@ -1513,8 +1659,17 @@
       <c r="F19" s="3">
         <v>366.00000000001398</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>72</v>
       </c>
@@ -1533,8 +1688,17 @@
       <c r="F20" s="3">
         <v>688058509.35971904</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="3">
+        <v>781249111.00424302</v>
+      </c>
+      <c r="H20" s="3">
+        <v>2254809792.5641699</v>
+      </c>
+      <c r="I20" s="3">
+        <v>782559226.24499905</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>73</v>
       </c>
@@ -1553,8 +1717,17 @@
       <c r="F21" s="3">
         <v>1546565315.5455699</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G21" s="3">
+        <v>1552886671.3623099</v>
+      </c>
+      <c r="H21" s="3">
+        <v>2280278499.1943102</v>
+      </c>
+      <c r="I21" s="3">
+        <v>1552464869.32584</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>75</v>
       </c>
@@ -1573,8 +1746,17 @@
       <c r="F22" s="3">
         <v>2520216.1403508801</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G22" s="3">
+        <v>4910932.8070173999</v>
+      </c>
+      <c r="H22" s="3">
+        <v>52885090.855262503</v>
+      </c>
+      <c r="I22" s="3">
+        <v>4910932.8070171699</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -1593,8 +1775,17 @@
       <c r="F23" s="3">
         <v>66086422.465755902</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G23" s="3">
+        <v>292109571.36183399</v>
+      </c>
+      <c r="H23" s="3">
+        <v>150615745.52630201</v>
+      </c>
+      <c r="I23" s="3">
+        <v>296474483.20394403</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>76</v>
       </c>
@@ -1613,8 +1804,17 @@
       <c r="F24" s="3">
         <v>233850933.002204</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G24" s="3">
+        <v>241231766.574619</v>
+      </c>
+      <c r="H24" s="3">
+        <v>455453360.36141002</v>
+      </c>
+      <c r="I24" s="3">
+        <v>240463453.04391801</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>77</v>
       </c>
@@ -1623,8 +1823,11 @@
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>2</v>
       </c>
@@ -1643,12 +1846,21 @@
       <c r="F26" s="3">
         <v>54.917894736842101</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G26" s="3">
+        <v>84.317824561403498</v>
+      </c>
+      <c r="H26" s="3">
+        <v>84.317824561403498</v>
+      </c>
+      <c r="I26" s="3">
+        <v>84.317824561403498</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>0</v>
       </c>
-      <c r="B27" s="11">
+      <c r="B27" s="10">
         <v>0</v>
       </c>
       <c r="C27" s="3">
@@ -1663,8 +1875,17 @@
       <c r="F27" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G27" s="3">
+        <v>0</v>
+      </c>
+      <c r="H27" s="3">
+        <v>0</v>
+      </c>
+      <c r="I27" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>1</v>
       </c>
@@ -1683,8 +1904,17 @@
       <c r="F28" s="3">
         <v>33.104912280701697</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G28" s="3">
+        <v>0</v>
+      </c>
+      <c r="H28" s="3">
+        <v>0</v>
+      </c>
+      <c r="I28" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>15</v>
       </c>
@@ -1693,8 +1923,11 @@
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>2</v>
       </c>
@@ -1713,12 +1946,21 @@
       <c r="F30" s="3">
         <v>54.917894736842101</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G30" s="3">
+        <v>84.317824561403498</v>
+      </c>
+      <c r="H30" s="3">
+        <v>129.55468508771901</v>
+      </c>
+      <c r="I30" s="3">
+        <v>84.317824561403498</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>0</v>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="10">
         <v>0</v>
       </c>
       <c r="C31" s="3">
@@ -1733,8 +1975,17 @@
       <c r="F31" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G31" s="3">
+        <v>0</v>
+      </c>
+      <c r="H31" s="3">
+        <v>0</v>
+      </c>
+      <c r="I31" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>1</v>
       </c>
@@ -1753,8 +2004,17 @@
       <c r="F32" s="3">
         <v>33.104912280701697</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G32" s="3">
+        <v>0</v>
+      </c>
+      <c r="H32" s="3">
+        <v>0</v>
+      </c>
+      <c r="I32" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>78</v>
       </c>
@@ -1763,8 +2023,11 @@
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>2</v>
       </c>
@@ -1783,12 +2046,21 @@
       <c r="F34" s="3">
         <v>158108334.629866</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G34" s="3">
+        <v>241231766.574619</v>
+      </c>
+      <c r="H34" s="3">
+        <v>455453360.36141002</v>
+      </c>
+      <c r="I34" s="3">
+        <v>240463453.04391801</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>0</v>
       </c>
-      <c r="B35" s="11">
+      <c r="B35" s="10">
         <v>0</v>
       </c>
       <c r="C35" s="3">
@@ -1803,8 +2075,17 @@
       <c r="F35" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G35" s="3">
+        <v>0</v>
+      </c>
+      <c r="H35" s="3">
+        <v>0</v>
+      </c>
+      <c r="I35" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>1</v>
       </c>
@@ -1820,12 +2101,21 @@
       <c r="E36" s="3">
         <v>77425708.665584803</v>
       </c>
-      <c r="F36" s="14">
+      <c r="F36" s="13">
         <v>75742598.372338593</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="10" t="s">
+      <c r="G36" s="3">
+        <v>0</v>
+      </c>
+      <c r="H36" s="3">
+        <v>0</v>
+      </c>
+      <c r="I36" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="9" t="s">
         <v>80</v>
       </c>
       <c r="B37" s="3"/>
@@ -1833,8 +2123,11 @@
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
+      <c r="I37" s="3"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>45</v>
       </c>
@@ -1843,8 +2136,11 @@
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>2</v>
       </c>
@@ -1863,12 +2159,21 @@
       <c r="F39" s="3">
         <v>54.917894736842101</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G39" s="3">
+        <v>84.317824561403498</v>
+      </c>
+      <c r="H39" s="3">
+        <v>84.317824561403498</v>
+      </c>
+      <c r="I39" s="3">
+        <v>84.317824561403498</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>0</v>
       </c>
-      <c r="B40" s="11">
+      <c r="B40" s="10">
         <v>38</v>
       </c>
       <c r="C40" s="3">
@@ -1880,11 +2185,20 @@
       <c r="E40" s="3">
         <v>74</v>
       </c>
-      <c r="F40" s="13">
+      <c r="F40" s="12">
         <v>74</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G40" s="3">
+        <v>74</v>
+      </c>
+      <c r="H40" s="3">
+        <v>38</v>
+      </c>
+      <c r="I40" s="3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>1</v>
       </c>
@@ -1903,8 +2217,17 @@
       <c r="F41" s="3">
         <v>33.104912280701697</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G41" s="3">
+        <v>0</v>
+      </c>
+      <c r="H41" s="3">
+        <v>0</v>
+      </c>
+      <c r="I41" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>79</v>
       </c>
@@ -1923,8 +2246,17 @@
       <c r="F42" s="3">
         <v>12.721192982456101</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G42" s="3">
+        <v>15.366</v>
+      </c>
+      <c r="H42" s="3">
+        <v>22.4947894736842</v>
+      </c>
+      <c r="I42" s="3">
+        <v>15.366</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>46</v>
       </c>
@@ -1933,12 +2265,15 @@
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+      <c r="I43" s="3"/>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>0</v>
       </c>
-      <c r="B44" s="11">
+      <c r="B44" s="10">
         <v>32.533356835617603</v>
       </c>
       <c r="C44" s="3">
@@ -1953,8 +2288,17 @@
       <c r="F44" s="3">
         <v>38</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G44" s="3">
+        <v>30.0063157894736</v>
+      </c>
+      <c r="H44" s="3">
+        <v>33.555754385964903</v>
+      </c>
+      <c r="I44" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>24</v>
       </c>
@@ -1970,11 +2314,20 @@
       <c r="E45" s="3">
         <v>95.02</v>
       </c>
-      <c r="F45" s="13">
+      <c r="F45" s="12">
         <v>95.02</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G45" s="3">
+        <v>95.02</v>
+      </c>
+      <c r="H45" s="3">
+        <v>95.02</v>
+      </c>
+      <c r="I45" s="3">
+        <v>95.02</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>1</v>
       </c>
@@ -1993,8 +2346,17 @@
       <c r="F46" s="3">
         <v>33.104912280701697</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G46" s="3">
+        <v>6</v>
+      </c>
+      <c r="H46" s="3">
+        <v>0</v>
+      </c>
+      <c r="I46" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>23</v>
       </c>
@@ -2003,8 +2365,11 @@
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>2</v>
       </c>
@@ -2023,8 +2388,17 @@
       <c r="F48" s="3">
         <v>1510482.5054732601</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G48" s="3">
+        <v>1741284.06034232</v>
+      </c>
+      <c r="H48" s="3">
+        <v>7330402.46816481</v>
+      </c>
+      <c r="I48" s="3">
+        <v>1736743.8276142499</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>0</v>
       </c>
@@ -2040,15 +2414,24 @@
       <c r="E49" s="3">
         <v>6278182.9098127401</v>
       </c>
-      <c r="F49" s="13">
+      <c r="F49" s="12">
         <v>6336354.5687585501</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G49" s="3">
+        <v>5943980.3882502103</v>
+      </c>
+      <c r="H49" s="3">
+        <v>335961.87677191099</v>
+      </c>
+      <c r="I49" s="3">
+        <v>5947935.8225923199</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>1</v>
       </c>
-      <c r="B50" s="12">
+      <c r="B50" s="11">
         <v>324696.16976015997</v>
       </c>
       <c r="C50" s="3">
@@ -2063,8 +2446,17 @@
       <c r="F50" s="3">
         <v>881256.44645368401</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G50" s="3">
+        <v>0</v>
+      </c>
+      <c r="H50" s="3">
+        <v>0</v>
+      </c>
+      <c r="I50" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>35</v>
       </c>
@@ -2083,8 +2475,17 @@
       <c r="F51" s="3">
         <v>1008.08645614035</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G51" s="3">
+        <v>1964.3731228069501</v>
+      </c>
+      <c r="H51" s="3">
+        <v>21154.036342104999</v>
+      </c>
+      <c r="I51" s="3">
+        <v>1964.37312280688</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>22</v>
       </c>
@@ -2093,8 +2494,11 @@
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G52" s="3"/>
+      <c r="H52" s="3"/>
+      <c r="I52" s="3"/>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>0</v>
       </c>
@@ -2113,8 +2517,17 @@
       <c r="F53" s="3">
         <v>2058.1905548631398</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G53" s="3">
+        <v>584.79838596491197</v>
+      </c>
+      <c r="H53" s="3">
+        <v>1656.9666456140301</v>
+      </c>
+      <c r="I53" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>24</v>
       </c>
@@ -2133,12 +2546,21 @@
       <c r="F54" s="3">
         <v>7684853.3281770796</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G54" s="3">
+        <v>7683897.04151031</v>
+      </c>
+      <c r="H54" s="3">
+        <v>7664707.3782909596</v>
+      </c>
+      <c r="I54" s="3">
+        <v>7683897.04151031</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>1</v>
       </c>
-      <c r="B55" s="12">
+      <c r="B55" s="11">
         <v>383620.23837449402</v>
       </c>
       <c r="C55" s="3">
@@ -2153,8 +2575,17 @@
       <c r="F55" s="3">
         <v>1041182.00195373</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G55" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="H55" s="3">
+        <v>0</v>
+      </c>
+      <c r="I55" s="3">
+        <v>782.60869565217297</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>27</v>
       </c>
@@ -2163,8 +2594,11 @@
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G56" s="3"/>
+      <c r="H56" s="3"/>
+      <c r="I56" s="3"/>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>2</v>
       </c>
@@ -2183,8 +2617,17 @@
       <c r="F57" s="3">
         <v>461148335.73813999</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G57" s="3">
+        <v>531611748.93757701</v>
+      </c>
+      <c r="H57" s="3">
+        <v>2237962297.6343999</v>
+      </c>
+      <c r="I57" s="3">
+        <v>530225621.81672299</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>0</v>
       </c>
@@ -2203,8 +2646,17 @@
       <c r="F58" s="3">
         <v>227413103.07681701</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G58" s="3">
+        <v>249860024.891193</v>
+      </c>
+      <c r="H58" s="3">
+        <v>17521742.9570923</v>
+      </c>
+      <c r="I58" s="3">
+        <v>252333604.42830101</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>1</v>
       </c>
@@ -2223,8 +2675,17 @@
       <c r="F59" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G59" s="3">
+        <v>0</v>
+      </c>
+      <c r="H59" s="3">
+        <v>0</v>
+      </c>
+      <c r="I59" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>28</v>
       </c>
@@ -2233,8 +2694,11 @@
       <c r="D60" s="3"/>
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G60" s="3"/>
+      <c r="H60" s="3"/>
+      <c r="I60" s="3"/>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>0</v>
       </c>
@@ -2253,8 +2717,17 @@
       <c r="F61" s="3">
         <v>502929.45532035403</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G61" s="3">
+        <v>222662.824504385</v>
+      </c>
+      <c r="H61" s="3">
+        <v>674248.02661492105</v>
+      </c>
+      <c r="I61" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>24</v>
       </c>
@@ -2273,8 +2746,17 @@
       <c r="F62" s="3">
         <v>19212133320.439201</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G62" s="3">
+        <v>19209742603.772499</v>
+      </c>
+      <c r="H62" s="3">
+        <v>19161768445.724098</v>
+      </c>
+      <c r="I62" s="3">
+        <v>19209742603.772499</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>1</v>
       </c>
@@ -2293,9 +2775,18 @@
       <c r="F63" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="10" t="s">
+      <c r="G63" s="3">
+        <v>0</v>
+      </c>
+      <c r="H63" s="3">
+        <v>0</v>
+      </c>
+      <c r="I63" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A64" s="9" t="s">
         <v>81</v>
       </c>
       <c r="B64" s="3"/>
@@ -2303,8 +2794,11 @@
       <c r="D64" s="3"/>
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G64" s="3"/>
+      <c r="H64" s="3"/>
+      <c r="I64" s="3"/>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>45</v>
       </c>
@@ -2313,8 +2807,11 @@
       <c r="D65" s="3"/>
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G65" s="3"/>
+      <c r="H65" s="3"/>
+      <c r="I65" s="3"/>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>2</v>
       </c>
@@ -2333,12 +2830,21 @@
       <c r="F66" s="3">
         <v>54.917894736842101</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G66" s="3">
+        <v>84.317824561403498</v>
+      </c>
+      <c r="H66" s="3">
+        <v>84.317824561403498</v>
+      </c>
+      <c r="I66" s="3">
+        <v>84.317824561403498</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>0</v>
       </c>
-      <c r="B67" s="12">
+      <c r="B67" s="11">
         <v>36</v>
       </c>
       <c r="C67" s="3">
@@ -2353,8 +2859,17 @@
       <c r="F67" s="3">
         <v>36</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G67" s="3">
+        <v>36</v>
+      </c>
+      <c r="H67" s="3">
+        <v>36</v>
+      </c>
+      <c r="I67" s="3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>1</v>
       </c>
@@ -2373,8 +2888,17 @@
       <c r="F68" s="3">
         <v>33.104912280701697</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G68" s="3">
+        <v>0</v>
+      </c>
+      <c r="H68" s="3">
+        <v>0</v>
+      </c>
+      <c r="I68" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>79</v>
       </c>
@@ -2393,8 +2917,17 @@
       <c r="F69" s="3">
         <v>24.891352674537298</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G69" s="3">
+        <v>34.685052631578898</v>
+      </c>
+      <c r="H69" s="3">
+        <v>33.602350877192897</v>
+      </c>
+      <c r="I69" s="3">
+        <v>34.685052631578898</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>46</v>
       </c>
@@ -2403,8 +2936,11 @@
       <c r="D70" s="3"/>
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G70" s="3"/>
+      <c r="H70" s="3"/>
+      <c r="I70" s="3"/>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>0</v>
       </c>
@@ -2423,8 +2959,17 @@
       <c r="F71" s="3">
         <v>20.737122807017499</v>
       </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G71" s="3">
+        <v>30.0063157894736</v>
+      </c>
+      <c r="H71" s="3">
+        <v>33.555754385964903</v>
+      </c>
+      <c r="I71" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>24</v>
       </c>
@@ -2443,8 +2988,17 @@
       <c r="F72" s="3">
         <v>88.022807017543798</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G72" s="3">
+        <v>84.317824561403498</v>
+      </c>
+      <c r="H72" s="3">
+        <v>84.317824561403498</v>
+      </c>
+      <c r="I72" s="3">
+        <v>84.317824561403498</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>1</v>
       </c>
@@ -2463,8 +3017,17 @@
       <c r="F73" s="3">
         <v>32.547859649122799</v>
       </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G73" s="3">
+        <v>6</v>
+      </c>
+      <c r="H73" s="3">
+        <v>0</v>
+      </c>
+      <c r="I73" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>23</v>
       </c>
@@ -2473,8 +3036,11 @@
       <c r="D74" s="3"/>
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G74" s="3"/>
+      <c r="H74" s="3"/>
+      <c r="I74" s="3"/>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>2</v>
       </c>
@@ -2493,8 +3059,17 @@
       <c r="F75" s="3">
         <v>4695316.8599934299</v>
       </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G75" s="3">
+        <v>4690467.1677328302</v>
+      </c>
+      <c r="H75" s="3">
+        <v>7438674.0150634302</v>
+      </c>
+      <c r="I75" s="3">
+        <v>4687607.1544554103</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>0</v>
       </c>
@@ -2513,8 +3088,17 @@
       <c r="F76" s="3">
         <v>3092471.8310868102</v>
       </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G76" s="3">
+        <v>2879761.3036968498</v>
+      </c>
+      <c r="H76" s="3">
+        <v>188598.06800528901</v>
+      </c>
+      <c r="I76" s="3">
+        <v>2880290.5538512398</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>1</v>
       </c>
@@ -2533,8 +3117,17 @@
       <c r="F77" s="3">
         <v>704228.27824355895</v>
       </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G77" s="3">
+        <v>0</v>
+      </c>
+      <c r="H77" s="3">
+        <v>0</v>
+      </c>
+      <c r="I77" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>35</v>
       </c>
@@ -2553,8 +3146,17 @@
       <c r="F78" s="3">
         <v>26434.568986302202</v>
       </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G78" s="3">
+        <v>116843.828544738</v>
+      </c>
+      <c r="H78" s="3">
+        <v>60246.298210522204</v>
+      </c>
+      <c r="I78" s="3">
+        <v>118589.79328158101</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>22</v>
       </c>
@@ -2563,8 +3165,11 @@
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G79" s="3"/>
+      <c r="H79" s="3"/>
+      <c r="I79" s="3"/>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>0</v>
       </c>
@@ -2583,8 +3188,17 @@
       <c r="F80" s="3">
         <v>562.38473322931497</v>
       </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G80" s="3">
+        <v>584.79838596491197</v>
+      </c>
+      <c r="H80" s="3">
+        <v>1656.9666456140101</v>
+      </c>
+      <c r="I80" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>24</v>
       </c>
@@ -2603,8 +3217,17 @@
       <c r="F81" s="3">
         <v>7659426.8456469998</v>
       </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G81" s="3">
+        <v>7569017.5860898104</v>
+      </c>
+      <c r="H81" s="3">
+        <v>7625615.1164232604</v>
+      </c>
+      <c r="I81" s="3">
+        <v>7567271.6213527499</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>1</v>
       </c>
@@ -2623,8 +3246,17 @@
       <c r="F82" s="3">
         <v>832027.73894551501</v>
       </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G82" s="3">
+        <v>626.08695652173901</v>
+      </c>
+      <c r="H82" s="3">
+        <v>0</v>
+      </c>
+      <c r="I82" s="3">
+        <v>626.08695652173901</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>27</v>
       </c>
@@ -2633,8 +3265,11 @@
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G83" s="3"/>
+      <c r="H83" s="3"/>
+      <c r="I83" s="3"/>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>2</v>
       </c>
@@ -2653,8 +3288,17 @@
       <c r="F84" s="3">
         <v>1433474103.7413399</v>
       </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G84" s="3">
+        <v>1431993499.0292101</v>
+      </c>
+      <c r="H84" s="3">
+        <v>2271017459.4651499</v>
+      </c>
+      <c r="I84" s="3">
+        <v>1431120340.7116201</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>0</v>
       </c>
@@ -2673,8 +3317,17 @@
       <c r="F85" s="3">
         <v>113312298.149334</v>
       </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G85" s="3">
+        <v>121115835.15784</v>
+      </c>
+      <c r="H85" s="3">
+        <v>9935287.7570965104</v>
+      </c>
+      <c r="I85" s="3">
+        <v>121344528.61445101</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>1</v>
       </c>
@@ -2693,8 +3346,17 @@
       <c r="F86" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G86" s="3">
+        <v>0</v>
+      </c>
+      <c r="H86" s="3">
+        <v>0</v>
+      </c>
+      <c r="I86" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>28</v>
       </c>
@@ -2703,8 +3365,11 @@
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G87" s="3"/>
+      <c r="H87" s="3"/>
+      <c r="I87" s="3"/>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>0</v>
       </c>
@@ -2723,8 +3388,17 @@
       <c r="F88" s="3">
         <v>221086.345003836</v>
       </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G88" s="3">
+        <v>222662.824504385</v>
+      </c>
+      <c r="H88" s="3">
+        <v>674248.02661490894</v>
+      </c>
+      <c r="I88" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>24</v>
       </c>
@@ -2743,8 +3417,17 @@
       <c r="F89" s="3">
         <v>19148567114.1133</v>
       </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G89" s="3">
+        <v>18922543965.2178</v>
+      </c>
+      <c r="H89" s="3">
+        <v>19064037791.0508</v>
+      </c>
+      <c r="I89" s="3">
+        <v>18918179053.377602</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>1</v>
       </c>
@@ -2761,6 +3444,15 @@
         <v>0</v>
       </c>
       <c r="F90" s="3">
+        <v>0</v>
+      </c>
+      <c r="G90" s="3">
+        <v>0</v>
+      </c>
+      <c r="H90" s="3">
+        <v>0</v>
+      </c>
+      <c r="I90" s="3">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated notes and results
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\Desktop\ongoing_projects\MVS\dev\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED03EADD-B819-4D93-9AC8-393788651A76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{249CD2E5-B4ED-4086-BDCA-D8209FF9B313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16950" yWindow="-8910" windowWidth="17055" windowHeight="15585" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-15945" yWindow="-8910" windowWidth="15855" windowHeight="15585" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Experiments" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="92">
   <si>
     <t>Grid</t>
   </si>
@@ -332,6 +332,9 @@
   </si>
   <si>
     <t>updated sum in market constraint</t>
+  </si>
+  <si>
+    <t>corrected capital costs</t>
   </si>
 </sst>
 </file>
@@ -1169,30 +1172,36 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEB77188-4C54-4D05-A0BB-AB8E292CE16E}">
-  <dimension ref="A1:I90"/>
+  <dimension ref="A1:L90"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="9" width="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="12" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="G1">
         <v>250617</v>
       </c>
-      <c r="I1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1">
+        <v>250618</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>62</v>
       </c>
@@ -1220,8 +1229,17 @@
       <c r="I3" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J3" s="3">
+        <v>0</v>
+      </c>
+      <c r="K3" s="3">
+        <v>0</v>
+      </c>
+      <c r="L3" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>63</v>
       </c>
@@ -1249,8 +1267,17 @@
       <c r="I4" s="3">
         <v>2500</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J4" s="3">
+        <v>2500</v>
+      </c>
+      <c r="K4" s="3">
+        <v>10000</v>
+      </c>
+      <c r="L4" s="3">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>57</v>
       </c>
@@ -1278,8 +1305,17 @@
       <c r="I5" s="3">
         <v>8783</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J5" s="3">
+        <v>8783</v>
+      </c>
+      <c r="K5" s="3">
+        <v>8783</v>
+      </c>
+      <c r="L5" s="3">
+        <v>8783</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>85</v>
       </c>
@@ -1307,8 +1343,17 @@
       <c r="I6" s="3">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J6" s="3">
+        <v>20</v>
+      </c>
+      <c r="K6" s="3">
+        <v>20</v>
+      </c>
+      <c r="L6" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>86</v>
       </c>
@@ -1336,8 +1381,17 @@
       <c r="I7" s="3">
         <v>80</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J7" s="3">
+        <v>80</v>
+      </c>
+      <c r="K7" s="3">
+        <v>80</v>
+      </c>
+      <c r="L7" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>64</v>
       </c>
@@ -1365,8 +1419,17 @@
       <c r="I8" s="3" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1394,8 +1457,17 @@
       <c r="I9" s="3" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J9" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>65</v>
       </c>
@@ -1423,8 +1495,17 @@
       <c r="I10" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J10" s="3">
+        <v>0</v>
+      </c>
+      <c r="K10" s="3">
+        <v>0</v>
+      </c>
+      <c r="L10" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -1436,8 +1517,11 @@
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>67</v>
       </c>
@@ -1465,8 +1549,17 @@
       <c r="I12" s="3">
         <v>17974426085.787498</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J12" s="3">
+        <v>18593036278.072899</v>
+      </c>
+      <c r="K12" s="3">
+        <v>76224539327.009293</v>
+      </c>
+      <c r="L12" s="3">
+        <v>76217736292.399704</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>66</v>
       </c>
@@ -1494,8 +1587,17 @@
       <c r="I13" s="3">
         <v>639.23342490196205</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J13" s="3">
+        <v>900.37050890922501</v>
+      </c>
+      <c r="K13" s="3">
+        <v>273.27420210838301</v>
+      </c>
+      <c r="L13" s="3">
+        <v>896.81816506385803</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>84</v>
       </c>
@@ -1523,8 +1625,17 @@
       <c r="I14" s="3">
         <v>7.9187216723792002E-4</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J14" s="3">
+        <v>0.46124892082726399</v>
+      </c>
+      <c r="K14" s="3">
+        <v>8.9406250560400302E-2</v>
+      </c>
+      <c r="L14" s="3">
+        <v>5.36780805316764E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>87</v>
       </c>
@@ -1552,8 +1663,17 @@
       <c r="I15" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J15" s="3">
+        <v>0</v>
+      </c>
+      <c r="K15" s="3">
+        <v>0</v>
+      </c>
+      <c r="L15" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>70</v>
       </c>
@@ -1581,8 +1701,17 @@
       <c r="I16" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J16" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>68</v>
       </c>
@@ -1610,8 +1739,17 @@
       <c r="I17" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>71</v>
       </c>
@@ -1639,8 +1777,17 @@
       <c r="I18" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>69</v>
       </c>
@@ -1668,8 +1815,17 @@
       <c r="I19" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>72</v>
       </c>
@@ -1697,8 +1853,17 @@
       <c r="I20" s="3">
         <v>782559226.24499905</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J20" s="3">
+        <v>330621930.02920002</v>
+      </c>
+      <c r="K20" s="3">
+        <v>331006591.66265798</v>
+      </c>
+      <c r="L20" s="3">
+        <v>330994041.82959598</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>73</v>
       </c>
@@ -1726,8 +1891,17 @@
       <c r="I21" s="3">
         <v>1552464869.32584</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J21" s="3">
+        <v>358593463.57974303</v>
+      </c>
+      <c r="K21" s="3">
+        <v>359443995.13158298</v>
+      </c>
+      <c r="L21" s="3">
+        <v>330184107.53514099</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>75</v>
       </c>
@@ -1755,8 +1929,17 @@
       <c r="I22" s="3">
         <v>4910932.8070171699</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J22" s="3">
+        <v>8056899.64912281</v>
+      </c>
+      <c r="K22" s="3">
+        <v>4.1389114358025803E-8</v>
+      </c>
+      <c r="L22" s="3">
+        <v>3.7125857943465202E-8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -1784,8 +1967,17 @@
       <c r="I23" s="3">
         <v>296474483.20394403</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J23" s="3">
+        <v>546027524.90788198</v>
+      </c>
+      <c r="K23" s="3">
+        <v>449542641.58762902</v>
+      </c>
+      <c r="L23" s="3">
+        <v>67318308.771929905</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>76</v>
       </c>
@@ -1813,8 +2005,17 @@
       <c r="I24" s="3">
         <v>240463453.04391801</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J24" s="3">
+        <v>169749997.06638101</v>
+      </c>
+      <c r="K24" s="3">
+        <v>207472218.63668799</v>
+      </c>
+      <c r="L24" s="3">
+        <v>276629624.84891802</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>77</v>
       </c>
@@ -1826,8 +2027,11 @@
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>2</v>
       </c>
@@ -1855,8 +2059,17 @@
       <c r="I26" s="3">
         <v>84.317824561403498</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J26" s="3">
+        <v>0</v>
+      </c>
+      <c r="K26" s="3">
+        <v>0</v>
+      </c>
+      <c r="L26" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>0</v>
       </c>
@@ -1884,8 +2097,17 @@
       <c r="I27" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J27" s="3">
+        <v>80</v>
+      </c>
+      <c r="K27" s="3">
+        <v>120</v>
+      </c>
+      <c r="L27" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>1</v>
       </c>
@@ -1913,8 +2135,17 @@
       <c r="I28" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J28" s="3">
+        <v>0</v>
+      </c>
+      <c r="K28" s="3">
+        <v>0</v>
+      </c>
+      <c r="L28" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>15</v>
       </c>
@@ -1926,8 +2157,11 @@
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
       <c r="I29" s="3"/>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+      <c r="L29" s="3"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>2</v>
       </c>
@@ -1955,8 +2189,17 @@
       <c r="I30" s="3">
         <v>84.317824561403498</v>
       </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J30" s="3">
+        <v>0</v>
+      </c>
+      <c r="K30" s="3">
+        <v>0</v>
+      </c>
+      <c r="L30" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>0</v>
       </c>
@@ -1984,8 +2227,17 @@
       <c r="I31" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J31" s="3">
+        <v>80</v>
+      </c>
+      <c r="K31" s="3">
+        <v>120</v>
+      </c>
+      <c r="L31" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>1</v>
       </c>
@@ -2013,8 +2265,17 @@
       <c r="I32" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J32" s="3">
+        <v>0</v>
+      </c>
+      <c r="K32" s="3">
+        <v>0</v>
+      </c>
+      <c r="L32" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>78</v>
       </c>
@@ -2026,8 +2287,11 @@
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J33" s="3"/>
+      <c r="K33" s="3"/>
+      <c r="L33" s="3"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>2</v>
       </c>
@@ -2055,8 +2319,17 @@
       <c r="I34" s="3">
         <v>240463453.04391801</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J34" s="3">
+        <v>0</v>
+      </c>
+      <c r="K34" s="3">
+        <v>0</v>
+      </c>
+      <c r="L34" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>0</v>
       </c>
@@ -2084,8 +2357,17 @@
       <c r="I35" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J35" s="3">
+        <v>169749997.06638101</v>
+      </c>
+      <c r="K35" s="3">
+        <v>207472218.63668799</v>
+      </c>
+      <c r="L35" s="3">
+        <v>276629624.84891802</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>1</v>
       </c>
@@ -2113,8 +2395,17 @@
       <c r="I36" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J36" s="3">
+        <v>0</v>
+      </c>
+      <c r="K36" s="3">
+        <v>0</v>
+      </c>
+      <c r="L36" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
         <v>80</v>
       </c>
@@ -2126,8 +2417,11 @@
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
       <c r="I37" s="3"/>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J37" s="3"/>
+      <c r="K37" s="3"/>
+      <c r="L37" s="3"/>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>45</v>
       </c>
@@ -2139,8 +2433,11 @@
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
       <c r="I38" s="3"/>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J38" s="3"/>
+      <c r="K38" s="3"/>
+      <c r="L38" s="3"/>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>2</v>
       </c>
@@ -2168,8 +2465,17 @@
       <c r="I39" s="3">
         <v>84.317824561403498</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J39" s="3">
+        <v>12.92135</v>
+      </c>
+      <c r="K39" s="3">
+        <v>12.92135</v>
+      </c>
+      <c r="L39" s="3">
+        <v>12.92135</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>0</v>
       </c>
@@ -2197,8 +2503,17 @@
       <c r="I40" s="3">
         <v>74</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J40" s="3">
+        <v>95.019999999999897</v>
+      </c>
+      <c r="K40" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="L40" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>1</v>
       </c>
@@ -2226,8 +2541,17 @@
       <c r="I41" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J41" s="3">
+        <v>0</v>
+      </c>
+      <c r="K41" s="3">
+        <v>0</v>
+      </c>
+      <c r="L41" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>79</v>
       </c>
@@ -2255,8 +2579,17 @@
       <c r="I42" s="3">
         <v>15.366</v>
       </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J42" s="3">
+        <v>18.084</v>
+      </c>
+      <c r="K42" s="3">
+        <v>1.4210854715202001E-14</v>
+      </c>
+      <c r="L42" s="3">
+        <v>1.4210854715202001E-14</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>46</v>
       </c>
@@ -2268,8 +2601,11 @@
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
       <c r="I43" s="3"/>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J43" s="3"/>
+      <c r="K43" s="3"/>
+      <c r="L43" s="3"/>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>0</v>
       </c>
@@ -2297,8 +2633,17 @@
       <c r="I44" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J44" s="3">
+        <v>0</v>
+      </c>
+      <c r="K44" s="3">
+        <v>0</v>
+      </c>
+      <c r="L44" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>24</v>
       </c>
@@ -2326,8 +2671,17 @@
       <c r="I45" s="3">
         <v>95.02</v>
       </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J45" s="3">
+        <v>95.02</v>
+      </c>
+      <c r="K45" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="L45" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>1</v>
       </c>
@@ -2355,8 +2709,17 @@
       <c r="I46" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J46" s="3">
+        <v>6</v>
+      </c>
+      <c r="K46" s="3">
+        <v>6</v>
+      </c>
+      <c r="L46" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>23</v>
       </c>
@@ -2368,8 +2731,11 @@
       <c r="G47" s="3"/>
       <c r="H47" s="3"/>
       <c r="I47" s="3"/>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J47" s="3"/>
+      <c r="K47" s="3"/>
+      <c r="L47" s="3"/>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>2</v>
       </c>
@@ -2397,8 +2763,17 @@
       <c r="I48" s="3">
         <v>1736743.8276142499</v>
       </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J48" s="3">
+        <v>2095.8063421052598</v>
+      </c>
+      <c r="K48" s="3">
+        <v>1993.33316666666</v>
+      </c>
+      <c r="L48" s="3">
+        <v>1938.2025000000001</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>0</v>
       </c>
@@ -2426,8 +2801,17 @@
       <c r="I49" s="3">
         <v>5947935.8225923199</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J49" s="3">
+        <v>7681325.4571270896</v>
+      </c>
+      <c r="K49" s="3">
+        <v>7684650.6901621604</v>
+      </c>
+      <c r="L49" s="3">
+        <v>7684705.8208288299</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>1</v>
       </c>
@@ -2455,8 +2839,17 @@
       <c r="I50" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J50" s="3">
+        <v>0</v>
+      </c>
+      <c r="K50" s="3">
+        <v>0</v>
+      </c>
+      <c r="L50" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>35</v>
       </c>
@@ -2484,8 +2877,17 @@
       <c r="I51" s="3">
         <v>1964.37312280688</v>
       </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J51" s="3">
+        <v>3222.7598596491198</v>
+      </c>
+      <c r="K51" s="3">
+        <v>4.1389114358025804E-12</v>
+      </c>
+      <c r="L51" s="3">
+        <v>3.7125857943465202E-12</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>22</v>
       </c>
@@ -2497,8 +2899,11 @@
       <c r="G52" s="3"/>
       <c r="H52" s="3"/>
       <c r="I52" s="3"/>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J52" s="3"/>
+      <c r="K52" s="3"/>
+      <c r="L52" s="3"/>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>0</v>
       </c>
@@ -2526,8 +2931,17 @@
       <c r="I53" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J53" s="3">
+        <v>0</v>
+      </c>
+      <c r="K53" s="3">
+        <v>0</v>
+      </c>
+      <c r="L53" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>24</v>
       </c>
@@ -2555,8 +2969,17 @@
       <c r="I54" s="3">
         <v>7683897.04151031</v>
       </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J54" s="3">
+        <v>7682638.6547735296</v>
+      </c>
+      <c r="K54" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+      <c r="L54" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>1</v>
       </c>
@@ -2584,8 +3007,17 @@
       <c r="I55" s="3">
         <v>782.60869565217297</v>
       </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J55" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="K55" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="L55" s="3">
+        <v>782.60869565217297</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>27</v>
       </c>
@@ -2597,8 +3029,11 @@
       <c r="G56" s="3"/>
       <c r="H56" s="3"/>
       <c r="I56" s="3"/>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J56" s="3"/>
+      <c r="K56" s="3"/>
+      <c r="L56" s="3"/>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>2</v>
       </c>
@@ -2626,8 +3061,17 @@
       <c r="I57" s="3">
         <v>530225621.81672299</v>
       </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J57" s="3">
+        <v>639846.93843812495</v>
+      </c>
+      <c r="K57" s="3">
+        <v>608562.01184010797</v>
+      </c>
+      <c r="L57" s="3">
+        <v>591730.69132540701</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>0</v>
       </c>
@@ -2655,8 +3099,17 @@
       <c r="I58" s="3">
         <v>252333604.42830101</v>
       </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J58" s="3">
+        <v>329982083.09076297</v>
+      </c>
+      <c r="K58" s="3">
+        <v>330398029.65081698</v>
+      </c>
+      <c r="L58" s="3">
+        <v>330402311.13827002</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>1</v>
       </c>
@@ -2684,8 +3137,17 @@
       <c r="I59" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J59" s="3">
+        <v>0</v>
+      </c>
+      <c r="K59" s="3">
+        <v>0</v>
+      </c>
+      <c r="L59" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>28</v>
       </c>
@@ -2697,8 +3159,11 @@
       <c r="G60" s="3"/>
       <c r="H60" s="3"/>
       <c r="I60" s="3"/>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J60" s="3"/>
+      <c r="K60" s="3"/>
+      <c r="L60" s="3"/>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>0</v>
       </c>
@@ -2726,8 +3191,17 @@
       <c r="I61" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J61" s="3">
+        <v>0</v>
+      </c>
+      <c r="K61" s="3">
+        <v>0</v>
+      </c>
+      <c r="L61" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>24</v>
       </c>
@@ -2755,8 +3229,17 @@
       <c r="I62" s="3">
         <v>19209742603.772499</v>
       </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J62" s="3">
+        <v>19206596636.9305</v>
+      </c>
+      <c r="K62" s="3">
+        <v>76858614146.318405</v>
+      </c>
+      <c r="L62" s="3">
+        <v>76858614146.318405</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>1</v>
       </c>
@@ -2784,8 +3267,17 @@
       <c r="I63" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J63" s="3">
+        <v>0</v>
+      </c>
+      <c r="K63" s="3">
+        <v>0</v>
+      </c>
+      <c r="L63" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" s="9" t="s">
         <v>81</v>
       </c>
@@ -2797,8 +3289,11 @@
       <c r="G64" s="3"/>
       <c r="H64" s="3"/>
       <c r="I64" s="3"/>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J64" s="3"/>
+      <c r="K64" s="3"/>
+      <c r="L64" s="3"/>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>45</v>
       </c>
@@ -2810,8 +3305,11 @@
       <c r="G65" s="3"/>
       <c r="H65" s="3"/>
       <c r="I65" s="3"/>
-    </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J65" s="3"/>
+      <c r="K65" s="3"/>
+      <c r="L65" s="3"/>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>2</v>
       </c>
@@ -2839,8 +3337,17 @@
       <c r="I66" s="3">
         <v>84.317824561403498</v>
       </c>
-    </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J66" s="3">
+        <v>12.9213500000059</v>
+      </c>
+      <c r="K66" s="3">
+        <v>12.921350000011</v>
+      </c>
+      <c r="L66" s="3">
+        <v>12.92135</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>0</v>
       </c>
@@ -2868,8 +3375,17 @@
       <c r="I67" s="3">
         <v>36</v>
       </c>
-    </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J67" s="3">
+        <v>78</v>
+      </c>
+      <c r="K67" s="3">
+        <v>80</v>
+      </c>
+      <c r="L67" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>1</v>
       </c>
@@ -2897,8 +3413,17 @@
       <c r="I68" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J68" s="3">
+        <v>0</v>
+      </c>
+      <c r="K68" s="3">
+        <v>0</v>
+      </c>
+      <c r="L68" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>79</v>
       </c>
@@ -2926,8 +3451,17 @@
       <c r="I69" s="3">
         <v>34.685052631578898</v>
       </c>
-    </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J69" s="3">
+        <v>58.084000000000003</v>
+      </c>
+      <c r="K69" s="3">
+        <v>30.007649999998101</v>
+      </c>
+      <c r="L69" s="3">
+        <v>18.084</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>46</v>
       </c>
@@ -2939,8 +3473,11 @@
       <c r="G70" s="3"/>
       <c r="H70" s="3"/>
       <c r="I70" s="3"/>
-    </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J70" s="3"/>
+      <c r="K70" s="3"/>
+      <c r="L70" s="3"/>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>0</v>
       </c>
@@ -2968,8 +3505,17 @@
       <c r="I71" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J71" s="3">
+        <v>0</v>
+      </c>
+      <c r="K71" s="3">
+        <v>0</v>
+      </c>
+      <c r="L71" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>24</v>
       </c>
@@ -2997,8 +3543,17 @@
       <c r="I72" s="3">
         <v>84.317824561403498</v>
       </c>
-    </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J72" s="3">
+        <v>86.207999999999998</v>
+      </c>
+      <c r="K72" s="3">
+        <v>86.207999999999998</v>
+      </c>
+      <c r="L72" s="3">
+        <v>86.207999999999998</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>1</v>
       </c>
@@ -3026,8 +3581,17 @@
       <c r="I73" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J73" s="3">
+        <v>6</v>
+      </c>
+      <c r="K73" s="3">
+        <v>6</v>
+      </c>
+      <c r="L73" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>23</v>
       </c>
@@ -3039,8 +3603,11 @@
       <c r="G74" s="3"/>
       <c r="H74" s="3"/>
       <c r="I74" s="3"/>
-    </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J74" s="3"/>
+      <c r="K74" s="3"/>
+      <c r="L74" s="3"/>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>2</v>
       </c>
@@ -3068,8 +3635,17 @@
       <c r="I75" s="3">
         <v>4687607.1544554103</v>
       </c>
-    </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J75" s="3">
+        <v>161205.78516666399</v>
+      </c>
+      <c r="K75" s="3">
+        <v>127240.23469737</v>
+      </c>
+      <c r="L75" s="3">
+        <v>2271.6272543858399</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>0</v>
       </c>
@@ -3097,8 +3673,17 @@
       <c r="I76" s="3">
         <v>2880290.5538512398</v>
       </c>
-    </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J76" s="3">
+        <v>7307027.2281987704</v>
+      </c>
+      <c r="K76" s="3">
+        <v>7514449.5244724201</v>
+      </c>
+      <c r="L76" s="3">
+        <v>7677640.5651971698</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>1</v>
       </c>
@@ -3126,8 +3711,17 @@
       <c r="I77" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J77" s="3">
+        <v>0</v>
+      </c>
+      <c r="K77" s="3">
+        <v>0</v>
+      </c>
+      <c r="L77" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>35</v>
       </c>
@@ -3155,8 +3749,17 @@
       <c r="I78" s="3">
         <v>118589.79328158101</v>
       </c>
-    </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J78" s="3">
+        <v>218411.00996315401</v>
+      </c>
+      <c r="K78" s="3">
+        <v>44954.264158763101</v>
+      </c>
+      <c r="L78" s="3">
+        <v>6731.8308771929796</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>22</v>
       </c>
@@ -3168,8 +3771,11 @@
       <c r="G79" s="3"/>
       <c r="H79" s="3"/>
       <c r="I79" s="3"/>
-    </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J79" s="3"/>
+      <c r="K79" s="3"/>
+      <c r="L79" s="3"/>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>0</v>
       </c>
@@ -3197,8 +3803,17 @@
       <c r="I80" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J80" s="3">
+        <v>0</v>
+      </c>
+      <c r="K80" s="3">
+        <v>0</v>
+      </c>
+      <c r="L80" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>24</v>
       </c>
@@ -3226,8 +3841,17 @@
       <c r="I81" s="3">
         <v>7567271.6213527499</v>
       </c>
-    </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J81" s="3">
+        <v>7467450.4046713598</v>
+      </c>
+      <c r="K81" s="3">
+        <v>7640907.1504754797</v>
+      </c>
+      <c r="L81" s="3">
+        <v>7679129.5837559802</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>1</v>
       </c>
@@ -3255,8 +3879,17 @@
       <c r="I82" s="3">
         <v>626.08695652173901</v>
       </c>
-    </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J82" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="K82" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="L82" s="3">
+        <v>782.60869565217297</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>27</v>
       </c>
@@ -3268,8 +3901,11 @@
       <c r="G83" s="3"/>
       <c r="H83" s="3"/>
       <c r="I83" s="3"/>
-    </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J83" s="3"/>
+      <c r="K83" s="3"/>
+      <c r="L83" s="3"/>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>2</v>
       </c>
@@ -3297,8 +3933,17 @@
       <c r="I84" s="3">
         <v>1431120340.7116201</v>
       </c>
-    </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J84" s="3">
+        <v>49215915.624048501</v>
+      </c>
+      <c r="K84" s="3">
+        <v>38846277.435859099</v>
+      </c>
+      <c r="L84" s="3">
+        <v>693524.83327793004</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>0</v>
       </c>
@@ -3326,8 +3971,17 @@
       <c r="I85" s="3">
         <v>121344528.61445101</v>
       </c>
-    </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J85" s="3">
+        <v>309377547.95568901</v>
+      </c>
+      <c r="K85" s="3">
+        <v>320597717.69572097</v>
+      </c>
+      <c r="L85" s="3">
+        <v>329490582.70186299</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>1</v>
       </c>
@@ -3355,8 +4009,17 @@
       <c r="I86" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J86" s="3">
+        <v>0</v>
+      </c>
+      <c r="K86" s="3">
+        <v>0</v>
+      </c>
+      <c r="L86" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>28</v>
       </c>
@@ -3368,8 +4031,11 @@
       <c r="G87" s="3"/>
       <c r="H87" s="3"/>
       <c r="I87" s="3"/>
-    </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J87" s="3"/>
+      <c r="K87" s="3"/>
+      <c r="L87" s="3"/>
+    </row>
+    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>0</v>
       </c>
@@ -3397,8 +4063,17 @@
       <c r="I88" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J88" s="3">
+        <v>0</v>
+      </c>
+      <c r="K88" s="3">
+        <v>0</v>
+      </c>
+      <c r="L88" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>24</v>
       </c>
@@ -3426,8 +4101,17 @@
       <c r="I89" s="3">
         <v>18918179053.377602</v>
       </c>
-    </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J89" s="3">
+        <v>18668626011.671001</v>
+      </c>
+      <c r="K89" s="3">
+        <v>76409071504.731094</v>
+      </c>
+      <c r="L89" s="3">
+        <v>76791295837.546799</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>1</v>
       </c>
@@ -3453,6 +4137,15 @@
         <v>0</v>
       </c>
       <c r="I90" s="3">
+        <v>0</v>
+      </c>
+      <c r="J90" s="3">
+        <v>0</v>
+      </c>
+      <c r="K90" s="3">
+        <v>0</v>
+      </c>
+      <c r="L90" s="3">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update results and progress notes
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\Desktop\ongoing_projects\MVS\dev\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{249CD2E5-B4ED-4086-BDCA-D8209FF9B313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30E7DC95-E666-4774-AD6E-586A72F06D54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15945" yWindow="-8910" windowWidth="15855" windowHeight="15585" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-16440" yWindow="-8910" windowWidth="16275" windowHeight="15585" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Experiments" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="94">
   <si>
     <t>Grid</t>
   </si>
@@ -335,6 +335,12 @@
   </si>
   <si>
     <t>corrected capital costs</t>
+  </si>
+  <si>
+    <t>updated backup generation cost</t>
+  </si>
+  <si>
+    <t>no load shedding</t>
   </si>
 </sst>
 </file>
@@ -1172,14 +1178,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEB77188-4C54-4D05-A0BB-AB8E292CE16E}">
-  <dimension ref="A1:L90"/>
+  <dimension ref="A1:U90"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="12" width="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="13" width="18" bestFit="1" customWidth="1"/>
+    <col min="14" max="16" width="19" bestFit="1" customWidth="1"/>
+    <col min="17" max="21" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -1189,8 +1197,11 @@
       <c r="J1">
         <v>250618</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M1">
+        <v>250623</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -1200,8 +1211,14 @@
       <c r="J2" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M2" t="s">
+        <v>92</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>62</v>
       </c>
@@ -1238,8 +1255,35 @@
       <c r="L3" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M3" s="3">
+        <v>0</v>
+      </c>
+      <c r="N3" s="3">
+        <v>0</v>
+      </c>
+      <c r="O3" s="3">
+        <v>0</v>
+      </c>
+      <c r="P3" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="3">
+        <v>0</v>
+      </c>
+      <c r="R3" s="3">
+        <v>0</v>
+      </c>
+      <c r="S3" s="3">
+        <v>0</v>
+      </c>
+      <c r="T3" s="3">
+        <v>0</v>
+      </c>
+      <c r="U3" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>63</v>
       </c>
@@ -1276,8 +1320,35 @@
       <c r="L4" s="3">
         <v>10000</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M4" s="3">
+        <v>10000</v>
+      </c>
+      <c r="N4" s="3">
+        <v>20000</v>
+      </c>
+      <c r="O4" s="3">
+        <v>50000</v>
+      </c>
+      <c r="P4" s="3">
+        <v>100000</v>
+      </c>
+      <c r="Q4" s="3">
+        <v>10000</v>
+      </c>
+      <c r="R4" s="3">
+        <v>10000</v>
+      </c>
+      <c r="S4" s="3">
+        <v>10000</v>
+      </c>
+      <c r="T4" s="3">
+        <v>10000</v>
+      </c>
+      <c r="U4" s="3">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>57</v>
       </c>
@@ -1314,8 +1385,35 @@
       <c r="L5" s="3">
         <v>8783</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M5" s="3">
+        <v>8783</v>
+      </c>
+      <c r="N5" s="3">
+        <v>8783</v>
+      </c>
+      <c r="O5" s="3">
+        <v>8783</v>
+      </c>
+      <c r="P5" s="3">
+        <v>8783</v>
+      </c>
+      <c r="Q5" s="3">
+        <v>8783</v>
+      </c>
+      <c r="R5" s="3">
+        <v>8783</v>
+      </c>
+      <c r="S5" s="3">
+        <v>8783</v>
+      </c>
+      <c r="T5" s="3">
+        <v>8783</v>
+      </c>
+      <c r="U5" s="3">
+        <v>8783</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>85</v>
       </c>
@@ -1352,8 +1450,35 @@
       <c r="L6" s="3">
         <v>50</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M6" s="3">
+        <v>50</v>
+      </c>
+      <c r="N6" s="3">
+        <v>50</v>
+      </c>
+      <c r="O6" s="3">
+        <v>50</v>
+      </c>
+      <c r="P6" s="3">
+        <v>50</v>
+      </c>
+      <c r="Q6" s="3">
+        <v>50</v>
+      </c>
+      <c r="R6" s="3">
+        <v>50</v>
+      </c>
+      <c r="S6" s="3">
+        <v>50</v>
+      </c>
+      <c r="T6" s="3">
+        <v>10</v>
+      </c>
+      <c r="U6" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>86</v>
       </c>
@@ -1390,8 +1515,35 @@
       <c r="L7" s="3">
         <v>50</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M7" s="3">
+        <v>50</v>
+      </c>
+      <c r="N7" s="3">
+        <v>50</v>
+      </c>
+      <c r="O7" s="3">
+        <v>50</v>
+      </c>
+      <c r="P7" s="3">
+        <v>50</v>
+      </c>
+      <c r="Q7" s="3">
+        <v>50</v>
+      </c>
+      <c r="R7" s="3">
+        <v>50</v>
+      </c>
+      <c r="S7" s="3">
+        <v>50</v>
+      </c>
+      <c r="T7" s="3">
+        <v>89.999999999999901</v>
+      </c>
+      <c r="U7" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>64</v>
       </c>
@@ -1428,8 +1580,35 @@
       <c r="L8" s="3" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="N8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="O8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="P8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="R8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="S8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="T8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="U8" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1466,8 +1645,35 @@
       <c r="L9" s="3" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M9" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="N9" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="O9" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="P9" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q9" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="R9" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="S9" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="T9" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="U9" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>65</v>
       </c>
@@ -1504,8 +1710,35 @@
       <c r="L10" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M10" s="3">
+        <v>0</v>
+      </c>
+      <c r="N10" s="3">
+        <v>0</v>
+      </c>
+      <c r="O10" s="3">
+        <v>0</v>
+      </c>
+      <c r="P10" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="3">
+        <v>0</v>
+      </c>
+      <c r="R10" s="3">
+        <v>0</v>
+      </c>
+      <c r="S10" s="3">
+        <v>0</v>
+      </c>
+      <c r="T10" s="3">
+        <v>0</v>
+      </c>
+      <c r="U10" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -1520,8 +1753,17 @@
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
+      <c r="O11" s="3"/>
+      <c r="P11" s="3"/>
+      <c r="Q11" s="3"/>
+      <c r="R11" s="3"/>
+      <c r="S11" s="3"/>
+      <c r="T11" s="3"/>
+      <c r="U11" s="3"/>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>67</v>
       </c>
@@ -1558,8 +1800,35 @@
       <c r="L12" s="3">
         <v>76217736292.399704</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M12" s="3">
+        <v>76165214305.257706</v>
+      </c>
+      <c r="N12" s="3">
+        <v>153032254731.38199</v>
+      </c>
+      <c r="O12" s="3">
+        <v>383571698888.06702</v>
+      </c>
+      <c r="P12" s="3">
+        <v>767724129880.96497</v>
+      </c>
+      <c r="Q12" s="3">
+        <v>76124934482.425995</v>
+      </c>
+      <c r="R12" s="3">
+        <v>76173580853.066895</v>
+      </c>
+      <c r="S12" s="3">
+        <v>76173580853.066895</v>
+      </c>
+      <c r="T12" s="3">
+        <v>76164262211.796997</v>
+      </c>
+      <c r="U12" s="3">
+        <v>76172224499.505005</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>66</v>
       </c>
@@ -1596,8 +1865,35 @@
       <c r="L13" s="3">
         <v>896.81816506385803</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M13" s="3">
+        <v>900.37372994422901</v>
+      </c>
+      <c r="N13" s="3">
+        <v>131.198789834976</v>
+      </c>
+      <c r="O13" s="3">
+        <v>113.707083940505</v>
+      </c>
+      <c r="P13" s="3">
+        <v>106.06011509895301</v>
+      </c>
+      <c r="Q13" s="3">
+        <v>153.08726406097401</v>
+      </c>
+      <c r="R13" s="3">
+        <v>632.70238184928803</v>
+      </c>
+      <c r="S13" s="3">
+        <v>918.17074990272499</v>
+      </c>
+      <c r="T13" s="3">
+        <v>868.10124802589405</v>
+      </c>
+      <c r="U13" s="3">
+        <v>252.44026494026099</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>84</v>
       </c>
@@ -1634,8 +1930,35 @@
       <c r="L14" s="3">
         <v>5.36780805316764E-2</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M14" s="3">
+        <v>0.13957344871392799</v>
+      </c>
+      <c r="N14" s="3">
+        <v>7.2096942926495294E-2</v>
+      </c>
+      <c r="O14" s="3">
+        <v>3.6623316735996697E-2</v>
+      </c>
+      <c r="P14" s="3">
+        <v>3.6270064287868303E-2</v>
+      </c>
+      <c r="Q14" s="3">
+        <v>0.17372019824815901</v>
+      </c>
+      <c r="R14" s="3">
+        <v>8.7765403753448906E-2</v>
+      </c>
+      <c r="S14" s="3">
+        <v>8.7664105567513195E-2</v>
+      </c>
+      <c r="T14" s="3">
+        <v>9.1096398205322393E-2</v>
+      </c>
+      <c r="U14" s="3">
+        <v>9.0839974476340596E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>87</v>
       </c>
@@ -1672,8 +1995,35 @@
       <c r="L15" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M15" s="3">
+        <v>0</v>
+      </c>
+      <c r="N15" s="3">
+        <v>0</v>
+      </c>
+      <c r="O15" s="3">
+        <v>0</v>
+      </c>
+      <c r="P15" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="3">
+        <v>0</v>
+      </c>
+      <c r="R15" s="3">
+        <v>0</v>
+      </c>
+      <c r="S15" s="3">
+        <v>0</v>
+      </c>
+      <c r="T15" s="3">
+        <v>0</v>
+      </c>
+      <c r="U15" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>70</v>
       </c>
@@ -1710,8 +2060,35 @@
       <c r="L16" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M16" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="N16" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="O16" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="P16" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q16" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="R16" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="S16" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="T16" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="U16" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>68</v>
       </c>
@@ -1748,8 +2125,35 @@
       <c r="L17" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="N17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="O17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="P17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="R17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="S17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="T17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="U17" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>71</v>
       </c>
@@ -1786,8 +2190,35 @@
       <c r="L18" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="N18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="O18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="P18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="R18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="S18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="T18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="U18" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>69</v>
       </c>
@@ -1824,8 +2255,35 @@
       <c r="L19" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="N19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="O19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="P19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="R19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="S19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="T19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="U19" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>72</v>
       </c>
@@ -1862,8 +2320,35 @@
       <c r="L20" s="3">
         <v>330994041.82959598</v>
       </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M20" s="3">
+        <v>330994041.82959598</v>
+      </c>
+      <c r="N20" s="3">
+        <v>330994041.82959598</v>
+      </c>
+      <c r="O20" s="3">
+        <v>330994041.82959598</v>
+      </c>
+      <c r="P20" s="3">
+        <v>330994041.82959598</v>
+      </c>
+      <c r="Q20" s="3">
+        <v>329990111.97349298</v>
+      </c>
+      <c r="R20" s="3">
+        <v>329962306.48000401</v>
+      </c>
+      <c r="S20" s="3">
+        <v>329962306.48000401</v>
+      </c>
+      <c r="T20" s="3">
+        <v>327936407.60196102</v>
+      </c>
+      <c r="U20" s="3">
+        <v>329802700.98608899</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>73</v>
       </c>
@@ -1900,8 +2385,35 @@
       <c r="L21" s="3">
         <v>330184107.53514099</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M21" s="3">
+        <v>330791618.59320599</v>
+      </c>
+      <c r="N21" s="3">
+        <v>330795394.83175099</v>
+      </c>
+      <c r="O21" s="3">
+        <v>330894906.50536197</v>
+      </c>
+      <c r="P21" s="3">
+        <v>330818140.491925</v>
+      </c>
+      <c r="Q21" s="3">
+        <v>370935323.57837898</v>
+      </c>
+      <c r="R21" s="3">
+        <v>331270901.09938103</v>
+      </c>
+      <c r="S21" s="3">
+        <v>331270901.09938103</v>
+      </c>
+      <c r="T21" s="3">
+        <v>502522863.426009</v>
+      </c>
+      <c r="U21" s="3">
+        <v>331373976.621975</v>
+      </c>
+    </row>
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>75</v>
       </c>
@@ -1938,8 +2450,35 @@
       <c r="L22" s="3">
         <v>3.7125857943465202E-8</v>
       </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M22" s="3">
+        <v>3.14415160573844E-8</v>
+      </c>
+      <c r="N22" s="3">
+        <v>6.28830321147688E-8</v>
+      </c>
+      <c r="O22" s="3">
+        <v>1.5720758028692201E-7</v>
+      </c>
+      <c r="P22" s="3">
+        <v>3.1441516057384401E-7</v>
+      </c>
+      <c r="Q22" s="3">
+        <v>0</v>
+      </c>
+      <c r="R22" s="3">
+        <v>0</v>
+      </c>
+      <c r="S22" s="3">
+        <v>0</v>
+      </c>
+      <c r="T22" s="3">
+        <v>0</v>
+      </c>
+      <c r="U22" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -1976,8 +2515,35 @@
       <c r="L23" s="3">
         <v>67318308.771929905</v>
       </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M23" s="3">
+        <v>46014033.429824598</v>
+      </c>
+      <c r="N23" s="3">
+        <v>92028066.859649196</v>
+      </c>
+      <c r="O23" s="3">
+        <v>139576972.017544</v>
+      </c>
+      <c r="P23" s="3">
+        <v>332914698.42105299</v>
+      </c>
+      <c r="Q23" s="3">
+        <v>0</v>
+      </c>
+      <c r="R23" s="3">
+        <v>0</v>
+      </c>
+      <c r="S23" s="3">
+        <v>0</v>
+      </c>
+      <c r="T23" s="3">
+        <v>0</v>
+      </c>
+      <c r="U23" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>76</v>
       </c>
@@ -2014,8 +2580,35 @@
       <c r="L24" s="3">
         <v>276629624.84891802</v>
       </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M24" s="3">
+        <v>339499994.13276303</v>
+      </c>
+      <c r="N24" s="3">
+        <v>308064809.49084097</v>
+      </c>
+      <c r="O24" s="3">
+        <v>320638883.34761</v>
+      </c>
+      <c r="P24" s="3">
+        <v>364648141.84630102</v>
+      </c>
+      <c r="Q24" s="3">
+        <v>383216946.11499298</v>
+      </c>
+      <c r="R24" s="3">
+        <v>354416689.46027398</v>
+      </c>
+      <c r="S24" s="3">
+        <v>354416689.46027398</v>
+      </c>
+      <c r="T24" s="3">
+        <v>348956881.34175003</v>
+      </c>
+      <c r="U24" s="3">
+        <v>356272690.69953698</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>77</v>
       </c>
@@ -2030,8 +2623,17 @@
       <c r="J25" s="3"/>
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+      <c r="O25" s="3"/>
+      <c r="P25" s="3"/>
+      <c r="Q25" s="3"/>
+      <c r="R25" s="3"/>
+      <c r="S25" s="3"/>
+      <c r="T25" s="3"/>
+      <c r="U25" s="3"/>
+    </row>
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>2</v>
       </c>
@@ -2068,8 +2670,35 @@
       <c r="L26" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M26" s="3">
+        <v>0</v>
+      </c>
+      <c r="N26" s="3">
+        <v>0</v>
+      </c>
+      <c r="O26" s="3">
+        <v>0</v>
+      </c>
+      <c r="P26" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="3">
+        <v>58.083999999991399</v>
+      </c>
+      <c r="R26" s="3">
+        <v>19.954999999999899</v>
+      </c>
+      <c r="S26" s="3">
+        <v>19.954999999999899</v>
+      </c>
+      <c r="T26" s="3">
+        <v>59.317999999996601</v>
+      </c>
+      <c r="U26" s="3">
+        <v>18.084</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>0</v>
       </c>
@@ -2106,8 +2735,35 @@
       <c r="L27" s="3">
         <v>120</v>
       </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M27" s="3">
+        <v>120</v>
+      </c>
+      <c r="N27" s="3">
+        <v>120</v>
+      </c>
+      <c r="O27" s="3">
+        <v>160</v>
+      </c>
+      <c r="P27" s="3">
+        <v>160</v>
+      </c>
+      <c r="Q27" s="3">
+        <v>80</v>
+      </c>
+      <c r="R27" s="3">
+        <v>120</v>
+      </c>
+      <c r="S27" s="3">
+        <v>120</v>
+      </c>
+      <c r="T27" s="3">
+        <v>80</v>
+      </c>
+      <c r="U27" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>1</v>
       </c>
@@ -2144,8 +2800,35 @@
       <c r="L28" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M28" s="3">
+        <v>0</v>
+      </c>
+      <c r="N28" s="3">
+        <v>0</v>
+      </c>
+      <c r="O28" s="3">
+        <v>0</v>
+      </c>
+      <c r="P28" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="3">
+        <v>0</v>
+      </c>
+      <c r="R28" s="3">
+        <v>0</v>
+      </c>
+      <c r="S28" s="3">
+        <v>0</v>
+      </c>
+      <c r="T28" s="3">
+        <v>0</v>
+      </c>
+      <c r="U28" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>15</v>
       </c>
@@ -2160,8 +2843,17 @@
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M29" s="3"/>
+      <c r="N29" s="3"/>
+      <c r="O29" s="3"/>
+      <c r="P29" s="3"/>
+      <c r="Q29" s="3"/>
+      <c r="R29" s="3"/>
+      <c r="S29" s="3"/>
+      <c r="T29" s="3"/>
+      <c r="U29" s="3"/>
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>2</v>
       </c>
@@ -2198,8 +2890,35 @@
       <c r="L30" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M30" s="3">
+        <v>0</v>
+      </c>
+      <c r="N30" s="3">
+        <v>0</v>
+      </c>
+      <c r="O30" s="3">
+        <v>0</v>
+      </c>
+      <c r="P30" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="3">
+        <v>58.083999999991399</v>
+      </c>
+      <c r="R30" s="3">
+        <v>21.954999999999899</v>
+      </c>
+      <c r="S30" s="3">
+        <v>21.954999999999899</v>
+      </c>
+      <c r="T30" s="3">
+        <v>80.513649999996602</v>
+      </c>
+      <c r="U30" s="3">
+        <v>25.149650000000001</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>0</v>
       </c>
@@ -2236,8 +2955,35 @@
       <c r="L31" s="3">
         <v>120</v>
       </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M31" s="3">
+        <v>120</v>
+      </c>
+      <c r="N31" s="3">
+        <v>120</v>
+      </c>
+      <c r="O31" s="3">
+        <v>160</v>
+      </c>
+      <c r="P31" s="3">
+        <v>160</v>
+      </c>
+      <c r="Q31" s="3">
+        <v>80</v>
+      </c>
+      <c r="R31" s="3">
+        <v>120</v>
+      </c>
+      <c r="S31" s="3">
+        <v>120</v>
+      </c>
+      <c r="T31" s="3">
+        <v>80</v>
+      </c>
+      <c r="U31" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>1</v>
       </c>
@@ -2274,8 +3020,35 @@
       <c r="L32" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M32" s="3">
+        <v>0</v>
+      </c>
+      <c r="N32" s="3">
+        <v>0</v>
+      </c>
+      <c r="O32" s="3">
+        <v>0</v>
+      </c>
+      <c r="P32" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="3">
+        <v>0</v>
+      </c>
+      <c r="R32" s="3">
+        <v>0</v>
+      </c>
+      <c r="S32" s="3">
+        <v>0</v>
+      </c>
+      <c r="T32" s="3">
+        <v>0</v>
+      </c>
+      <c r="U32" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>78</v>
       </c>
@@ -2290,8 +3063,17 @@
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
       <c r="L33" s="3"/>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M33" s="3"/>
+      <c r="N33" s="3"/>
+      <c r="O33" s="3"/>
+      <c r="P33" s="3"/>
+      <c r="Q33" s="3"/>
+      <c r="R33" s="3"/>
+      <c r="S33" s="3"/>
+      <c r="T33" s="3"/>
+      <c r="U33" s="3"/>
+    </row>
+    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>2</v>
       </c>
@@ -2328,8 +3110,35 @@
       <c r="L34" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M34" s="3">
+        <v>0</v>
+      </c>
+      <c r="N34" s="3">
+        <v>0</v>
+      </c>
+      <c r="O34" s="3">
+        <v>0</v>
+      </c>
+      <c r="P34" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="3">
+        <v>87726210.480921701</v>
+      </c>
+      <c r="R34" s="3">
+        <v>52638916.897818103</v>
+      </c>
+      <c r="S34" s="3">
+        <v>52638916.897818103</v>
+      </c>
+      <c r="T34" s="3">
+        <v>235790216.63082799</v>
+      </c>
+      <c r="U34" s="3">
+        <v>60781955.0654651</v>
+      </c>
+    </row>
+    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>0</v>
       </c>
@@ -2366,8 +3175,35 @@
       <c r="L35" s="3">
         <v>276629624.84891802</v>
       </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M35" s="3">
+        <v>339499994.13276303</v>
+      </c>
+      <c r="N35" s="3">
+        <v>308064809.49084097</v>
+      </c>
+      <c r="O35" s="3">
+        <v>320638883.34761</v>
+      </c>
+      <c r="P35" s="3">
+        <v>364648141.84630102</v>
+      </c>
+      <c r="Q35" s="3">
+        <v>295490735.63407201</v>
+      </c>
+      <c r="R35" s="3">
+        <v>301777772.56245601</v>
+      </c>
+      <c r="S35" s="3">
+        <v>301777772.56245601</v>
+      </c>
+      <c r="T35" s="3">
+        <v>113166664.710921</v>
+      </c>
+      <c r="U35" s="3">
+        <v>295490735.63407201</v>
+      </c>
+    </row>
+    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>1</v>
       </c>
@@ -2404,8 +3240,35 @@
       <c r="L36" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M36" s="3">
+        <v>0</v>
+      </c>
+      <c r="N36" s="3">
+        <v>0</v>
+      </c>
+      <c r="O36" s="3">
+        <v>0</v>
+      </c>
+      <c r="P36" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="3">
+        <v>0</v>
+      </c>
+      <c r="R36" s="3">
+        <v>0</v>
+      </c>
+      <c r="S36" s="3">
+        <v>0</v>
+      </c>
+      <c r="T36" s="3">
+        <v>0</v>
+      </c>
+      <c r="U36" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
         <v>80</v>
       </c>
@@ -2420,8 +3283,17 @@
       <c r="J37" s="3"/>
       <c r="K37" s="3"/>
       <c r="L37" s="3"/>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M37" s="3"/>
+      <c r="N37" s="3"/>
+      <c r="O37" s="3"/>
+      <c r="P37" s="3"/>
+      <c r="Q37" s="3"/>
+      <c r="R37" s="3"/>
+      <c r="S37" s="3"/>
+      <c r="T37" s="3"/>
+      <c r="U37" s="3"/>
+    </row>
+    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>45</v>
       </c>
@@ -2436,8 +3308,17 @@
       <c r="J38" s="3"/>
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M38" s="3"/>
+      <c r="N38" s="3"/>
+      <c r="O38" s="3"/>
+      <c r="P38" s="3"/>
+      <c r="Q38" s="3"/>
+      <c r="R38" s="3"/>
+      <c r="S38" s="3"/>
+      <c r="T38" s="3"/>
+      <c r="U38" s="3"/>
+    </row>
+    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>2</v>
       </c>
@@ -2474,8 +3355,35 @@
       <c r="L39" s="3">
         <v>12.92135</v>
       </c>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M39" s="3">
+        <v>12.92135</v>
+      </c>
+      <c r="N39" s="3">
+        <v>12.92135</v>
+      </c>
+      <c r="O39" s="3">
+        <v>12.92135</v>
+      </c>
+      <c r="P39" s="3">
+        <v>12.92135</v>
+      </c>
+      <c r="Q39" s="3">
+        <v>58.083999999991399</v>
+      </c>
+      <c r="R39" s="3">
+        <v>26.876349999999899</v>
+      </c>
+      <c r="S39" s="3">
+        <v>26.876349999999899</v>
+      </c>
+      <c r="T39" s="3">
+        <v>75.150649999998507</v>
+      </c>
+      <c r="U39" s="3">
+        <v>28.02535</v>
+      </c>
+    </row>
+    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>0</v>
       </c>
@@ -2512,8 +3420,35 @@
       <c r="L40" s="3">
         <v>98.084000000000003</v>
       </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M40" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="N40" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="O40" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="P40" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="Q40" s="3">
+        <v>95.02</v>
+      </c>
+      <c r="R40" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="S40" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="T40" s="3">
+        <v>80</v>
+      </c>
+      <c r="U40" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>1</v>
       </c>
@@ -2550,8 +3485,35 @@
       <c r="L41" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M41" s="3">
+        <v>0</v>
+      </c>
+      <c r="N41" s="3">
+        <v>0</v>
+      </c>
+      <c r="O41" s="3">
+        <v>0</v>
+      </c>
+      <c r="P41" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="3">
+        <v>0</v>
+      </c>
+      <c r="R41" s="3">
+        <v>0</v>
+      </c>
+      <c r="S41" s="3">
+        <v>0</v>
+      </c>
+      <c r="T41" s="3">
+        <v>0</v>
+      </c>
+      <c r="U41" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>79</v>
       </c>
@@ -2588,8 +3550,35 @@
       <c r="L42" s="3">
         <v>1.4210854715202001E-14</v>
       </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M42" s="3">
+        <v>7.1054273576010003E-15</v>
+      </c>
+      <c r="N42" s="3">
+        <v>7.1054273576010003E-15</v>
+      </c>
+      <c r="O42" s="3">
+        <v>7.1054273576010003E-15</v>
+      </c>
+      <c r="P42" s="3">
+        <v>7.1054273576010003E-15</v>
+      </c>
+      <c r="Q42" s="3">
+        <v>0</v>
+      </c>
+      <c r="R42" s="3">
+        <v>0</v>
+      </c>
+      <c r="S42" s="3">
+        <v>0</v>
+      </c>
+      <c r="T42" s="3">
+        <v>0</v>
+      </c>
+      <c r="U42" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>46</v>
       </c>
@@ -2604,8 +3593,17 @@
       <c r="J43" s="3"/>
       <c r="K43" s="3"/>
       <c r="L43" s="3"/>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M43" s="3"/>
+      <c r="N43" s="3"/>
+      <c r="O43" s="3"/>
+      <c r="P43" s="3"/>
+      <c r="Q43" s="3"/>
+      <c r="R43" s="3"/>
+      <c r="S43" s="3"/>
+      <c r="T43" s="3"/>
+      <c r="U43" s="3"/>
+    </row>
+    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>0</v>
       </c>
@@ -2642,8 +3640,35 @@
       <c r="L44" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M44" s="3">
+        <v>0</v>
+      </c>
+      <c r="N44" s="3">
+        <v>0</v>
+      </c>
+      <c r="O44" s="3">
+        <v>0</v>
+      </c>
+      <c r="P44" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q44" s="3">
+        <v>24.474877192972698</v>
+      </c>
+      <c r="R44" s="3">
+        <v>0</v>
+      </c>
+      <c r="S44" s="3">
+        <v>0</v>
+      </c>
+      <c r="T44" s="3">
+        <v>42.482579824558499</v>
+      </c>
+      <c r="U44" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>24</v>
       </c>
@@ -2680,8 +3705,35 @@
       <c r="L45" s="3">
         <v>98.084000000000003</v>
       </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M45" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="N45" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="O45" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="P45" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="Q45" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="R45" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="S45" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="T45" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="U45" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>1</v>
       </c>
@@ -2718,8 +3770,35 @@
       <c r="L46" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M46" s="3">
+        <v>6</v>
+      </c>
+      <c r="N46" s="3">
+        <v>6</v>
+      </c>
+      <c r="O46" s="3">
+        <v>6</v>
+      </c>
+      <c r="P46" s="3">
+        <v>6</v>
+      </c>
+      <c r="Q46" s="3">
+        <v>6</v>
+      </c>
+      <c r="R46" s="3">
+        <v>6</v>
+      </c>
+      <c r="S46" s="3">
+        <v>6</v>
+      </c>
+      <c r="T46" s="3">
+        <v>6</v>
+      </c>
+      <c r="U46" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>23</v>
       </c>
@@ -2734,8 +3813,17 @@
       <c r="J47" s="3"/>
       <c r="K47" s="3"/>
       <c r="L47" s="3"/>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M47" s="3"/>
+      <c r="N47" s="3"/>
+      <c r="O47" s="3"/>
+      <c r="P47" s="3"/>
+      <c r="Q47" s="3"/>
+      <c r="R47" s="3"/>
+      <c r="S47" s="3"/>
+      <c r="T47" s="3"/>
+      <c r="U47" s="3"/>
+    </row>
+    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>2</v>
       </c>
@@ -2772,8 +3860,35 @@
       <c r="L48" s="3">
         <v>1938.2025000000001</v>
       </c>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M48" s="3">
+        <v>1938.2025000000001</v>
+      </c>
+      <c r="N48" s="3">
+        <v>1938.2025000000001</v>
+      </c>
+      <c r="O48" s="3">
+        <v>1938.2025000000001</v>
+      </c>
+      <c r="P48" s="3">
+        <v>1938.2025000000001</v>
+      </c>
+      <c r="Q48" s="3">
+        <v>9299.9844999957495</v>
+      </c>
+      <c r="R48" s="3">
+        <v>4511.9024999999901</v>
+      </c>
+      <c r="S48" s="3">
+        <v>4511.9024999999901</v>
+      </c>
+      <c r="T48" s="3">
+        <v>20203.975131574</v>
+      </c>
+      <c r="U48" s="3">
+        <v>4910.0439999999999</v>
+      </c>
+    </row>
+    <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>0</v>
       </c>
@@ -2810,8 +3925,35 @@
       <c r="L49" s="3">
         <v>7684705.8208288299</v>
       </c>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M49" s="3">
+        <v>7684705.8208288299</v>
+      </c>
+      <c r="N49" s="3">
+        <v>7684705.8208288299</v>
+      </c>
+      <c r="O49" s="3">
+        <v>7684705.8208288299</v>
+      </c>
+      <c r="P49" s="3">
+        <v>7684705.8208288299</v>
+      </c>
+      <c r="Q49" s="3">
+        <v>7677538.35377621</v>
+      </c>
+      <c r="R49" s="3">
+        <v>7682132.1208288204</v>
+      </c>
+      <c r="S49" s="3">
+        <v>7682132.1208288204</v>
+      </c>
+      <c r="T49" s="3">
+        <v>7667881.3627358396</v>
+      </c>
+      <c r="U49" s="3">
+        <v>7681733.9793288196</v>
+      </c>
+    </row>
+    <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>1</v>
       </c>
@@ -2848,8 +3990,35 @@
       <c r="L50" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M50" s="3">
+        <v>0</v>
+      </c>
+      <c r="N50" s="3">
+        <v>0</v>
+      </c>
+      <c r="O50" s="3">
+        <v>0</v>
+      </c>
+      <c r="P50" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q50" s="3">
+        <v>0</v>
+      </c>
+      <c r="R50" s="3">
+        <v>0</v>
+      </c>
+      <c r="S50" s="3">
+        <v>0</v>
+      </c>
+      <c r="T50" s="3">
+        <v>0</v>
+      </c>
+      <c r="U50" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>35</v>
       </c>
@@ -2886,8 +4055,35 @@
       <c r="L51" s="3">
         <v>3.7125857943465202E-12</v>
       </c>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M51" s="3">
+        <v>3.1441516057384401E-12</v>
+      </c>
+      <c r="N51" s="3">
+        <v>3.1441516057384401E-12</v>
+      </c>
+      <c r="O51" s="3">
+        <v>3.1441516057384401E-12</v>
+      </c>
+      <c r="P51" s="3">
+        <v>3.1441516057384401E-12</v>
+      </c>
+      <c r="Q51" s="3">
+        <v>0</v>
+      </c>
+      <c r="R51" s="3">
+        <v>0</v>
+      </c>
+      <c r="S51" s="3">
+        <v>0</v>
+      </c>
+      <c r="T51" s="3">
+        <v>0</v>
+      </c>
+      <c r="U51" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>22</v>
       </c>
@@ -2902,8 +4098,17 @@
       <c r="J52" s="3"/>
       <c r="K52" s="3"/>
       <c r="L52" s="3"/>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M52" s="3"/>
+      <c r="N52" s="3"/>
+      <c r="O52" s="3"/>
+      <c r="P52" s="3"/>
+      <c r="Q52" s="3"/>
+      <c r="R52" s="3"/>
+      <c r="S52" s="3"/>
+      <c r="T52" s="3"/>
+      <c r="U52" s="3"/>
+    </row>
+    <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>0</v>
       </c>
@@ -2940,8 +4145,35 @@
       <c r="L53" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M53" s="3">
+        <v>0</v>
+      </c>
+      <c r="N53" s="3">
+        <v>0</v>
+      </c>
+      <c r="O53" s="3">
+        <v>0</v>
+      </c>
+      <c r="P53" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q53" s="3">
+        <v>194.31494736827901</v>
+      </c>
+      <c r="R53" s="3">
+        <v>0</v>
+      </c>
+      <c r="S53" s="3">
+        <v>0</v>
+      </c>
+      <c r="T53" s="3">
+        <v>1441.3145385963601</v>
+      </c>
+      <c r="U53" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>24</v>
       </c>
@@ -2978,8 +4210,35 @@
       <c r="L54" s="3">
         <v>7685861.4146331698</v>
       </c>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M54" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+      <c r="N54" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+      <c r="O54" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+      <c r="P54" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+      <c r="Q54" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+      <c r="R54" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+      <c r="S54" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+      <c r="T54" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+      <c r="U54" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+    </row>
+    <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>1</v>
       </c>
@@ -3016,8 +4275,35 @@
       <c r="L55" s="3">
         <v>782.60869565217297</v>
       </c>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M55" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="N55" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="O55" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="P55" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="Q55" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="R55" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="S55" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="T55" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="U55" s="3">
+        <v>782.60869565217297</v>
+      </c>
+    </row>
+    <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>27</v>
       </c>
@@ -3032,8 +4318,17 @@
       <c r="J56" s="3"/>
       <c r="K56" s="3"/>
       <c r="L56" s="3"/>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M56" s="3"/>
+      <c r="N56" s="3"/>
+      <c r="O56" s="3"/>
+      <c r="P56" s="3"/>
+      <c r="Q56" s="3"/>
+      <c r="R56" s="3"/>
+      <c r="S56" s="3"/>
+      <c r="T56" s="3"/>
+      <c r="U56" s="3"/>
+    </row>
+    <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>2</v>
       </c>
@@ -3070,8 +4365,35 @@
       <c r="L57" s="3">
         <v>591730.69132540701</v>
       </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M57" s="3">
+        <v>591730.69132540701</v>
+      </c>
+      <c r="N57" s="3">
+        <v>591730.69132540701</v>
+      </c>
+      <c r="O57" s="3">
+        <v>591730.69132540701</v>
+      </c>
+      <c r="P57" s="3">
+        <v>591730.69132540701</v>
+      </c>
+      <c r="Q57" s="3">
+        <v>2839273.1190358298</v>
+      </c>
+      <c r="R57" s="3">
+        <v>1377477.9392338099</v>
+      </c>
+      <c r="S57" s="3">
+        <v>1377477.9392338099</v>
+      </c>
+      <c r="T57" s="3">
+        <v>6168247.2146886503</v>
+      </c>
+      <c r="U57" s="3">
+        <v>1499030.01908116</v>
+      </c>
+    </row>
+    <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>0</v>
       </c>
@@ -3108,8 +4430,35 @@
       <c r="L58" s="3">
         <v>330402311.13827002</v>
       </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M58" s="3">
+        <v>330402311.13827002</v>
+      </c>
+      <c r="N58" s="3">
+        <v>330402311.13827002</v>
+      </c>
+      <c r="O58" s="3">
+        <v>330402311.13827002</v>
+      </c>
+      <c r="P58" s="3">
+        <v>330402311.13827002</v>
+      </c>
+      <c r="Q58" s="3">
+        <v>327219838.05708098</v>
+      </c>
+      <c r="R58" s="3">
+        <v>328584828.54076999</v>
+      </c>
+      <c r="S58" s="3">
+        <v>328584828.54076999</v>
+      </c>
+      <c r="T58" s="3">
+        <v>322334999.496795</v>
+      </c>
+      <c r="U58" s="3">
+        <v>328303670.96700698</v>
+      </c>
+    </row>
+    <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>1</v>
       </c>
@@ -3146,8 +4495,35 @@
       <c r="L59" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M59" s="3">
+        <v>0</v>
+      </c>
+      <c r="N59" s="3">
+        <v>0</v>
+      </c>
+      <c r="O59" s="3">
+        <v>0</v>
+      </c>
+      <c r="P59" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q59" s="3">
+        <v>0</v>
+      </c>
+      <c r="R59" s="3">
+        <v>0</v>
+      </c>
+      <c r="S59" s="3">
+        <v>0</v>
+      </c>
+      <c r="T59" s="3">
+        <v>0</v>
+      </c>
+      <c r="U59" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>28</v>
       </c>
@@ -3162,8 +4538,17 @@
       <c r="J60" s="3"/>
       <c r="K60" s="3"/>
       <c r="L60" s="3"/>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M60" s="3"/>
+      <c r="N60" s="3"/>
+      <c r="O60" s="3"/>
+      <c r="P60" s="3"/>
+      <c r="Q60" s="3"/>
+      <c r="R60" s="3"/>
+      <c r="S60" s="3"/>
+      <c r="T60" s="3"/>
+      <c r="U60" s="3"/>
+    </row>
+    <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>0</v>
       </c>
@@ -3200,8 +4585,35 @@
       <c r="L61" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M61" s="3">
+        <v>0</v>
+      </c>
+      <c r="N61" s="3">
+        <v>0</v>
+      </c>
+      <c r="O61" s="3">
+        <v>0</v>
+      </c>
+      <c r="P61" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q61" s="3">
+        <v>68999.202625197096</v>
+      </c>
+      <c r="R61" s="3">
+        <v>0</v>
+      </c>
+      <c r="S61" s="3">
+        <v>0</v>
+      </c>
+      <c r="T61" s="3">
+        <v>566839.10952401999</v>
+      </c>
+      <c r="U61" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>24</v>
       </c>
@@ -3238,8 +4650,35 @@
       <c r="L62" s="3">
         <v>76858614146.318405</v>
       </c>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M62" s="3">
+        <v>76858614146.318405</v>
+      </c>
+      <c r="N62" s="3">
+        <v>153717228292.63599</v>
+      </c>
+      <c r="O62" s="3">
+        <v>384293070731.54797</v>
+      </c>
+      <c r="P62" s="3">
+        <v>768586141463.09595</v>
+      </c>
+      <c r="Q62" s="3">
+        <v>76858614146.318405</v>
+      </c>
+      <c r="R62" s="3">
+        <v>76858614146.318405</v>
+      </c>
+      <c r="S62" s="3">
+        <v>76858614146.318405</v>
+      </c>
+      <c r="T62" s="3">
+        <v>76858614146.318405</v>
+      </c>
+      <c r="U62" s="3">
+        <v>76858614146.318405</v>
+      </c>
+    </row>
+    <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>1</v>
       </c>
@@ -3276,8 +4715,35 @@
       <c r="L63" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M63" s="3">
+        <v>0</v>
+      </c>
+      <c r="N63" s="3">
+        <v>0</v>
+      </c>
+      <c r="O63" s="3">
+        <v>0</v>
+      </c>
+      <c r="P63" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q63" s="3">
+        <v>0</v>
+      </c>
+      <c r="R63" s="3">
+        <v>0</v>
+      </c>
+      <c r="S63" s="3">
+        <v>0</v>
+      </c>
+      <c r="T63" s="3">
+        <v>0</v>
+      </c>
+      <c r="U63" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="9" t="s">
         <v>81</v>
       </c>
@@ -3292,8 +4758,17 @@
       <c r="J64" s="3"/>
       <c r="K64" s="3"/>
       <c r="L64" s="3"/>
-    </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M64" s="3"/>
+      <c r="N64" s="3"/>
+      <c r="O64" s="3"/>
+      <c r="P64" s="3"/>
+      <c r="Q64" s="3"/>
+      <c r="R64" s="3"/>
+      <c r="S64" s="3"/>
+      <c r="T64" s="3"/>
+      <c r="U64" s="3"/>
+    </row>
+    <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>45</v>
       </c>
@@ -3308,8 +4783,17 @@
       <c r="J65" s="3"/>
       <c r="K65" s="3"/>
       <c r="L65" s="3"/>
-    </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M65" s="3"/>
+      <c r="N65" s="3"/>
+      <c r="O65" s="3"/>
+      <c r="P65" s="3"/>
+      <c r="Q65" s="3"/>
+      <c r="R65" s="3"/>
+      <c r="S65" s="3"/>
+      <c r="T65" s="3"/>
+      <c r="U65" s="3"/>
+    </row>
+    <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>2</v>
       </c>
@@ -3346,8 +4830,35 @@
       <c r="L66" s="3">
         <v>12.92135</v>
       </c>
-    </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M66" s="3">
+        <v>12.92135</v>
+      </c>
+      <c r="N66" s="3">
+        <v>12.92135</v>
+      </c>
+      <c r="O66" s="3">
+        <v>12.92135</v>
+      </c>
+      <c r="P66" s="3">
+        <v>12.92135</v>
+      </c>
+      <c r="Q66" s="3">
+        <v>58.083999999997602</v>
+      </c>
+      <c r="R66" s="3">
+        <v>26.876349999999899</v>
+      </c>
+      <c r="S66" s="3">
+        <v>26.876349999999899</v>
+      </c>
+      <c r="T66" s="3">
+        <v>75.150649999998507</v>
+      </c>
+      <c r="U66" s="3">
+        <v>28.02535</v>
+      </c>
+    </row>
+    <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>0</v>
       </c>
@@ -3384,8 +4895,35 @@
       <c r="L67" s="3">
         <v>80</v>
       </c>
-    </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M67" s="3">
+        <v>95.02</v>
+      </c>
+      <c r="N67" s="3">
+        <v>95.02</v>
+      </c>
+      <c r="O67" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="P67" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="Q67" s="3">
+        <v>80.653000000000006</v>
+      </c>
+      <c r="R67" s="3">
+        <v>95.02</v>
+      </c>
+      <c r="S67" s="3">
+        <v>95.02</v>
+      </c>
+      <c r="T67" s="3">
+        <v>40</v>
+      </c>
+      <c r="U67" s="3">
+        <v>95.02</v>
+      </c>
+    </row>
+    <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>1</v>
       </c>
@@ -3422,8 +4960,35 @@
       <c r="L68" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M68" s="3">
+        <v>0</v>
+      </c>
+      <c r="N68" s="3">
+        <v>0</v>
+      </c>
+      <c r="O68" s="3">
+        <v>0</v>
+      </c>
+      <c r="P68" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q68" s="3">
+        <v>0</v>
+      </c>
+      <c r="R68" s="3">
+        <v>0</v>
+      </c>
+      <c r="S68" s="3">
+        <v>0</v>
+      </c>
+      <c r="T68" s="3">
+        <v>0</v>
+      </c>
+      <c r="U68" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>79</v>
       </c>
@@ -3460,8 +5025,35 @@
       <c r="L69" s="3">
         <v>18.084</v>
       </c>
-    </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M69" s="3">
+        <v>18.084</v>
+      </c>
+      <c r="N69" s="3">
+        <v>18.084</v>
+      </c>
+      <c r="O69" s="3">
+        <v>16.744</v>
+      </c>
+      <c r="P69" s="3">
+        <v>15.87</v>
+      </c>
+      <c r="Q69" s="3">
+        <v>0</v>
+      </c>
+      <c r="R69" s="3">
+        <v>0</v>
+      </c>
+      <c r="S69" s="3">
+        <v>0</v>
+      </c>
+      <c r="T69" s="3">
+        <v>0</v>
+      </c>
+      <c r="U69" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>46</v>
       </c>
@@ -3476,8 +5068,17 @@
       <c r="J70" s="3"/>
       <c r="K70" s="3"/>
       <c r="L70" s="3"/>
-    </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M70" s="3"/>
+      <c r="N70" s="3"/>
+      <c r="O70" s="3"/>
+      <c r="P70" s="3"/>
+      <c r="Q70" s="3"/>
+      <c r="R70" s="3"/>
+      <c r="S70" s="3"/>
+      <c r="T70" s="3"/>
+      <c r="U70" s="3"/>
+    </row>
+    <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>0</v>
       </c>
@@ -3514,8 +5115,35 @@
       <c r="L71" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M71" s="3">
+        <v>0</v>
+      </c>
+      <c r="N71" s="3">
+        <v>0</v>
+      </c>
+      <c r="O71" s="3">
+        <v>0</v>
+      </c>
+      <c r="P71" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q71" s="3">
+        <v>24.474877192971501</v>
+      </c>
+      <c r="R71" s="3">
+        <v>0</v>
+      </c>
+      <c r="S71" s="3">
+        <v>0</v>
+      </c>
+      <c r="T71" s="3">
+        <v>38</v>
+      </c>
+      <c r="U71" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>24</v>
       </c>
@@ -3552,8 +5180,35 @@
       <c r="L72" s="3">
         <v>86.207999999999998</v>
       </c>
-    </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M72" s="3">
+        <v>95.02</v>
+      </c>
+      <c r="N72" s="3">
+        <v>95.02</v>
+      </c>
+      <c r="O72" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="P72" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="Q72" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="R72" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="S72" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="T72" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="U72" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>1</v>
       </c>
@@ -3590,8 +5245,35 @@
       <c r="L73" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M73" s="3">
+        <v>6</v>
+      </c>
+      <c r="N73" s="3">
+        <v>6</v>
+      </c>
+      <c r="O73" s="3">
+        <v>6</v>
+      </c>
+      <c r="P73" s="3">
+        <v>6</v>
+      </c>
+      <c r="Q73" s="3">
+        <v>6</v>
+      </c>
+      <c r="R73" s="3">
+        <v>6</v>
+      </c>
+      <c r="S73" s="3">
+        <v>6</v>
+      </c>
+      <c r="T73" s="3">
+        <v>6</v>
+      </c>
+      <c r="U73" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>23</v>
       </c>
@@ -3606,8 +5288,17 @@
       <c r="J74" s="3"/>
       <c r="K74" s="3"/>
       <c r="L74" s="3"/>
-    </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M74" s="3"/>
+      <c r="N74" s="3"/>
+      <c r="O74" s="3"/>
+      <c r="P74" s="3"/>
+      <c r="Q74" s="3"/>
+      <c r="R74" s="3"/>
+      <c r="S74" s="3"/>
+      <c r="T74" s="3"/>
+      <c r="U74" s="3"/>
+    </row>
+    <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>2</v>
       </c>
@@ -3644,8 +5335,35 @@
       <c r="L75" s="3">
         <v>2271.6272543858399</v>
       </c>
-    </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M75" s="3">
+        <v>3655.7006833333298</v>
+      </c>
+      <c r="N75" s="3">
+        <v>3672.1242096491201</v>
+      </c>
+      <c r="O75" s="3">
+        <v>3163.6046385964901</v>
+      </c>
+      <c r="P75" s="3">
+        <v>3147.1811122806998</v>
+      </c>
+      <c r="Q75" s="3">
+        <v>169282.024271809</v>
+      </c>
+      <c r="R75" s="3">
+        <v>10135.2488333333</v>
+      </c>
+      <c r="S75" s="3">
+        <v>10135.2488333333</v>
+      </c>
+      <c r="T75" s="3">
+        <v>701317.29067674396</v>
+      </c>
+      <c r="U75" s="3">
+        <v>11637.4284385964</v>
+      </c>
+    </row>
+    <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>0</v>
       </c>
@@ -3682,8 +5400,35 @@
       <c r="L76" s="3">
         <v>7677640.5651971698</v>
       </c>
-    </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M76" s="3">
+        <v>7678386.9193024999</v>
+      </c>
+      <c r="N76" s="3">
+        <v>7678370.4957761904</v>
+      </c>
+      <c r="O76" s="3">
+        <v>7680688.8792498698</v>
+      </c>
+      <c r="P76" s="3">
+        <v>7680167.6952323196</v>
+      </c>
+      <c r="Q76" s="3">
+        <v>7517556.31400433</v>
+      </c>
+      <c r="R76" s="3">
+        <v>7676508.7744954899</v>
+      </c>
+      <c r="S76" s="3">
+        <v>7676508.7744954899</v>
+      </c>
+      <c r="T76" s="3">
+        <v>6986753.9513499904</v>
+      </c>
+      <c r="U76" s="3">
+        <v>7675006.5948902201</v>
+      </c>
+    </row>
+    <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>1</v>
       </c>
@@ -3720,8 +5465,35 @@
       <c r="L77" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M77" s="3">
+        <v>0</v>
+      </c>
+      <c r="N77" s="3">
+        <v>0</v>
+      </c>
+      <c r="O77" s="3">
+        <v>0</v>
+      </c>
+      <c r="P77" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q77" s="3">
+        <v>0</v>
+      </c>
+      <c r="R77" s="3">
+        <v>0</v>
+      </c>
+      <c r="S77" s="3">
+        <v>0</v>
+      </c>
+      <c r="T77" s="3">
+        <v>0</v>
+      </c>
+      <c r="U77" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>35</v>
       </c>
@@ -3758,8 +5530,35 @@
       <c r="L78" s="3">
         <v>6731.8308771929796</v>
       </c>
-    </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M78" s="3">
+        <v>4601.4033429824503</v>
+      </c>
+      <c r="N78" s="3">
+        <v>4601.4033429824503</v>
+      </c>
+      <c r="O78" s="3">
+        <v>2791.5394403508699</v>
+      </c>
+      <c r="P78" s="3">
+        <v>3329.1469842105198</v>
+      </c>
+      <c r="Q78" s="3">
+        <v>0</v>
+      </c>
+      <c r="R78" s="3">
+        <v>0</v>
+      </c>
+      <c r="S78" s="3">
+        <v>0</v>
+      </c>
+      <c r="T78" s="3">
+        <v>0</v>
+      </c>
+      <c r="U78" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>22</v>
       </c>
@@ -3774,8 +5573,17 @@
       <c r="J79" s="3"/>
       <c r="K79" s="3"/>
       <c r="L79" s="3"/>
-    </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M79" s="3"/>
+      <c r="N79" s="3"/>
+      <c r="O79" s="3"/>
+      <c r="P79" s="3"/>
+      <c r="Q79" s="3"/>
+      <c r="R79" s="3"/>
+      <c r="S79" s="3"/>
+      <c r="T79" s="3"/>
+      <c r="U79" s="3"/>
+    </row>
+    <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>0</v>
       </c>
@@ -3812,8 +5620,35 @@
       <c r="L80" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M80" s="3">
+        <v>0</v>
+      </c>
+      <c r="N80" s="3">
+        <v>0</v>
+      </c>
+      <c r="O80" s="3">
+        <v>0</v>
+      </c>
+      <c r="P80" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q80" s="3">
+        <v>194.31494736824601</v>
+      </c>
+      <c r="R80" s="3">
+        <v>0</v>
+      </c>
+      <c r="S80" s="3">
+        <v>0</v>
+      </c>
+      <c r="T80" s="3">
+        <v>1427.21869824544</v>
+      </c>
+      <c r="U80" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>24</v>
       </c>
@@ -3850,8 +5685,35 @@
       <c r="L81" s="3">
         <v>7679129.5837559802</v>
       </c>
-    </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M81" s="3">
+        <v>7681260.0112901898</v>
+      </c>
+      <c r="N81" s="3">
+        <v>7681260.0112901898</v>
+      </c>
+      <c r="O81" s="3">
+        <v>7683069.8751928201</v>
+      </c>
+      <c r="P81" s="3">
+        <v>7682532.2676489502</v>
+      </c>
+      <c r="Q81" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+      <c r="R81" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+      <c r="S81" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+      <c r="T81" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+      <c r="U81" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+    </row>
+    <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>1</v>
       </c>
@@ -3888,8 +5750,35 @@
       <c r="L82" s="3">
         <v>782.60869565217297</v>
       </c>
-    </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M82" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="N82" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="O82" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="P82" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="Q82" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="R82" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="S82" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="T82" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="U82" s="3">
+        <v>782.60869565217297</v>
+      </c>
+    </row>
+    <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>27</v>
       </c>
@@ -3904,8 +5793,17 @@
       <c r="J83" s="3"/>
       <c r="K83" s="3"/>
       <c r="L83" s="3"/>
-    </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M83" s="3"/>
+      <c r="N83" s="3"/>
+      <c r="O83" s="3"/>
+      <c r="P83" s="3"/>
+      <c r="Q83" s="3"/>
+      <c r="R83" s="3"/>
+      <c r="S83" s="3"/>
+      <c r="T83" s="3"/>
+      <c r="U83" s="3"/>
+    </row>
+    <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>2</v>
       </c>
@@ -3942,8 +5840,35 @@
       <c r="L84" s="3">
         <v>693524.83327793004</v>
       </c>
-    </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M84" s="3">
+        <v>1116080.6430843</v>
+      </c>
+      <c r="N84" s="3">
+        <v>1121094.72421403</v>
+      </c>
+      <c r="O84" s="3">
+        <v>965844.36346406897</v>
+      </c>
+      <c r="P84" s="3">
+        <v>960830.28233434097</v>
+      </c>
+      <c r="Q84" s="3">
+        <v>51681580.872651801</v>
+      </c>
+      <c r="R84" s="3">
+        <v>3094278.2288761698</v>
+      </c>
+      <c r="S84" s="3">
+        <v>3094278.2288761698</v>
+      </c>
+      <c r="T84" s="3">
+        <v>214111252.69451299</v>
+      </c>
+      <c r="U84" s="3">
+        <v>3552891.7000265201</v>
+      </c>
+    </row>
+    <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>0</v>
       </c>
@@ -3980,8 +5905,35 @@
       <c r="L85" s="3">
         <v>329490582.70186299</v>
       </c>
-    </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M85" s="3">
+        <v>329675537.950122</v>
+      </c>
+      <c r="N85" s="3">
+        <v>329674300.10753798</v>
+      </c>
+      <c r="O85" s="3">
+        <v>329929062.14189899</v>
+      </c>
+      <c r="P85" s="3">
+        <v>329857310.20959097</v>
+      </c>
+      <c r="Q85" s="3">
+        <v>319322741.90834802</v>
+      </c>
+      <c r="R85" s="3">
+        <v>328176622.87050301</v>
+      </c>
+      <c r="S85" s="3">
+        <v>328176622.87050301</v>
+      </c>
+      <c r="T85" s="3">
+        <v>288973625.39870203</v>
+      </c>
+      <c r="U85" s="3">
+        <v>327821084.92194599</v>
+      </c>
+    </row>
+    <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>1</v>
       </c>
@@ -4018,8 +5970,35 @@
       <c r="L86" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M86" s="3">
+        <v>0</v>
+      </c>
+      <c r="N86" s="3">
+        <v>0</v>
+      </c>
+      <c r="O86" s="3">
+        <v>0</v>
+      </c>
+      <c r="P86" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q86" s="3">
+        <v>0</v>
+      </c>
+      <c r="R86" s="3">
+        <v>0</v>
+      </c>
+      <c r="S86" s="3">
+        <v>0</v>
+      </c>
+      <c r="T86" s="3">
+        <v>0</v>
+      </c>
+      <c r="U86" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>28</v>
       </c>
@@ -4034,8 +6013,17 @@
       <c r="J87" s="3"/>
       <c r="K87" s="3"/>
       <c r="L87" s="3"/>
-    </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M87" s="3"/>
+      <c r="N87" s="3"/>
+      <c r="O87" s="3"/>
+      <c r="P87" s="3"/>
+      <c r="Q87" s="3"/>
+      <c r="R87" s="3"/>
+      <c r="S87" s="3"/>
+      <c r="T87" s="3"/>
+      <c r="U87" s="3"/>
+    </row>
+    <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>0</v>
       </c>
@@ -4072,8 +6060,35 @@
       <c r="L88" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M88" s="3">
+        <v>0</v>
+      </c>
+      <c r="N88" s="3">
+        <v>0</v>
+      </c>
+      <c r="O88" s="3">
+        <v>0</v>
+      </c>
+      <c r="P88" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q88" s="3">
+        <v>68999.202625181701</v>
+      </c>
+      <c r="R88" s="3">
+        <v>0</v>
+      </c>
+      <c r="S88" s="3">
+        <v>0</v>
+      </c>
+      <c r="T88" s="3">
+        <v>562014.66720550996</v>
+      </c>
+      <c r="U88" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>24</v>
       </c>
@@ -4110,8 +6125,35 @@
       <c r="L89" s="3">
         <v>76791295837.546799</v>
       </c>
-    </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M89" s="3">
+        <v>76812600112.888901</v>
+      </c>
+      <c r="N89" s="3">
+        <v>153625200225.77701</v>
+      </c>
+      <c r="O89" s="3">
+        <v>384153493759.52899</v>
+      </c>
+      <c r="P89" s="3">
+        <v>768253226764.672</v>
+      </c>
+      <c r="Q89" s="3">
+        <v>76858614146.318405</v>
+      </c>
+      <c r="R89" s="3">
+        <v>76858614146.318405</v>
+      </c>
+      <c r="S89" s="3">
+        <v>76858614146.318405</v>
+      </c>
+      <c r="T89" s="3">
+        <v>76858614146.318405</v>
+      </c>
+      <c r="U89" s="3">
+        <v>76858614146.318405</v>
+      </c>
+    </row>
+    <row r="90" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>1</v>
       </c>
@@ -4146,6 +6188,33 @@
         <v>0</v>
       </c>
       <c r="L90" s="3">
+        <v>0</v>
+      </c>
+      <c r="M90" s="3">
+        <v>0</v>
+      </c>
+      <c r="N90" s="3">
+        <v>0</v>
+      </c>
+      <c r="O90" s="3">
+        <v>0</v>
+      </c>
+      <c r="P90" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q90" s="3">
+        <v>0</v>
+      </c>
+      <c r="R90" s="3">
+        <v>0</v>
+      </c>
+      <c r="S90" s="3">
+        <v>0</v>
+      </c>
+      <c r="T90" s="3">
+        <v>0</v>
+      </c>
+      <c r="U90" s="3">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update notes and results
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\Desktop\ongoing_projects\MVS\dev\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{108C223F-8AB0-463F-A0C4-78862CD8E2E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F6A4C4D-0CF0-4175-AE4B-3AD526E6959F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Experiments" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="250601_ops" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -59,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="96">
   <si>
     <t>Grid</t>
   </si>
@@ -344,6 +345,9 @@
   </si>
   <si>
     <t>Load shedding</t>
+  </si>
+  <si>
+    <t>updated cycle analysis</t>
   </si>
 </sst>
 </file>
@@ -746,28 +750,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J46"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.33203125" customWidth="1"/>
-    <col min="7" max="8" width="9.33203125" customWidth="1"/>
+    <col min="1" max="1" width="29.28515625" customWidth="1"/>
+    <col min="7" max="8" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -799,7 +803,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -831,7 +835,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -863,12 +867,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -900,7 +904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -932,7 +936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -964,7 +968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -996,179 +1000,179 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E12" s="1"/>
       <c r="H12" s="1"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>1</v>
       </c>
@@ -1181,17 +1185,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEB77188-4C54-4D05-A0BB-AB8E292CE16E}">
-  <dimension ref="A1:Z92"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AB92"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="42.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="13" width="18" bestFit="1" customWidth="1"/>
     <col min="14" max="16" width="19" bestFit="1" customWidth="1"/>
-    <col min="17" max="21" width="18" bestFit="1" customWidth="1"/>
-    <col min="22" max="26" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="17" max="28" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -1208,7 +1211,7 @@
         <v>250624</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -1224,8 +1227,11 @@
       <c r="Q2" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>62</v>
       </c>
@@ -1304,8 +1310,14 @@
       <c r="Z3" s="3">
         <v>150</v>
       </c>
-    </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA3" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="3">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>63</v>
       </c>
@@ -1384,8 +1396,14 @@
       <c r="Z4" s="3">
         <v>10000</v>
       </c>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA4" s="3">
+        <v>10000</v>
+      </c>
+      <c r="AB4" s="3">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>94</v>
       </c>
@@ -1426,8 +1444,14 @@
       <c r="Z5" s="3" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA5" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>57</v>
       </c>
@@ -1506,8 +1530,14 @@
       <c r="Z6" s="3">
         <v>8783</v>
       </c>
-    </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA6" s="3">
+        <v>8783</v>
+      </c>
+      <c r="AB6" s="3">
+        <v>8783</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>85</v>
       </c>
@@ -1586,8 +1616,14 @@
       <c r="Z7" s="3">
         <v>20</v>
       </c>
-    </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA7" s="3">
+        <v>20</v>
+      </c>
+      <c r="AB7" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>86</v>
       </c>
@@ -1666,8 +1702,14 @@
       <c r="Z8" s="3">
         <v>80</v>
       </c>
-    </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA8" s="3">
+        <v>80</v>
+      </c>
+      <c r="AB8" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>64</v>
       </c>
@@ -1746,8 +1788,14 @@
       <c r="Z9" s="3" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA9" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="AB9" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -1826,8 +1874,14 @@
       <c r="Z10" s="3" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA10" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="AB10" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>65</v>
       </c>
@@ -1906,8 +1960,14 @@
       <c r="Z11" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA11" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB11" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
@@ -1936,8 +1996,10 @@
       <c r="X12" s="3"/>
       <c r="Y12" s="3"/>
       <c r="Z12" s="3"/>
-    </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA12" s="3"/>
+      <c r="AB12" s="3"/>
+    </row>
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>67</v>
       </c>
@@ -2016,8 +2078,14 @@
       <c r="Z13" s="3">
         <v>53815076863.977097</v>
       </c>
-    </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA13" s="3">
+        <v>76172224499.505005</v>
+      </c>
+      <c r="AB13" s="3">
+        <v>76190255242.415695</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>66</v>
       </c>
@@ -2096,8 +2164,14 @@
       <c r="Z14" s="3">
         <v>28835.2907481193</v>
       </c>
-    </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA14" s="3">
+        <v>214.88944911956699</v>
+      </c>
+      <c r="AB14" s="3">
+        <v>7721.0674748420697</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>84</v>
       </c>
@@ -2176,8 +2250,14 @@
       <c r="Z15" s="3">
         <v>41.816229661111997</v>
       </c>
-    </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA15" s="3">
+        <v>9.0839974476340596E-2</v>
+      </c>
+      <c r="AB15" s="3">
+        <v>9.7156968396968094E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>87</v>
       </c>
@@ -2256,8 +2336,14 @@
       <c r="Z16" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA16" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB16" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>70</v>
       </c>
@@ -2336,8 +2422,14 @@
       <c r="Z17" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA17" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB17" s="3">
+        <v>149.99999999999699</v>
+      </c>
+    </row>
+    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>68</v>
       </c>
@@ -2416,8 +2508,14 @@
       <c r="Z18" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA18" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB18" s="3">
+        <v>149.99999999999901</v>
+      </c>
+    </row>
+    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>71</v>
       </c>
@@ -2496,8 +2594,14 @@
       <c r="Z19" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA19" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB19" s="3">
+        <v>149.99999999999699</v>
+      </c>
+    </row>
+    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>69</v>
       </c>
@@ -2576,8 +2680,14 @@
       <c r="Z20" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB20" s="3">
+        <v>149.99999999999901</v>
+      </c>
+    </row>
+    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>72</v>
       </c>
@@ -2656,8 +2766,14 @@
       <c r="Z21" s="3">
         <v>260665530.39608899</v>
       </c>
-    </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA21" s="3">
+        <v>329802700.98608899</v>
+      </c>
+      <c r="AB21" s="3">
+        <v>311781514.42136002</v>
+      </c>
+    </row>
+    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>73</v>
       </c>
@@ -2736,8 +2852,14 @@
       <c r="Z22" s="3">
         <v>162304542.981278</v>
       </c>
-    </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA22" s="3">
+        <v>331373976.621975</v>
+      </c>
+      <c r="AB22" s="3">
+        <v>314094436.03966099</v>
+      </c>
+    </row>
+    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>75</v>
       </c>
@@ -2816,8 +2938,14 @@
       <c r="Z23" s="3">
         <v>16985244411.447201</v>
       </c>
-    </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA23" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB23" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>74</v>
       </c>
@@ -2896,8 +3024,14 @@
       <c r="Z24" s="3">
         <v>46062139636.980499</v>
       </c>
-    </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA24" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB24" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>76</v>
       </c>
@@ -2976,8 +3110,14 @@
       <c r="Z25" s="3">
         <v>1920492.86937599</v>
       </c>
-    </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA25" s="3">
+        <v>356272690.69953698</v>
+      </c>
+      <c r="AB25" s="3">
+        <v>356114805.157166</v>
+      </c>
+    </row>
+    <row r="26" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>77</v>
       </c>
@@ -3006,8 +3146,10 @@
       <c r="X26" s="3"/>
       <c r="Y26" s="3"/>
       <c r="Z26" s="3"/>
-    </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA26" s="3"/>
+      <c r="AB26" s="3"/>
+    </row>
+    <row r="27" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>2</v>
       </c>
@@ -3086,8 +3228,14 @@
       <c r="Z27" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA27" s="3">
+        <v>18.084</v>
+      </c>
+      <c r="AB27" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>0</v>
       </c>
@@ -3166,8 +3314,14 @@
       <c r="Z28" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA28" s="3">
+        <v>120</v>
+      </c>
+      <c r="AB28" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="29" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>1</v>
       </c>
@@ -3246,8 +3400,14 @@
       <c r="Z29" s="3">
         <v>2</v>
       </c>
-    </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB29" s="3">
+        <v>18.083999999993299</v>
+      </c>
+    </row>
+    <row r="30" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>15</v>
       </c>
@@ -3276,8 +3436,10 @@
       <c r="X30" s="3"/>
       <c r="Y30" s="3"/>
       <c r="Z30" s="3"/>
-    </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA30" s="3"/>
+      <c r="AB30" s="3"/>
+    </row>
+    <row r="31" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>2</v>
       </c>
@@ -3356,8 +3518,14 @@
       <c r="Z31" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA31" s="3">
+        <v>25.149650000000001</v>
+      </c>
+      <c r="AB31" s="3">
+        <v>9.0656499999999802</v>
+      </c>
+    </row>
+    <row r="32" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>0</v>
       </c>
@@ -3436,8 +3604,14 @@
       <c r="Z32" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA32" s="3">
+        <v>120</v>
+      </c>
+      <c r="AB32" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="33" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>1</v>
       </c>
@@ -3516,8 +3690,14 @@
       <c r="Z33" s="3">
         <v>2</v>
       </c>
-    </row>
-    <row r="34" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB33" s="3">
+        <v>18.083999999993299</v>
+      </c>
+    </row>
+    <row r="34" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>78</v>
       </c>
@@ -3546,8 +3726,10 @@
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
       <c r="Z34" s="3"/>
-    </row>
-    <row r="35" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA34" s="3"/>
+      <c r="AB34" s="3"/>
+    </row>
+    <row r="35" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>2</v>
       </c>
@@ -3626,8 +3808,14 @@
       <c r="Z35" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA35" s="3">
+        <v>60781955.0654651</v>
+      </c>
+      <c r="AB35" s="3">
+        <v>37083265.102747403</v>
+      </c>
+    </row>
+    <row r="36" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>0</v>
       </c>
@@ -3706,8 +3894,14 @@
       <c r="Z36" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA36" s="3">
+        <v>295490735.63407201</v>
+      </c>
+      <c r="AB36" s="3">
+        <v>289203698.70568699</v>
+      </c>
+    </row>
+    <row r="37" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>1</v>
       </c>
@@ -3786,8 +3980,14 @@
       <c r="Z37" s="3">
         <v>1920492.86937599</v>
       </c>
-    </row>
-    <row r="38" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB37" s="3">
+        <v>29827841.348731399</v>
+      </c>
+    </row>
+    <row r="38" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
         <v>80</v>
       </c>
@@ -3816,8 +4016,10 @@
       <c r="X38" s="3"/>
       <c r="Y38" s="3"/>
       <c r="Z38" s="3"/>
-    </row>
-    <row r="39" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA38" s="3"/>
+      <c r="AB38" s="3"/>
+    </row>
+    <row r="39" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>45</v>
       </c>
@@ -3846,8 +4048,10 @@
       <c r="X39" s="3"/>
       <c r="Y39" s="3"/>
       <c r="Z39" s="3"/>
-    </row>
-    <row r="40" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA39" s="3"/>
+      <c r="AB39" s="3"/>
+    </row>
+    <row r="40" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>2</v>
       </c>
@@ -3926,8 +4130,14 @@
       <c r="Z40" s="3">
         <v>12.921350000002301</v>
       </c>
-    </row>
-    <row r="41" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA40" s="3">
+        <v>28.02535</v>
+      </c>
+      <c r="AB40" s="3">
+        <v>21.986999999999899</v>
+      </c>
+    </row>
+    <row r="41" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>0</v>
       </c>
@@ -4006,8 +4216,14 @@
       <c r="Z41" s="3">
         <v>74</v>
       </c>
-    </row>
-    <row r="42" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA41" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AB41" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="42" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>1</v>
       </c>
@@ -4086,8 +4302,14 @@
       <c r="Z42" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="43" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB42" s="3">
+        <v>18.083999999993299</v>
+      </c>
+    </row>
+    <row r="43" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>79</v>
       </c>
@@ -4166,8 +4388,14 @@
       <c r="Z43" s="3">
         <v>98.084000000000003</v>
       </c>
-    </row>
-    <row r="44" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA43" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB43" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>46</v>
       </c>
@@ -4196,8 +4424,10 @@
       <c r="X44" s="3"/>
       <c r="Y44" s="3"/>
       <c r="Z44" s="3"/>
-    </row>
-    <row r="45" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA44" s="3"/>
+      <c r="AB44" s="3"/>
+    </row>
+    <row r="45" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>0</v>
       </c>
@@ -4276,8 +4506,14 @@
       <c r="Z45" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA45" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB45" s="3">
+        <v>6.0729649122806801</v>
+      </c>
+    </row>
+    <row r="46" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>24</v>
       </c>
@@ -4356,8 +4592,14 @@
       <c r="Z46" s="3">
         <v>80.653000000000006</v>
       </c>
-    </row>
-    <row r="47" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA46" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AB46" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="47" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>1</v>
       </c>
@@ -4436,8 +4678,14 @@
       <c r="Z47" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="48" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA47" s="3">
+        <v>6</v>
+      </c>
+      <c r="AB47" s="3">
+        <v>18.083999999993299</v>
+      </c>
+    </row>
+    <row r="48" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>23</v>
       </c>
@@ -4466,8 +4714,10 @@
       <c r="X48" s="3"/>
       <c r="Y48" s="3"/>
       <c r="Z48" s="3"/>
-    </row>
-    <row r="49" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA48" s="3"/>
+      <c r="AB48" s="3"/>
+    </row>
+    <row r="49" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>2</v>
       </c>
@@ -4546,8 +4796,14 @@
       <c r="Z49" s="3">
         <v>26412.406416667302</v>
       </c>
-    </row>
-    <row r="50" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA49" s="3">
+        <v>4910.0439999999999</v>
+      </c>
+      <c r="AB49" s="3">
+        <v>3751.33249999996</v>
+      </c>
+    </row>
+    <row r="50" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>0</v>
       </c>
@@ -4626,8 +4882,14 @@
       <c r="Z50" s="3">
         <v>5964037.8031871403</v>
       </c>
-    </row>
-    <row r="51" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA50" s="3">
+        <v>7681733.9793288196</v>
+      </c>
+      <c r="AB50" s="3">
+        <v>7723147.0301441904</v>
+      </c>
+    </row>
+    <row r="51" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>1</v>
       </c>
@@ -4706,8 +4968,14 @@
       <c r="Z51" s="3">
         <v>13771.3531754377</v>
       </c>
-    </row>
-    <row r="52" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB51" s="3">
+        <v>225883.31279995001</v>
+      </c>
+    </row>
+    <row r="52" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>35</v>
       </c>
@@ -4786,8 +5054,14 @@
       <c r="Z52" s="3">
         <v>1698524.44114494</v>
       </c>
-    </row>
-    <row r="53" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA52" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB52" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>22</v>
       </c>
@@ -4816,8 +5090,10 @@
       <c r="X53" s="3"/>
       <c r="Y53" s="3"/>
       <c r="Z53" s="3"/>
-    </row>
-    <row r="54" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA53" s="3"/>
+      <c r="AB53" s="3"/>
+    </row>
+    <row r="54" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>0</v>
       </c>
@@ -4896,8 +5172,14 @@
       <c r="Z54" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="55" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB54" s="3">
+        <v>44.891245614034702</v>
+      </c>
+    </row>
+    <row r="55" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>24</v>
       </c>
@@ -4976,8 +5258,14 @@
       <c r="Z55" s="3">
         <v>5987336.9734887797</v>
       </c>
-    </row>
-    <row r="56" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA55" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+      <c r="AB55" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+    </row>
+    <row r="56" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>1</v>
       </c>
@@ -5056,8 +5344,14 @@
       <c r="Z56" s="3">
         <v>16884.589290453299</v>
       </c>
-    </row>
-    <row r="57" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA56" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="AB56" s="3">
+        <v>266875.36956515198</v>
+      </c>
+    </row>
+    <row r="57" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>27</v>
       </c>
@@ -5086,8 +5380,10 @@
       <c r="X57" s="3"/>
       <c r="Y57" s="3"/>
       <c r="Z57" s="3"/>
-    </row>
-    <row r="58" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA57" s="3"/>
+      <c r="AB57" s="3"/>
+    </row>
+    <row r="58" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>2</v>
       </c>
@@ -5166,8 +5462,14 @@
       <c r="Z58" s="3">
         <v>8063673.1757917404</v>
       </c>
-    </row>
-    <row r="59" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA58" s="3">
+        <v>1499030.01908116</v>
+      </c>
+      <c r="AB58" s="3">
+        <v>1145276.9117862701</v>
+      </c>
+    </row>
+    <row r="59" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>0</v>
       </c>
@@ -5246,8 +5548,14 @@
       <c r="Z59" s="3">
         <v>252601857.22029799</v>
       </c>
-    </row>
-    <row r="60" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA59" s="3">
+        <v>328303670.96700698</v>
+      </c>
+      <c r="AB59" s="3">
+        <v>310651371.83779597</v>
+      </c>
+    </row>
+    <row r="60" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>1</v>
       </c>
@@ -5326,8 +5634,14 @@
       <c r="Z60" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="61" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA60" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB60" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>28</v>
       </c>
@@ -5356,8 +5670,10 @@
       <c r="X61" s="3"/>
       <c r="Y61" s="3"/>
       <c r="Z61" s="3"/>
-    </row>
-    <row r="62" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA61" s="3"/>
+      <c r="AB61" s="3"/>
+    </row>
+    <row r="62" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>0</v>
       </c>
@@ -5436,8 +5752,14 @@
       <c r="Z62" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA62" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB62" s="3">
+        <v>15134.328222105099</v>
+      </c>
+    </row>
+    <row r="63" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>24</v>
       </c>
@@ -5516,8 +5838,14 @@
       <c r="Z63" s="3">
         <v>59873369734.866302</v>
       </c>
-    </row>
-    <row r="64" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA63" s="3">
+        <v>76858614146.318405</v>
+      </c>
+      <c r="AB63" s="3">
+        <v>76858614146.318405</v>
+      </c>
+    </row>
+    <row r="64" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>1</v>
       </c>
@@ -5596,8 +5924,14 @@
       <c r="Z64" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="65" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA64" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB64" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A65" s="9" t="s">
         <v>81</v>
       </c>
@@ -5626,8 +5960,10 @@
       <c r="X65" s="3"/>
       <c r="Y65" s="3"/>
       <c r="Z65" s="3"/>
-    </row>
-    <row r="66" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA65" s="3"/>
+      <c r="AB65" s="3"/>
+    </row>
+    <row r="66" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>45</v>
       </c>
@@ -5656,8 +5992,10 @@
       <c r="X66" s="3"/>
       <c r="Y66" s="3"/>
       <c r="Z66" s="3"/>
-    </row>
-    <row r="67" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA66" s="3"/>
+      <c r="AB66" s="3"/>
+    </row>
+    <row r="67" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>2</v>
       </c>
@@ -5736,8 +6074,14 @@
       <c r="Z67" s="3">
         <v>12.9213500000025</v>
       </c>
-    </row>
-    <row r="68" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA67" s="3">
+        <v>28.02535</v>
+      </c>
+      <c r="AB67" s="3">
+        <v>21.986999999999998</v>
+      </c>
+    </row>
+    <row r="68" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>0</v>
       </c>
@@ -5816,8 +6160,14 @@
       <c r="Z68" s="3">
         <v>36</v>
       </c>
-    </row>
-    <row r="69" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA68" s="3">
+        <v>95.02</v>
+      </c>
+      <c r="AB68" s="3">
+        <v>95.02</v>
+      </c>
+    </row>
+    <row r="69" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>1</v>
       </c>
@@ -5896,8 +6246,14 @@
       <c r="Z69" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="70" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA69" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB69" s="3">
+        <v>18.083999999993299</v>
+      </c>
+    </row>
+    <row r="70" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>79</v>
       </c>
@@ -5976,8 +6332,14 @@
       <c r="Z70" s="3">
         <v>98.084000000000003</v>
       </c>
-    </row>
-    <row r="71" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA70" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB70" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>46</v>
       </c>
@@ -6006,8 +6368,10 @@
       <c r="X71" s="3"/>
       <c r="Y71" s="3"/>
       <c r="Z71" s="3"/>
-    </row>
-    <row r="72" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA71" s="3"/>
+      <c r="AB71" s="3"/>
+    </row>
+    <row r="72" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>0</v>
       </c>
@@ -6086,8 +6450,14 @@
       <c r="Z72" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="73" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB72" s="3">
+        <v>6.0729649122806801</v>
+      </c>
+    </row>
+    <row r="73" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>24</v>
       </c>
@@ -6166,8 +6536,14 @@
       <c r="Z73" s="3">
         <v>54.9213500000048</v>
       </c>
-    </row>
-    <row r="74" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA73" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AB73" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="74" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>1</v>
       </c>
@@ -6246,8 +6622,14 @@
       <c r="Z74" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="75" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA74" s="3">
+        <v>6</v>
+      </c>
+      <c r="AB74" s="3">
+        <v>18.083999999993299</v>
+      </c>
+    </row>
+    <row r="75" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>23</v>
       </c>
@@ -6276,8 +6658,10 @@
       <c r="X75" s="3"/>
       <c r="Y75" s="3"/>
       <c r="Z75" s="3"/>
-    </row>
-    <row r="76" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA75" s="3"/>
+      <c r="AB75" s="3"/>
+    </row>
+    <row r="76" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>2</v>
       </c>
@@ -6356,8 +6740,14 @@
       <c r="Z76" s="3">
         <v>129573.199616677</v>
       </c>
-    </row>
-    <row r="77" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA76" s="3">
+        <v>11637.4284385964</v>
+      </c>
+      <c r="AB76" s="3">
+        <v>11753.176635087601</v>
+      </c>
+    </row>
+    <row r="77" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>0</v>
       </c>
@@ -6436,8 +6826,14 @@
       <c r="Z77" s="3">
         <v>2962920.4938157098</v>
       </c>
-    </row>
-    <row r="78" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA77" s="3">
+        <v>7675006.5948902201</v>
+      </c>
+      <c r="AB77" s="3">
+        <v>7715145.1860090699</v>
+      </c>
+    </row>
+    <row r="78" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>1</v>
       </c>
@@ -6516,8 +6912,14 @@
       <c r="Z78" s="3">
         <v>70409.784421051794</v>
       </c>
-    </row>
-    <row r="79" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB78" s="3">
+        <v>225883.31279994699</v>
+      </c>
+    </row>
+    <row r="79" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>35</v>
       </c>
@@ -6596,8 +6998,14 @@
       <c r="Z79" s="3">
         <v>4606213.96369908</v>
       </c>
-    </row>
-    <row r="80" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA79" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB79" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>22</v>
       </c>
@@ -6626,8 +7034,10 @@
       <c r="X80" s="3"/>
       <c r="Y80" s="3"/>
       <c r="Z80" s="3"/>
-    </row>
-    <row r="81" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA80" s="3"/>
+      <c r="AB80" s="3"/>
+    </row>
+    <row r="81" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>0</v>
       </c>
@@ -6706,8 +7116,14 @@
       <c r="Z81" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="82" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB81" s="3">
+        <v>44.891245614034801</v>
+      </c>
+    </row>
+    <row r="82" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>24</v>
       </c>
@@ -6786,8 +7202,14 @@
       <c r="Z82" s="3">
         <v>3079647.45093212</v>
       </c>
-    </row>
-    <row r="83" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA82" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+      <c r="AB82" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+    </row>
+    <row r="83" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>1</v>
       </c>
@@ -6866,8 +7288,14 @@
       <c r="Z83" s="3">
         <v>83256.0269210353</v>
       </c>
-    </row>
-    <row r="84" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA83" s="3">
+        <v>782.60869565217297</v>
+      </c>
+      <c r="AB83" s="3">
+        <v>266875.36956515198</v>
+      </c>
+    </row>
+    <row r="84" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>27</v>
       </c>
@@ -6896,8 +7324,10 @@
       <c r="X84" s="3"/>
       <c r="Y84" s="3"/>
       <c r="Z84" s="3"/>
-    </row>
-    <row r="85" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA84" s="3"/>
+      <c r="AB84" s="3"/>
+    </row>
+    <row r="85" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>2</v>
       </c>
@@ -6976,8 +7406,14 @@
       <c r="Z85" s="3">
         <v>39558528.578106299</v>
       </c>
-    </row>
-    <row r="86" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA85" s="3">
+        <v>3552891.7000265201</v>
+      </c>
+      <c r="AB85" s="3">
+        <v>3588229.4732103799</v>
+      </c>
+    </row>
+    <row r="86" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>0</v>
       </c>
@@ -7056,8 +7492,14 @@
       <c r="Z86" s="3">
         <v>122746014.403165</v>
       </c>
-    </row>
-    <row r="87" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA86" s="3">
+        <v>327821084.92194599</v>
+      </c>
+      <c r="AB86" s="3">
+        <v>310521340.89467198</v>
+      </c>
+    </row>
+    <row r="87" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>1</v>
       </c>
@@ -7136,8 +7578,14 @@
       <c r="Z87" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="88" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA87" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB87" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>28</v>
       </c>
@@ -7166,8 +7614,10 @@
       <c r="X88" s="3"/>
       <c r="Y88" s="3"/>
       <c r="Z88" s="3"/>
-    </row>
-    <row r="89" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA88" s="3"/>
+      <c r="AB88" s="3"/>
+    </row>
+    <row r="89" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>0</v>
       </c>
@@ -7246,8 +7696,14 @@
       <c r="Z89" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="90" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB89" s="3">
+        <v>15134.328222105099</v>
+      </c>
+    </row>
+    <row r="90" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>24</v>
       </c>
@@ -7326,8 +7782,14 @@
       <c r="Z90" s="3">
         <v>30796474509.321899</v>
       </c>
-    </row>
-    <row r="91" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA90" s="3">
+        <v>76858614146.318405</v>
+      </c>
+      <c r="AB90" s="3">
+        <v>76858614146.318405</v>
+      </c>
+    </row>
+    <row r="91" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>1</v>
       </c>
@@ -7406,8 +7868,14 @@
       <c r="Z91" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="92" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA91" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB91" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:28" x14ac:dyDescent="0.25">
       <c r="V92" s="3"/>
     </row>
   </sheetData>
@@ -7418,30 +7886,30 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00CD46BB-A2D1-4791-8AAC-69869F785713}">
   <dimension ref="A1:M52"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="4" max="5" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="9.33203125" customWidth="1"/>
-    <col min="11" max="13" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.28515625" customWidth="1"/>
+    <col min="11" max="13" width="19.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -7461,7 +7929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -7475,7 +7943,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>36</v>
       </c>
@@ -7489,7 +7957,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>37</v>
       </c>
@@ -7503,12 +7971,12 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -7549,7 +8017,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -7590,7 +8058,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -7631,12 +8099,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -7677,7 +8145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -7718,7 +8186,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -7759,7 +8227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -7800,14 +8268,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E17" s="3"/>
       <c r="H17" s="1"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>10</v>
       </c>
@@ -7827,7 +8295,7 @@
         <v>-13456893997.0168</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -7847,7 +8315,7 @@
         <v>34.491999864578197</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -7867,7 +8335,7 @@
         <v>8.0815127926575099E-5</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -7887,7 +8355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>11</v>
       </c>
@@ -7897,7 +8365,7 @@
       <c r="L22" s="3"/>
       <c r="M22" s="3"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>2</v>
       </c>
@@ -7917,7 +8385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -7937,7 +8405,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>1</v>
       </c>
@@ -7957,7 +8425,7 @@
         <v>15.427141887890601</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>29</v>
       </c>
@@ -7977,7 +8445,7 @@
         <v>98.084000000000003</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>30</v>
       </c>
@@ -7997,7 +8465,7 @@
         <v>2.65685811210931</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>15</v>
       </c>
@@ -8007,7 +8475,7 @@
       <c r="L28" s="3"/>
       <c r="M28" s="3"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>2</v>
       </c>
@@ -8027,7 +8495,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>0</v>
       </c>
@@ -8047,7 +8515,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>1</v>
       </c>
@@ -8067,7 +8535,7 @@
         <v>15.427141887890601</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>16</v>
       </c>
@@ -8077,7 +8545,7 @@
       <c r="L32" s="3"/>
       <c r="M32" s="3"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -8097,7 +8565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>0</v>
       </c>
@@ -8117,7 +8585,7 @@
         <v>249617260.626542</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>1</v>
       </c>
@@ -8137,7 +8605,7 @@
         <v>30544228.586336799</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>23</v>
       </c>
@@ -8147,7 +8615,7 @@
       <c r="L36" s="3"/>
       <c r="M36" s="3"/>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>2</v>
       </c>
@@ -8167,7 +8635,7 @@
         <v>3421.3094646414202</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>0</v>
       </c>
@@ -8187,7 +8655,7 @@
         <v>1772151.2791056901</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>1</v>
       </c>
@@ -8207,7 +8675,7 @@
         <v>7524.5956312832805</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>22</v>
       </c>
@@ -8217,7 +8685,7 @@
       <c r="L40" s="3"/>
       <c r="M40" s="3"/>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>0</v>
       </c>
@@ -8237,7 +8705,7 @@
         <v>392888.13096246601</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>24</v>
       </c>
@@ -8257,7 +8725,7 @@
         <v>1381318.93552733</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>35</v>
       </c>
@@ -8277,7 +8745,7 @@
         <v>2522.7416867100901</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -8297,7 +8765,7 @@
         <v>8890.1177118186097</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>27</v>
       </c>
@@ -8307,7 +8775,7 @@
       <c r="L45" s="3"/>
       <c r="M45" s="3"/>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>2</v>
       </c>
@@ -8327,7 +8795,7 @@
         <v>1044521.3102090301</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>0</v>
       </c>
@@ -8347,7 +8815,7 @@
         <v>96512651.699123099</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>1</v>
       </c>
@@ -8367,7 +8835,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>28</v>
       </c>
@@ -8377,7 +8845,7 @@
       <c r="L49" s="3"/>
       <c r="M49" s="3"/>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>0</v>
       </c>
@@ -8397,7 +8865,7 @@
         <v>21423303.9657369</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>24</v>
       </c>
@@ -8417,7 +8885,7 @@
         <v>13813189355.2733</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>1</v>
       </c>
@@ -8446,30 +8914,30 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4317E227-4F2F-4766-80E7-4A0C11DC1BA8}">
   <dimension ref="A1:J48"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.33203125" customWidth="1"/>
-    <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="9.33203125" customWidth="1"/>
+    <col min="1" max="1" width="29.28515625" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -8480,12 +8948,12 @@
         <v>6.8500000000000005E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -8517,7 +8985,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -8549,7 +9017,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -8581,12 +9049,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -8618,7 +9086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -8650,7 +9118,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -8682,7 +9150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -8714,14 +9182,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E14" s="3"/>
       <c r="H14" s="1"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -8732,7 +9200,7 @@
         <v>-566684168.67891097</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>32</v>
       </c>
@@ -8743,7 +9211,7 @@
         <v>2.5789999961853001</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -8754,7 +9222,7 @@
         <v>9.2925621330612702E-5</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>31</v>
       </c>
@@ -8765,14 +9233,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>2</v>
       </c>
@@ -8783,7 +9251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>0</v>
       </c>
@@ -8794,7 +9262,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>1</v>
       </c>
@@ -8805,7 +9273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>29</v>
       </c>
@@ -8816,7 +9284,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>30</v>
       </c>
@@ -8827,14 +9295,14 @@
         <v>58.084000000000003</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>2</v>
       </c>
@@ -8845,7 +9313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>0</v>
       </c>
@@ -8856,7 +9324,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>1</v>
       </c>
@@ -8867,14 +9335,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>2</v>
       </c>
@@ -8885,7 +9353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>0</v>
       </c>
@@ -8896,7 +9364,7 @@
         <v>93383545.771093696</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>1</v>
       </c>
@@ -8907,14 +9375,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>2</v>
       </c>
@@ -8925,7 +9393,7 @@
         <v>10839.670693578801</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>0</v>
       </c>
@@ -8936,7 +9404,7 @@
         <v>755352.36146108399</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>1</v>
       </c>
@@ -8947,14 +9415,14 @@
         <v>8697.9159292100794</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>0</v>
       </c>
@@ -8965,7 +9433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>24</v>
       </c>
@@ -8976,7 +9444,7 @@
         <v>764613.58238300995</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>1</v>
       </c>
@@ -8987,14 +9455,14 @@
         <v>10276.3657008625</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>2</v>
       </c>
@@ -9005,7 +9473,7 @@
         <v>1636903.5360916599</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>0</v>
       </c>
@@ -9016,7 +9484,7 @@
         <v>14194345.611482101</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -9027,14 +9495,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>28</v>
       </c>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>0</v>
       </c>
@@ -9045,7 +9513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>24</v>
       </c>
@@ -9056,7 +9524,7 @@
         <v>675898963.597579</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>1</v>
       </c>
@@ -9076,19 +9544,19 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CDE5EF9-418E-4572-AF84-E6DEF6E71829}">
   <dimension ref="A1:M49"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="2" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="19.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -9096,12 +9564,12 @@
         <v>45810</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>52</v>
       </c>
@@ -9118,7 +9586,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>51</v>
       </c>
@@ -9132,13 +9600,13 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>44</v>
       </c>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -9170,7 +9638,7 @@
         <v>12.920999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -9202,7 +9670,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -9234,7 +9702,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -9247,7 +9715,7 @@
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -9279,7 +9747,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -9311,7 +9779,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -9343,7 +9811,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>47</v>
       </c>
@@ -9375,7 +9843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>39</v>
       </c>
@@ -9389,7 +9857,7 @@
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>40</v>
       </c>
@@ -9421,7 +9889,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>42</v>
       </c>
@@ -9435,7 +9903,7 @@
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -9467,7 +9935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>9</v>
       </c>
@@ -9481,7 +9949,7 @@
       <c r="I18" s="3"/>
       <c r="J18" s="3"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>48</v>
       </c>
@@ -9516,7 +9984,7 @@
       <c r="L19" s="3"/>
       <c r="M19" s="3"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -9551,7 +10019,7 @@
       <c r="L20" s="3"/>
       <c r="M20" s="3"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>17</v>
       </c>
@@ -9586,7 +10054,7 @@
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -9621,7 +10089,7 @@
       <c r="L22" s="3"/>
       <c r="M22" s="3"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>41</v>
       </c>
@@ -9656,7 +10124,7 @@
       <c r="L23" s="3"/>
       <c r="M23" s="3"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>45</v>
       </c>
@@ -9673,7 +10141,7 @@
       <c r="L24" s="3"/>
       <c r="M24" s="3"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>2</v>
       </c>
@@ -9708,7 +10176,7 @@
       <c r="L25" s="3"/>
       <c r="M25" s="3"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>0</v>
       </c>
@@ -9743,7 +10211,7 @@
       <c r="L26" s="3"/>
       <c r="M26" s="3"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>1</v>
       </c>
@@ -9778,7 +10246,7 @@
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>46</v>
       </c>
@@ -9795,7 +10263,7 @@
       <c r="L28" s="3"/>
       <c r="M28" s="3"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>0</v>
       </c>
@@ -9830,7 +10298,7 @@
       <c r="L29" s="3"/>
       <c r="M29" s="3"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>24</v>
       </c>
@@ -9865,7 +10333,7 @@
       <c r="L30" s="3"/>
       <c r="M30" s="3"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>1</v>
       </c>
@@ -9900,7 +10368,7 @@
       <c r="L31" s="3"/>
       <c r="M31" s="3"/>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>23</v>
       </c>
@@ -9917,7 +10385,7 @@
       <c r="L32" s="3"/>
       <c r="M32" s="3"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -9952,7 +10420,7 @@
       <c r="L33" s="3"/>
       <c r="M33" s="3"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>0</v>
       </c>
@@ -9987,7 +10455,7 @@
       <c r="L34" s="3"/>
       <c r="M34" s="3"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>1</v>
       </c>
@@ -10022,7 +10490,7 @@
       <c r="L35" s="3"/>
       <c r="M35" s="3"/>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>22</v>
       </c>
@@ -10039,7 +10507,7 @@
       <c r="L36" s="3"/>
       <c r="M36" s="3"/>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>0</v>
       </c>
@@ -10074,7 +10542,7 @@
       <c r="L37" s="3"/>
       <c r="M37" s="3"/>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>24</v>
       </c>
@@ -10109,7 +10577,7 @@
       <c r="L38" s="3"/>
       <c r="M38" s="3"/>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>1</v>
       </c>
@@ -10144,7 +10612,7 @@
       <c r="L39" s="3"/>
       <c r="M39" s="3"/>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>35</v>
       </c>
@@ -10179,7 +10647,7 @@
       <c r="L40" s="3"/>
       <c r="M40" s="3"/>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>27</v>
       </c>
@@ -10196,7 +10664,7 @@
       <c r="L41" s="3"/>
       <c r="M41" s="3"/>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>2</v>
       </c>
@@ -10231,7 +10699,7 @@
       <c r="L42" s="3"/>
       <c r="M42" s="3"/>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>0</v>
       </c>
@@ -10266,7 +10734,7 @@
       <c r="L43" s="3"/>
       <c r="M43" s="3"/>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -10298,7 +10766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>28</v>
       </c>
@@ -10312,7 +10780,7 @@
       <c r="I45" s="3"/>
       <c r="J45" s="3"/>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>0</v>
       </c>
@@ -10344,7 +10812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>24</v>
       </c>
@@ -10376,7 +10844,7 @@
         <v>10737630</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>1</v>
       </c>
@@ -10408,7 +10876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D49" s="3"/>
     </row>
   </sheetData>
@@ -10421,16 +10889,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4F0EF5-9E64-45A3-AF76-8FD0E53934FE}">
   <dimension ref="A1:G53"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" customWidth="1"/>
+    <col min="1" max="1" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" customWidth="1"/>
     <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.88671875" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -10438,12 +10906,12 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>55</v>
       </c>
@@ -10451,7 +10919,7 @@
         <v>6624</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>52</v>
       </c>
@@ -10471,7 +10939,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>57</v>
       </c>
@@ -10491,7 +10959,7 @@
         <v>8783</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>58</v>
       </c>
@@ -10507,7 +10975,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>44</v>
       </c>
@@ -10517,7 +10985,7 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -10537,7 +11005,7 @@
         <v>12.920999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -10557,7 +11025,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -10577,7 +11045,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -10587,7 +11055,7 @@
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -10607,7 +11075,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -10627,7 +11095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -10647,7 +11115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>47</v>
       </c>
@@ -10667,7 +11135,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>39</v>
       </c>
@@ -10677,7 +11145,7 @@
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -10697,7 +11165,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>42</v>
       </c>
@@ -10707,7 +11175,7 @@
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>43</v>
       </c>
@@ -10727,7 +11195,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>9</v>
       </c>
@@ -10737,7 +11205,7 @@
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>48</v>
       </c>
@@ -10757,7 +11225,7 @@
         <v>-503145897.59350002</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>54</v>
       </c>
@@ -10777,7 +11245,7 @@
         <v>9546602.4064993802</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -10797,7 +11265,7 @@
         <v>0.26200008392333901</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>17</v>
       </c>
@@ -10817,7 +11285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>31</v>
       </c>
@@ -10837,7 +11305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>41</v>
       </c>
@@ -10857,7 +11325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>56</v>
       </c>
@@ -10871,7 +11339,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>59</v>
       </c>
@@ -10888,7 +11356,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>45</v>
       </c>
@@ -10898,7 +11366,7 @@
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>2</v>
       </c>
@@ -10918,7 +11386,7 @@
         <v>12.920999999999999</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>0</v>
       </c>
@@ -10938,7 +11406,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>1</v>
       </c>
@@ -10958,7 +11426,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>46</v>
       </c>
@@ -10968,7 +11436,7 @@
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>0</v>
       </c>
@@ -10988,7 +11456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>24</v>
       </c>
@@ -11008,7 +11476,7 @@
         <v>54.920999999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>1</v>
       </c>
@@ -11028,7 +11496,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>23</v>
       </c>
@@ -11038,7 +11506,7 @@
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>2</v>
       </c>
@@ -11058,7 +11526,7 @@
         <v>3000.0191999999902</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>0</v>
       </c>
@@ -11078,7 +11546,7 @@
         <v>202367.83931946999</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>1</v>
       </c>
@@ -11098,7 +11566,7 @@
         <v>1685.0463999999899</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>22</v>
       </c>
@@ -11108,7 +11576,7 @@
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>0</v>
       </c>
@@ -11128,7 +11596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>24</v>
       </c>
@@ -11148,7 +11616,7 @@
         <v>205050.0656</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -11168,7 +11636,7 @@
         <v>2002.83931947069</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>35</v>
       </c>
@@ -11188,7 +11656,7 @@
         <v>26.9344</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>27</v>
       </c>
@@ -11198,7 +11666,7 @@
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>2</v>
       </c>
@@ -11218,7 +11686,7 @@
         <v>915901.94275649404</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>0</v>
       </c>
@@ -11238,7 +11706,7 @@
         <v>8563364.4637428895</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>1</v>
       </c>
@@ -11258,7 +11726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>28</v>
       </c>
@@ -11268,7 +11736,7 @@
       <c r="E50" s="4"/>
       <c r="F50" s="4"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>0</v>
       </c>
@@ -11288,7 +11756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>24</v>
       </c>
@@ -11308,7 +11776,7 @@
         <v>512625164</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
updating notes and results with tightened big-M
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\Desktop\ongoing_projects\MVS\dev\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFB18BEB-3666-4226-9E18-B5ABE9A804FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A24F2D0-85E3-4798-A222-708F5A54D7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="101">
   <si>
     <t>Grid</t>
   </si>
@@ -265,18 +265,6 @@
     <t>Objective (Surplus in $)</t>
   </si>
   <si>
-    <t>Max. storage supply  cycles base case (-)</t>
-  </si>
-  <si>
-    <t>Max. storage supply  cycles contingency (-)</t>
-  </si>
-  <si>
-    <t>Avg. storage supply  cycles base case (-)</t>
-  </si>
-  <si>
-    <t>Avg. storage supply  cycles contingency (-)</t>
-  </si>
-  <si>
     <t>Total operating cost -- base case ($)</t>
   </si>
   <si>
@@ -359,6 +347,21 @@
   </si>
   <si>
     <t>All logs are insample, in practice reoptimize, given investment decisions, may need to allow for load shedding; would of course depend on scenarios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">updated M </t>
+  </si>
+  <si>
+    <t>Avg. yearly storage supply  cycles base case (-)</t>
+  </si>
+  <si>
+    <t>Max. yearly storage supply  cycles base case (-)</t>
+  </si>
+  <si>
+    <t>Avg. yearly storage supply  cycles contingency (-)</t>
+  </si>
+  <si>
+    <t>Max. yearly storage supply  cycles contingency (-)</t>
   </si>
 </sst>
 </file>
@@ -1196,21 +1199,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEB77188-4C54-4D05-A0BB-AB8E292CE16E}">
-  <dimension ref="A1:AI94"/>
+  <dimension ref="A1:AJ94"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="45" customWidth="1"/>
     <col min="2" max="13" width="18" bestFit="1" customWidth="1"/>
     <col min="14" max="16" width="19" bestFit="1" customWidth="1"/>
-    <col min="17" max="35" width="18" bestFit="1" customWidth="1"/>
+    <col min="17" max="36" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1232,34 +1235,40 @@
       <c r="AF2">
         <v>250707</v>
       </c>
-    </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ2">
+        <v>250708</v>
+      </c>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
       <c r="I3" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="J3" t="s">
+        <v>87</v>
+      </c>
+      <c r="M3" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>89</v>
+      </c>
+      <c r="AA3" t="s">
         <v>91</v>
       </c>
-      <c r="M3" t="s">
+      <c r="AD3" t="s">
         <v>92</v>
       </c>
-      <c r="Q3" t="s">
-        <v>93</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>95</v>
-      </c>
-      <c r="AD3" t="s">
+      <c r="AF3" t="s">
+        <v>94</v>
+      </c>
+      <c r="AJ3" t="s">
         <v>96</v>
       </c>
-      <c r="AF3" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>62</v>
       </c>
@@ -1365,8 +1374,11 @@
       <c r="AI4" s="3">
         <v>150</v>
       </c>
-    </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ4" s="3">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>63</v>
       </c>
@@ -1472,10 +1484,13 @@
       <c r="AI5" s="3">
         <v>10000</v>
       </c>
-    </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ5" s="3">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -1541,8 +1556,11 @@
       <c r="AI6" s="3" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ6" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>57</v>
       </c>
@@ -1648,10 +1666,13 @@
       <c r="AI7" s="3">
         <v>24</v>
       </c>
-    </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ7" s="3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -1699,10 +1720,13 @@
       <c r="AI8" s="3">
         <v>31</v>
       </c>
-    </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ8" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B9" s="3">
         <v>0.2</v>
@@ -1806,10 +1830,13 @@
       <c r="AI9" s="3">
         <v>19.999999999999901</v>
       </c>
-    </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ9" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B10" s="3">
         <v>1</v>
@@ -1913,222 +1940,231 @@
       <c r="AI10" s="3">
         <v>79.999999999999602</v>
       </c>
-    </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ10" s="3">
+        <v>80.000000000000099</v>
+      </c>
+    </row>
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>64</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="P11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="Q11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="R11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="S11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="T11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="U11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="V11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="W11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="X11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="Y11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="Z11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AA11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AB11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AC11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AD11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AE11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AF11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AG11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AH11" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI11" s="3" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+      <c r="AJ11" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>20</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="P12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="Q12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="R12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="S12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="T12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="U12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="V12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="W12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="X12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="Y12" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="Z12" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="AA12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="AB12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="AC12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="AD12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="AE12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="AF12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="AG12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="AH12" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="AI12" s="3" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+      <c r="AJ12" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>65</v>
       </c>
@@ -2234,8 +2270,11 @@
       <c r="AI13" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ13" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>9</v>
       </c>
@@ -2273,8 +2312,9 @@
       <c r="AG14" s="3"/>
       <c r="AH14" s="3"/>
       <c r="AI14" s="3"/>
-    </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ14" s="3"/>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>67</v>
       </c>
@@ -2380,8 +2420,11 @@
       <c r="AI15" s="5">
         <v>75466664528.569199</v>
       </c>
-    </row>
-    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ15" s="5">
+        <v>80348048910.696899</v>
+      </c>
+    </row>
+    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>66</v>
       </c>
@@ -2487,10 +2530,13 @@
       <c r="AI16" s="5">
         <v>82.082669973373399</v>
       </c>
-    </row>
-    <row r="17" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ16" s="5">
+        <v>33.474738836288402</v>
+      </c>
+    </row>
+    <row r="17" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B17" s="3">
         <v>5.0159819466078998E-3</v>
@@ -2594,10 +2640,13 @@
       <c r="AI17" s="5">
         <v>8.5320634778948398E-2</v>
       </c>
-    </row>
-    <row r="18" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ17" s="5">
+        <v>6.2993654033391203E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B18" s="3">
         <v>0</v>
@@ -2701,16 +2750,19 @@
       <c r="AI18" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ18" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>70</v>
+        <v>97</v>
       </c>
       <c r="B19" s="3">
         <v>60.420364466636798</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D19" s="3">
         <v>60.453825953486898</v>
@@ -2722,64 +2774,64 @@
         <v>249.106177578238</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="P19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="Q19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="R19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="S19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="T19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="U19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="V19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="W19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="X19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="Y19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="Z19" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="AA19" s="3">
         <v>0</v>
@@ -2808,16 +2860,19 @@
       <c r="AI19" s="3">
         <v>109.615384615384</v>
       </c>
-    </row>
-    <row r="20" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ19" s="3">
+        <v>0.48793109975197602</v>
+      </c>
+    </row>
+    <row r="20" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="B20" s="3">
         <v>117.511996639882</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D20" s="3">
         <v>121.52741218059001</v>
@@ -2829,64 +2884,64 @@
         <v>366.000000000017</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="O20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="P20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="Q20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="R20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="S20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="T20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="U20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="V20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="W20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="X20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="Y20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="Z20" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="AA20" s="3">
         <v>0</v>
@@ -2915,16 +2970,19 @@
       <c r="AI20" s="3">
         <v>150</v>
       </c>
-    </row>
-    <row r="21" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ20" s="3">
+        <v>6.0224303966438102</v>
+      </c>
+    </row>
+    <row r="21" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>99</v>
       </c>
       <c r="B21" s="3">
         <v>75.955726389845793</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D21" s="3">
         <v>77.744130515221698</v>
@@ -2936,64 +2994,64 @@
         <v>212.36105235593601</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="O21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="P21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="Q21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="R21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="S21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="T21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="U21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="V21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="W21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="X21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="Y21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="Z21" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="AA21" s="3">
         <v>0</v>
@@ -3022,16 +3080,19 @@
       <c r="AI21" s="3">
         <v>109.615384615384</v>
       </c>
-    </row>
-    <row r="22" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ21" s="3">
+        <v>15.436822181531699</v>
+      </c>
+    </row>
+    <row r="22" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>69</v>
+        <v>100</v>
       </c>
       <c r="B22" s="3">
         <v>149.99999999999699</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D22" s="3">
         <v>152.83528225048701</v>
@@ -3043,64 +3104,64 @@
         <v>366.00000000001398</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="O22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="P22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="Q22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="R22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="S22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="T22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="U22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="V22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="W22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="X22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="Y22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="Z22" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="AA22" s="3">
         <v>0</v>
@@ -3129,10 +3190,13 @@
       <c r="AI22" s="3">
         <v>150</v>
       </c>
-    </row>
-    <row r="23" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ22" s="3">
+        <v>49.066885964912203</v>
+      </c>
+    </row>
+    <row r="23" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B23" s="3">
         <v>2276815636.0092702</v>
@@ -3236,10 +3300,13 @@
       <c r="AI23" s="3">
         <v>341095916.39237797</v>
       </c>
-    </row>
-    <row r="24" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ23" s="3">
+        <v>445384864.54277402</v>
+      </c>
+    </row>
+    <row r="24" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B24" s="3">
         <v>2314736549.2487898</v>
@@ -3343,10 +3410,13 @@
       <c r="AI24" s="3">
         <v>362229658.04327297</v>
       </c>
-    </row>
-    <row r="25" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ24" s="3">
+        <v>536021286.85959601</v>
+      </c>
+    </row>
+    <row r="25" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B25" s="3">
         <v>16882345.0438595</v>
@@ -3450,10 +3520,13 @@
       <c r="AI25" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ25" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B26" s="3">
         <v>53005356.477268197</v>
@@ -3557,10 +3630,13 @@
       <c r="AI26" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ26" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B27" s="3">
         <v>375804542.65472698</v>
@@ -3664,10 +3740,13 @@
       <c r="AI27" s="3">
         <v>342803520.57327098</v>
       </c>
-    </row>
-    <row r="28" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ27" s="3">
+        <v>307544149.06881702</v>
+      </c>
+    </row>
+    <row r="28" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -3703,8 +3782,9 @@
       <c r="AG28" s="3"/>
       <c r="AH28" s="3"/>
       <c r="AI28" s="3"/>
-    </row>
-    <row r="29" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ28" s="3"/>
+    </row>
+    <row r="29" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>2</v>
       </c>
@@ -3810,8 +3890,11 @@
       <c r="AI29" s="3">
         <v>2.8052631578947498</v>
       </c>
-    </row>
-    <row r="30" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ29" s="3">
+        <v>15.006105263157799</v>
+      </c>
+    </row>
+    <row r="30" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>0</v>
       </c>
@@ -3917,8 +4000,11 @@
       <c r="AI30" s="3">
         <v>120</v>
       </c>
-    </row>
-    <row r="31" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ30" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="31" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>1</v>
       </c>
@@ -4024,8 +4110,11 @@
       <c r="AI31" s="3">
         <v>11.8371929824561</v>
       </c>
-    </row>
-    <row r="32" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ31" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>15</v>
       </c>
@@ -4063,8 +4152,9 @@
       <c r="AG32" s="3"/>
       <c r="AH32" s="3"/>
       <c r="AI32" s="3"/>
-    </row>
-    <row r="33" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ32" s="3"/>
+    </row>
+    <row r="33" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -4170,8 +4260,11 @@
       <c r="AI33" s="5">
         <v>15.6928605263157</v>
       </c>
-    </row>
-    <row r="34" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ33" s="3">
+        <v>33.963702631578897</v>
+      </c>
+    </row>
+    <row r="34" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>0</v>
       </c>
@@ -4277,8 +4370,11 @@
       <c r="AI34" s="5">
         <v>120</v>
       </c>
-    </row>
-    <row r="35" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ34" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="35" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>1</v>
       </c>
@@ -4384,10 +4480,13 @@
       <c r="AI35" s="5">
         <v>11.8371929824561</v>
       </c>
-    </row>
-    <row r="36" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ35" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -4423,8 +4522,9 @@
       <c r="AG36" s="3"/>
       <c r="AH36" s="3"/>
       <c r="AI36" s="3"/>
-    </row>
-    <row r="37" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ36" s="3"/>
+    </row>
+    <row r="37" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>2</v>
       </c>
@@ -4530,8 +4630,11 @@
       <c r="AI37" s="3">
         <v>64192033.347615398</v>
       </c>
-    </row>
-    <row r="38" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ37" s="3">
+        <v>125220078.145666</v>
+      </c>
+    </row>
+    <row r="38" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>0</v>
       </c>
@@ -4637,8 +4740,11 @@
       <c r="AI38" s="3">
         <v>270342587.92053401</v>
       </c>
-    </row>
-    <row r="39" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ38" s="3">
+        <v>182324070.92315</v>
+      </c>
+    </row>
+    <row r="39" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>1</v>
       </c>
@@ -4744,10 +4850,13 @@
       <c r="AI39" s="3">
         <v>8268899.3051215401</v>
       </c>
-    </row>
-    <row r="40" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ39" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -4783,8 +4892,9 @@
       <c r="AG40" s="3"/>
       <c r="AH40" s="3"/>
       <c r="AI40" s="3"/>
-    </row>
-    <row r="41" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ40" s="3"/>
+    </row>
+    <row r="41" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>45</v>
       </c>
@@ -4822,8 +4932,9 @@
       <c r="AG41" s="3"/>
       <c r="AH41" s="3"/>
       <c r="AI41" s="3"/>
-    </row>
-    <row r="42" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ41" s="3"/>
+    </row>
+    <row r="42" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>2</v>
       </c>
@@ -4929,8 +5040,11 @@
       <c r="AI42" s="3">
         <v>28.614210526315802</v>
       </c>
-    </row>
-    <row r="43" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ42" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>0</v>
       </c>
@@ -5036,8 +5150,11 @@
       <c r="AI43" s="3">
         <v>94.642456140350802</v>
       </c>
-    </row>
-    <row r="44" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ43" s="3">
+        <v>92.921684210526294</v>
+      </c>
+    </row>
+    <row r="44" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -5143,10 +5260,13 @@
       <c r="AI44" s="3">
         <v>11.8371929824561</v>
       </c>
-    </row>
-    <row r="45" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ44" s="3">
+        <v>3.6707368421052702</v>
+      </c>
+    </row>
+    <row r="45" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B45" s="3">
         <v>13.0106842105263</v>
@@ -5250,8 +5370,11 @@
       <c r="AI45" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ45" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>46</v>
       </c>
@@ -5289,8 +5412,9 @@
       <c r="AG46" s="3"/>
       <c r="AH46" s="3"/>
       <c r="AI46" s="3"/>
-    </row>
-    <row r="47" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ46" s="3"/>
+    </row>
+    <row r="47" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>0</v>
       </c>
@@ -5396,8 +5520,11 @@
       <c r="AI47" s="3">
         <v>5.7028070175438703</v>
       </c>
-    </row>
-    <row r="48" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ47" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>24</v>
       </c>
@@ -5503,8 +5630,11 @@
       <c r="AI48" s="3">
         <v>94.642456140350802</v>
       </c>
-    </row>
-    <row r="49" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ48" s="3">
+        <v>92.921684210526294</v>
+      </c>
+    </row>
+    <row r="49" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>1</v>
       </c>
@@ -5610,8 +5740,11 @@
       <c r="AI49" s="3">
         <v>11.8371929824561</v>
       </c>
-    </row>
-    <row r="50" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ49" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>23</v>
       </c>
@@ -5649,8 +5782,9 @@
       <c r="AG50" s="3"/>
       <c r="AH50" s="3"/>
       <c r="AI50" s="3"/>
-    </row>
-    <row r="51" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ50" s="3"/>
+    </row>
+    <row r="51" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>2</v>
       </c>
@@ -5756,8 +5890,11 @@
       <c r="AI51" s="3">
         <v>17932.478041171398</v>
       </c>
-    </row>
-    <row r="52" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ51" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>0</v>
       </c>
@@ -5863,8 +6000,11 @@
       <c r="AI52" s="3">
         <v>7623012.1342303902</v>
       </c>
-    </row>
-    <row r="53" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ52" s="3">
+        <v>8112012.18704974</v>
+      </c>
+    </row>
+    <row r="53" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>1</v>
       </c>
@@ -5970,8 +6110,11 @@
       <c r="AI53" s="3">
         <v>137867.519999999</v>
       </c>
-    </row>
-    <row r="54" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ53" s="3">
+        <v>560.22297149122903</v>
+      </c>
+    </row>
+    <row r="54" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>35</v>
       </c>
@@ -6077,8 +6220,11 @@
       <c r="AI54" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="55" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ54" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>22</v>
       </c>
@@ -6116,8 +6262,9 @@
       <c r="AG55" s="3"/>
       <c r="AH55" s="3"/>
       <c r="AI55" s="3"/>
-    </row>
-    <row r="56" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ55" s="3"/>
+    </row>
+    <row r="56" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>0</v>
       </c>
@@ -6223,8 +6370,11 @@
       <c r="AI56" s="3">
         <v>446.10436332767398</v>
       </c>
-    </row>
-    <row r="57" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ56" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>24</v>
       </c>
@@ -6330,8 +6480,11 @@
       <c r="AI57" s="3">
         <v>7615479.0713864798</v>
       </c>
-    </row>
-    <row r="58" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ57" s="3">
+        <v>8111910.5208772197</v>
+      </c>
+    </row>
+    <row r="58" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>1</v>
       </c>
@@ -6437,8 +6590,11 @@
       <c r="AI58" s="3">
         <v>162886.956521741</v>
       </c>
-    </row>
-    <row r="59" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ58" s="3">
+        <v>661.88914401137595</v>
+      </c>
+    </row>
+    <row r="59" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>27</v>
       </c>
@@ -6476,8 +6632,9 @@
       <c r="AG59" s="3"/>
       <c r="AH59" s="3"/>
       <c r="AI59" s="3"/>
-    </row>
-    <row r="60" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ59" s="3"/>
+    </row>
+    <row r="60" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>2</v>
       </c>
@@ -6583,8 +6740,11 @@
       <c r="AI60" s="3">
         <v>5474762.1203048099</v>
       </c>
-    </row>
-    <row r="61" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ60" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>0</v>
       </c>
@@ -6690,8 +6850,11 @@
       <c r="AI61" s="3">
         <v>335761213.19798303</v>
       </c>
-    </row>
-    <row r="62" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ61" s="3">
+        <v>445384864.54277402</v>
+      </c>
+    </row>
+    <row r="62" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>1</v>
       </c>
@@ -6797,8 +6960,11 @@
       <c r="AI62" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ62" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>28</v>
       </c>
@@ -6836,8 +7002,9 @@
       <c r="AG63" s="3"/>
       <c r="AH63" s="3"/>
       <c r="AI63" s="3"/>
-    </row>
-    <row r="64" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ63" s="3"/>
+    </row>
+    <row r="64" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>0</v>
       </c>
@@ -6943,8 +7110,11 @@
       <c r="AI64" s="3">
         <v>140058.92591035599</v>
       </c>
-    </row>
-    <row r="65" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ64" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>24</v>
       </c>
@@ -7050,8 +7220,11 @@
       <c r="AI65" s="3">
         <v>76154790713.864807</v>
       </c>
-    </row>
-    <row r="66" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ65" s="3">
+        <v>81119105208.772095</v>
+      </c>
+    </row>
+    <row r="66" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>1</v>
       </c>
@@ -7157,10 +7330,13 @@
       <c r="AI66" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="67" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ66" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A67" s="9" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
@@ -7196,8 +7372,9 @@
       <c r="AG67" s="3"/>
       <c r="AH67" s="3"/>
       <c r="AI67" s="3"/>
-    </row>
-    <row r="68" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ67" s="3"/>
+    </row>
+    <row r="68" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>45</v>
       </c>
@@ -7235,8 +7412,9 @@
       <c r="AG68" s="3"/>
       <c r="AH68" s="3"/>
       <c r="AI68" s="3"/>
-    </row>
-    <row r="69" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ68" s="3"/>
+    </row>
+    <row r="69" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>2</v>
       </c>
@@ -7342,8 +7520,11 @@
       <c r="AI69" s="3">
         <v>28.614210526315802</v>
       </c>
-    </row>
-    <row r="70" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ69" s="3">
+        <v>46.885052631578901</v>
+      </c>
+    </row>
+    <row r="70" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>0</v>
       </c>
@@ -7449,8 +7630,11 @@
       <c r="AI70" s="3">
         <v>91.685964912280696</v>
       </c>
-    </row>
-    <row r="71" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ70" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="71" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>1</v>
       </c>
@@ -7556,10 +7740,13 @@
       <c r="AI71" s="3">
         <v>11.8371929824561</v>
       </c>
-    </row>
-    <row r="72" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ71" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="72" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B72" s="3">
         <v>26.4866431643824</v>
@@ -7663,8 +7850,11 @@
       <c r="AI72" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="73" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ72" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>46</v>
       </c>
@@ -7702,8 +7892,9 @@
       <c r="AG73" s="3"/>
       <c r="AH73" s="3"/>
       <c r="AI73" s="3"/>
-    </row>
-    <row r="74" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ73" s="3"/>
+    </row>
+    <row r="74" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>0</v>
       </c>
@@ -7809,8 +8000,11 @@
       <c r="AI74" s="3">
         <v>5.7028070175438703</v>
       </c>
-    </row>
-    <row r="75" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ74" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>24</v>
       </c>
@@ -7916,8 +8110,11 @@
       <c r="AI75" s="3">
         <v>94.642456140350802</v>
       </c>
-    </row>
-    <row r="76" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ75" s="3">
+        <v>92.921684210526294</v>
+      </c>
+    </row>
+    <row r="76" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>1</v>
       </c>
@@ -8023,8 +8220,11 @@
       <c r="AI76" s="3">
         <v>11.8371929824561</v>
       </c>
-    </row>
-    <row r="77" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ76" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="77" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>23</v>
       </c>
@@ -8062,8 +8262,9 @@
       <c r="AG77" s="3"/>
       <c r="AH77" s="3"/>
       <c r="AI77" s="3"/>
-    </row>
-    <row r="78" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ77" s="3"/>
+    </row>
+    <row r="78" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>2</v>
       </c>
@@ -8169,8 +8370,11 @@
       <c r="AI78" s="3">
         <v>96589.410716585699</v>
       </c>
-    </row>
-    <row r="79" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ78" s="3">
+        <v>358180.011412911</v>
+      </c>
+    </row>
+    <row r="79" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>0</v>
       </c>
@@ -8276,8 +8480,11 @@
       <c r="AI79" s="3">
         <v>7544355.2015550602</v>
       </c>
-    </row>
-    <row r="80" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ79" s="3">
+        <v>7756946.9525807202</v>
+      </c>
+    </row>
+    <row r="80" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>1</v>
       </c>
@@ -8383,8 +8590,11 @@
       <c r="AI80" s="3">
         <v>137867.519999999</v>
       </c>
-    </row>
-    <row r="81" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ80" s="3">
+        <v>17723.941755947399</v>
+      </c>
+    </row>
+    <row r="81" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>35</v>
       </c>
@@ -8490,8 +8700,11 @@
       <c r="AI81" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="82" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ81" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>22</v>
       </c>
@@ -8529,8 +8742,9 @@
       <c r="AG82" s="3"/>
       <c r="AH82" s="3"/>
       <c r="AI82" s="3"/>
-    </row>
-    <row r="83" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ82" s="3"/>
+    </row>
+    <row r="83" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>0</v>
       </c>
@@ -8636,8 +8850,11 @@
       <c r="AI83" s="3">
         <v>446.10436332767398</v>
       </c>
-    </row>
-    <row r="84" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ83" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>24</v>
       </c>
@@ -8743,8 +8960,11 @@
       <c r="AI84" s="3">
         <v>7615479.0713864798</v>
       </c>
-    </row>
-    <row r="85" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ84" s="3">
+        <v>8111910.5208772197</v>
+      </c>
+    </row>
+    <row r="85" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>1</v>
       </c>
@@ -8850,8 +9070,11 @@
       <c r="AI85" s="3">
         <v>162886.95652174001</v>
       </c>
-    </row>
-    <row r="86" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ85" s="3">
+        <v>20940.3848723386</v>
+      </c>
+    </row>
+    <row r="86" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>27</v>
       </c>
@@ -8889,8 +9112,9 @@
       <c r="AG86" s="3"/>
       <c r="AH86" s="3"/>
       <c r="AI86" s="3"/>
-    </row>
-    <row r="87" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ86" s="3"/>
+    </row>
+    <row r="87" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>2</v>
       </c>
@@ -8996,8 +9220,11 @@
       <c r="AI87" s="3">
         <v>29488620.914501499</v>
       </c>
-    </row>
-    <row r="88" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ87" s="3">
+        <v>109351889.58444899</v>
+      </c>
+    </row>
+    <row r="88" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>0</v>
       </c>
@@ -9103,8 +9330,11 @@
       <c r="AI88" s="3">
         <v>332881096.054681</v>
       </c>
-    </row>
-    <row r="89" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ88" s="3">
+        <v>426669397.27514702</v>
+      </c>
+    </row>
+    <row r="89" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>1</v>
       </c>
@@ -9210,8 +9440,11 @@
       <c r="AI89" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="90" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ89" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>28</v>
       </c>
@@ -9249,8 +9482,9 @@
       <c r="AG90" s="3"/>
       <c r="AH90" s="3"/>
       <c r="AI90" s="3"/>
-    </row>
-    <row r="91" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ90" s="3"/>
+    </row>
+    <row r="91" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>0</v>
       </c>
@@ -9356,8 +9590,11 @@
       <c r="AI91" s="3">
         <v>140058.92591035599</v>
       </c>
-    </row>
-    <row r="92" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ91" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>24</v>
       </c>
@@ -9463,8 +9700,11 @@
       <c r="AI92" s="3">
         <v>76154790713.864807</v>
       </c>
-    </row>
-    <row r="93" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ92" s="3">
+        <v>81119105208.772095</v>
+      </c>
+    </row>
+    <row r="93" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>1</v>
       </c>
@@ -9570,8 +9810,11 @@
       <c r="AI93" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="94" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ93" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:36" x14ac:dyDescent="0.25">
       <c r="V94" s="3"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update results with strided peak-shaving runs
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\Desktop\ongoing_projects\MVS\dev\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A24F2D0-85E3-4798-A222-708F5A54D7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FAA5D51-9DCE-4BDE-9B49-CA563642770A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="101">
   <si>
     <t>Grid</t>
   </si>
@@ -1199,21 +1199,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEB77188-4C54-4D05-A0BB-AB8E292CE16E}">
-  <dimension ref="A1:AJ94"/>
+  <dimension ref="A1:AQ94"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
     <col min="2" max="13" width="18" bestFit="1" customWidth="1"/>
     <col min="14" max="16" width="19" bestFit="1" customWidth="1"/>
-    <col min="17" max="36" width="18" bestFit="1" customWidth="1"/>
+    <col min="17" max="43" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1239,7 +1239,7 @@
         <v>250708</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1268,7 +1268,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>62</v>
       </c>
@@ -1377,8 +1377,29 @@
       <c r="AJ4" s="3">
         <v>150</v>
       </c>
-    </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK4" s="3">
+        <v>150</v>
+      </c>
+      <c r="AL4" s="3">
+        <v>150</v>
+      </c>
+      <c r="AM4" s="3">
+        <v>150</v>
+      </c>
+      <c r="AN4" s="3">
+        <v>150</v>
+      </c>
+      <c r="AO4" s="3">
+        <v>150</v>
+      </c>
+      <c r="AP4" s="3">
+        <v>150</v>
+      </c>
+      <c r="AQ4" s="3">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="5" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>63</v>
       </c>
@@ -1487,8 +1508,29 @@
       <c r="AJ5" s="3">
         <v>10000</v>
       </c>
-    </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK5" s="3">
+        <v>10000</v>
+      </c>
+      <c r="AL5" s="3">
+        <v>10000</v>
+      </c>
+      <c r="AM5" s="3">
+        <v>10000</v>
+      </c>
+      <c r="AN5" s="3">
+        <v>10000</v>
+      </c>
+      <c r="AO5" s="3">
+        <v>10000</v>
+      </c>
+      <c r="AP5" s="3">
+        <v>10000</v>
+      </c>
+      <c r="AQ5" s="3">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>90</v>
       </c>
@@ -1559,8 +1601,29 @@
       <c r="AJ6" s="3" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AO6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AP6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ6" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>57</v>
       </c>
@@ -1669,8 +1732,29 @@
       <c r="AJ7" s="3">
         <v>24</v>
       </c>
-    </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK7" s="3">
+        <v>24</v>
+      </c>
+      <c r="AL7" s="3">
+        <v>24</v>
+      </c>
+      <c r="AM7" s="3">
+        <v>24</v>
+      </c>
+      <c r="AN7" s="3">
+        <v>24</v>
+      </c>
+      <c r="AO7" s="3">
+        <v>24</v>
+      </c>
+      <c r="AP7" s="3">
+        <v>24</v>
+      </c>
+      <c r="AQ7" s="3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>93</v>
       </c>
@@ -1708,23 +1792,44 @@
       <c r="AE8" s="3">
         <v>365</v>
       </c>
-      <c r="AF8" s="3">
+      <c r="AF8" s="5">
         <v>73</v>
       </c>
-      <c r="AG8" s="3">
+      <c r="AG8" s="5">
         <v>73</v>
       </c>
-      <c r="AH8" s="3">
+      <c r="AH8" s="5">
         <v>73</v>
       </c>
-      <c r="AI8" s="3">
+      <c r="AI8" s="5">
         <v>31</v>
       </c>
-      <c r="AJ8" s="3">
+      <c r="AJ8" s="5">
         <v>8</v>
       </c>
-    </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK8" s="5">
+        <v>16</v>
+      </c>
+      <c r="AL8" s="5">
+        <v>31</v>
+      </c>
+      <c r="AM8" s="5">
+        <v>61</v>
+      </c>
+      <c r="AN8" s="5">
+        <v>92</v>
+      </c>
+      <c r="AO8" s="5">
+        <v>122</v>
+      </c>
+      <c r="AP8" s="5">
+        <v>183</v>
+      </c>
+      <c r="AQ8" s="5">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="9" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>81</v>
       </c>
@@ -1833,8 +1938,29 @@
       <c r="AJ9" s="3">
         <v>20</v>
       </c>
-    </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK9" s="3">
+        <v>20.000000000000099</v>
+      </c>
+      <c r="AL9" s="3">
+        <v>19.999999999999901</v>
+      </c>
+      <c r="AM9" s="3">
+        <v>19.9999999999994</v>
+      </c>
+      <c r="AN9" s="3">
+        <v>19.999999999999201</v>
+      </c>
+      <c r="AO9" s="3">
+        <v>20.000000000000199</v>
+      </c>
+      <c r="AP9" s="3">
+        <v>20.000000000001599</v>
+      </c>
+      <c r="AQ9" s="3">
+        <v>20.000000000003102</v>
+      </c>
+    </row>
+    <row r="10" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>82</v>
       </c>
@@ -1943,8 +2069,29 @@
       <c r="AJ10" s="3">
         <v>80.000000000000099</v>
       </c>
-    </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK10" s="3">
+        <v>80.000000000000597</v>
+      </c>
+      <c r="AL10" s="3">
+        <v>79.999999999999602</v>
+      </c>
+      <c r="AM10" s="3">
+        <v>79.999999999997598</v>
+      </c>
+      <c r="AN10" s="3">
+        <v>79.999999999996803</v>
+      </c>
+      <c r="AO10" s="3">
+        <v>80.000000000000895</v>
+      </c>
+      <c r="AP10" s="3">
+        <v>80.000000000006594</v>
+      </c>
+      <c r="AQ10" s="3">
+        <v>80.000000000012406</v>
+      </c>
+    </row>
+    <row r="11" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>64</v>
       </c>
@@ -2053,8 +2200,29 @@
       <c r="AJ11" s="3" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK11" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="AL11" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="AM11" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="AN11" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="AO11" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="AP11" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="AQ11" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="12" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -2163,8 +2331,29 @@
       <c r="AJ12" s="3" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK12" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AL12" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AM12" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AN12" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AO12" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AP12" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AQ12" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>65</v>
       </c>
@@ -2273,8 +2462,29 @@
       <c r="AJ13" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ13" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>9</v>
       </c>
@@ -2313,8 +2523,15 @@
       <c r="AH14" s="3"/>
       <c r="AI14" s="3"/>
       <c r="AJ14" s="3"/>
-    </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK14" s="3"/>
+      <c r="AL14" s="3"/>
+      <c r="AM14" s="3"/>
+      <c r="AN14" s="3"/>
+      <c r="AO14" s="3"/>
+      <c r="AP14" s="3"/>
+      <c r="AQ14" s="3"/>
+    </row>
+    <row r="15" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>67</v>
       </c>
@@ -2423,8 +2640,29 @@
       <c r="AJ15" s="5">
         <v>80348048910.696899</v>
       </c>
-    </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK15" s="5">
+        <v>77792956759.908997</v>
+      </c>
+      <c r="AL15" s="5">
+        <v>75489803133.828903</v>
+      </c>
+      <c r="AM15" s="5">
+        <v>75911219997.949707</v>
+      </c>
+      <c r="AN15" s="5">
+        <v>76144326710.2052</v>
+      </c>
+      <c r="AO15" s="5">
+        <v>76148220420.443405</v>
+      </c>
+      <c r="AP15" s="5">
+        <v>75773314787.084</v>
+      </c>
+      <c r="AQ15" s="5">
+        <v>75978820499.906204</v>
+      </c>
+    </row>
+    <row r="16" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>66</v>
       </c>
@@ -2533,8 +2771,29 @@
       <c r="AJ16" s="5">
         <v>33.474738836288402</v>
       </c>
-    </row>
-    <row r="17" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK16" s="5">
+        <v>91.536086797714205</v>
+      </c>
+      <c r="AL16" s="5">
+        <v>609.251305103302</v>
+      </c>
+      <c r="AM16" s="5">
+        <v>1369.1989958286199</v>
+      </c>
+      <c r="AN16" s="5">
+        <v>3760.6898629665302</v>
+      </c>
+      <c r="AO16" s="5">
+        <v>4332.8456928730002</v>
+      </c>
+      <c r="AP16" s="5">
+        <v>13099.7239570617</v>
+      </c>
+      <c r="AQ16" s="5">
+        <v>41532.982882022799</v>
+      </c>
+    </row>
+    <row r="17" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>80</v>
       </c>
@@ -2643,8 +2902,29 @@
       <c r="AJ17" s="5">
         <v>6.2993654033391203E-2</v>
       </c>
-    </row>
-    <row r="18" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK17" s="5">
+        <v>9.8230637327631695E-2</v>
+      </c>
+      <c r="AL17" s="5">
+        <v>7.2780797586374193E-2</v>
+      </c>
+      <c r="AM17" s="5">
+        <v>9.1965468685320698E-2</v>
+      </c>
+      <c r="AN17" s="5">
+        <v>9.1867765788054501E-2</v>
+      </c>
+      <c r="AO17" s="5">
+        <v>9.9240102473112699E-2</v>
+      </c>
+      <c r="AP17" s="5">
+        <v>9.7016347395388794E-2</v>
+      </c>
+      <c r="AQ17" s="5">
+        <v>0.172875483053822</v>
+      </c>
+    </row>
+    <row r="18" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>83</v>
       </c>
@@ -2753,8 +3033,29 @@
       <c r="AJ18" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK18" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL18" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM18" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN18" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO18" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP18" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ18" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>97</v>
       </c>
@@ -2863,8 +3164,29 @@
       <c r="AJ19" s="3">
         <v>0.48793109975197602</v>
       </c>
-    </row>
-    <row r="20" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK19" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL19" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM19" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN19" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO19" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP19" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ19" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>98</v>
       </c>
@@ -2973,8 +3295,29 @@
       <c r="AJ20" s="3">
         <v>6.0224303966438102</v>
       </c>
-    </row>
-    <row r="21" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ20" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>99</v>
       </c>
@@ -3083,8 +3426,29 @@
       <c r="AJ21" s="3">
         <v>15.436822181531699</v>
       </c>
-    </row>
-    <row r="22" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK21" s="3">
+        <v>10.3403818266356</v>
+      </c>
+      <c r="AL21" s="3">
+        <v>4.64137485285893</v>
+      </c>
+      <c r="AM21" s="3">
+        <v>17.138369690872</v>
+      </c>
+      <c r="AN21" s="3">
+        <v>7.4963002476406704</v>
+      </c>
+      <c r="AO21" s="3">
+        <v>11.216330059432501</v>
+      </c>
+      <c r="AP21" s="3">
+        <v>9.8119212302309293</v>
+      </c>
+      <c r="AQ21" s="3">
+        <v>3.8172441275996301E-3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>100</v>
       </c>
@@ -3193,8 +3557,29 @@
       <c r="AJ22" s="3">
         <v>49.066885964912203</v>
       </c>
-    </row>
-    <row r="23" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK22" s="3">
+        <v>23.3202108064011</v>
+      </c>
+      <c r="AL22" s="3">
+        <v>21.4589170203731</v>
+      </c>
+      <c r="AM22" s="3">
+        <v>45.325050155681502</v>
+      </c>
+      <c r="AN22" s="3">
+        <v>27.8075629489603</v>
+      </c>
+      <c r="AO22" s="3">
+        <v>28.0804315784784</v>
+      </c>
+      <c r="AP22" s="3">
+        <v>26.134002474785699</v>
+      </c>
+      <c r="AQ22" s="3">
+        <v>9.9248347317590593E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>68</v>
       </c>
@@ -3303,8 +3688,29 @@
       <c r="AJ23" s="3">
         <v>445384864.54277402</v>
       </c>
-    </row>
-    <row r="24" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK23" s="3">
+        <v>431447564.16910702</v>
+      </c>
+      <c r="AL23" s="3">
+        <v>351808996.53383201</v>
+      </c>
+      <c r="AM23" s="3">
+        <v>333523585.99850601</v>
+      </c>
+      <c r="AN23" s="3">
+        <v>380189251.57179201</v>
+      </c>
+      <c r="AO23" s="3">
+        <v>326831944.91225201</v>
+      </c>
+      <c r="AP23" s="3">
+        <v>341287726.17254299</v>
+      </c>
+      <c r="AQ23" s="3">
+        <v>331464587.11156601</v>
+      </c>
+    </row>
+    <row r="24" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>69</v>
       </c>
@@ -3413,8 +3819,29 @@
       <c r="AJ24" s="3">
         <v>536021286.85959601</v>
       </c>
-    </row>
-    <row r="25" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK24" s="3">
+        <v>460586779.718243</v>
+      </c>
+      <c r="AL24" s="3">
+        <v>355012188.52074897</v>
+      </c>
+      <c r="AM24" s="3">
+        <v>350361321.09619802</v>
+      </c>
+      <c r="AN24" s="3">
+        <v>379594776.64917201</v>
+      </c>
+      <c r="AO24" s="3">
+        <v>329099395.46098399</v>
+      </c>
+      <c r="AP24" s="3">
+        <v>341869994.67594999</v>
+      </c>
+      <c r="AQ24" s="3">
+        <v>331470220.01673001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>71</v>
       </c>
@@ -3523,8 +3950,29 @@
       <c r="AJ25" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK25" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL25" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM25" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN25" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO25" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP25" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ25" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>70</v>
       </c>
@@ -3633,8 +4081,29 @@
       <c r="AJ26" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK26" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL26" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM26" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN26" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO26" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP26" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ26" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>72</v>
       </c>
@@ -3743,8 +4212,29 @@
       <c r="AJ27" s="3">
         <v>307544149.06881702</v>
       </c>
-    </row>
-    <row r="28" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK27" s="3">
+        <v>349626177.43916398</v>
+      </c>
+      <c r="AL27" s="3">
+        <v>312537945.10486901</v>
+      </c>
+      <c r="AM27" s="3">
+        <v>325381984.30439699</v>
+      </c>
+      <c r="AN27" s="3">
+        <v>327316252.01008898</v>
+      </c>
+      <c r="AO27" s="3">
+        <v>345787031.06114799</v>
+      </c>
+      <c r="AP27" s="3">
+        <v>345152533.742212</v>
+      </c>
+      <c r="AQ27" s="3">
+        <v>389796289.55983901</v>
+      </c>
+    </row>
+    <row r="28" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>73</v>
       </c>
@@ -3783,8 +4273,15 @@
       <c r="AH28" s="3"/>
       <c r="AI28" s="3"/>
       <c r="AJ28" s="3"/>
-    </row>
-    <row r="29" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK28" s="3"/>
+      <c r="AL28" s="3"/>
+      <c r="AM28" s="3"/>
+      <c r="AN28" s="3"/>
+      <c r="AO28" s="3"/>
+      <c r="AP28" s="3"/>
+      <c r="AQ28" s="3"/>
+    </row>
+    <row r="29" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>2</v>
       </c>
@@ -3893,8 +4390,29 @@
       <c r="AJ29" s="3">
         <v>15.006105263157799</v>
       </c>
-    </row>
-    <row r="30" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK29" s="3">
+        <v>3.5230751438585299</v>
+      </c>
+      <c r="AL29" s="3">
+        <v>14.642456140350401</v>
+      </c>
+      <c r="AM29" s="3">
+        <v>14.6424561403508</v>
+      </c>
+      <c r="AN29" s="3">
+        <v>16.3632280701752</v>
+      </c>
+      <c r="AO29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP29" s="3">
+        <v>20.552210526021199</v>
+      </c>
+      <c r="AQ29" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>0</v>
       </c>
@@ -4003,8 +4521,29 @@
       <c r="AJ30" s="3">
         <v>120</v>
       </c>
-    </row>
-    <row r="31" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK30" s="3">
+        <v>160</v>
+      </c>
+      <c r="AL30" s="3">
+        <v>120</v>
+      </c>
+      <c r="AM30" s="3">
+        <v>120</v>
+      </c>
+      <c r="AN30" s="3">
+        <v>120</v>
+      </c>
+      <c r="AO30" s="3">
+        <v>160</v>
+      </c>
+      <c r="AP30" s="3">
+        <v>120</v>
+      </c>
+      <c r="AQ30" s="13">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="31" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>1</v>
       </c>
@@ -4113,8 +4652,29 @@
       <c r="AJ31" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ31" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>15</v>
       </c>
@@ -4153,8 +4713,15 @@
       <c r="AH32" s="3"/>
       <c r="AI32" s="3"/>
       <c r="AJ32" s="3"/>
-    </row>
-    <row r="33" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK32" s="3"/>
+      <c r="AL32" s="3"/>
+      <c r="AM32" s="3"/>
+      <c r="AN32" s="3"/>
+      <c r="AO32" s="3"/>
+      <c r="AP32" s="3"/>
+      <c r="AQ32" s="3"/>
+    </row>
+    <row r="33" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -4260,11 +4827,32 @@
       <c r="AI33" s="5">
         <v>15.6928605263157</v>
       </c>
-      <c r="AJ33" s="3">
+      <c r="AJ33" s="5">
         <v>33.963702631578897</v>
       </c>
-    </row>
-    <row r="34" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK33" s="5">
+        <v>23.737690056139201</v>
+      </c>
+      <c r="AL33" s="5">
+        <v>14.642456140350401</v>
+      </c>
+      <c r="AM33" s="5">
+        <v>31.2654421403508</v>
+      </c>
+      <c r="AN33" s="5">
+        <v>16.3632280701752</v>
+      </c>
+      <c r="AO33" s="5">
+        <v>0</v>
+      </c>
+      <c r="AP33" s="5">
+        <v>20.552210526021899</v>
+      </c>
+      <c r="AQ33" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>0</v>
       </c>
@@ -4370,11 +4958,32 @@
       <c r="AI34" s="5">
         <v>120</v>
       </c>
-      <c r="AJ34" s="3">
+      <c r="AJ34" s="5">
         <v>120</v>
       </c>
-    </row>
-    <row r="35" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK34" s="5">
+        <v>160</v>
+      </c>
+      <c r="AL34" s="5">
+        <v>120</v>
+      </c>
+      <c r="AM34" s="5">
+        <v>120</v>
+      </c>
+      <c r="AN34" s="5">
+        <v>120</v>
+      </c>
+      <c r="AO34" s="5">
+        <v>160</v>
+      </c>
+      <c r="AP34" s="5">
+        <v>120</v>
+      </c>
+      <c r="AQ34" s="5">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="35" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>1</v>
       </c>
@@ -4480,11 +5089,32 @@
       <c r="AI35" s="5">
         <v>11.8371929824561</v>
       </c>
-      <c r="AJ35" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AJ35" s="5">
+        <v>0</v>
+      </c>
+      <c r="AK35" s="5">
+        <v>0</v>
+      </c>
+      <c r="AL35" s="5">
+        <v>0</v>
+      </c>
+      <c r="AM35" s="5">
+        <v>0</v>
+      </c>
+      <c r="AN35" s="5">
+        <v>0</v>
+      </c>
+      <c r="AO35" s="5">
+        <v>0</v>
+      </c>
+      <c r="AP35" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ35" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>74</v>
       </c>
@@ -4523,8 +5153,15 @@
       <c r="AH36" s="3"/>
       <c r="AI36" s="3"/>
       <c r="AJ36" s="3"/>
-    </row>
-    <row r="37" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK36" s="3"/>
+      <c r="AL36" s="3"/>
+      <c r="AM36" s="3"/>
+      <c r="AN36" s="3"/>
+      <c r="AO36" s="3"/>
+      <c r="AP36" s="3"/>
+      <c r="AQ36" s="3"/>
+    </row>
+    <row r="37" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>2</v>
       </c>
@@ -4633,8 +5270,29 @@
       <c r="AJ37" s="3">
         <v>125220078.145666</v>
       </c>
-    </row>
-    <row r="38" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK37" s="3">
+        <v>85570626.447014704</v>
+      </c>
+      <c r="AL37" s="3">
+        <v>29621283.3275664</v>
+      </c>
+      <c r="AM37" s="3">
+        <v>80187544.097401798</v>
+      </c>
+      <c r="AN37" s="3">
+        <v>31825516.376017202</v>
+      </c>
+      <c r="AO37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP37" s="3">
+        <v>43374761.1797553</v>
+      </c>
+      <c r="AQ37" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>0</v>
       </c>
@@ -4743,8 +5401,29 @@
       <c r="AJ38" s="3">
         <v>182324070.92315</v>
       </c>
-    </row>
-    <row r="39" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK38" s="3">
+        <v>264055550.992149</v>
+      </c>
+      <c r="AL38" s="3">
+        <v>282916661.77730298</v>
+      </c>
+      <c r="AM38" s="3">
+        <v>245194440.20699599</v>
+      </c>
+      <c r="AN38" s="3">
+        <v>295490735.63407201</v>
+      </c>
+      <c r="AO38" s="3">
+        <v>345787031.06114799</v>
+      </c>
+      <c r="AP38" s="3">
+        <v>301777772.56245601</v>
+      </c>
+      <c r="AQ38" s="3">
+        <v>389796289.55983901</v>
+      </c>
+    </row>
+    <row r="39" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>1</v>
       </c>
@@ -4853,8 +5532,29 @@
       <c r="AJ39" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ39" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
         <v>76</v>
       </c>
@@ -4893,8 +5593,15 @@
       <c r="AH40" s="3"/>
       <c r="AI40" s="3"/>
       <c r="AJ40" s="3"/>
-    </row>
-    <row r="41" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK40" s="3"/>
+      <c r="AL40" s="3"/>
+      <c r="AM40" s="3"/>
+      <c r="AN40" s="3"/>
+      <c r="AO40" s="3"/>
+      <c r="AP40" s="3"/>
+      <c r="AQ40" s="3"/>
+    </row>
+    <row r="41" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>45</v>
       </c>
@@ -4933,8 +5640,15 @@
       <c r="AH41" s="3"/>
       <c r="AI41" s="3"/>
       <c r="AJ41" s="3"/>
-    </row>
-    <row r="42" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK41" s="3"/>
+      <c r="AL41" s="3"/>
+      <c r="AM41" s="3"/>
+      <c r="AN41" s="3"/>
+      <c r="AO41" s="3"/>
+      <c r="AP41" s="3"/>
+      <c r="AQ41" s="3"/>
+    </row>
+    <row r="42" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>2</v>
       </c>
@@ -5043,8 +5757,29 @@
       <c r="AJ42" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ42" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>0</v>
       </c>
@@ -5153,8 +5888,29 @@
       <c r="AJ43" s="3">
         <v>92.921684210526294</v>
       </c>
-    </row>
-    <row r="44" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK43" s="3">
+        <v>94.642456140350802</v>
+      </c>
+      <c r="AL43" s="3">
+        <v>94.642456140350802</v>
+      </c>
+      <c r="AM43" s="3">
+        <v>94.642456140350802</v>
+      </c>
+      <c r="AN43" s="3">
+        <v>96.363228069863297</v>
+      </c>
+      <c r="AO43" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AP43" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AQ43" s="3">
+        <v>98.083999999999406</v>
+      </c>
+    </row>
+    <row r="44" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -5263,8 +6019,29 @@
       <c r="AJ44" s="3">
         <v>3.6707368421052702</v>
       </c>
-    </row>
-    <row r="45" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK44" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL44" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM44" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN44" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO44" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP44" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ44" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>75</v>
       </c>
@@ -5373,8 +6150,29 @@
       <c r="AJ45" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK45" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL45" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM45" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN45" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO45" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP45" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ45" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>46</v>
       </c>
@@ -5413,8 +6211,15 @@
       <c r="AH46" s="3"/>
       <c r="AI46" s="3"/>
       <c r="AJ46" s="3"/>
-    </row>
-    <row r="47" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK46" s="3"/>
+      <c r="AL46" s="3"/>
+      <c r="AM46" s="3"/>
+      <c r="AN46" s="3"/>
+      <c r="AO46" s="3"/>
+      <c r="AP46" s="3"/>
+      <c r="AQ46" s="3"/>
+    </row>
+    <row r="47" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>0</v>
       </c>
@@ -5523,8 +6328,29 @@
       <c r="AJ47" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK47" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL47" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM47" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN47" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO47" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP47" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ47" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>24</v>
       </c>
@@ -5633,8 +6459,29 @@
       <c r="AJ48" s="3">
         <v>92.921684210526294</v>
       </c>
-    </row>
-    <row r="49" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK48" s="3">
+        <v>94.642456140350802</v>
+      </c>
+      <c r="AL48" s="3">
+        <v>94.642456140350802</v>
+      </c>
+      <c r="AM48" s="3">
+        <v>94.642456140350802</v>
+      </c>
+      <c r="AN48" s="3">
+        <v>96.363228070175396</v>
+      </c>
+      <c r="AO48" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AP48" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AQ48" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="49" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>1</v>
       </c>
@@ -5743,8 +6590,29 @@
       <c r="AJ49" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="50" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK49" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL49" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM49" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN49" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO49" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP49" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ49" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>23</v>
       </c>
@@ -5783,8 +6651,15 @@
       <c r="AH50" s="3"/>
       <c r="AI50" s="3"/>
       <c r="AJ50" s="3"/>
-    </row>
-    <row r="51" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK50" s="3"/>
+      <c r="AL50" s="3"/>
+      <c r="AM50" s="3"/>
+      <c r="AN50" s="3"/>
+      <c r="AO50" s="3"/>
+      <c r="AP50" s="3"/>
+      <c r="AQ50" s="3"/>
+    </row>
+    <row r="51" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>2</v>
       </c>
@@ -5893,8 +6768,29 @@
       <c r="AJ51" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="52" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ51" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>0</v>
       </c>
@@ -6003,8 +6899,29 @@
       <c r="AJ52" s="3">
         <v>8112012.18704974</v>
       </c>
-    </row>
-    <row r="53" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK52" s="3">
+        <v>7857985.8344626203</v>
+      </c>
+      <c r="AL52" s="3">
+        <v>7615479.0713864798</v>
+      </c>
+      <c r="AM52" s="3">
+        <v>7657349.3115268704</v>
+      </c>
+      <c r="AN52" s="3">
+        <v>7685171.3318801597</v>
+      </c>
+      <c r="AO52" s="3">
+        <v>7682129.2886530804</v>
+      </c>
+      <c r="AP52" s="3">
+        <v>7645987.1500695003</v>
+      </c>
+      <c r="AQ52" s="3">
+        <v>7670008.2503163796</v>
+      </c>
+    </row>
+    <row r="53" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>1</v>
       </c>
@@ -6113,8 +7030,29 @@
       <c r="AJ53" s="3">
         <v>560.22297149122903</v>
       </c>
-    </row>
-    <row r="54" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK53" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL53" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM53" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN53" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO53" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP53" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ53" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>35</v>
       </c>
@@ -6223,8 +7161,29 @@
       <c r="AJ54" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="55" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ54" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>22</v>
       </c>
@@ -6263,8 +7222,15 @@
       <c r="AH55" s="3"/>
       <c r="AI55" s="3"/>
       <c r="AJ55" s="3"/>
-    </row>
-    <row r="56" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK55" s="3"/>
+      <c r="AL55" s="3"/>
+      <c r="AM55" s="3"/>
+      <c r="AN55" s="3"/>
+      <c r="AO55" s="3"/>
+      <c r="AP55" s="3"/>
+      <c r="AQ55" s="3"/>
+    </row>
+    <row r="56" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>0</v>
       </c>
@@ -6373,8 +7339,29 @@
       <c r="AJ56" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="57" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK56" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL56" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM56" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN56" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO56" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP56" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ56" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>24</v>
       </c>
@@ -6483,8 +7470,29 @@
       <c r="AJ57" s="3">
         <v>8111910.5208772197</v>
       </c>
-    </row>
-    <row r="58" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK57" s="3">
+        <v>7857985.8344626203</v>
+      </c>
+      <c r="AL57" s="3">
+        <v>7615479.0713864798</v>
+      </c>
+      <c r="AM57" s="3">
+        <v>7657349.3115268704</v>
+      </c>
+      <c r="AN57" s="3">
+        <v>7685171.3318804</v>
+      </c>
+      <c r="AO57" s="3">
+        <v>7682129.2886527795</v>
+      </c>
+      <c r="AP57" s="3">
+        <v>7645987.1500695003</v>
+      </c>
+      <c r="AQ57" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+    </row>
+    <row r="58" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>1</v>
       </c>
@@ -6593,8 +7601,29 @@
       <c r="AJ58" s="3">
         <v>661.88914401137595</v>
       </c>
-    </row>
-    <row r="59" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK58" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL58" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM58" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN58" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO58" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP58" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ58" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>27</v>
       </c>
@@ -6633,8 +7662,15 @@
       <c r="AH59" s="3"/>
       <c r="AI59" s="3"/>
       <c r="AJ59" s="3"/>
-    </row>
-    <row r="60" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK59" s="3"/>
+      <c r="AL59" s="3"/>
+      <c r="AM59" s="3"/>
+      <c r="AN59" s="3"/>
+      <c r="AO59" s="3"/>
+      <c r="AP59" s="3"/>
+      <c r="AQ59" s="3"/>
+    </row>
+    <row r="60" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>2</v>
       </c>
@@ -6743,8 +7779,29 @@
       <c r="AJ60" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="61" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK60" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL60" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM60" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN60" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO60" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP60" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ60" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>0</v>
       </c>
@@ -6853,8 +7910,29 @@
       <c r="AJ61" s="3">
         <v>445384864.54277402</v>
       </c>
-    </row>
-    <row r="62" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK61" s="3">
+        <v>431447564.16910702</v>
+      </c>
+      <c r="AL61" s="3">
+        <v>351808996.53383201</v>
+      </c>
+      <c r="AM61" s="3">
+        <v>333523585.99850601</v>
+      </c>
+      <c r="AN61" s="3">
+        <v>380189251.57179201</v>
+      </c>
+      <c r="AO61" s="3">
+        <v>326831944.91225201</v>
+      </c>
+      <c r="AP61" s="3">
+        <v>341287726.17254299</v>
+      </c>
+      <c r="AQ61" s="3">
+        <v>331464587.11156601</v>
+      </c>
+    </row>
+    <row r="62" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>1</v>
       </c>
@@ -6963,8 +8041,29 @@
       <c r="AJ62" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK62" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL62" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM62" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN62" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO62" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP62" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ62" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>28</v>
       </c>
@@ -7003,8 +8102,15 @@
       <c r="AH63" s="3"/>
       <c r="AI63" s="3"/>
       <c r="AJ63" s="3"/>
-    </row>
-    <row r="64" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK63" s="3"/>
+      <c r="AL63" s="3"/>
+      <c r="AM63" s="3"/>
+      <c r="AN63" s="3"/>
+      <c r="AO63" s="3"/>
+      <c r="AP63" s="3"/>
+      <c r="AQ63" s="3"/>
+    </row>
+    <row r="64" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>0</v>
       </c>
@@ -7113,8 +8219,29 @@
       <c r="AJ64" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="65" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK64" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL64" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM64" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN64" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO64" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP64" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ64" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>24</v>
       </c>
@@ -7223,8 +8350,29 @@
       <c r="AJ65" s="3">
         <v>81119105208.772095</v>
       </c>
-    </row>
-    <row r="66" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK65" s="3">
+        <v>78579858344.627502</v>
+      </c>
+      <c r="AL65" s="3">
+        <v>76154790713.864807</v>
+      </c>
+      <c r="AM65" s="3">
+        <v>76573493115.274597</v>
+      </c>
+      <c r="AN65" s="3">
+        <v>76851713318.801193</v>
+      </c>
+      <c r="AO65" s="3">
+        <v>76821292886.530594</v>
+      </c>
+      <c r="AP65" s="3">
+        <v>76459871500.705399</v>
+      </c>
+      <c r="AQ65" s="3">
+        <v>76700082503.154099</v>
+      </c>
+    </row>
+    <row r="66" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>1</v>
       </c>
@@ -7333,8 +8481,29 @@
       <c r="AJ66" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="67" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ66" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A67" s="9" t="s">
         <v>77</v>
       </c>
@@ -7373,8 +8542,15 @@
       <c r="AH67" s="3"/>
       <c r="AI67" s="3"/>
       <c r="AJ67" s="3"/>
-    </row>
-    <row r="68" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK67" s="3"/>
+      <c r="AL67" s="3"/>
+      <c r="AM67" s="3"/>
+      <c r="AN67" s="3"/>
+      <c r="AO67" s="3"/>
+      <c r="AP67" s="3"/>
+      <c r="AQ67" s="3"/>
+    </row>
+    <row r="68" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>45</v>
       </c>
@@ -7413,8 +8589,15 @@
       <c r="AH68" s="3"/>
       <c r="AI68" s="3"/>
       <c r="AJ68" s="3"/>
-    </row>
-    <row r="69" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK68" s="3"/>
+      <c r="AL68" s="3"/>
+      <c r="AM68" s="3"/>
+      <c r="AN68" s="3"/>
+      <c r="AO68" s="3"/>
+      <c r="AP68" s="3"/>
+      <c r="AQ68" s="3"/>
+    </row>
+    <row r="69" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>2</v>
       </c>
@@ -7523,8 +8706,29 @@
       <c r="AJ69" s="3">
         <v>46.885052631578901</v>
       </c>
-    </row>
-    <row r="70" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK69" s="3">
+        <v>33.135964912280699</v>
+      </c>
+      <c r="AL69" s="3">
+        <v>14.6424561403505</v>
+      </c>
+      <c r="AM69" s="3">
+        <v>29.544335999999898</v>
+      </c>
+      <c r="AN69" s="3">
+        <v>16.363228070175399</v>
+      </c>
+      <c r="AO69" s="3">
+        <v>12.921350000001601</v>
+      </c>
+      <c r="AP69" s="3">
+        <v>18.552210526315701</v>
+      </c>
+      <c r="AQ69" s="3">
+        <v>4.3828070175438896</v>
+      </c>
+    </row>
+    <row r="70" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>0</v>
       </c>
@@ -7633,8 +8837,29 @@
       <c r="AJ70" s="3">
         <v>80</v>
       </c>
-    </row>
-    <row r="71" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK70" s="3">
+        <v>94.642456140350802</v>
+      </c>
+      <c r="AL70" s="3">
+        <v>80</v>
+      </c>
+      <c r="AM70" s="3">
+        <v>80</v>
+      </c>
+      <c r="AN70" s="3">
+        <v>80</v>
+      </c>
+      <c r="AO70" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AP70" s="3">
+        <v>95.02</v>
+      </c>
+      <c r="AQ70" s="3">
+        <v>98.083999999995996</v>
+      </c>
+    </row>
+    <row r="71" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>1</v>
       </c>
@@ -7743,8 +8968,29 @@
       <c r="AJ71" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="72" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK71" s="3">
+        <v>6</v>
+      </c>
+      <c r="AL71" s="3">
+        <v>6</v>
+      </c>
+      <c r="AM71" s="3">
+        <v>6</v>
+      </c>
+      <c r="AN71" s="3">
+        <v>6</v>
+      </c>
+      <c r="AO71" s="3">
+        <v>6</v>
+      </c>
+      <c r="AP71" s="3">
+        <v>6</v>
+      </c>
+      <c r="AQ71" s="3">
+        <v>4.3828070175448</v>
+      </c>
+    </row>
+    <row r="72" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>75</v>
       </c>
@@ -7853,8 +9099,29 @@
       <c r="AJ72" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="73" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ72" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>46</v>
       </c>
@@ -7893,8 +9160,15 @@
       <c r="AH73" s="3"/>
       <c r="AI73" s="3"/>
       <c r="AJ73" s="3"/>
-    </row>
-    <row r="74" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK73" s="3"/>
+      <c r="AL73" s="3"/>
+      <c r="AM73" s="3"/>
+      <c r="AN73" s="3"/>
+      <c r="AO73" s="3"/>
+      <c r="AP73" s="3"/>
+      <c r="AQ73" s="3"/>
+    </row>
+    <row r="74" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>0</v>
       </c>
@@ -8003,8 +9277,29 @@
       <c r="AJ74" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="75" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK74" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL74" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM74" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN74" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO74" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP74" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ74" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>24</v>
       </c>
@@ -8113,8 +9408,29 @@
       <c r="AJ75" s="3">
         <v>92.921684210526294</v>
       </c>
-    </row>
-    <row r="76" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK75" s="3">
+        <v>94.642456140350802</v>
+      </c>
+      <c r="AL75" s="3">
+        <v>94.642456140350802</v>
+      </c>
+      <c r="AM75" s="3">
+        <v>94.642456140350802</v>
+      </c>
+      <c r="AN75" s="3">
+        <v>96.363228070175396</v>
+      </c>
+      <c r="AO75" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AP75" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AQ75" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="76" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>1</v>
       </c>
@@ -8223,8 +9539,29 @@
       <c r="AJ76" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="77" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK76" s="3">
+        <v>6</v>
+      </c>
+      <c r="AL76" s="3">
+        <v>6</v>
+      </c>
+      <c r="AM76" s="3">
+        <v>6</v>
+      </c>
+      <c r="AN76" s="3">
+        <v>6</v>
+      </c>
+      <c r="AO76" s="3">
+        <v>6</v>
+      </c>
+      <c r="AP76" s="3">
+        <v>6</v>
+      </c>
+      <c r="AQ76" s="3">
+        <v>2.98677113388483</v>
+      </c>
+    </row>
+    <row r="77" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>23</v>
       </c>
@@ -8263,8 +9600,15 @@
       <c r="AH77" s="3"/>
       <c r="AI77" s="3"/>
       <c r="AJ77" s="3"/>
-    </row>
-    <row r="78" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK77" s="3"/>
+      <c r="AL77" s="3"/>
+      <c r="AM77" s="3"/>
+      <c r="AN77" s="3"/>
+      <c r="AO77" s="3"/>
+      <c r="AP77" s="3"/>
+      <c r="AQ77" s="3"/>
+    </row>
+    <row r="78" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>2</v>
       </c>
@@ -8373,8 +9717,29 @@
       <c r="AJ78" s="3">
         <v>358180.011412911</v>
       </c>
-    </row>
-    <row r="79" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK78" s="3">
+        <v>114435.099597758</v>
+      </c>
+      <c r="AL78" s="3">
+        <v>13017.5249940064</v>
+      </c>
+      <c r="AM78" s="3">
+        <v>66480.374027198093</v>
+      </c>
+      <c r="AN78" s="3">
+        <v>14009.789790531901</v>
+      </c>
+      <c r="AO78" s="3">
+        <v>10904.490845226101</v>
+      </c>
+      <c r="AP78" s="3">
+        <v>12102.8770382291</v>
+      </c>
+      <c r="AQ78" s="3">
+        <v>35.0624561403515</v>
+      </c>
+    </row>
+    <row r="79" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>0</v>
       </c>
@@ -8483,8 +9848,29 @@
       <c r="AJ79" s="3">
         <v>7756946.9525807202</v>
       </c>
-    </row>
-    <row r="80" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK79" s="3">
+        <v>7745705.2748055002</v>
+      </c>
+      <c r="AL79" s="3">
+        <v>7603428.6313284496</v>
+      </c>
+      <c r="AM79" s="3">
+        <v>7594439.9180144696</v>
+      </c>
+      <c r="AN79" s="3">
+        <v>7672723.4842454204</v>
+      </c>
+      <c r="AO79" s="3">
+        <v>7673561.85184603</v>
+      </c>
+      <c r="AP79" s="3">
+        <v>7635928.7020027703</v>
+      </c>
+      <c r="AQ79" s="3">
+        <v>7669973.9832275799</v>
+      </c>
+    </row>
+    <row r="80" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>1</v>
       </c>
@@ -8593,8 +9979,29 @@
       <c r="AJ80" s="3">
         <v>17723.941755947399</v>
       </c>
-    </row>
-    <row r="81" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK80" s="3">
+        <v>11872.4127980699</v>
+      </c>
+      <c r="AL80" s="3">
+        <v>5329.0409510585096</v>
+      </c>
+      <c r="AM80" s="3">
+        <v>19677.590544271501</v>
+      </c>
+      <c r="AN80" s="3">
+        <v>8606.9520923311102</v>
+      </c>
+      <c r="AO80" s="3">
+        <v>12878.141521038</v>
+      </c>
+      <c r="AP80" s="3">
+        <v>11265.655479702</v>
+      </c>
+      <c r="AQ80" s="3">
+        <v>4.3828070175448</v>
+      </c>
+    </row>
+    <row r="81" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>35</v>
       </c>
@@ -8703,8 +10110,29 @@
       <c r="AJ81" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="82" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ81" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>22</v>
       </c>
@@ -8743,8 +10171,15 @@
       <c r="AH82" s="3"/>
       <c r="AI82" s="3"/>
       <c r="AJ82" s="3"/>
-    </row>
-    <row r="83" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK82" s="3"/>
+      <c r="AL82" s="3"/>
+      <c r="AM82" s="3"/>
+      <c r="AN82" s="3"/>
+      <c r="AO82" s="3"/>
+      <c r="AP82" s="3"/>
+      <c r="AQ82" s="3"/>
+    </row>
+    <row r="83" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>0</v>
       </c>
@@ -8853,8 +10288,29 @@
       <c r="AJ83" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="84" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK83" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL83" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM83" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN83" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO83" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP83" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ83" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>24</v>
       </c>
@@ -8963,8 +10419,29 @@
       <c r="AJ84" s="3">
         <v>8111910.5208772197</v>
       </c>
-    </row>
-    <row r="85" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK84" s="3">
+        <v>7857985.8344626203</v>
+      </c>
+      <c r="AL84" s="3">
+        <v>7615479.0713864798</v>
+      </c>
+      <c r="AM84" s="3">
+        <v>7657349.3115268704</v>
+      </c>
+      <c r="AN84" s="3">
+        <v>7685171.3318804</v>
+      </c>
+      <c r="AO84" s="3">
+        <v>7682129.2886527795</v>
+      </c>
+      <c r="AP84" s="3">
+        <v>7645987.1500695003</v>
+      </c>
+      <c r="AQ84" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+    </row>
+    <row r="85" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>1</v>
       </c>
@@ -9073,8 +10550,29 @@
       <c r="AJ85" s="3">
         <v>20940.3848723386</v>
       </c>
-    </row>
-    <row r="86" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK85" s="3">
+        <v>14026.9527387502</v>
+      </c>
+      <c r="AL85" s="3">
+        <v>6296.1258873564102</v>
+      </c>
+      <c r="AM85" s="3">
+        <v>23248.571058922</v>
+      </c>
+      <c r="AN85" s="3">
+        <v>10168.8942489734</v>
+      </c>
+      <c r="AO85" s="3">
+        <v>15215.1955588822</v>
+      </c>
+      <c r="AP85" s="3">
+        <v>13310.084451444</v>
+      </c>
+      <c r="AQ85" s="3">
+        <v>5.1781746426569004</v>
+      </c>
+    </row>
+    <row r="86" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>27</v>
       </c>
@@ -9113,8 +10611,15 @@
       <c r="AH86" s="3"/>
       <c r="AI86" s="3"/>
       <c r="AJ86" s="3"/>
-    </row>
-    <row r="87" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK86" s="3"/>
+      <c r="AL86" s="3"/>
+      <c r="AM86" s="3"/>
+      <c r="AN86" s="3"/>
+      <c r="AO86" s="3"/>
+      <c r="AP86" s="3"/>
+      <c r="AQ86" s="3"/>
+    </row>
+    <row r="87" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>2</v>
       </c>
@@ -9223,8 +10728,29 @@
       <c r="AJ87" s="3">
         <v>109351889.58444899</v>
       </c>
-    </row>
-    <row r="88" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK87" s="3">
+        <v>34936886.417633399</v>
+      </c>
+      <c r="AL87" s="3">
+        <v>3974233.3755369699</v>
+      </c>
+      <c r="AM87" s="3">
+        <v>20296371.345453098</v>
+      </c>
+      <c r="AN87" s="3">
+        <v>4277170.5216947598</v>
+      </c>
+      <c r="AO87" s="3">
+        <v>3329126.81022608</v>
+      </c>
+      <c r="AP87" s="3">
+        <v>3694992.5494666998</v>
+      </c>
+      <c r="AQ87" s="3">
+        <v>10704.522056646199</v>
+      </c>
+    </row>
+    <row r="88" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>0</v>
       </c>
@@ -9333,8 +10859,29 @@
       <c r="AJ88" s="3">
         <v>426669397.27514702</v>
       </c>
-    </row>
-    <row r="89" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK88" s="3">
+        <v>425649893.30061001</v>
+      </c>
+      <c r="AL88" s="3">
+        <v>351037955.14521199</v>
+      </c>
+      <c r="AM88" s="3">
+        <v>330064949.75074601</v>
+      </c>
+      <c r="AN88" s="3">
+        <v>375317606.127478</v>
+      </c>
+      <c r="AO88" s="3">
+        <v>325770268.65075803</v>
+      </c>
+      <c r="AP88" s="3">
+        <v>338175002.12648302</v>
+      </c>
+      <c r="AQ88" s="3">
+        <v>331459515.49467301</v>
+      </c>
+    </row>
+    <row r="89" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>1</v>
       </c>
@@ -9443,8 +10990,29 @@
       <c r="AJ89" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="90" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ89" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>28</v>
       </c>
@@ -9483,8 +11051,15 @@
       <c r="AH90" s="3"/>
       <c r="AI90" s="3"/>
       <c r="AJ90" s="3"/>
-    </row>
-    <row r="91" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK90" s="3"/>
+      <c r="AL90" s="3"/>
+      <c r="AM90" s="3"/>
+      <c r="AN90" s="3"/>
+      <c r="AO90" s="3"/>
+      <c r="AP90" s="3"/>
+      <c r="AQ90" s="3"/>
+    </row>
+    <row r="91" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>0</v>
       </c>
@@ -9593,8 +11168,29 @@
       <c r="AJ91" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="92" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK91" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL91" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM91" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN91" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO91" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP91" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ91" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>24</v>
       </c>
@@ -9703,8 +11299,29 @@
       <c r="AJ92" s="3">
         <v>81119105208.772095</v>
       </c>
-    </row>
-    <row r="93" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK92" s="3">
+        <v>78579858344.627502</v>
+      </c>
+      <c r="AL92" s="3">
+        <v>76154790713.864807</v>
+      </c>
+      <c r="AM92" s="3">
+        <v>76573493115.274597</v>
+      </c>
+      <c r="AN92" s="3">
+        <v>76851713318.801193</v>
+      </c>
+      <c r="AO92" s="3">
+        <v>76821292886.530594</v>
+      </c>
+      <c r="AP92" s="3">
+        <v>76459871500.705399</v>
+      </c>
+      <c r="AQ92" s="3">
+        <v>76700082503.154099</v>
+      </c>
+    </row>
+    <row r="93" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>1</v>
       </c>
@@ -9813,8 +11430,29 @@
       <c r="AJ93" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="94" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK93" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL93" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM93" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN93" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO93" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP93" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ93" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:43" x14ac:dyDescent="0.25">
       <c r="V94" s="3"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add no backup option
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\Desktop\ongoing_projects\MVS\dev\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FAA5D51-9DCE-4BDE-9B49-CA563642770A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64E1FE99-4847-4C52-A1B4-95B198788DB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Experiments" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="106">
   <si>
     <t>Grid</t>
   </si>
@@ -363,6 +363,21 @@
   <si>
     <t>Max. yearly storage supply  cycles contingency (-)</t>
   </si>
+  <si>
+    <t>no backup</t>
+  </si>
+  <si>
+    <t>["g", "s"]</t>
+  </si>
+  <si>
+    <t>lower optimality gap</t>
+  </si>
+  <si>
+    <t>benefit per year</t>
+  </si>
+  <si>
+    <t>lower optimality gap; zero new backup installation; no lock-in effect</t>
+  </si>
 </sst>
 </file>
 
@@ -451,7 +466,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -466,6 +481,7 @@
     <xf numFmtId="43" fontId="4" fillId="2" borderId="0" xfId="2" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Bad" xfId="3" builtinId="27"/>
@@ -764,28 +780,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J46"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.28515625" customWidth="1"/>
-    <col min="7" max="8" width="9.28515625" customWidth="1"/>
+    <col min="1" max="1" width="29.33203125" customWidth="1"/>
+    <col min="7" max="8" width="9.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -817,7 +833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -849,7 +865,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -881,12 +897,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -918,7 +934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -950,7 +966,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -982,7 +998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -1014,179 +1030,179 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E12" s="1"/>
       <c r="H12" s="1"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>1</v>
       </c>
@@ -1199,21 +1215,22 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEB77188-4C54-4D05-A0BB-AB8E292CE16E}">
-  <dimension ref="A1:AQ94"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AZ94"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
     <col min="2" max="13" width="18" bestFit="1" customWidth="1"/>
     <col min="14" max="16" width="19" bestFit="1" customWidth="1"/>
-    <col min="17" max="43" width="18" bestFit="1" customWidth="1"/>
+    <col min="17" max="50" width="18" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="14.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1238,8 +1255,14 @@
       <c r="AJ2">
         <v>250708</v>
       </c>
-    </row>
-    <row r="3" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR2">
+        <v>250713</v>
+      </c>
+      <c r="AU2">
+        <v>250714</v>
+      </c>
+    </row>
+    <row r="3" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1267,8 +1290,17 @@
       <c r="AJ3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="4" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR3" t="s">
+        <v>101</v>
+      </c>
+      <c r="AU3" t="s">
+        <v>103</v>
+      </c>
+      <c r="AY3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>62</v>
       </c>
@@ -1398,8 +1430,29 @@
       <c r="AQ4" s="3">
         <v>150</v>
       </c>
-    </row>
-    <row r="5" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR4" s="3">
+        <v>150</v>
+      </c>
+      <c r="AS4" s="3">
+        <v>150</v>
+      </c>
+      <c r="AT4" s="3">
+        <v>150</v>
+      </c>
+      <c r="AU4" s="3">
+        <v>150</v>
+      </c>
+      <c r="AV4" s="3">
+        <v>150</v>
+      </c>
+      <c r="AW4" s="3">
+        <v>150</v>
+      </c>
+      <c r="AX4" s="3">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="5" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>63</v>
       </c>
@@ -1529,8 +1582,29 @@
       <c r="AQ5" s="3">
         <v>10000</v>
       </c>
-    </row>
-    <row r="6" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR5" s="3">
+        <v>10000</v>
+      </c>
+      <c r="AS5" s="3">
+        <v>10000</v>
+      </c>
+      <c r="AT5" s="3">
+        <v>10000</v>
+      </c>
+      <c r="AU5" s="3">
+        <v>10000</v>
+      </c>
+      <c r="AV5" s="3">
+        <v>10000</v>
+      </c>
+      <c r="AW5" s="3">
+        <v>10000</v>
+      </c>
+      <c r="AX5" s="3">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>90</v>
       </c>
@@ -1622,8 +1696,29 @@
       <c r="AQ6" s="3" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AU6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AV6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AW6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AX6" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>57</v>
       </c>
@@ -1753,8 +1848,29 @@
       <c r="AQ7" s="3">
         <v>24</v>
       </c>
-    </row>
-    <row r="8" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR7" s="3">
+        <v>24</v>
+      </c>
+      <c r="AS7" s="3">
+        <v>24</v>
+      </c>
+      <c r="AT7" s="3">
+        <v>24</v>
+      </c>
+      <c r="AU7" s="3">
+        <v>24</v>
+      </c>
+      <c r="AV7" s="3">
+        <v>24</v>
+      </c>
+      <c r="AW7" s="3">
+        <v>24</v>
+      </c>
+      <c r="AX7" s="3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>93</v>
       </c>
@@ -1828,8 +1944,29 @@
       <c r="AQ8" s="5">
         <v>365</v>
       </c>
-    </row>
-    <row r="9" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR8" s="3">
+        <v>183</v>
+      </c>
+      <c r="AS8" s="3">
+        <v>183</v>
+      </c>
+      <c r="AT8" s="3">
+        <v>365</v>
+      </c>
+      <c r="AU8" s="3">
+        <v>183</v>
+      </c>
+      <c r="AV8" s="3">
+        <v>183</v>
+      </c>
+      <c r="AW8" s="3">
+        <v>365</v>
+      </c>
+      <c r="AX8" s="3">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="9" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>81</v>
       </c>
@@ -1959,8 +2096,29 @@
       <c r="AQ9" s="3">
         <v>20.000000000003102</v>
       </c>
-    </row>
-    <row r="10" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR9" s="3">
+        <v>20.000000000001599</v>
+      </c>
+      <c r="AS9" s="3">
+        <v>20.000000000001599</v>
+      </c>
+      <c r="AT9" s="3">
+        <v>20.000000000003102</v>
+      </c>
+      <c r="AU9" s="3">
+        <v>20.000000000001599</v>
+      </c>
+      <c r="AV9" s="3">
+        <v>20.000000000001599</v>
+      </c>
+      <c r="AW9" s="3">
+        <v>20.000000000003102</v>
+      </c>
+      <c r="AX9" s="3">
+        <v>20.000000000003102</v>
+      </c>
+    </row>
+    <row r="10" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>82</v>
       </c>
@@ -2090,8 +2248,29 @@
       <c r="AQ10" s="3">
         <v>80.000000000012406</v>
       </c>
-    </row>
-    <row r="11" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR10" s="3">
+        <v>80.000000000006594</v>
+      </c>
+      <c r="AS10" s="3">
+        <v>80.000000000006594</v>
+      </c>
+      <c r="AT10" s="3">
+        <v>80.000000000012406</v>
+      </c>
+      <c r="AU10" s="3">
+        <v>80.000000000006594</v>
+      </c>
+      <c r="AV10" s="3">
+        <v>80.000000000006594</v>
+      </c>
+      <c r="AW10" s="3">
+        <v>80.000000000012406</v>
+      </c>
+      <c r="AX10" s="3">
+        <v>80.000000000012406</v>
+      </c>
+    </row>
+    <row r="11" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>64</v>
       </c>
@@ -2221,8 +2400,29 @@
       <c r="AQ11" s="3" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="12" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR11" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="AS11" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="AT11" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="AU11" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="AV11" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="AW11" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="AX11" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -2352,8 +2552,29 @@
       <c r="AQ12" s="3" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="13" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="AS12" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AT12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="AU12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="AV12" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="AX12" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>65</v>
       </c>
@@ -2483,8 +2704,33 @@
       <c r="AQ13" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ13" s="3">
+        <f>AW17*AW15/100</f>
+        <v>5613440.4115295373</v>
+      </c>
+    </row>
+    <row r="14" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>9</v>
       </c>
@@ -2530,8 +2776,19 @@
       <c r="AO14" s="3"/>
       <c r="AP14" s="3"/>
       <c r="AQ14" s="3"/>
-    </row>
-    <row r="15" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR14" s="3"/>
+      <c r="AS14" s="3"/>
+      <c r="AT14" s="3"/>
+      <c r="AU14" s="3"/>
+      <c r="AV14" s="3"/>
+      <c r="AW14" s="3"/>
+      <c r="AX14" s="3"/>
+      <c r="AZ14" s="3">
+        <f>AX17*AX15/100</f>
+        <v>7517855.6325683566</v>
+      </c>
+    </row>
+    <row r="15" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>67</v>
       </c>
@@ -2661,8 +2918,33 @@
       <c r="AQ15" s="5">
         <v>75978820499.906204</v>
       </c>
-    </row>
-    <row r="16" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR15" s="5">
+        <v>75782031705.381897</v>
+      </c>
+      <c r="AS15" s="5">
+        <v>75735074506.153198</v>
+      </c>
+      <c r="AT15" s="5">
+        <v>75995963340.847595</v>
+      </c>
+      <c r="AU15" s="5">
+        <v>75806177393.352905</v>
+      </c>
+      <c r="AV15" s="5">
+        <v>75790646421.535095</v>
+      </c>
+      <c r="AW15" s="5">
+        <v>76054556803.439194</v>
+      </c>
+      <c r="AX15" s="5">
+        <v>76036916539.554596</v>
+      </c>
+      <c r="AZ15" s="14">
+        <f>AW15-AX15</f>
+        <v>17640263.884597778</v>
+      </c>
+    </row>
+    <row r="16" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>66</v>
       </c>
@@ -2792,8 +3074,29 @@
       <c r="AQ16" s="5">
         <v>41532.982882022799</v>
       </c>
-    </row>
-    <row r="17" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR16" s="5">
+        <v>176.44134807586599</v>
+      </c>
+      <c r="AS16" s="5">
+        <v>119.42701101303101</v>
+      </c>
+      <c r="AT16" s="5">
+        <v>390.318123102188</v>
+      </c>
+      <c r="AU16" s="5">
+        <v>254.60152578353799</v>
+      </c>
+      <c r="AV16" s="5">
+        <v>264.71024703979401</v>
+      </c>
+      <c r="AW16" s="5">
+        <v>2050.3553199767998</v>
+      </c>
+      <c r="AX16" s="5">
+        <v>718.28705191612198</v>
+      </c>
+    </row>
+    <row r="17" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>80</v>
       </c>
@@ -2923,8 +3226,32 @@
       <c r="AQ17" s="5">
         <v>0.172875483053822</v>
       </c>
-    </row>
-    <row r="18" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR17" s="5">
+        <v>5.1328254728459602E-2</v>
+      </c>
+      <c r="AS17" s="5">
+        <v>9.7308277561418896E-2</v>
+      </c>
+      <c r="AT17" s="5">
+        <v>9.8112912386183096E-2</v>
+      </c>
+      <c r="AU17" s="5">
+        <v>5.7470911815349201E-3</v>
+      </c>
+      <c r="AV17" s="5">
+        <v>4.0122701148495301E-3</v>
+      </c>
+      <c r="AW17" s="5">
+        <v>7.3808074722430004E-3</v>
+      </c>
+      <c r="AX17" s="5">
+        <v>9.8871127009175202E-3</v>
+      </c>
+      <c r="AZ17" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="18" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>83</v>
       </c>
@@ -3054,8 +3381,33 @@
       <c r="AQ18" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR18" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS18" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT18" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU18" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV18" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW18" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX18" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ18" s="14">
+        <f>AZ15/26</f>
+        <v>678471.6878691453</v>
+      </c>
+    </row>
+    <row r="19" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>97</v>
       </c>
@@ -3185,8 +3537,29 @@
       <c r="AQ19" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR19" s="3">
+        <v>150.00000000000099</v>
+      </c>
+      <c r="AS19" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT19" s="3">
+        <v>86.5384615384597</v>
+      </c>
+      <c r="AU19" s="3">
+        <v>150</v>
+      </c>
+      <c r="AV19" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW19" s="3">
+        <v>149.99999999999901</v>
+      </c>
+      <c r="AX19" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>98</v>
       </c>
@@ -3316,8 +3689,29 @@
       <c r="AQ20" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR20" s="3">
+        <v>150.00000000000199</v>
+      </c>
+      <c r="AS20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT20" s="3">
+        <v>149.99999999999599</v>
+      </c>
+      <c r="AU20" s="3">
+        <v>150.00000000000199</v>
+      </c>
+      <c r="AV20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW20" s="3">
+        <v>150.000000000005</v>
+      </c>
+      <c r="AX20" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>99</v>
       </c>
@@ -3447,8 +3841,29 @@
       <c r="AQ21" s="3">
         <v>3.8172441275996301E-3</v>
       </c>
-    </row>
-    <row r="22" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR21" s="3">
+        <v>150.00000000000099</v>
+      </c>
+      <c r="AS21" s="3">
+        <v>1.9073996655494E-3</v>
+      </c>
+      <c r="AT21" s="3">
+        <v>86.5384615384597</v>
+      </c>
+      <c r="AU21" s="3">
+        <v>150</v>
+      </c>
+      <c r="AV21" s="3">
+        <v>3.69933259123076</v>
+      </c>
+      <c r="AW21" s="3">
+        <v>149.99999999999901</v>
+      </c>
+      <c r="AX21" s="3">
+        <v>3.2362526863760599</v>
+      </c>
+    </row>
+    <row r="22" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>100</v>
       </c>
@@ -3578,8 +3993,29 @@
       <c r="AQ22" s="3">
         <v>9.9248347317590593E-2</v>
       </c>
-    </row>
-    <row r="23" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR22" s="3">
+        <v>150.00000000000199</v>
+      </c>
+      <c r="AS22" s="3">
+        <v>4.9592391304284597E-2</v>
+      </c>
+      <c r="AT22" s="3">
+        <v>149.99999999999599</v>
+      </c>
+      <c r="AU22" s="3">
+        <v>150.00000000000199</v>
+      </c>
+      <c r="AV22" s="3">
+        <v>8.4255329488747801</v>
+      </c>
+      <c r="AW22" s="3">
+        <v>150.000000000005</v>
+      </c>
+      <c r="AX22" s="3">
+        <v>7.7939723320161498</v>
+      </c>
+    </row>
+    <row r="23" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>68</v>
       </c>
@@ -3709,8 +4145,29 @@
       <c r="AQ23" s="3">
         <v>331464587.11156601</v>
       </c>
-    </row>
-    <row r="24" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR23" s="3">
+        <v>321195123.62479901</v>
+      </c>
+      <c r="AS23" s="3">
+        <v>341287726.17254299</v>
+      </c>
+      <c r="AT23" s="3">
+        <v>326896914.53985</v>
+      </c>
+      <c r="AU23" s="3">
+        <v>325908952.656555</v>
+      </c>
+      <c r="AV23" s="3">
+        <v>341287726.17254299</v>
+      </c>
+      <c r="AW23" s="3">
+        <v>317355520.34808803</v>
+      </c>
+      <c r="AX23" s="3">
+        <v>331464587.11163098</v>
+      </c>
+    </row>
+    <row r="24" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>69</v>
       </c>
@@ -3840,8 +4297,29 @@
       <c r="AQ24" s="3">
         <v>331470220.01673001</v>
       </c>
-    </row>
-    <row r="25" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR24" s="3">
+        <v>321368757.37180197</v>
+      </c>
+      <c r="AS24" s="3">
+        <v>341287804.88261598</v>
+      </c>
+      <c r="AT24" s="3">
+        <v>326897074.889341</v>
+      </c>
+      <c r="AU24" s="3">
+        <v>326054995.69194901</v>
+      </c>
+      <c r="AV24" s="3">
+        <v>339864580.35255897</v>
+      </c>
+      <c r="AW24" s="3">
+        <v>317483522.54990101</v>
+      </c>
+      <c r="AX24" s="3">
+        <v>330594342.69532299</v>
+      </c>
+    </row>
+    <row r="25" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>71</v>
       </c>
@@ -3971,8 +4449,29 @@
       <c r="AQ25" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR25" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS25" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT25" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU25" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV25" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW25" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX25" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>70</v>
       </c>
@@ -4102,8 +4601,29 @@
       <c r="AQ26" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR26" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS26" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT26" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU26" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV26" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW26" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX26" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>72</v>
       </c>
@@ -4233,8 +4753,29 @@
       <c r="AQ27" s="3">
         <v>389796289.55983901</v>
       </c>
-    </row>
-    <row r="28" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR27" s="3">
+        <v>356609944.94310701</v>
+      </c>
+      <c r="AS27" s="3">
+        <v>383509252.631455</v>
+      </c>
+      <c r="AT27" s="3">
+        <v>377222215.70306998</v>
+      </c>
+      <c r="AU27" s="3">
+        <v>327755946.08269399</v>
+      </c>
+      <c r="AV27" s="3">
+        <v>328221982.155626</v>
+      </c>
+      <c r="AW27" s="3">
+        <v>328144578.93234497</v>
+      </c>
+      <c r="AX27" s="3">
+        <v>331875425.37673599</v>
+      </c>
+    </row>
+    <row r="28" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>73</v>
       </c>
@@ -4280,8 +4821,15 @@
       <c r="AO28" s="3"/>
       <c r="AP28" s="3"/>
       <c r="AQ28" s="3"/>
-    </row>
-    <row r="29" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR28" s="3"/>
+      <c r="AS28" s="3"/>
+      <c r="AT28" s="3"/>
+      <c r="AU28" s="3"/>
+      <c r="AV28" s="3"/>
+      <c r="AW28" s="3"/>
+      <c r="AX28" s="3"/>
+    </row>
+    <row r="29" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>2</v>
       </c>
@@ -4411,8 +4959,29 @@
       <c r="AQ29" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX29" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>0</v>
       </c>
@@ -4542,8 +5111,29 @@
       <c r="AQ30" s="13">
         <v>160</v>
       </c>
-    </row>
-    <row r="31" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR30" s="5">
+        <v>120.000000000014</v>
+      </c>
+      <c r="AS30" s="5">
+        <v>160</v>
+      </c>
+      <c r="AT30" s="5">
+        <v>160</v>
+      </c>
+      <c r="AU30" s="5">
+        <v>120</v>
+      </c>
+      <c r="AV30" s="5">
+        <v>120</v>
+      </c>
+      <c r="AW30" s="5">
+        <v>120</v>
+      </c>
+      <c r="AX30" s="5">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="31" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>1</v>
       </c>
@@ -4673,8 +5263,29 @@
       <c r="AQ31" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR31" s="5">
+        <v>18.0839999999857</v>
+      </c>
+      <c r="AS31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU31" s="5">
+        <v>18.083999999990301</v>
+      </c>
+      <c r="AV31" s="5">
+        <v>18.9284912280689</v>
+      </c>
+      <c r="AW31" s="5">
+        <v>19.103999999993601</v>
+      </c>
+      <c r="AX31" s="5">
+        <v>18.928491228068498</v>
+      </c>
+    </row>
+    <row r="32" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>15</v>
       </c>
@@ -4720,8 +5331,15 @@
       <c r="AO32" s="3"/>
       <c r="AP32" s="3"/>
       <c r="AQ32" s="3"/>
-    </row>
-    <row r="33" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR32" s="3"/>
+      <c r="AS32" s="3"/>
+      <c r="AT32" s="3"/>
+      <c r="AU32" s="3"/>
+      <c r="AV32" s="3"/>
+      <c r="AW32" s="3"/>
+      <c r="AX32" s="3"/>
+    </row>
+    <row r="33" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -4851,8 +5469,29 @@
       <c r="AQ33" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX33" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>0</v>
       </c>
@@ -4982,8 +5621,29 @@
       <c r="AQ34" s="5">
         <v>160</v>
       </c>
-    </row>
-    <row r="35" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR34" s="5">
+        <v>120.000000000014</v>
+      </c>
+      <c r="AS34" s="5">
+        <v>160</v>
+      </c>
+      <c r="AT34" s="5">
+        <v>160</v>
+      </c>
+      <c r="AU34" s="5">
+        <v>120</v>
+      </c>
+      <c r="AV34" s="5">
+        <v>120</v>
+      </c>
+      <c r="AW34" s="5">
+        <v>120</v>
+      </c>
+      <c r="AX34" s="5">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="35" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>1</v>
       </c>
@@ -5113,8 +5773,29 @@
       <c r="AQ35" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR35" s="5">
+        <v>18.0839999999857</v>
+      </c>
+      <c r="AS35" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT35" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU35" s="5">
+        <v>18.083999999987899</v>
+      </c>
+      <c r="AV35" s="5">
+        <v>18.928491228067099</v>
+      </c>
+      <c r="AW35" s="5">
+        <v>19.103999999993601</v>
+      </c>
+      <c r="AX35" s="5">
+        <v>18.928491228068498</v>
+      </c>
+    </row>
+    <row r="36" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>74</v>
       </c>
@@ -5160,8 +5841,15 @@
       <c r="AO36" s="3"/>
       <c r="AP36" s="3"/>
       <c r="AQ36" s="3"/>
-    </row>
-    <row r="37" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR36" s="3"/>
+      <c r="AS36" s="3"/>
+      <c r="AT36" s="3"/>
+      <c r="AU36" s="3"/>
+      <c r="AV36" s="3"/>
+      <c r="AW36" s="3"/>
+      <c r="AX36" s="3"/>
+    </row>
+    <row r="37" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>2</v>
       </c>
@@ -5291,8 +5979,29 @@
       <c r="AQ37" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX37" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>0</v>
       </c>
@@ -5422,8 +6131,29 @@
       <c r="AQ38" s="3">
         <v>389796289.55983901</v>
       </c>
-    </row>
-    <row r="39" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR38" s="3">
+        <v>276629624.84891999</v>
+      </c>
+      <c r="AS38" s="3">
+        <v>383509252.631455</v>
+      </c>
+      <c r="AT38" s="3">
+        <v>377222215.70306998</v>
+      </c>
+      <c r="AU38" s="3">
+        <v>276629624.84891802</v>
+      </c>
+      <c r="AV38" s="3">
+        <v>276629624.84891802</v>
+      </c>
+      <c r="AW38" s="3">
+        <v>276629624.84891802</v>
+      </c>
+      <c r="AX38" s="3">
+        <v>276629624.84891802</v>
+      </c>
+    </row>
+    <row r="39" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>1</v>
       </c>
@@ -5553,8 +6283,29 @@
       <c r="AQ39" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR39" s="3">
+        <v>79980320.094186097</v>
+      </c>
+      <c r="AS39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU39" s="3">
+        <v>51126321.233776003</v>
+      </c>
+      <c r="AV39" s="3">
+        <v>51592357.306707896</v>
+      </c>
+      <c r="AW39" s="3">
+        <v>51514954.083426997</v>
+      </c>
+      <c r="AX39" s="3">
+        <v>55245800.527817801</v>
+      </c>
+    </row>
+    <row r="40" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A40" s="9" t="s">
         <v>76</v>
       </c>
@@ -5600,8 +6351,15 @@
       <c r="AO40" s="3"/>
       <c r="AP40" s="3"/>
       <c r="AQ40" s="3"/>
-    </row>
-    <row r="41" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR40" s="3"/>
+      <c r="AS40" s="3"/>
+      <c r="AT40" s="3"/>
+      <c r="AU40" s="3"/>
+      <c r="AV40" s="3"/>
+      <c r="AW40" s="3"/>
+      <c r="AX40" s="3"/>
+    </row>
+    <row r="41" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>45</v>
       </c>
@@ -5647,8 +6405,15 @@
       <c r="AO41" s="3"/>
       <c r="AP41" s="3"/>
       <c r="AQ41" s="3"/>
-    </row>
-    <row r="42" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR41" s="3"/>
+      <c r="AS41" s="3"/>
+      <c r="AT41" s="3"/>
+      <c r="AU41" s="3"/>
+      <c r="AV41" s="3"/>
+      <c r="AW41" s="3"/>
+      <c r="AX41" s="3"/>
+    </row>
+    <row r="42" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>2</v>
       </c>
@@ -5778,8 +6543,29 @@
       <c r="AQ42" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX42" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>0</v>
       </c>
@@ -5909,8 +6695,29 @@
       <c r="AQ43" s="3">
         <v>98.083999999999406</v>
       </c>
-    </row>
-    <row r="44" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR43" s="3">
+        <v>104.122596491213</v>
+      </c>
+      <c r="AS43" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AT43" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AU43" s="3">
+        <v>104.122596491218</v>
+      </c>
+      <c r="AV43" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AW43" s="3">
+        <v>108.58414035087</v>
+      </c>
+      <c r="AX43" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="44" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -6040,8 +6847,29 @@
       <c r="AQ44" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR44" s="3">
+        <v>24.083999999980801</v>
+      </c>
+      <c r="AS44" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT44" s="3">
+        <v>6</v>
+      </c>
+      <c r="AU44" s="3">
+        <v>18.083999999990301</v>
+      </c>
+      <c r="AV44" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW44" s="3">
+        <v>19.103999999993601</v>
+      </c>
+      <c r="AX44" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>75</v>
       </c>
@@ -6171,8 +6999,29 @@
       <c r="AQ45" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR45" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS45" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT45" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU45" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV45" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW45" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX45" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>46</v>
       </c>
@@ -6218,8 +7067,15 @@
       <c r="AO46" s="3"/>
       <c r="AP46" s="3"/>
       <c r="AQ46" s="3"/>
-    </row>
-    <row r="47" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR46" s="3"/>
+      <c r="AS46" s="3"/>
+      <c r="AT46" s="3"/>
+      <c r="AU46" s="3"/>
+      <c r="AV46" s="3"/>
+      <c r="AW46" s="3"/>
+      <c r="AX46" s="3"/>
+    </row>
+    <row r="47" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>0</v>
       </c>
@@ -6349,8 +7205,29 @@
       <c r="AQ47" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR47" s="3">
+        <v>5.6894561403317097</v>
+      </c>
+      <c r="AS47" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT47" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU47" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV47" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW47" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX47" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>24</v>
       </c>
@@ -6480,8 +7357,29 @@
       <c r="AQ48" s="3">
         <v>98.084000000000003</v>
       </c>
-    </row>
-    <row r="49" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR48" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AS48" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AT48" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AU48" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AV48" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AW48" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AX48" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="49" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>1</v>
       </c>
@@ -6611,8 +7509,29 @@
       <c r="AQ49" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR49" s="3">
+        <v>24.083999999980801</v>
+      </c>
+      <c r="AS49" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT49" s="3">
+        <v>6</v>
+      </c>
+      <c r="AU49" s="3">
+        <v>18.083999999990301</v>
+      </c>
+      <c r="AV49" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW49" s="3">
+        <v>19.103999999993601</v>
+      </c>
+      <c r="AX49" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>23</v>
       </c>
@@ -6658,8 +7577,15 @@
       <c r="AO50" s="3"/>
       <c r="AP50" s="3"/>
       <c r="AQ50" s="3"/>
-    </row>
-    <row r="51" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR50" s="3"/>
+      <c r="AS50" s="3"/>
+      <c r="AT50" s="3"/>
+      <c r="AU50" s="3"/>
+      <c r="AV50" s="3"/>
+      <c r="AW50" s="3"/>
+      <c r="AX50" s="3"/>
+    </row>
+    <row r="51" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>2</v>
       </c>
@@ -6789,8 +7715,29 @@
       <c r="AQ51" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="52" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX51" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>0</v>
       </c>
@@ -6920,8 +7867,29 @@
       <c r="AQ52" s="3">
         <v>7670008.2503163796</v>
       </c>
-    </row>
-    <row r="53" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR52" s="3">
+        <v>7718560.1127042398</v>
+      </c>
+      <c r="AS52" s="3">
+        <v>7645987.1500695003</v>
+      </c>
+      <c r="AT52" s="3">
+        <v>7688039.5546650495</v>
+      </c>
+      <c r="AU52" s="3">
+        <v>7701385.7281562602</v>
+      </c>
+      <c r="AV52" s="3">
+        <v>7645987.1500695003</v>
+      </c>
+      <c r="AW52" s="3">
+        <v>7725720.7734476104</v>
+      </c>
+      <c r="AX52" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+    </row>
+    <row r="53" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>1</v>
       </c>
@@ -7051,8 +8019,29 @@
       <c r="AQ53" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR53" s="3">
+        <v>398831.03999970399</v>
+      </c>
+      <c r="AS53" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT53" s="3">
+        <v>99359.999999997701</v>
+      </c>
+      <c r="AU53" s="3">
+        <v>305269.24799992499</v>
+      </c>
+      <c r="AV53" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW53" s="3">
+        <v>306999.21599986602</v>
+      </c>
+      <c r="AX53" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>35</v>
       </c>
@@ -7182,8 +8171,29 @@
       <c r="AQ54" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="55" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX54" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>22</v>
       </c>
@@ -7229,8 +8239,15 @@
       <c r="AO55" s="3"/>
       <c r="AP55" s="3"/>
       <c r="AQ55" s="3"/>
-    </row>
-    <row r="56" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR55" s="3"/>
+      <c r="AS55" s="3"/>
+      <c r="AT55" s="3"/>
+      <c r="AU55" s="3"/>
+      <c r="AV55" s="3"/>
+      <c r="AW55" s="3"/>
+      <c r="AX55" s="3"/>
+    </row>
+    <row r="56" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>0</v>
       </c>
@@ -7360,8 +8377,29 @@
       <c r="AQ56" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="57" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR56" s="3">
+        <v>195.30698254971401</v>
+      </c>
+      <c r="AS56" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT56" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU56" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV56" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW56" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX56" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>24</v>
       </c>
@@ -7491,8 +8529,29 @@
       <c r="AQ57" s="3">
         <v>7670008.2503171796</v>
       </c>
-    </row>
-    <row r="58" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR57" s="3">
+        <v>7645987.1500695003</v>
+      </c>
+      <c r="AS57" s="3">
+        <v>7645987.1500695003</v>
+      </c>
+      <c r="AT57" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+      <c r="AU57" s="3">
+        <v>7645987.1500695003</v>
+      </c>
+      <c r="AV57" s="3">
+        <v>7645987.1500695003</v>
+      </c>
+      <c r="AW57" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+      <c r="AX57" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+    </row>
+    <row r="58" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>1</v>
       </c>
@@ -7622,8 +8681,29 @@
       <c r="AQ58" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="59" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR58" s="3">
+        <v>471208.69565183698</v>
+      </c>
+      <c r="AS58" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT58" s="3">
+        <v>117391.304347824</v>
+      </c>
+      <c r="AU58" s="3">
+        <v>360667.82608691702</v>
+      </c>
+      <c r="AV58" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW58" s="3">
+        <v>362711.73913027602</v>
+      </c>
+      <c r="AX58" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>27</v>
       </c>
@@ -7669,8 +8749,15 @@
       <c r="AO59" s="3"/>
       <c r="AP59" s="3"/>
       <c r="AQ59" s="3"/>
-    </row>
-    <row r="60" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR59" s="3"/>
+      <c r="AS59" s="3"/>
+      <c r="AT59" s="3"/>
+      <c r="AU59" s="3"/>
+      <c r="AV59" s="3"/>
+      <c r="AW59" s="3"/>
+      <c r="AX59" s="3"/>
+    </row>
+    <row r="60" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>2</v>
       </c>
@@ -7800,8 +8887,29 @@
       <c r="AQ60" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="61" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR60" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS60" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT60" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU60" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV60" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW60" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX60" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>0</v>
       </c>
@@ -7931,8 +9039,29 @@
       <c r="AQ61" s="3">
         <v>331464587.11156601</v>
       </c>
-    </row>
-    <row r="62" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR61" s="3">
+        <v>321206562.43709701</v>
+      </c>
+      <c r="AS61" s="3">
+        <v>341287726.17254299</v>
+      </c>
+      <c r="AT61" s="3">
+        <v>326896914.53985</v>
+      </c>
+      <c r="AU61" s="3">
+        <v>325908952.656555</v>
+      </c>
+      <c r="AV61" s="3">
+        <v>341287726.17254299</v>
+      </c>
+      <c r="AW61" s="3">
+        <v>317355520.34808803</v>
+      </c>
+      <c r="AX61" s="3">
+        <v>331464587.11163098</v>
+      </c>
+    </row>
+    <row r="62" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>1</v>
       </c>
@@ -8062,8 +9191,29 @@
       <c r="AQ62" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR62" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS62" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT62" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU62" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV62" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW62" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX62" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>28</v>
       </c>
@@ -8109,8 +9259,15 @@
       <c r="AO63" s="3"/>
       <c r="AP63" s="3"/>
       <c r="AQ63" s="3"/>
-    </row>
-    <row r="64" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR63" s="3"/>
+      <c r="AS63" s="3"/>
+      <c r="AT63" s="3"/>
+      <c r="AU63" s="3"/>
+      <c r="AV63" s="3"/>
+      <c r="AW63" s="3"/>
+      <c r="AX63" s="3"/>
+    </row>
+    <row r="64" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>0</v>
       </c>
@@ -8240,8 +9397,29 @@
       <c r="AQ64" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="65" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR64" s="3">
+        <v>11438.8122982648</v>
+      </c>
+      <c r="AS64" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT64" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU64" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV64" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW64" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX64" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>24</v>
       </c>
@@ -8371,8 +9549,29 @@
       <c r="AQ65" s="3">
         <v>76700082503.154099</v>
       </c>
-    </row>
-    <row r="66" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR65" s="3">
+        <v>76459871500.705399</v>
+      </c>
+      <c r="AS65" s="3">
+        <v>76459871500.705399</v>
+      </c>
+      <c r="AT65" s="3">
+        <v>76700082503.154099</v>
+      </c>
+      <c r="AU65" s="3">
+        <v>76459871500.705399</v>
+      </c>
+      <c r="AV65" s="3">
+        <v>76459871500.705399</v>
+      </c>
+      <c r="AW65" s="3">
+        <v>76700082503.154099</v>
+      </c>
+      <c r="AX65" s="3">
+        <v>76700082503.154099</v>
+      </c>
+    </row>
+    <row r="66" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>1</v>
       </c>
@@ -8502,8 +9701,29 @@
       <c r="AQ66" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="67" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX66" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A67" s="9" t="s">
         <v>77</v>
       </c>
@@ -8549,8 +9769,15 @@
       <c r="AO67" s="3"/>
       <c r="AP67" s="3"/>
       <c r="AQ67" s="3"/>
-    </row>
-    <row r="68" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR67" s="3"/>
+      <c r="AS67" s="3"/>
+      <c r="AT67" s="3"/>
+      <c r="AU67" s="3"/>
+      <c r="AV67" s="3"/>
+      <c r="AW67" s="3"/>
+      <c r="AX67" s="3"/>
+    </row>
+    <row r="68" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>45</v>
       </c>
@@ -8596,8 +9823,15 @@
       <c r="AO68" s="3"/>
       <c r="AP68" s="3"/>
       <c r="AQ68" s="3"/>
-    </row>
-    <row r="69" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR68" s="3"/>
+      <c r="AS68" s="3"/>
+      <c r="AT68" s="3"/>
+      <c r="AU68" s="3"/>
+      <c r="AV68" s="3"/>
+      <c r="AW68" s="3"/>
+      <c r="AX68" s="3"/>
+    </row>
+    <row r="69" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>2</v>
       </c>
@@ -8727,8 +9961,29 @@
       <c r="AQ69" s="3">
         <v>4.3828070175438896</v>
       </c>
-    </row>
-    <row r="70" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR69" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS69" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT69" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU69" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV69" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW69" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX69" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>0</v>
       </c>
@@ -8858,8 +10113,29 @@
       <c r="AQ70" s="3">
         <v>98.083999999995996</v>
       </c>
-    </row>
-    <row r="71" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR70" s="3">
+        <v>80.000000000015802</v>
+      </c>
+      <c r="AS70" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AT70" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AU70" s="3">
+        <v>80</v>
+      </c>
+      <c r="AV70" s="3">
+        <v>79.7713684210526</v>
+      </c>
+      <c r="AW70" s="3">
+        <v>80</v>
+      </c>
+      <c r="AX70" s="3">
+        <v>79.155508771931395</v>
+      </c>
+    </row>
+    <row r="71" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>1</v>
       </c>
@@ -8989,8 +10265,29 @@
       <c r="AQ71" s="3">
         <v>4.3828070175448</v>
       </c>
-    </row>
-    <row r="72" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR71" s="3">
+        <v>24.083999999980801</v>
+      </c>
+      <c r="AS71" s="3">
+        <v>1.0979999999986001</v>
+      </c>
+      <c r="AT71" s="3">
+        <v>6</v>
+      </c>
+      <c r="AU71" s="3">
+        <v>18.083999999990301</v>
+      </c>
+      <c r="AV71" s="3">
+        <v>18.9284912280689</v>
+      </c>
+      <c r="AW71" s="3">
+        <v>19.103999999993601</v>
+      </c>
+      <c r="AX71" s="3">
+        <v>18.928491228068498</v>
+      </c>
+    </row>
+    <row r="72" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>75</v>
       </c>
@@ -9120,8 +10417,29 @@
       <c r="AQ72" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="73" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX72" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>46</v>
       </c>
@@ -9167,8 +10485,15 @@
       <c r="AO73" s="3"/>
       <c r="AP73" s="3"/>
       <c r="AQ73" s="3"/>
-    </row>
-    <row r="74" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR73" s="3"/>
+      <c r="AS73" s="3"/>
+      <c r="AT73" s="3"/>
+      <c r="AU73" s="3"/>
+      <c r="AV73" s="3"/>
+      <c r="AW73" s="3"/>
+      <c r="AX73" s="3"/>
+    </row>
+    <row r="74" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>0</v>
       </c>
@@ -9298,8 +10623,29 @@
       <c r="AQ74" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="75" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR74" s="3">
+        <v>5.6894561403317097</v>
+      </c>
+      <c r="AS74" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT74" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU74" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV74" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW74" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX74" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>24</v>
       </c>
@@ -9429,8 +10775,29 @@
       <c r="AQ75" s="3">
         <v>98.084000000000003</v>
       </c>
-    </row>
-    <row r="76" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR75" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AS75" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AT75" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AU75" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AV75" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AW75" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AX75" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="76" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>1</v>
       </c>
@@ -9560,8 +10927,29 @@
       <c r="AQ76" s="3">
         <v>2.98677113388483</v>
       </c>
-    </row>
-    <row r="77" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR76" s="3">
+        <v>24.083999999980801</v>
+      </c>
+      <c r="AS76" s="3">
+        <v>1.07775020725311</v>
+      </c>
+      <c r="AT76" s="3">
+        <v>6</v>
+      </c>
+      <c r="AU76" s="3">
+        <v>18.083999999990301</v>
+      </c>
+      <c r="AV76" s="3">
+        <v>18.9284912280689</v>
+      </c>
+      <c r="AW76" s="3">
+        <v>19.103999999993601</v>
+      </c>
+      <c r="AX76" s="3">
+        <v>18.928491228068498</v>
+      </c>
+    </row>
+    <row r="77" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>23</v>
       </c>
@@ -9607,8 +10995,15 @@
       <c r="AO77" s="3"/>
       <c r="AP77" s="3"/>
       <c r="AQ77" s="3"/>
-    </row>
-    <row r="78" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR77" s="3"/>
+      <c r="AS77" s="3"/>
+      <c r="AT77" s="3"/>
+      <c r="AU77" s="3"/>
+      <c r="AV77" s="3"/>
+      <c r="AW77" s="3"/>
+      <c r="AX77" s="3"/>
+    </row>
+    <row r="78" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>2</v>
       </c>
@@ -9738,8 +11133,29 @@
       <c r="AQ78" s="3">
         <v>35.0624561403515</v>
       </c>
-    </row>
-    <row r="79" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX78" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>0</v>
       </c>
@@ -9869,8 +11285,29 @@
       <c r="AQ79" s="3">
         <v>7669973.9832275799</v>
       </c>
-    </row>
-    <row r="80" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR79" s="3">
+        <v>7718560.1127040498</v>
+      </c>
+      <c r="AS79" s="3">
+        <v>7645987.5474986099</v>
+      </c>
+      <c r="AT79" s="3">
+        <v>7688039.5546650495</v>
+      </c>
+      <c r="AU79" s="3">
+        <v>7701385.7281561298</v>
+      </c>
+      <c r="AV79" s="3">
+        <v>7647772.8690141803</v>
+      </c>
+      <c r="AW79" s="3">
+        <v>7725720.7734477501</v>
+      </c>
+      <c r="AX79" s="3">
+        <v>7671740.7152322195</v>
+      </c>
+    </row>
+    <row r="80" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>1</v>
       </c>
@@ -10000,8 +11437,29 @@
       <c r="AQ80" s="3">
         <v>4.3828070175448</v>
       </c>
-    </row>
-    <row r="81" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR80" s="3">
+        <v>398831.03999970399</v>
+      </c>
+      <c r="AS80" s="3">
+        <v>2.1899999999972</v>
+      </c>
+      <c r="AT80" s="3">
+        <v>99359.999999997701</v>
+      </c>
+      <c r="AU80" s="3">
+        <v>305269.24799992499</v>
+      </c>
+      <c r="AV80" s="3">
+        <v>9840.0554352409108</v>
+      </c>
+      <c r="AW80" s="3">
+        <v>306999.21599986602</v>
+      </c>
+      <c r="AX80" s="3">
+        <v>9546.6035438602194</v>
+      </c>
+    </row>
+    <row r="81" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>35</v>
       </c>
@@ -10131,8 +11589,29 @@
       <c r="AQ81" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="82" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX81" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>22</v>
       </c>
@@ -10178,8 +11657,15 @@
       <c r="AO82" s="3"/>
       <c r="AP82" s="3"/>
       <c r="AQ82" s="3"/>
-    </row>
-    <row r="83" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR82" s="3"/>
+      <c r="AS82" s="3"/>
+      <c r="AT82" s="3"/>
+      <c r="AU82" s="3"/>
+      <c r="AV82" s="3"/>
+      <c r="AW82" s="3"/>
+      <c r="AX82" s="3"/>
+    </row>
+    <row r="83" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>0</v>
       </c>
@@ -10309,8 +11795,29 @@
       <c r="AQ83" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="84" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR83" s="3">
+        <v>195.30698254971401</v>
+      </c>
+      <c r="AS83" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT83" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU83" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV83" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW83" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX83" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>24</v>
       </c>
@@ -10440,8 +11947,29 @@
       <c r="AQ84" s="3">
         <v>7670008.2503171796</v>
       </c>
-    </row>
-    <row r="85" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR84" s="3">
+        <v>7645987.1500695003</v>
+      </c>
+      <c r="AS84" s="3">
+        <v>7645987.1500695003</v>
+      </c>
+      <c r="AT84" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+      <c r="AU84" s="3">
+        <v>7645987.1500695003</v>
+      </c>
+      <c r="AV84" s="3">
+        <v>7645987.1500695003</v>
+      </c>
+      <c r="AW84" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+      <c r="AX84" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+    </row>
+    <row r="85" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>1</v>
       </c>
@@ -10571,8 +12099,29 @@
       <c r="AQ85" s="3">
         <v>5.1781746426569004</v>
       </c>
-    </row>
-    <row r="86" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR85" s="3">
+        <v>471208.69565184298</v>
+      </c>
+      <c r="AS85" s="3">
+        <v>2.5874291115096399</v>
+      </c>
+      <c r="AT85" s="3">
+        <v>117391.304347824</v>
+      </c>
+      <c r="AU85" s="3">
+        <v>360667.82608691801</v>
+      </c>
+      <c r="AV85" s="3">
+        <v>11625.7743800105</v>
+      </c>
+      <c r="AW85" s="3">
+        <v>362711.739130278</v>
+      </c>
+      <c r="AX85" s="3">
+        <v>11279.0684591919</v>
+      </c>
+    </row>
+    <row r="86" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>27</v>
       </c>
@@ -10618,8 +12167,15 @@
       <c r="AO86" s="3"/>
       <c r="AP86" s="3"/>
       <c r="AQ86" s="3"/>
-    </row>
-    <row r="87" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR86" s="3"/>
+      <c r="AS86" s="3"/>
+      <c r="AT86" s="3"/>
+      <c r="AU86" s="3"/>
+      <c r="AV86" s="3"/>
+      <c r="AW86" s="3"/>
+      <c r="AX86" s="3"/>
+    </row>
+    <row r="87" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>2</v>
       </c>
@@ -10749,8 +12305,29 @@
       <c r="AQ87" s="3">
         <v>10704.522056646199</v>
       </c>
-    </row>
-    <row r="88" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR87" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS87" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT87" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU87" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV87" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW87" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX87" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>0</v>
       </c>
@@ -10880,8 +12457,29 @@
       <c r="AQ88" s="3">
         <v>331459515.49467301</v>
       </c>
-    </row>
-    <row r="89" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR88" s="3">
+        <v>321380196.18409997</v>
+      </c>
+      <c r="AS88" s="3">
+        <v>341287804.88261598</v>
+      </c>
+      <c r="AT88" s="3">
+        <v>326897074.889341</v>
+      </c>
+      <c r="AU88" s="3">
+        <v>326054995.69194901</v>
+      </c>
+      <c r="AV88" s="3">
+        <v>339864580.35255897</v>
+      </c>
+      <c r="AW88" s="3">
+        <v>317483522.54990101</v>
+      </c>
+      <c r="AX88" s="3">
+        <v>330594342.69532299</v>
+      </c>
+    </row>
+    <row r="89" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>1</v>
       </c>
@@ -11011,8 +12609,29 @@
       <c r="AQ89" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="90" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX89" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>28</v>
       </c>
@@ -11058,8 +12677,15 @@
       <c r="AO90" s="3"/>
       <c r="AP90" s="3"/>
       <c r="AQ90" s="3"/>
-    </row>
-    <row r="91" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR90" s="3"/>
+      <c r="AS90" s="3"/>
+      <c r="AT90" s="3"/>
+      <c r="AU90" s="3"/>
+      <c r="AV90" s="3"/>
+      <c r="AW90" s="3"/>
+      <c r="AX90" s="3"/>
+    </row>
+    <row r="91" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>0</v>
       </c>
@@ -11189,8 +12815,29 @@
       <c r="AQ91" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="92" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR91" s="3">
+        <v>11438.8122982648</v>
+      </c>
+      <c r="AS91" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT91" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU91" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV91" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW91" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX91" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>24</v>
       </c>
@@ -11320,8 +12967,29 @@
       <c r="AQ92" s="3">
         <v>76700082503.154099</v>
       </c>
-    </row>
-    <row r="93" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR92" s="3">
+        <v>76459871500.705399</v>
+      </c>
+      <c r="AS92" s="3">
+        <v>76459871500.705399</v>
+      </c>
+      <c r="AT92" s="3">
+        <v>76700082503.154099</v>
+      </c>
+      <c r="AU92" s="3">
+        <v>76459871500.705399</v>
+      </c>
+      <c r="AV92" s="3">
+        <v>76459871500.705399</v>
+      </c>
+      <c r="AW92" s="3">
+        <v>76700082503.154099</v>
+      </c>
+      <c r="AX92" s="3">
+        <v>76700082503.154099</v>
+      </c>
+    </row>
+    <row r="93" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>1</v>
       </c>
@@ -11451,8 +13119,29 @@
       <c r="AQ93" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="94" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AR93" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS93" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT93" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU93" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV93" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW93" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX93" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:50" x14ac:dyDescent="0.3">
       <c r="V94" s="3"/>
     </row>
   </sheetData>
@@ -11464,30 +13153,30 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00CD46BB-A2D1-4791-8AAC-69869F785713}">
   <dimension ref="A1:M52"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="4" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="9.28515625" customWidth="1"/>
-    <col min="11" max="13" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.33203125" customWidth="1"/>
+    <col min="11" max="13" width="19.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -11507,7 +13196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -11521,7 +13210,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>36</v>
       </c>
@@ -11535,7 +13224,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>37</v>
       </c>
@@ -11549,12 +13238,12 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -11595,7 +13284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -11636,7 +13325,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -11677,12 +13366,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -11723,7 +13412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -11764,7 +13453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -11805,7 +13494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -11846,14 +13535,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E17" s="3"/>
       <c r="H17" s="1"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>10</v>
       </c>
@@ -11873,7 +13562,7 @@
         <v>-13456893997.0168</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -11893,7 +13582,7 @@
         <v>34.491999864578197</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -11913,7 +13602,7 @@
         <v>8.0815127926575099E-5</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -11933,7 +13622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>11</v>
       </c>
@@ -11943,7 +13632,7 @@
       <c r="L22" s="3"/>
       <c r="M22" s="3"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>2</v>
       </c>
@@ -11963,7 +13652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -11983,7 +13672,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>1</v>
       </c>
@@ -12003,7 +13692,7 @@
         <v>15.427141887890601</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>29</v>
       </c>
@@ -12023,7 +13712,7 @@
         <v>98.084000000000003</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>30</v>
       </c>
@@ -12043,7 +13732,7 @@
         <v>2.65685811210931</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>15</v>
       </c>
@@ -12053,7 +13742,7 @@
       <c r="L28" s="3"/>
       <c r="M28" s="3"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>2</v>
       </c>
@@ -12073,7 +13762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>0</v>
       </c>
@@ -12093,7 +13782,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>1</v>
       </c>
@@ -12113,7 +13802,7 @@
         <v>15.427141887890601</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>16</v>
       </c>
@@ -12123,7 +13812,7 @@
       <c r="L32" s="3"/>
       <c r="M32" s="3"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -12143,7 +13832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>0</v>
       </c>
@@ -12163,7 +13852,7 @@
         <v>249617260.626542</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>1</v>
       </c>
@@ -12183,7 +13872,7 @@
         <v>30544228.586336799</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>23</v>
       </c>
@@ -12193,7 +13882,7 @@
       <c r="L36" s="3"/>
       <c r="M36" s="3"/>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>2</v>
       </c>
@@ -12213,7 +13902,7 @@
         <v>3421.3094646414202</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>0</v>
       </c>
@@ -12233,7 +13922,7 @@
         <v>1772151.2791056901</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>1</v>
       </c>
@@ -12253,7 +13942,7 @@
         <v>7524.5956312832805</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>22</v>
       </c>
@@ -12263,7 +13952,7 @@
       <c r="L40" s="3"/>
       <c r="M40" s="3"/>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>0</v>
       </c>
@@ -12283,7 +13972,7 @@
         <v>392888.13096246601</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>24</v>
       </c>
@@ -12303,7 +13992,7 @@
         <v>1381318.93552733</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>35</v>
       </c>
@@ -12323,7 +14012,7 @@
         <v>2522.7416867100901</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -12343,7 +14032,7 @@
         <v>8890.1177118186097</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>27</v>
       </c>
@@ -12353,7 +14042,7 @@
       <c r="L45" s="3"/>
       <c r="M45" s="3"/>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>2</v>
       </c>
@@ -12373,7 +14062,7 @@
         <v>1044521.3102090301</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>0</v>
       </c>
@@ -12393,7 +14082,7 @@
         <v>96512651.699123099</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>1</v>
       </c>
@@ -12413,7 +14102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>28</v>
       </c>
@@ -12423,7 +14112,7 @@
       <c r="L49" s="3"/>
       <c r="M49" s="3"/>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>0</v>
       </c>
@@ -12443,7 +14132,7 @@
         <v>21423303.9657369</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>24</v>
       </c>
@@ -12463,7 +14152,7 @@
         <v>13813189355.2733</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>1</v>
       </c>
@@ -12492,30 +14181,30 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4317E227-4F2F-4766-80E7-4A0C11DC1BA8}">
   <dimension ref="A1:J48"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.28515625" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="9.28515625" customWidth="1"/>
+    <col min="1" max="1" width="29.33203125" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -12526,12 +14215,12 @@
         <v>6.8500000000000005E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -12563,7 +14252,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -12595,7 +14284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -12627,12 +14316,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -12664,7 +14353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -12696,7 +14385,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -12728,7 +14417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -12760,14 +14449,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E14" s="3"/>
       <c r="H14" s="1"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -12778,7 +14467,7 @@
         <v>-566684168.67891097</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>32</v>
       </c>
@@ -12789,7 +14478,7 @@
         <v>2.5789999961853001</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -12800,7 +14489,7 @@
         <v>9.2925621330612702E-5</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>31</v>
       </c>
@@ -12811,14 +14500,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>2</v>
       </c>
@@ -12829,7 +14518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>0</v>
       </c>
@@ -12840,7 +14529,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>1</v>
       </c>
@@ -12851,7 +14540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>29</v>
       </c>
@@ -12862,7 +14551,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>30</v>
       </c>
@@ -12873,14 +14562,14 @@
         <v>58.084000000000003</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>2</v>
       </c>
@@ -12891,7 +14580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>0</v>
       </c>
@@ -12902,7 +14591,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>1</v>
       </c>
@@ -12913,14 +14602,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>2</v>
       </c>
@@ -12931,7 +14620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>0</v>
       </c>
@@ -12942,7 +14631,7 @@
         <v>93383545.771093696</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>1</v>
       </c>
@@ -12953,14 +14642,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>2</v>
       </c>
@@ -12971,7 +14660,7 @@
         <v>10839.670693578801</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>0</v>
       </c>
@@ -12982,7 +14671,7 @@
         <v>755352.36146108399</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>1</v>
       </c>
@@ -12993,14 +14682,14 @@
         <v>8697.9159292100794</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>0</v>
       </c>
@@ -13011,7 +14700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>24</v>
       </c>
@@ -13022,7 +14711,7 @@
         <v>764613.58238300995</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>1</v>
       </c>
@@ -13033,14 +14722,14 @@
         <v>10276.3657008625</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>2</v>
       </c>
@@ -13051,7 +14740,7 @@
         <v>1636903.5360916599</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>0</v>
       </c>
@@ -13062,7 +14751,7 @@
         <v>14194345.611482101</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -13073,14 +14762,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>28</v>
       </c>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>0</v>
       </c>
@@ -13091,7 +14780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>24</v>
       </c>
@@ -13102,7 +14791,7 @@
         <v>675898963.597579</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>1</v>
       </c>
@@ -13122,19 +14811,19 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CDE5EF9-418E-4572-AF84-E6DEF6E71829}">
   <dimension ref="A1:M49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="2" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="19.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -13142,12 +14831,12 @@
         <v>45810</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>52</v>
       </c>
@@ -13164,7 +14853,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>51</v>
       </c>
@@ -13178,13 +14867,13 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>44</v>
       </c>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -13216,7 +14905,7 @@
         <v>12.920999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -13248,7 +14937,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -13280,7 +14969,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -13293,7 +14982,7 @@
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -13325,7 +15014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -13357,7 +15046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -13389,7 +15078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>47</v>
       </c>
@@ -13421,7 +15110,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>39</v>
       </c>
@@ -13435,7 +15124,7 @@
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>40</v>
       </c>
@@ -13467,7 +15156,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>42</v>
       </c>
@@ -13481,7 +15170,7 @@
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -13513,7 +15202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>9</v>
       </c>
@@ -13527,7 +15216,7 @@
       <c r="I18" s="3"/>
       <c r="J18" s="3"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>48</v>
       </c>
@@ -13562,7 +15251,7 @@
       <c r="L19" s="3"/>
       <c r="M19" s="3"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -13597,7 +15286,7 @@
       <c r="L20" s="3"/>
       <c r="M20" s="3"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>17</v>
       </c>
@@ -13632,7 +15321,7 @@
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -13667,7 +15356,7 @@
       <c r="L22" s="3"/>
       <c r="M22" s="3"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>41</v>
       </c>
@@ -13702,7 +15391,7 @@
       <c r="L23" s="3"/>
       <c r="M23" s="3"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>45</v>
       </c>
@@ -13719,7 +15408,7 @@
       <c r="L24" s="3"/>
       <c r="M24" s="3"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>2</v>
       </c>
@@ -13754,7 +15443,7 @@
       <c r="L25" s="3"/>
       <c r="M25" s="3"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>0</v>
       </c>
@@ -13789,7 +15478,7 @@
       <c r="L26" s="3"/>
       <c r="M26" s="3"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>1</v>
       </c>
@@ -13824,7 +15513,7 @@
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>46</v>
       </c>
@@ -13841,7 +15530,7 @@
       <c r="L28" s="3"/>
       <c r="M28" s="3"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>0</v>
       </c>
@@ -13876,7 +15565,7 @@
       <c r="L29" s="3"/>
       <c r="M29" s="3"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>24</v>
       </c>
@@ -13911,7 +15600,7 @@
       <c r="L30" s="3"/>
       <c r="M30" s="3"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>1</v>
       </c>
@@ -13946,7 +15635,7 @@
       <c r="L31" s="3"/>
       <c r="M31" s="3"/>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>23</v>
       </c>
@@ -13963,7 +15652,7 @@
       <c r="L32" s="3"/>
       <c r="M32" s="3"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -13998,7 +15687,7 @@
       <c r="L33" s="3"/>
       <c r="M33" s="3"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>0</v>
       </c>
@@ -14033,7 +15722,7 @@
       <c r="L34" s="3"/>
       <c r="M34" s="3"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>1</v>
       </c>
@@ -14068,7 +15757,7 @@
       <c r="L35" s="3"/>
       <c r="M35" s="3"/>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>22</v>
       </c>
@@ -14085,7 +15774,7 @@
       <c r="L36" s="3"/>
       <c r="M36" s="3"/>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>0</v>
       </c>
@@ -14120,7 +15809,7 @@
       <c r="L37" s="3"/>
       <c r="M37" s="3"/>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>24</v>
       </c>
@@ -14155,7 +15844,7 @@
       <c r="L38" s="3"/>
       <c r="M38" s="3"/>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>1</v>
       </c>
@@ -14190,7 +15879,7 @@
       <c r="L39" s="3"/>
       <c r="M39" s="3"/>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>35</v>
       </c>
@@ -14225,7 +15914,7 @@
       <c r="L40" s="3"/>
       <c r="M40" s="3"/>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>27</v>
       </c>
@@ -14242,7 +15931,7 @@
       <c r="L41" s="3"/>
       <c r="M41" s="3"/>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>2</v>
       </c>
@@ -14277,7 +15966,7 @@
       <c r="L42" s="3"/>
       <c r="M42" s="3"/>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>0</v>
       </c>
@@ -14312,7 +16001,7 @@
       <c r="L43" s="3"/>
       <c r="M43" s="3"/>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -14344,7 +16033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>28</v>
       </c>
@@ -14358,7 +16047,7 @@
       <c r="I45" s="3"/>
       <c r="J45" s="3"/>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>0</v>
       </c>
@@ -14390,7 +16079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>24</v>
       </c>
@@ -14422,7 +16111,7 @@
         <v>10737630</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>1</v>
       </c>
@@ -14454,7 +16143,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D49" s="3"/>
     </row>
   </sheetData>
@@ -14467,16 +16156,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4F0EF5-9E64-45A3-AF76-8FD0E53934FE}">
   <dimension ref="A1:G53"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" customWidth="1"/>
+    <col min="1" max="1" width="36.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" customWidth="1"/>
     <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.85546875" customWidth="1"/>
+    <col min="6" max="6" width="13.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -14484,12 +16173,12 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>55</v>
       </c>
@@ -14497,7 +16186,7 @@
         <v>6624</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>52</v>
       </c>
@@ -14517,7 +16206,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>57</v>
       </c>
@@ -14537,7 +16226,7 @@
         <v>8783</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>58</v>
       </c>
@@ -14553,7 +16242,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>44</v>
       </c>
@@ -14563,7 +16252,7 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -14583,7 +16272,7 @@
         <v>12.920999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -14603,7 +16292,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -14623,7 +16312,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -14633,7 +16322,7 @@
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -14653,7 +16342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -14673,7 +16362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -14693,7 +16382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>47</v>
       </c>
@@ -14713,7 +16402,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>39</v>
       </c>
@@ -14723,7 +16412,7 @@
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -14743,7 +16432,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>42</v>
       </c>
@@ -14753,7 +16442,7 @@
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>43</v>
       </c>
@@ -14773,7 +16462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>9</v>
       </c>
@@ -14783,7 +16472,7 @@
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>48</v>
       </c>
@@ -14803,7 +16492,7 @@
         <v>-503145897.59350002</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>54</v>
       </c>
@@ -14823,7 +16512,7 @@
         <v>9546602.4064993802</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -14843,7 +16532,7 @@
         <v>0.26200008392333901</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>17</v>
       </c>
@@ -14863,7 +16552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>31</v>
       </c>
@@ -14883,7 +16572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>41</v>
       </c>
@@ -14903,7 +16592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>56</v>
       </c>
@@ -14917,7 +16606,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>59</v>
       </c>
@@ -14934,7 +16623,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>45</v>
       </c>
@@ -14944,7 +16633,7 @@
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>2</v>
       </c>
@@ -14964,7 +16653,7 @@
         <v>12.920999999999999</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>0</v>
       </c>
@@ -14984,7 +16673,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>1</v>
       </c>
@@ -15004,7 +16693,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>46</v>
       </c>
@@ -15014,7 +16703,7 @@
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>0</v>
       </c>
@@ -15034,7 +16723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>24</v>
       </c>
@@ -15054,7 +16743,7 @@
         <v>54.920999999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>1</v>
       </c>
@@ -15074,7 +16763,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>23</v>
       </c>
@@ -15084,7 +16773,7 @@
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>2</v>
       </c>
@@ -15104,7 +16793,7 @@
         <v>3000.0191999999902</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>0</v>
       </c>
@@ -15124,7 +16813,7 @@
         <v>202367.83931946999</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>1</v>
       </c>
@@ -15144,7 +16833,7 @@
         <v>1685.0463999999899</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>22</v>
       </c>
@@ -15154,7 +16843,7 @@
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>0</v>
       </c>
@@ -15174,7 +16863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>24</v>
       </c>
@@ -15194,7 +16883,7 @@
         <v>205050.0656</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -15214,7 +16903,7 @@
         <v>2002.83931947069</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>35</v>
       </c>
@@ -15234,7 +16923,7 @@
         <v>26.9344</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>27</v>
       </c>
@@ -15244,7 +16933,7 @@
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>2</v>
       </c>
@@ -15264,7 +16953,7 @@
         <v>915901.94275649404</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>0</v>
       </c>
@@ -15284,7 +16973,7 @@
         <v>8563364.4637428895</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>1</v>
       </c>
@@ -15304,7 +16993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>28</v>
       </c>
@@ -15314,7 +17003,7 @@
       <c r="E50" s="4"/>
       <c r="F50" s="4"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>0</v>
       </c>
@@ -15334,7 +17023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>24</v>
       </c>
@@ -15354,7 +17043,7 @@
         <v>512625164</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
add option to disallow new backup generation
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\Desktop\ongoing_projects\MVS\dev\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64E1FE99-4847-4C52-A1B4-95B198788DB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3B7575E-8CFE-4749-B767-C34A9A1CBE2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Experiments" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="105">
   <si>
     <t>Grid</t>
   </si>
@@ -374,9 +374,6 @@
   </si>
   <si>
     <t>benefit per year</t>
-  </si>
-  <si>
-    <t>lower optimality gap; zero new backup installation; no lock-in effect</t>
   </si>
 </sst>
 </file>
@@ -780,28 +777,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J46"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.33203125" customWidth="1"/>
-    <col min="7" max="8" width="9.33203125" customWidth="1"/>
+    <col min="1" max="1" width="29.28515625" customWidth="1"/>
+    <col min="7" max="8" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -833,7 +830,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -865,7 +862,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -897,12 +894,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -934,7 +931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -966,7 +963,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -998,7 +995,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -1030,179 +1027,179 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E12" s="1"/>
       <c r="H12" s="1"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>1</v>
       </c>
@@ -1216,21 +1213,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEB77188-4C54-4D05-A0BB-AB8E292CE16E}">
   <dimension ref="A1:AZ94"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
     <col min="2" max="13" width="18" bestFit="1" customWidth="1"/>
     <col min="14" max="16" width="19" bestFit="1" customWidth="1"/>
     <col min="17" max="50" width="18" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="2" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1262,7 +1259,7 @@
         <v>250714</v>
       </c>
     </row>
-    <row r="3" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1296,11 +1293,8 @@
       <c r="AU3" t="s">
         <v>103</v>
       </c>
-      <c r="AY3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="4" spans="1:52" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>62</v>
       </c>
@@ -1452,7 +1446,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="5" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>63</v>
       </c>
@@ -1604,7 +1598,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="6" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>90</v>
       </c>
@@ -1718,7 +1712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>57</v>
       </c>
@@ -1870,7 +1864,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>93</v>
       </c>
@@ -1966,7 +1960,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="9" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>81</v>
       </c>
@@ -2118,7 +2112,7 @@
         <v>20.000000000003102</v>
       </c>
     </row>
-    <row r="10" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>82</v>
       </c>
@@ -2270,7 +2264,7 @@
         <v>80.000000000012406</v>
       </c>
     </row>
-    <row r="11" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>64</v>
       </c>
@@ -2422,7 +2416,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="12" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -2574,7 +2568,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>65</v>
       </c>
@@ -2730,7 +2724,7 @@
         <v>5613440.4115295373</v>
       </c>
     </row>
-    <row r="14" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>9</v>
       </c>
@@ -2788,7 +2782,7 @@
         <v>7517855.6325683566</v>
       </c>
     </row>
-    <row r="15" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>67</v>
       </c>
@@ -2944,7 +2938,7 @@
         <v>17640263.884597778</v>
       </c>
     </row>
-    <row r="16" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>66</v>
       </c>
@@ -3096,7 +3090,7 @@
         <v>718.28705191612198</v>
       </c>
     </row>
-    <row r="17" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>80</v>
       </c>
@@ -3251,7 +3245,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="18" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>83</v>
       </c>
@@ -3407,7 +3401,7 @@
         <v>678471.6878691453</v>
       </c>
     </row>
-    <row r="19" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>97</v>
       </c>
@@ -3559,7 +3553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>98</v>
       </c>
@@ -3711,7 +3705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>99</v>
       </c>
@@ -3863,7 +3857,7 @@
         <v>3.2362526863760599</v>
       </c>
     </row>
-    <row r="22" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>100</v>
       </c>
@@ -4015,7 +4009,7 @@
         <v>7.7939723320161498</v>
       </c>
     </row>
-    <row r="23" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>68</v>
       </c>
@@ -4167,7 +4161,7 @@
         <v>331464587.11163098</v>
       </c>
     </row>
-    <row r="24" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>69</v>
       </c>
@@ -4319,7 +4313,7 @@
         <v>330594342.69532299</v>
       </c>
     </row>
-    <row r="25" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>71</v>
       </c>
@@ -4471,7 +4465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>70</v>
       </c>
@@ -4623,7 +4617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>72</v>
       </c>
@@ -4775,7 +4769,7 @@
         <v>331875425.37673599</v>
       </c>
     </row>
-    <row r="28" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>73</v>
       </c>
@@ -4829,7 +4823,7 @@
       <c r="AW28" s="3"/>
       <c r="AX28" s="3"/>
     </row>
-    <row r="29" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>2</v>
       </c>
@@ -4981,7 +4975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>0</v>
       </c>
@@ -5133,7 +5127,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="31" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>1</v>
       </c>
@@ -5285,7 +5279,7 @@
         <v>18.928491228068498</v>
       </c>
     </row>
-    <row r="32" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>15</v>
       </c>
@@ -5339,7 +5333,7 @@
       <c r="AW32" s="3"/>
       <c r="AX32" s="3"/>
     </row>
-    <row r="33" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -5491,7 +5485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>0</v>
       </c>
@@ -5643,7 +5637,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="35" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>1</v>
       </c>
@@ -5795,7 +5789,7 @@
         <v>18.928491228068498</v>
       </c>
     </row>
-    <row r="36" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>74</v>
       </c>
@@ -5849,7 +5843,7 @@
       <c r="AW36" s="3"/>
       <c r="AX36" s="3"/>
     </row>
-    <row r="37" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>2</v>
       </c>
@@ -6001,7 +5995,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>0</v>
       </c>
@@ -6153,7 +6147,7 @@
         <v>276629624.84891802</v>
       </c>
     </row>
-    <row r="39" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>1</v>
       </c>
@@ -6305,7 +6299,7 @@
         <v>55245800.527817801</v>
       </c>
     </row>
-    <row r="40" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
         <v>76</v>
       </c>
@@ -6359,7 +6353,7 @@
       <c r="AW40" s="3"/>
       <c r="AX40" s="3"/>
     </row>
-    <row r="41" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>45</v>
       </c>
@@ -6413,7 +6407,7 @@
       <c r="AW41" s="3"/>
       <c r="AX41" s="3"/>
     </row>
-    <row r="42" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>2</v>
       </c>
@@ -6565,7 +6559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>0</v>
       </c>
@@ -6717,7 +6711,7 @@
         <v>98.084000000000003</v>
       </c>
     </row>
-    <row r="44" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -6869,7 +6863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>75</v>
       </c>
@@ -7021,7 +7015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>46</v>
       </c>
@@ -7075,7 +7069,7 @@
       <c r="AW46" s="3"/>
       <c r="AX46" s="3"/>
     </row>
-    <row r="47" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>0</v>
       </c>
@@ -7227,7 +7221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>24</v>
       </c>
@@ -7379,7 +7373,7 @@
         <v>98.084000000000003</v>
       </c>
     </row>
-    <row r="49" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>1</v>
       </c>
@@ -7531,7 +7525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>23</v>
       </c>
@@ -7585,7 +7579,7 @@
       <c r="AW50" s="3"/>
       <c r="AX50" s="3"/>
     </row>
-    <row r="51" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>2</v>
       </c>
@@ -7737,7 +7731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>0</v>
       </c>
@@ -7889,7 +7883,7 @@
         <v>7670008.2503171796</v>
       </c>
     </row>
-    <row r="53" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>1</v>
       </c>
@@ -8041,7 +8035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>35</v>
       </c>
@@ -8193,7 +8187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>22</v>
       </c>
@@ -8247,7 +8241,7 @@
       <c r="AW55" s="3"/>
       <c r="AX55" s="3"/>
     </row>
-    <row r="56" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>0</v>
       </c>
@@ -8399,7 +8393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>24</v>
       </c>
@@ -8551,7 +8545,7 @@
         <v>7670008.2503171796</v>
       </c>
     </row>
-    <row r="58" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>1</v>
       </c>
@@ -8703,7 +8697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>27</v>
       </c>
@@ -8757,7 +8751,7 @@
       <c r="AW59" s="3"/>
       <c r="AX59" s="3"/>
     </row>
-    <row r="60" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>2</v>
       </c>
@@ -8909,7 +8903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>0</v>
       </c>
@@ -9061,7 +9055,7 @@
         <v>331464587.11163098</v>
       </c>
     </row>
-    <row r="62" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>1</v>
       </c>
@@ -9213,7 +9207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>28</v>
       </c>
@@ -9267,7 +9261,7 @@
       <c r="AW63" s="3"/>
       <c r="AX63" s="3"/>
     </row>
-    <row r="64" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>0</v>
       </c>
@@ -9419,7 +9413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>24</v>
       </c>
@@ -9571,7 +9565,7 @@
         <v>76700082503.154099</v>
       </c>
     </row>
-    <row r="66" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>1</v>
       </c>
@@ -9723,7 +9717,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A67" s="9" t="s">
         <v>77</v>
       </c>
@@ -9777,7 +9771,7 @@
       <c r="AW67" s="3"/>
       <c r="AX67" s="3"/>
     </row>
-    <row r="68" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>45</v>
       </c>
@@ -9831,7 +9825,7 @@
       <c r="AW68" s="3"/>
       <c r="AX68" s="3"/>
     </row>
-    <row r="69" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>2</v>
       </c>
@@ -9983,7 +9977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>0</v>
       </c>
@@ -10135,7 +10129,7 @@
         <v>79.155508771931395</v>
       </c>
     </row>
-    <row r="71" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>1</v>
       </c>
@@ -10287,7 +10281,7 @@
         <v>18.928491228068498</v>
       </c>
     </row>
-    <row r="72" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>75</v>
       </c>
@@ -10439,7 +10433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>46</v>
       </c>
@@ -10493,7 +10487,7 @@
       <c r="AW73" s="3"/>
       <c r="AX73" s="3"/>
     </row>
-    <row r="74" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>0</v>
       </c>
@@ -10645,7 +10639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>24</v>
       </c>
@@ -10797,7 +10791,7 @@
         <v>98.084000000000003</v>
       </c>
     </row>
-    <row r="76" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>1</v>
       </c>
@@ -10949,7 +10943,7 @@
         <v>18.928491228068498</v>
       </c>
     </row>
-    <row r="77" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>23</v>
       </c>
@@ -11003,7 +10997,7 @@
       <c r="AW77" s="3"/>
       <c r="AX77" s="3"/>
     </row>
-    <row r="78" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>2</v>
       </c>
@@ -11155,7 +11149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>0</v>
       </c>
@@ -11307,7 +11301,7 @@
         <v>7671740.7152322195</v>
       </c>
     </row>
-    <row r="80" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>1</v>
       </c>
@@ -11459,7 +11453,7 @@
         <v>9546.6035438602194</v>
       </c>
     </row>
-    <row r="81" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>35</v>
       </c>
@@ -11611,7 +11605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>22</v>
       </c>
@@ -11665,7 +11659,7 @@
       <c r="AW82" s="3"/>
       <c r="AX82" s="3"/>
     </row>
-    <row r="83" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>0</v>
       </c>
@@ -11817,7 +11811,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>24</v>
       </c>
@@ -11969,7 +11963,7 @@
         <v>7670008.2503171796</v>
       </c>
     </row>
-    <row r="85" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>1</v>
       </c>
@@ -12121,7 +12115,7 @@
         <v>11279.0684591919</v>
       </c>
     </row>
-    <row r="86" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>27</v>
       </c>
@@ -12175,7 +12169,7 @@
       <c r="AW86" s="3"/>
       <c r="AX86" s="3"/>
     </row>
-    <row r="87" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>2</v>
       </c>
@@ -12327,7 +12321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>0</v>
       </c>
@@ -12479,7 +12473,7 @@
         <v>330594342.69532299</v>
       </c>
     </row>
-    <row r="89" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>1</v>
       </c>
@@ -12631,7 +12625,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>28</v>
       </c>
@@ -12685,7 +12679,7 @@
       <c r="AW90" s="3"/>
       <c r="AX90" s="3"/>
     </row>
-    <row r="91" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>0</v>
       </c>
@@ -12837,7 +12831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>24</v>
       </c>
@@ -12989,7 +12983,7 @@
         <v>76700082503.154099</v>
       </c>
     </row>
-    <row r="93" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>1</v>
       </c>
@@ -13141,7 +13135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:50" x14ac:dyDescent="0.25">
       <c r="V94" s="3"/>
     </row>
   </sheetData>
@@ -13153,30 +13147,30 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00CD46BB-A2D1-4791-8AAC-69869F785713}">
   <dimension ref="A1:M52"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="4" max="5" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="9.33203125" customWidth="1"/>
-    <col min="11" max="13" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.28515625" customWidth="1"/>
+    <col min="11" max="13" width="19.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -13196,7 +13190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -13210,7 +13204,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>36</v>
       </c>
@@ -13224,7 +13218,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>37</v>
       </c>
@@ -13238,12 +13232,12 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -13284,7 +13278,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -13325,7 +13319,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -13366,12 +13360,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -13412,7 +13406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -13453,7 +13447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -13494,7 +13488,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -13535,14 +13529,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E17" s="3"/>
       <c r="H17" s="1"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>10</v>
       </c>
@@ -13562,7 +13556,7 @@
         <v>-13456893997.0168</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -13582,7 +13576,7 @@
         <v>34.491999864578197</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -13602,7 +13596,7 @@
         <v>8.0815127926575099E-5</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -13622,7 +13616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>11</v>
       </c>
@@ -13632,7 +13626,7 @@
       <c r="L22" s="3"/>
       <c r="M22" s="3"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>2</v>
       </c>
@@ -13652,7 +13646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -13672,7 +13666,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>1</v>
       </c>
@@ -13692,7 +13686,7 @@
         <v>15.427141887890601</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>29</v>
       </c>
@@ -13712,7 +13706,7 @@
         <v>98.084000000000003</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>30</v>
       </c>
@@ -13732,7 +13726,7 @@
         <v>2.65685811210931</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>15</v>
       </c>
@@ -13742,7 +13736,7 @@
       <c r="L28" s="3"/>
       <c r="M28" s="3"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>2</v>
       </c>
@@ -13762,7 +13756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>0</v>
       </c>
@@ -13782,7 +13776,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>1</v>
       </c>
@@ -13802,7 +13796,7 @@
         <v>15.427141887890601</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>16</v>
       </c>
@@ -13812,7 +13806,7 @@
       <c r="L32" s="3"/>
       <c r="M32" s="3"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -13832,7 +13826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>0</v>
       </c>
@@ -13852,7 +13846,7 @@
         <v>249617260.626542</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>1</v>
       </c>
@@ -13872,7 +13866,7 @@
         <v>30544228.586336799</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>23</v>
       </c>
@@ -13882,7 +13876,7 @@
       <c r="L36" s="3"/>
       <c r="M36" s="3"/>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>2</v>
       </c>
@@ -13902,7 +13896,7 @@
         <v>3421.3094646414202</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>0</v>
       </c>
@@ -13922,7 +13916,7 @@
         <v>1772151.2791056901</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>1</v>
       </c>
@@ -13942,7 +13936,7 @@
         <v>7524.5956312832805</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>22</v>
       </c>
@@ -13952,7 +13946,7 @@
       <c r="L40" s="3"/>
       <c r="M40" s="3"/>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>0</v>
       </c>
@@ -13972,7 +13966,7 @@
         <v>392888.13096246601</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>24</v>
       </c>
@@ -13992,7 +13986,7 @@
         <v>1381318.93552733</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>35</v>
       </c>
@@ -14012,7 +14006,7 @@
         <v>2522.7416867100901</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -14032,7 +14026,7 @@
         <v>8890.1177118186097</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>27</v>
       </c>
@@ -14042,7 +14036,7 @@
       <c r="L45" s="3"/>
       <c r="M45" s="3"/>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>2</v>
       </c>
@@ -14062,7 +14056,7 @@
         <v>1044521.3102090301</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>0</v>
       </c>
@@ -14082,7 +14076,7 @@
         <v>96512651.699123099</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>1</v>
       </c>
@@ -14102,7 +14096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>28</v>
       </c>
@@ -14112,7 +14106,7 @@
       <c r="L49" s="3"/>
       <c r="M49" s="3"/>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>0</v>
       </c>
@@ -14132,7 +14126,7 @@
         <v>21423303.9657369</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>24</v>
       </c>
@@ -14152,7 +14146,7 @@
         <v>13813189355.2733</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>1</v>
       </c>
@@ -14181,30 +14175,30 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4317E227-4F2F-4766-80E7-4A0C11DC1BA8}">
   <dimension ref="A1:J48"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.33203125" customWidth="1"/>
-    <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="9.33203125" customWidth="1"/>
+    <col min="1" max="1" width="29.28515625" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -14215,12 +14209,12 @@
         <v>6.8500000000000005E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -14252,7 +14246,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -14284,7 +14278,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -14316,12 +14310,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -14353,7 +14347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -14385,7 +14379,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -14417,7 +14411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -14449,14 +14443,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E14" s="3"/>
       <c r="H14" s="1"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -14467,7 +14461,7 @@
         <v>-566684168.67891097</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>32</v>
       </c>
@@ -14478,7 +14472,7 @@
         <v>2.5789999961853001</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -14489,7 +14483,7 @@
         <v>9.2925621330612702E-5</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>31</v>
       </c>
@@ -14500,14 +14494,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>2</v>
       </c>
@@ -14518,7 +14512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>0</v>
       </c>
@@ -14529,7 +14523,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>1</v>
       </c>
@@ -14540,7 +14534,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>29</v>
       </c>
@@ -14551,7 +14545,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>30</v>
       </c>
@@ -14562,14 +14556,14 @@
         <v>58.084000000000003</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>2</v>
       </c>
@@ -14580,7 +14574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>0</v>
       </c>
@@ -14591,7 +14585,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>1</v>
       </c>
@@ -14602,14 +14596,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>2</v>
       </c>
@@ -14620,7 +14614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>0</v>
       </c>
@@ -14631,7 +14625,7 @@
         <v>93383545.771093696</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>1</v>
       </c>
@@ -14642,14 +14636,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>2</v>
       </c>
@@ -14660,7 +14654,7 @@
         <v>10839.670693578801</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>0</v>
       </c>
@@ -14671,7 +14665,7 @@
         <v>755352.36146108399</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>1</v>
       </c>
@@ -14682,14 +14676,14 @@
         <v>8697.9159292100794</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>0</v>
       </c>
@@ -14700,7 +14694,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>24</v>
       </c>
@@ -14711,7 +14705,7 @@
         <v>764613.58238300995</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>1</v>
       </c>
@@ -14722,14 +14716,14 @@
         <v>10276.3657008625</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>2</v>
       </c>
@@ -14740,7 +14734,7 @@
         <v>1636903.5360916599</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>0</v>
       </c>
@@ -14751,7 +14745,7 @@
         <v>14194345.611482101</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -14762,14 +14756,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>28</v>
       </c>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>0</v>
       </c>
@@ -14780,7 +14774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>24</v>
       </c>
@@ -14791,7 +14785,7 @@
         <v>675898963.597579</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>1</v>
       </c>
@@ -14811,19 +14805,19 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CDE5EF9-418E-4572-AF84-E6DEF6E71829}">
   <dimension ref="A1:M49"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="2" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="19.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -14831,12 +14825,12 @@
         <v>45810</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>52</v>
       </c>
@@ -14853,7 +14847,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>51</v>
       </c>
@@ -14867,13 +14861,13 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>44</v>
       </c>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -14905,7 +14899,7 @@
         <v>12.920999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -14937,7 +14931,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -14969,7 +14963,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -14982,7 +14976,7 @@
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -15014,7 +15008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -15046,7 +15040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -15078,7 +15072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>47</v>
       </c>
@@ -15110,7 +15104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>39</v>
       </c>
@@ -15124,7 +15118,7 @@
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>40</v>
       </c>
@@ -15156,7 +15150,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>42</v>
       </c>
@@ -15170,7 +15164,7 @@
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -15202,7 +15196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>9</v>
       </c>
@@ -15216,7 +15210,7 @@
       <c r="I18" s="3"/>
       <c r="J18" s="3"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>48</v>
       </c>
@@ -15251,7 +15245,7 @@
       <c r="L19" s="3"/>
       <c r="M19" s="3"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -15286,7 +15280,7 @@
       <c r="L20" s="3"/>
       <c r="M20" s="3"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>17</v>
       </c>
@@ -15321,7 +15315,7 @@
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -15356,7 +15350,7 @@
       <c r="L22" s="3"/>
       <c r="M22" s="3"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>41</v>
       </c>
@@ -15391,7 +15385,7 @@
       <c r="L23" s="3"/>
       <c r="M23" s="3"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>45</v>
       </c>
@@ -15408,7 +15402,7 @@
       <c r="L24" s="3"/>
       <c r="M24" s="3"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>2</v>
       </c>
@@ -15443,7 +15437,7 @@
       <c r="L25" s="3"/>
       <c r="M25" s="3"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>0</v>
       </c>
@@ -15478,7 +15472,7 @@
       <c r="L26" s="3"/>
       <c r="M26" s="3"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>1</v>
       </c>
@@ -15513,7 +15507,7 @@
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>46</v>
       </c>
@@ -15530,7 +15524,7 @@
       <c r="L28" s="3"/>
       <c r="M28" s="3"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>0</v>
       </c>
@@ -15565,7 +15559,7 @@
       <c r="L29" s="3"/>
       <c r="M29" s="3"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>24</v>
       </c>
@@ -15600,7 +15594,7 @@
       <c r="L30" s="3"/>
       <c r="M30" s="3"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>1</v>
       </c>
@@ -15635,7 +15629,7 @@
       <c r="L31" s="3"/>
       <c r="M31" s="3"/>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>23</v>
       </c>
@@ -15652,7 +15646,7 @@
       <c r="L32" s="3"/>
       <c r="M32" s="3"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -15687,7 +15681,7 @@
       <c r="L33" s="3"/>
       <c r="M33" s="3"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>0</v>
       </c>
@@ -15722,7 +15716,7 @@
       <c r="L34" s="3"/>
       <c r="M34" s="3"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>1</v>
       </c>
@@ -15757,7 +15751,7 @@
       <c r="L35" s="3"/>
       <c r="M35" s="3"/>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>22</v>
       </c>
@@ -15774,7 +15768,7 @@
       <c r="L36" s="3"/>
       <c r="M36" s="3"/>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>0</v>
       </c>
@@ -15809,7 +15803,7 @@
       <c r="L37" s="3"/>
       <c r="M37" s="3"/>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>24</v>
       </c>
@@ -15844,7 +15838,7 @@
       <c r="L38" s="3"/>
       <c r="M38" s="3"/>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>1</v>
       </c>
@@ -15879,7 +15873,7 @@
       <c r="L39" s="3"/>
       <c r="M39" s="3"/>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>35</v>
       </c>
@@ -15914,7 +15908,7 @@
       <c r="L40" s="3"/>
       <c r="M40" s="3"/>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>27</v>
       </c>
@@ -15931,7 +15925,7 @@
       <c r="L41" s="3"/>
       <c r="M41" s="3"/>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>2</v>
       </c>
@@ -15966,7 +15960,7 @@
       <c r="L42" s="3"/>
       <c r="M42" s="3"/>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>0</v>
       </c>
@@ -16001,7 +15995,7 @@
       <c r="L43" s="3"/>
       <c r="M43" s="3"/>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -16033,7 +16027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>28</v>
       </c>
@@ -16047,7 +16041,7 @@
       <c r="I45" s="3"/>
       <c r="J45" s="3"/>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>0</v>
       </c>
@@ -16079,7 +16073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>24</v>
       </c>
@@ -16111,7 +16105,7 @@
         <v>10737630</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>1</v>
       </c>
@@ -16143,7 +16137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D49" s="3"/>
     </row>
   </sheetData>
@@ -16156,16 +16150,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4F0EF5-9E64-45A3-AF76-8FD0E53934FE}">
   <dimension ref="A1:G53"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" customWidth="1"/>
+    <col min="1" max="1" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" customWidth="1"/>
     <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.88671875" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -16173,12 +16167,12 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>55</v>
       </c>
@@ -16186,7 +16180,7 @@
         <v>6624</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>52</v>
       </c>
@@ -16206,7 +16200,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>57</v>
       </c>
@@ -16226,7 +16220,7 @@
         <v>8783</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>58</v>
       </c>
@@ -16242,7 +16236,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>44</v>
       </c>
@@ -16252,7 +16246,7 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -16272,7 +16266,7 @@
         <v>12.920999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -16292,7 +16286,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -16312,7 +16306,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -16322,7 +16316,7 @@
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -16342,7 +16336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -16362,7 +16356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -16382,7 +16376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>47</v>
       </c>
@@ -16402,7 +16396,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>39</v>
       </c>
@@ -16412,7 +16406,7 @@
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -16432,7 +16426,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>42</v>
       </c>
@@ -16442,7 +16436,7 @@
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>43</v>
       </c>
@@ -16462,7 +16456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>9</v>
       </c>
@@ -16472,7 +16466,7 @@
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>48</v>
       </c>
@@ -16492,7 +16486,7 @@
         <v>-503145897.59350002</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>54</v>
       </c>
@@ -16512,7 +16506,7 @@
         <v>9546602.4064993802</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -16532,7 +16526,7 @@
         <v>0.26200008392333901</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>17</v>
       </c>
@@ -16552,7 +16546,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>31</v>
       </c>
@@ -16572,7 +16566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>41</v>
       </c>
@@ -16592,7 +16586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>56</v>
       </c>
@@ -16606,7 +16600,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>59</v>
       </c>
@@ -16623,7 +16617,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>45</v>
       </c>
@@ -16633,7 +16627,7 @@
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>2</v>
       </c>
@@ -16653,7 +16647,7 @@
         <v>12.920999999999999</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>0</v>
       </c>
@@ -16673,7 +16667,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>1</v>
       </c>
@@ -16693,7 +16687,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>46</v>
       </c>
@@ -16703,7 +16697,7 @@
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>0</v>
       </c>
@@ -16723,7 +16717,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>24</v>
       </c>
@@ -16743,7 +16737,7 @@
         <v>54.920999999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>1</v>
       </c>
@@ -16763,7 +16757,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>23</v>
       </c>
@@ -16773,7 +16767,7 @@
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>2</v>
       </c>
@@ -16793,7 +16787,7 @@
         <v>3000.0191999999902</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>0</v>
       </c>
@@ -16813,7 +16807,7 @@
         <v>202367.83931946999</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>1</v>
       </c>
@@ -16833,7 +16827,7 @@
         <v>1685.0463999999899</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>22</v>
       </c>
@@ -16843,7 +16837,7 @@
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>0</v>
       </c>
@@ -16863,7 +16857,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>24</v>
       </c>
@@ -16883,7 +16877,7 @@
         <v>205050.0656</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -16903,7 +16897,7 @@
         <v>2002.83931947069</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>35</v>
       </c>
@@ -16923,7 +16917,7 @@
         <v>26.9344</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>27</v>
       </c>
@@ -16933,7 +16927,7 @@
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>2</v>
       </c>
@@ -16953,7 +16947,7 @@
         <v>915901.94275649404</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>0</v>
       </c>
@@ -16973,7 +16967,7 @@
         <v>8563364.4637428895</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>1</v>
       </c>
@@ -16993,7 +16987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>28</v>
       </c>
@@ -17003,7 +16997,7 @@
       <c r="E50" s="4"/>
       <c r="F50" s="4"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>0</v>
       </c>
@@ -17023,7 +17017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>24</v>
       </c>
@@ -17043,7 +17037,7 @@
         <v>512625164</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
update results and add group pressie
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\Desktop\ongoing_projects\MVS\dev\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3B7575E-8CFE-4749-B767-C34A9A1CBE2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{599E0BCF-CADF-4298-87E7-378C51F765E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="106">
   <si>
     <t>Grid</t>
   </si>
@@ -373,7 +373,10 @@
     <t>lower optimality gap</t>
   </si>
   <si>
-    <t>benefit per year</t>
+    <t>no new backup generation</t>
+  </si>
+  <si>
+    <t>shinserver</t>
   </si>
 </sst>
 </file>
@@ -1212,22 +1215,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEB77188-4C54-4D05-A0BB-AB8E292CE16E}">
-  <dimension ref="A1:AZ94"/>
+  <dimension ref="A1:BD94"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
     <col min="2" max="13" width="18" bestFit="1" customWidth="1"/>
     <col min="14" max="16" width="19" bestFit="1" customWidth="1"/>
-    <col min="17" max="50" width="18" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="55" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="2" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1258,8 +1260,14 @@
       <c r="AU2">
         <v>250714</v>
       </c>
-    </row>
-    <row r="3" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY2" t="s">
+        <v>105</v>
+      </c>
+      <c r="BA2">
+        <v>250715</v>
+      </c>
+    </row>
+    <row r="3" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1293,8 +1301,14 @@
       <c r="AU3" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="4" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY3" t="s">
+        <v>104</v>
+      </c>
+      <c r="BA3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>62</v>
       </c>
@@ -1445,8 +1459,23 @@
       <c r="AX4" s="3">
         <v>150</v>
       </c>
-    </row>
-    <row r="5" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY4" s="3">
+        <v>150</v>
+      </c>
+      <c r="AZ4" s="3">
+        <v>150</v>
+      </c>
+      <c r="BA4" s="3">
+        <v>150</v>
+      </c>
+      <c r="BB4" s="3">
+        <v>150</v>
+      </c>
+      <c r="BC4" s="3">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="5" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>63</v>
       </c>
@@ -1597,8 +1626,23 @@
       <c r="AX5" s="3">
         <v>10000</v>
       </c>
-    </row>
-    <row r="6" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY5" s="3">
+        <v>10000</v>
+      </c>
+      <c r="AZ5" s="3">
+        <v>10000</v>
+      </c>
+      <c r="BA5" s="3">
+        <v>10000</v>
+      </c>
+      <c r="BB5" s="3">
+        <v>10000</v>
+      </c>
+      <c r="BC5" s="3">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>90</v>
       </c>
@@ -1711,8 +1755,23 @@
       <c r="AX6" s="3" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AZ6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="BA6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="BB6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="BC6" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>57</v>
       </c>
@@ -1863,8 +1922,23 @@
       <c r="AX7" s="3">
         <v>24</v>
       </c>
-    </row>
-    <row r="8" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY7" s="3">
+        <v>24</v>
+      </c>
+      <c r="AZ7" s="3">
+        <v>24</v>
+      </c>
+      <c r="BA7" s="3">
+        <v>24</v>
+      </c>
+      <c r="BB7" s="3">
+        <v>24</v>
+      </c>
+      <c r="BC7" s="3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>93</v>
       </c>
@@ -1959,8 +2033,23 @@
       <c r="AX8" s="3">
         <v>365</v>
       </c>
-    </row>
-    <row r="9" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY8" s="3">
+        <v>183</v>
+      </c>
+      <c r="AZ8" s="3">
+        <v>365</v>
+      </c>
+      <c r="BA8" s="3">
+        <v>365</v>
+      </c>
+      <c r="BB8" s="3">
+        <v>365</v>
+      </c>
+      <c r="BC8" s="3">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="9" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>81</v>
       </c>
@@ -2111,8 +2200,23 @@
       <c r="AX9" s="3">
         <v>20.000000000003102</v>
       </c>
-    </row>
-    <row r="10" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY9" s="3">
+        <v>20.000000000001599</v>
+      </c>
+      <c r="AZ9" s="3">
+        <v>20.000000000003102</v>
+      </c>
+      <c r="BA9" s="3">
+        <v>20.000000000003102</v>
+      </c>
+      <c r="BB9" s="3">
+        <v>20.000000000003102</v>
+      </c>
+      <c r="BC9" s="3">
+        <v>20.000000000003102</v>
+      </c>
+    </row>
+    <row r="10" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>82</v>
       </c>
@@ -2263,8 +2367,23 @@
       <c r="AX10" s="3">
         <v>80.000000000012406</v>
       </c>
-    </row>
-    <row r="11" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY10" s="3">
+        <v>80.000000000006594</v>
+      </c>
+      <c r="AZ10" s="3">
+        <v>80.000000000012406</v>
+      </c>
+      <c r="BA10" s="3">
+        <v>80.000000000012406</v>
+      </c>
+      <c r="BB10" s="3">
+        <v>80.000000000012406</v>
+      </c>
+      <c r="BC10" s="3">
+        <v>80.000000000012406</v>
+      </c>
+    </row>
+    <row r="11" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>64</v>
       </c>
@@ -2415,8 +2534,23 @@
       <c r="AX11" s="3" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="12" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY11" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="AZ11" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="BA11" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="BB11" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="BC11" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -2567,8 +2701,23 @@
       <c r="AX12" s="3" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="13" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="AZ12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="BA12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="BB12" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="BC12" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>65</v>
       </c>
@@ -2719,12 +2868,24 @@
       <c r="AX13" s="3">
         <v>0</v>
       </c>
+      <c r="AY13" s="3">
+        <v>0</v>
+      </c>
       <c r="AZ13" s="3">
-        <f>AW17*AW15/100</f>
-        <v>5613440.4115295373</v>
-      </c>
-    </row>
-    <row r="14" spans="1:52" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="BA13" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB13" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC13" s="3">
+        <v>0</v>
+      </c>
+      <c r="BD13" s="3"/>
+    </row>
+    <row r="14" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>9</v>
       </c>
@@ -2777,12 +2938,14 @@
       <c r="AV14" s="3"/>
       <c r="AW14" s="3"/>
       <c r="AX14" s="3"/>
-      <c r="AZ14" s="3">
-        <f>AX17*AX15/100</f>
-        <v>7517855.6325683566</v>
-      </c>
-    </row>
-    <row r="15" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY14" s="3"/>
+      <c r="AZ14" s="3"/>
+      <c r="BA14" s="3"/>
+      <c r="BB14" s="3"/>
+      <c r="BC14" s="3"/>
+      <c r="BD14" s="3"/>
+    </row>
+    <row r="15" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>67</v>
       </c>
@@ -2933,12 +3096,24 @@
       <c r="AX15" s="5">
         <v>76036916539.554596</v>
       </c>
-      <c r="AZ15" s="14">
-        <f>AW15-AX15</f>
-        <v>17640263.884597778</v>
-      </c>
-    </row>
-    <row r="16" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY15" s="5">
+        <v>75805109783.920593</v>
+      </c>
+      <c r="AZ15" s="5">
+        <v>76059504933.349899</v>
+      </c>
+      <c r="BA15" s="5">
+        <v>76056090504.707596</v>
+      </c>
+      <c r="BB15" s="5">
+        <v>76042535168.811905</v>
+      </c>
+      <c r="BC15" s="5">
+        <v>76008537277.977295</v>
+      </c>
+      <c r="BD15" s="14"/>
+    </row>
+    <row r="16" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>66</v>
       </c>
@@ -3089,8 +3264,23 @@
       <c r="AX16" s="5">
         <v>718.28705191612198</v>
       </c>
-    </row>
-    <row r="17" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY16" s="5">
+        <v>2271.0799810886301</v>
+      </c>
+      <c r="AZ16" s="5">
+        <v>5864.1845259666397</v>
+      </c>
+      <c r="BA16" s="5">
+        <v>3874.6648027896799</v>
+      </c>
+      <c r="BB16" s="5">
+        <v>2720.983689785</v>
+      </c>
+      <c r="BC16" s="3">
+        <v>32.641910791397002</v>
+      </c>
+    </row>
+    <row r="17" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>80</v>
       </c>
@@ -3241,11 +3431,23 @@
       <c r="AX17" s="5">
         <v>9.8871127009175202E-3</v>
       </c>
-      <c r="AZ17" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="18" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY17" s="5">
+        <v>9.7384256526910195E-3</v>
+      </c>
+      <c r="AZ17" s="3">
+        <v>1.35094521307029E-3</v>
+      </c>
+      <c r="BA17" s="3">
+        <v>4.8822517031525502E-4</v>
+      </c>
+      <c r="BB17" s="3">
+        <v>2.8201050966829999E-4</v>
+      </c>
+      <c r="BC17" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>83</v>
       </c>
@@ -3396,12 +3598,24 @@
       <c r="AX18" s="3">
         <v>0</v>
       </c>
-      <c r="AZ18" s="14">
-        <f>AZ15/26</f>
-        <v>678471.6878691453</v>
-      </c>
-    </row>
-    <row r="19" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY18" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ18" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA18" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB18" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC18" s="3">
+        <v>0</v>
+      </c>
+      <c r="BD18" s="14"/>
+    </row>
+    <row r="19" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>97</v>
       </c>
@@ -3552,8 +3766,23 @@
       <c r="AX19" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY19" s="3">
+        <v>150.00000000000099</v>
+      </c>
+      <c r="AZ19" s="3">
+        <v>149.99999999999801</v>
+      </c>
+      <c r="BA19" s="3">
+        <v>149.99999999999801</v>
+      </c>
+      <c r="BB19" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC19" s="3">
+        <v>86.5384615384597</v>
+      </c>
+    </row>
+    <row r="20" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>98</v>
       </c>
@@ -3704,8 +3933,23 @@
       <c r="AX20" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY20" s="3">
+        <v>150.00000000000199</v>
+      </c>
+      <c r="AZ20" s="3">
+        <v>150.00000000000199</v>
+      </c>
+      <c r="BA20" s="3">
+        <v>150.00000000000401</v>
+      </c>
+      <c r="BB20" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC20" s="3">
+        <v>149.99999999999599</v>
+      </c>
+    </row>
+    <row r="21" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>99</v>
       </c>
@@ -3856,8 +4100,23 @@
       <c r="AX21" s="3">
         <v>3.2362526863760599</v>
       </c>
-    </row>
-    <row r="22" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY21" s="3">
+        <v>150.00000000000099</v>
+      </c>
+      <c r="AZ21" s="3">
+        <v>149.99999999999801</v>
+      </c>
+      <c r="BA21" s="3">
+        <v>149.99999999999801</v>
+      </c>
+      <c r="BB21" s="3">
+        <v>3.4608016950840002</v>
+      </c>
+      <c r="BC21" s="3">
+        <v>86.5384615384597</v>
+      </c>
+    </row>
+    <row r="22" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>100</v>
       </c>
@@ -4008,8 +4267,23 @@
       <c r="AX22" s="3">
         <v>7.7939723320161498</v>
       </c>
-    </row>
-    <row r="23" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY22" s="3">
+        <v>150.00000000000199</v>
+      </c>
+      <c r="AZ22" s="3">
+        <v>150.00000000000199</v>
+      </c>
+      <c r="BA22" s="3">
+        <v>150.00000000000401</v>
+      </c>
+      <c r="BB22" s="3">
+        <v>7.6368224929282302</v>
+      </c>
+      <c r="BC22" s="3">
+        <v>149.99999999999599</v>
+      </c>
+    </row>
+    <row r="23" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>68</v>
       </c>
@@ -4160,8 +4434,23 @@
       <c r="AX23" s="3">
         <v>331464587.11163098</v>
       </c>
-    </row>
-    <row r="24" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY23" s="3">
+        <v>325141274.67285299</v>
+      </c>
+      <c r="AZ23" s="3">
+        <v>317366318.5079</v>
+      </c>
+      <c r="BA23" s="3">
+        <v>317710687.31554198</v>
+      </c>
+      <c r="BB23" s="3">
+        <v>331464587.11163098</v>
+      </c>
+      <c r="BC23" s="3">
+        <v>326896914.53985</v>
+      </c>
+    </row>
+    <row r="24" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>69</v>
       </c>
@@ -4312,8 +4601,23 @@
       <c r="AX24" s="3">
         <v>330594342.69532299</v>
       </c>
-    </row>
-    <row r="25" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY24" s="3">
+        <v>325265666.21797502</v>
+      </c>
+      <c r="AZ24" s="3">
+        <v>317494578.07677799</v>
+      </c>
+      <c r="BA24" s="3">
+        <v>317835911.64261001</v>
+      </c>
+      <c r="BB24" s="3">
+        <v>330596991.93365598</v>
+      </c>
+      <c r="BC24" s="3">
+        <v>326897758.52137703</v>
+      </c>
+    </row>
+    <row r="25" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>71</v>
       </c>
@@ -4464,8 +4768,23 @@
       <c r="AX25" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY25" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ25" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA25" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB25" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC25" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>70</v>
       </c>
@@ -4616,8 +4935,23 @@
       <c r="AX26" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY26" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ26" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA26" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB26" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC26" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>72</v>
       </c>
@@ -4768,8 +5102,23 @@
       <c r="AX27" s="3">
         <v>331875425.37673599</v>
       </c>
-    </row>
-    <row r="28" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY27" s="3">
+        <v>329595563.79689097</v>
+      </c>
+      <c r="AZ27" s="3">
+        <v>323185599.387169</v>
+      </c>
+      <c r="BA27" s="3">
+        <v>326256266.27174997</v>
+      </c>
+      <c r="BB27" s="3">
+        <v>326256266.271761</v>
+      </c>
+      <c r="BC27" s="3">
+        <v>364648141.84630102</v>
+      </c>
+    </row>
+    <row r="28" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>73</v>
       </c>
@@ -4822,8 +5171,13 @@
       <c r="AV28" s="3"/>
       <c r="AW28" s="3"/>
       <c r="AX28" s="3"/>
-    </row>
-    <row r="29" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY28" s="3"/>
+      <c r="AZ28" s="3"/>
+      <c r="BA28" s="3"/>
+      <c r="BB28" s="3"/>
+      <c r="BC28" s="3"/>
+    </row>
+    <row r="29" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>2</v>
       </c>
@@ -4974,8 +5328,23 @@
       <c r="AX29" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ29" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA29" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB29" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC29" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>0</v>
       </c>
@@ -5126,8 +5495,23 @@
       <c r="AX30" s="5">
         <v>120</v>
       </c>
-    </row>
-    <row r="31" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY30" s="5">
+        <v>160</v>
+      </c>
+      <c r="AZ30" s="5">
+        <v>120</v>
+      </c>
+      <c r="BA30" s="5">
+        <v>120</v>
+      </c>
+      <c r="BB30" s="5">
+        <v>120</v>
+      </c>
+      <c r="BC30" s="3">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="31" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>1</v>
       </c>
@@ -5278,8 +5662,23 @@
       <c r="AX31" s="5">
         <v>18.928491228068498</v>
       </c>
-    </row>
-    <row r="32" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="AY31" s="5">
+        <v>17.87</v>
+      </c>
+      <c r="AZ31" s="5">
+        <v>19.103999999999001</v>
+      </c>
+      <c r="BA31" s="5">
+        <v>19.317999999990899</v>
+      </c>
+      <c r="BB31" s="5">
+        <v>19.317999999999302</v>
+      </c>
+      <c r="BC31" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>15</v>
       </c>
@@ -5332,8 +5731,13 @@
       <c r="AV32" s="3"/>
       <c r="AW32" s="3"/>
       <c r="AX32" s="3"/>
-    </row>
-    <row r="33" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY32" s="3"/>
+      <c r="AZ32" s="3"/>
+      <c r="BA32" s="3"/>
+      <c r="BB32" s="3"/>
+      <c r="BC32" s="3"/>
+    </row>
+    <row r="33" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -5484,8 +5888,23 @@
       <c r="AX33" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ33" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA33" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB33" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC33" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>0</v>
       </c>
@@ -5636,8 +6055,23 @@
       <c r="AX34" s="5">
         <v>120</v>
       </c>
-    </row>
-    <row r="35" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY34" s="5">
+        <v>160</v>
+      </c>
+      <c r="AZ34" s="5">
+        <v>120</v>
+      </c>
+      <c r="BA34" s="5">
+        <v>120</v>
+      </c>
+      <c r="BB34" s="5">
+        <v>120</v>
+      </c>
+      <c r="BC34" s="3">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="35" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>1</v>
       </c>
@@ -5788,8 +6222,23 @@
       <c r="AX35" s="5">
         <v>18.928491228068498</v>
       </c>
-    </row>
-    <row r="36" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY35" s="5">
+        <v>17.87</v>
+      </c>
+      <c r="AZ35" s="5">
+        <v>19.103999999999001</v>
+      </c>
+      <c r="BA35" s="5">
+        <v>19.317999999995699</v>
+      </c>
+      <c r="BB35" s="5">
+        <v>19.3179999999989</v>
+      </c>
+      <c r="BC35" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>74</v>
       </c>
@@ -5842,8 +6291,13 @@
       <c r="AV36" s="3"/>
       <c r="AW36" s="3"/>
       <c r="AX36" s="3"/>
-    </row>
-    <row r="37" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY36" s="3"/>
+      <c r="AZ36" s="3"/>
+      <c r="BA36" s="3"/>
+      <c r="BB36" s="3"/>
+      <c r="BC36" s="3"/>
+    </row>
+    <row r="37" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>2</v>
       </c>
@@ -5994,8 +6448,23 @@
       <c r="AX37" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ37" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA37" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB37" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC37" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>0</v>
       </c>
@@ -6146,8 +6615,23 @@
       <c r="AX38" s="3">
         <v>276629624.84891802</v>
       </c>
-    </row>
-    <row r="39" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY38" s="3">
+        <v>282916661.77730298</v>
+      </c>
+      <c r="AZ38" s="3">
+        <v>276629624.84891802</v>
+      </c>
+      <c r="BA38" s="13">
+        <v>276629624.84891802</v>
+      </c>
+      <c r="BB38" s="3">
+        <v>276629624.84891802</v>
+      </c>
+      <c r="BC38" s="3">
+        <v>364648141.84630102</v>
+      </c>
+    </row>
+    <row r="39" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>1</v>
       </c>
@@ -6298,8 +6782,23 @@
       <c r="AX39" s="3">
         <v>55245800.527817801</v>
       </c>
-    </row>
-    <row r="40" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY39" s="3">
+        <v>46678902.019588701</v>
+      </c>
+      <c r="AZ39" s="3">
+        <v>46555974.538251102</v>
+      </c>
+      <c r="BA39" s="3">
+        <v>49626641.422832303</v>
+      </c>
+      <c r="BB39" s="3">
+        <v>49626641.4228433</v>
+      </c>
+      <c r="BC39" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
         <v>76</v>
       </c>
@@ -6352,8 +6851,13 @@
       <c r="AV40" s="3"/>
       <c r="AW40" s="3"/>
       <c r="AX40" s="3"/>
-    </row>
-    <row r="41" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY40" s="3"/>
+      <c r="AZ40" s="3"/>
+      <c r="BA40" s="3"/>
+      <c r="BB40" s="3"/>
+      <c r="BC40" s="3"/>
+    </row>
+    <row r="41" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>45</v>
       </c>
@@ -6406,8 +6910,13 @@
       <c r="AV41" s="3"/>
       <c r="AW41" s="3"/>
       <c r="AX41" s="3"/>
-    </row>
-    <row r="42" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY41" s="3"/>
+      <c r="AZ41" s="3"/>
+      <c r="BA41" s="3"/>
+      <c r="BB41" s="3"/>
+      <c r="BC41" s="3"/>
+    </row>
+    <row r="42" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>2</v>
       </c>
@@ -6558,8 +7067,23 @@
       <c r="AX42" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY42" s="3">
+        <v>12.92135</v>
+      </c>
+      <c r="AZ42" s="3">
+        <v>12.92135</v>
+      </c>
+      <c r="BA42" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB42" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC42" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>0</v>
       </c>
@@ -6710,8 +7234,23 @@
       <c r="AX43" s="3">
         <v>98.084000000000003</v>
       </c>
-    </row>
-    <row r="44" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY43" s="3">
+        <v>103.908596491228</v>
+      </c>
+      <c r="AZ43" s="3">
+        <v>108.584140350876</v>
+      </c>
+      <c r="BA43" s="3">
+        <v>108.798140350868</v>
+      </c>
+      <c r="BB43" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="BC43" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="44" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -6862,8 +7401,23 @@
       <c r="AX44" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY44" s="3">
+        <v>17.87</v>
+      </c>
+      <c r="AZ44" s="3">
+        <v>19.103999999999001</v>
+      </c>
+      <c r="BA44" s="3">
+        <v>19.317999999990899</v>
+      </c>
+      <c r="BB44" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC44" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="45" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>75</v>
       </c>
@@ -7014,8 +7568,23 @@
       <c r="AX45" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY45" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ45" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA45" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB45" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC45" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>46</v>
       </c>
@@ -7068,8 +7637,13 @@
       <c r="AV46" s="3"/>
       <c r="AW46" s="3"/>
       <c r="AX46" s="3"/>
-    </row>
-    <row r="47" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY46" s="3"/>
+      <c r="AZ46" s="3"/>
+      <c r="BA46" s="3"/>
+      <c r="BB46" s="3"/>
+      <c r="BC46" s="3"/>
+    </row>
+    <row r="47" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>0</v>
       </c>
@@ -7220,8 +7794,23 @@
       <c r="AX47" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY47" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ47" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA47" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB47" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC47" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>24</v>
       </c>
@@ -7372,8 +7961,23 @@
       <c r="AX48" s="3">
         <v>98.084000000000003</v>
       </c>
-    </row>
-    <row r="49" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY48" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AZ48" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="BA48" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="BB48" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="BC48" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="49" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>1</v>
       </c>
@@ -7524,8 +8128,23 @@
       <c r="AX49" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY49" s="3">
+        <v>17.87</v>
+      </c>
+      <c r="AZ49" s="3">
+        <v>19.1039999999991</v>
+      </c>
+      <c r="BA49" s="3">
+        <v>19.317999999990899</v>
+      </c>
+      <c r="BB49" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC49" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>23</v>
       </c>
@@ -7578,8 +8197,13 @@
       <c r="AV50" s="3"/>
       <c r="AW50" s="3"/>
       <c r="AX50" s="3"/>
-    </row>
-    <row r="51" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY50" s="3"/>
+      <c r="AZ50" s="3"/>
+      <c r="BA50" s="3"/>
+      <c r="BB50" s="3"/>
+      <c r="BC50" s="3"/>
+    </row>
+    <row r="51" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>2</v>
       </c>
@@ -7730,8 +8354,23 @@
       <c r="AX51" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="52" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY51" s="5">
+        <v>3479.2323565573802</v>
+      </c>
+      <c r="AZ51" s="5">
+        <v>1938.2025000000001</v>
+      </c>
+      <c r="BA51" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB51" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC51" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>0</v>
       </c>
@@ -7882,8 +8521,23 @@
       <c r="AX52" s="3">
         <v>7670008.2503171796</v>
       </c>
-    </row>
-    <row r="53" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY52" s="3">
+        <v>7695137.8891912401</v>
+      </c>
+      <c r="AZ52" s="3">
+        <v>7720674.3747738795</v>
+      </c>
+      <c r="BA52" s="3">
+        <v>7724323.5477085998</v>
+      </c>
+      <c r="BB52" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+      <c r="BC52" s="3">
+        <v>7688039.5546650495</v>
+      </c>
+    </row>
+    <row r="53" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>1</v>
       </c>
@@ -8034,8 +8688,23 @@
       <c r="AX53" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY53" s="3">
+        <v>290013.07200001698</v>
+      </c>
+      <c r="AZ53" s="3">
+        <v>289871.75999992999</v>
+      </c>
+      <c r="BA53" s="5">
+        <v>299299.91999988299</v>
+      </c>
+      <c r="BB53" s="5">
+        <v>0</v>
+      </c>
+      <c r="BC53" s="3">
+        <v>99359.999999997701</v>
+      </c>
+    </row>
+    <row r="54" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>35</v>
       </c>
@@ -8186,8 +8855,23 @@
       <c r="AX54" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="55" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ54" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA54" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB54" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC54" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>22</v>
       </c>
@@ -8240,8 +8924,13 @@
       <c r="AV55" s="3"/>
       <c r="AW55" s="3"/>
       <c r="AX55" s="3"/>
-    </row>
-    <row r="56" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY55" s="3"/>
+      <c r="AZ55" s="3"/>
+      <c r="BA55" s="3"/>
+      <c r="BB55" s="3"/>
+      <c r="BC55" s="3"/>
+    </row>
+    <row r="56" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>0</v>
       </c>
@@ -8392,8 +9081,23 @@
       <c r="AX56" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="57" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY56" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ56" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA56" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB56" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC56" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>24</v>
       </c>
@@ -8544,8 +9248,23 @@
       <c r="AX57" s="3">
         <v>7670008.2503171796</v>
       </c>
-    </row>
-    <row r="58" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY57" s="3">
+        <v>7645987.1500695003</v>
+      </c>
+      <c r="AZ57" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+      <c r="BA57" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+      <c r="BB57" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+      <c r="BC57" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+    </row>
+    <row r="58" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>1</v>
       </c>
@@ -8696,8 +9415,23 @@
       <c r="AX58" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="59" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY58" s="3">
+        <v>342643.04347831698</v>
+      </c>
+      <c r="AZ58" s="3">
+        <v>342476.08695644501</v>
+      </c>
+      <c r="BA58" s="3">
+        <v>353615.21739113302</v>
+      </c>
+      <c r="BB58" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC58" s="3">
+        <v>117391.304347824</v>
+      </c>
+    </row>
+    <row r="59" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>27</v>
       </c>
@@ -8750,8 +9484,13 @@
       <c r="AV59" s="3"/>
       <c r="AW59" s="3"/>
       <c r="AX59" s="3"/>
-    </row>
-    <row r="60" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY59" s="3"/>
+      <c r="AZ59" s="3"/>
+      <c r="BA59" s="3"/>
+      <c r="BB59" s="3"/>
+      <c r="BC59" s="3"/>
+    </row>
+    <row r="60" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>2</v>
       </c>
@@ -8902,8 +9641,23 @@
       <c r="AX60" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="61" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY60" s="3">
+        <v>1062205.09344478</v>
+      </c>
+      <c r="AZ60" s="3">
+        <v>591730.69132540701</v>
+      </c>
+      <c r="BA60" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB60" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC60" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>0</v>
       </c>
@@ -9054,8 +9808,23 @@
       <c r="AX61" s="3">
         <v>331464587.11163098</v>
       </c>
-    </row>
-    <row r="62" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY61" s="3">
+        <v>324079069.57940698</v>
+      </c>
+      <c r="AZ61" s="3">
+        <v>316774587.81657398</v>
+      </c>
+      <c r="BA61" s="3">
+        <v>317710687.31554198</v>
+      </c>
+      <c r="BB61" s="3">
+        <v>331464587.11163098</v>
+      </c>
+      <c r="BC61" s="3">
+        <v>326896914.53985</v>
+      </c>
+    </row>
+    <row r="62" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>1</v>
       </c>
@@ -9206,8 +9975,23 @@
       <c r="AX62" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY62" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ62" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA62" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB62" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC62" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>28</v>
       </c>
@@ -9260,8 +10044,13 @@
       <c r="AV63" s="3"/>
       <c r="AW63" s="3"/>
       <c r="AX63" s="3"/>
-    </row>
-    <row r="64" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY63" s="3"/>
+      <c r="AZ63" s="3"/>
+      <c r="BA63" s="3"/>
+      <c r="BB63" s="3"/>
+      <c r="BC63" s="3"/>
+    </row>
+    <row r="64" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>0</v>
       </c>
@@ -9412,8 +10201,23 @@
       <c r="AX64" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="65" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY64" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ64" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA64" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB64" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC64" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>24</v>
       </c>
@@ -9564,8 +10368,23 @@
       <c r="AX65" s="3">
         <v>76700082503.154099</v>
       </c>
-    </row>
-    <row r="66" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY65" s="3">
+        <v>76459871500.705399</v>
+      </c>
+      <c r="AZ65" s="3">
+        <v>76700082503.154099</v>
+      </c>
+      <c r="BA65" s="3">
+        <v>76700082503.154099</v>
+      </c>
+      <c r="BB65" s="3">
+        <v>76700082503.154099</v>
+      </c>
+      <c r="BC65" s="3">
+        <v>76700082503.154099</v>
+      </c>
+    </row>
+    <row r="66" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>1</v>
       </c>
@@ -9716,8 +10535,23 @@
       <c r="AX66" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="67" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ66" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA66" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB66" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC66" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A67" s="9" t="s">
         <v>77</v>
       </c>
@@ -9770,8 +10604,13 @@
       <c r="AV67" s="3"/>
       <c r="AW67" s="3"/>
       <c r="AX67" s="3"/>
-    </row>
-    <row r="68" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY67" s="3"/>
+      <c r="AZ67" s="3"/>
+      <c r="BA67" s="3"/>
+      <c r="BB67" s="3"/>
+      <c r="BC67" s="3"/>
+    </row>
+    <row r="68" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>45</v>
       </c>
@@ -9824,8 +10663,13 @@
       <c r="AV68" s="3"/>
       <c r="AW68" s="3"/>
       <c r="AX68" s="3"/>
-    </row>
-    <row r="69" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY68" s="3"/>
+      <c r="AZ68" s="3"/>
+      <c r="BA68" s="3"/>
+      <c r="BB68" s="3"/>
+      <c r="BC68" s="3"/>
+    </row>
+    <row r="69" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>2</v>
       </c>
@@ -9976,8 +10820,23 @@
       <c r="AX69" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="70" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY69" s="3">
+        <v>12.92135</v>
+      </c>
+      <c r="AZ69" s="3">
+        <v>12.92135</v>
+      </c>
+      <c r="BA69" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB69" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC69" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>0</v>
       </c>
@@ -10128,8 +10987,23 @@
       <c r="AX70" s="3">
         <v>79.155508771931395</v>
       </c>
-    </row>
-    <row r="71" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY70" s="3">
+        <v>103.908596491228</v>
+      </c>
+      <c r="AZ70" s="3">
+        <v>80</v>
+      </c>
+      <c r="BA70" s="3">
+        <v>80</v>
+      </c>
+      <c r="BB70" s="3">
+        <v>80</v>
+      </c>
+      <c r="BC70" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="71" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>1</v>
       </c>
@@ -10280,8 +11154,23 @@
       <c r="AX71" s="3">
         <v>18.928491228068498</v>
       </c>
-    </row>
-    <row r="72" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY71" s="3">
+        <v>17.87</v>
+      </c>
+      <c r="AZ71" s="3">
+        <v>19.103999999999001</v>
+      </c>
+      <c r="BA71" s="3">
+        <v>19.317999999990899</v>
+      </c>
+      <c r="BB71" s="3">
+        <v>18.9284912280702</v>
+      </c>
+      <c r="BC71" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="72" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>75</v>
       </c>
@@ -10432,8 +11321,23 @@
       <c r="AX72" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="73" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ72" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA72" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB72" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC72" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>46</v>
       </c>
@@ -10486,8 +11390,13 @@
       <c r="AV73" s="3"/>
       <c r="AW73" s="3"/>
       <c r="AX73" s="3"/>
-    </row>
-    <row r="74" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY73" s="3"/>
+      <c r="AZ73" s="3"/>
+      <c r="BA73" s="3"/>
+      <c r="BB73" s="3"/>
+      <c r="BC73" s="3"/>
+    </row>
+    <row r="74" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>0</v>
       </c>
@@ -10638,8 +11547,23 @@
       <c r="AX74" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="75" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY74" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ74" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA74" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB74" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC74" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>24</v>
       </c>
@@ -10790,8 +11714,23 @@
       <c r="AX75" s="3">
         <v>98.084000000000003</v>
       </c>
-    </row>
-    <row r="76" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY75" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="AZ75" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="BA75" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="BB75" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="BC75" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="76" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>1</v>
       </c>
@@ -10942,8 +11881,23 @@
       <c r="AX76" s="3">
         <v>18.928491228068498</v>
       </c>
-    </row>
-    <row r="77" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY76" s="3">
+        <v>17.87</v>
+      </c>
+      <c r="AZ76" s="3">
+        <v>19.103999999999001</v>
+      </c>
+      <c r="BA76" s="3">
+        <v>19.317999999990899</v>
+      </c>
+      <c r="BB76" s="3">
+        <v>19.317999999999302</v>
+      </c>
+      <c r="BC76" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="77" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>23</v>
       </c>
@@ -10996,8 +11950,13 @@
       <c r="AV77" s="3"/>
       <c r="AW77" s="3"/>
       <c r="AX77" s="3"/>
-    </row>
-    <row r="78" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY77" s="3"/>
+      <c r="AZ77" s="3"/>
+      <c r="BA77" s="3"/>
+      <c r="BB77" s="3"/>
+      <c r="BC77" s="3"/>
+    </row>
+    <row r="78" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>2</v>
       </c>
@@ -11148,8 +12107,23 @@
       <c r="AX78" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="79" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY78" s="3">
+        <v>3489.6831977998299</v>
+      </c>
+      <c r="AZ78" s="3">
+        <v>1947.2908157894699</v>
+      </c>
+      <c r="BA78" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB78" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC78" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>0</v>
       </c>
@@ -11300,8 +12274,23 @@
       <c r="AX79" s="3">
         <v>7671740.7152322195</v>
       </c>
-    </row>
-    <row r="80" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY79" s="3">
+        <v>7695127.43834987</v>
+      </c>
+      <c r="AZ79" s="3">
+        <v>7720665.2864581002</v>
+      </c>
+      <c r="BA79" s="3">
+        <v>7724323.5477082897</v>
+      </c>
+      <c r="BB79" s="3">
+        <v>7671613.4336484103</v>
+      </c>
+      <c r="BC79" s="3">
+        <v>7688039.5546650495</v>
+      </c>
+    </row>
+    <row r="80" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>1</v>
       </c>
@@ -11452,8 +12441,23 @@
       <c r="AX80" s="3">
         <v>9546.6035438602194</v>
       </c>
-    </row>
-    <row r="81" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY80" s="3">
+        <v>290013.07200001599</v>
+      </c>
+      <c r="AZ80" s="3">
+        <v>289871.75999993098</v>
+      </c>
+      <c r="BA80" s="5">
+        <v>299299.919999882</v>
+      </c>
+      <c r="BB80" s="3">
+        <v>8845.22898245529</v>
+      </c>
+      <c r="BC80" s="3">
+        <v>99359.999999997701</v>
+      </c>
+    </row>
+    <row r="81" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>35</v>
       </c>
@@ -11604,8 +12608,23 @@
       <c r="AX81" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="82" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ81" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA81" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB81" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC81" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>22</v>
       </c>
@@ -11658,8 +12677,13 @@
       <c r="AV82" s="3"/>
       <c r="AW82" s="3"/>
       <c r="AX82" s="3"/>
-    </row>
-    <row r="83" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY82" s="3"/>
+      <c r="AZ82" s="3"/>
+      <c r="BA82" s="3"/>
+      <c r="BB82" s="3"/>
+      <c r="BC82" s="3"/>
+    </row>
+    <row r="83" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>0</v>
       </c>
@@ -11810,8 +12834,23 @@
       <c r="AX83" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="84" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY83" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ83" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA83" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB83" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC83" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>24</v>
       </c>
@@ -11962,8 +13001,23 @@
       <c r="AX84" s="3">
         <v>7670008.2503171796</v>
       </c>
-    </row>
-    <row r="85" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY84" s="3">
+        <v>7645987.1500695003</v>
+      </c>
+      <c r="AZ84" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+      <c r="BA84" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+      <c r="BB84" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+      <c r="BC84" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+    </row>
+    <row r="85" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>1</v>
       </c>
@@ -12114,8 +13168,23 @@
       <c r="AX85" s="3">
         <v>11279.0684591919</v>
       </c>
-    </row>
-    <row r="86" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY85" s="3">
+        <v>342643.04347832</v>
+      </c>
+      <c r="AZ85" s="3">
+        <v>342476.08695644798</v>
+      </c>
+      <c r="BA85" s="3">
+        <v>353615.21739113599</v>
+      </c>
+      <c r="BB85" s="3">
+        <v>10450.412313864799</v>
+      </c>
+      <c r="BC85" s="3">
+        <v>117391.304347824</v>
+      </c>
+    </row>
+    <row r="86" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>27</v>
       </c>
@@ -12168,8 +13237,13 @@
       <c r="AV86" s="3"/>
       <c r="AW86" s="3"/>
       <c r="AX86" s="3"/>
-    </row>
-    <row r="87" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY86" s="3"/>
+      <c r="AZ86" s="3"/>
+      <c r="BA86" s="3"/>
+      <c r="BB86" s="3"/>
+      <c r="BC86" s="3"/>
+    </row>
+    <row r="87" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>2</v>
       </c>
@@ -12320,8 +13394,23 @@
       <c r="AX87" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="88" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY87" s="3">
+        <v>1065395.7216238901</v>
+      </c>
+      <c r="AZ87" s="3">
+        <v>594505.34226362896</v>
+      </c>
+      <c r="BA87" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB87" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC87" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>0</v>
       </c>
@@ -12472,8 +13561,23 @@
       <c r="AX88" s="3">
         <v>330594342.69532299</v>
       </c>
-    </row>
-    <row r="89" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY88" s="3">
+        <v>324200270.49634999</v>
+      </c>
+      <c r="AZ88" s="3">
+        <v>316900072.73451501</v>
+      </c>
+      <c r="BA88" s="3">
+        <v>317835911.64261001</v>
+      </c>
+      <c r="BB88" s="3">
+        <v>330596991.93365598</v>
+      </c>
+      <c r="BC88" s="3">
+        <v>326897758.52137703</v>
+      </c>
+    </row>
+    <row r="89" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>1</v>
       </c>
@@ -12624,8 +13728,23 @@
       <c r="AX89" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="90" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ89" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA89" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB89" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC89" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>28</v>
       </c>
@@ -12678,8 +13797,13 @@
       <c r="AV90" s="3"/>
       <c r="AW90" s="3"/>
       <c r="AX90" s="3"/>
-    </row>
-    <row r="91" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY90" s="3"/>
+      <c r="AZ90" s="3"/>
+      <c r="BA90" s="3"/>
+      <c r="BB90" s="3"/>
+      <c r="BC90" s="3"/>
+    </row>
+    <row r="91" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>0</v>
       </c>
@@ -12830,8 +13954,23 @@
       <c r="AX91" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="92" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY91" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ91" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA91" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB91" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC91" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>24</v>
       </c>
@@ -12982,8 +14121,23 @@
       <c r="AX92" s="3">
         <v>76700082503.154099</v>
       </c>
-    </row>
-    <row r="93" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY92" s="3">
+        <v>76459871500.705399</v>
+      </c>
+      <c r="AZ92" s="3">
+        <v>76700082503.154099</v>
+      </c>
+      <c r="BA92" s="3">
+        <v>76700082503.154099</v>
+      </c>
+      <c r="BB92" s="3">
+        <v>76700082503.154099</v>
+      </c>
+      <c r="BC92" s="3">
+        <v>76700082503.154099</v>
+      </c>
+    </row>
+    <row r="93" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>1</v>
       </c>
@@ -13134,8 +14288,23 @@
       <c r="AX93" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="94" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AY93" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ93" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA93" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB93" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC93" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:55" x14ac:dyDescent="0.25">
       <c r="V94" s="3"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add results for low-cost storage on daily operations
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\Desktop\ongoing_projects\MVS\dev\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74988F05-330E-4EF1-AD51-30D28C308C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51193FEC-8BAF-41ED-A48A-DAC001171CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-9030" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Experiments" sheetId="1" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="141">
   <si>
     <t>Grid</t>
   </si>
@@ -467,9 +467,6 @@
     <t>grid_w_storage</t>
   </si>
   <si>
-    <t>free storage</t>
-  </si>
-  <si>
     <t>Max resource investments (MW)</t>
   </si>
   <si>
@@ -480,6 +477,12 @@
   </si>
   <si>
     <t>no_exports</t>
+  </si>
+  <si>
+    <t>low-cost storage</t>
+  </si>
+  <si>
+    <t>repeat runs with daily storage</t>
   </si>
 </sst>
 </file>
@@ -2625,7 +2628,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEB77188-4C54-4D05-A0BB-AB8E292CE16E}">
-  <dimension ref="A1:BO96"/>
+  <dimension ref="A1:BQ96"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
@@ -2635,17 +2638,20 @@
     <col min="57" max="57" width="19.5703125" customWidth="1"/>
     <col min="58" max="58" width="18.28515625" customWidth="1"/>
     <col min="59" max="60" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="61" max="64" width="17.7109375" customWidth="1"/>
-    <col min="66" max="66" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="61" max="66" width="17.7109375" customWidth="1"/>
+    <col min="68" max="68" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="2" spans="1:67" x14ac:dyDescent="0.25">
+      <c r="BL1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -2688,8 +2694,11 @@
       <c r="BI2">
         <v>250807</v>
       </c>
-    </row>
-    <row r="3" spans="1:67" x14ac:dyDescent="0.25">
+      <c r="BK2">
+        <v>250808</v>
+      </c>
+    </row>
+    <row r="3" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -2733,10 +2742,10 @@
         <v>118</v>
       </c>
       <c r="BI3" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="4" spans="1:67" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="4" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>62</v>
       </c>
@@ -2923,13 +2932,23 @@
       <c r="BJ4" s="3">
         <v>150</v>
       </c>
-      <c r="BK4" s="3"/>
-      <c r="BL4" s="3"/>
-      <c r="BN4" t="s">
+      <c r="BK4" s="3">
+        <v>150</v>
+      </c>
+      <c r="BL4" s="3">
+        <v>150</v>
+      </c>
+      <c r="BM4" s="3">
+        <v>150</v>
+      </c>
+      <c r="BN4" s="3">
+        <v>150</v>
+      </c>
+      <c r="BP4" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="5" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>63</v>
       </c>
@@ -3116,16 +3135,26 @@
       <c r="BJ5" s="3">
         <v>0</v>
       </c>
-      <c r="BK5" s="3"/>
-      <c r="BL5" s="3"/>
-      <c r="BN5" t="s">
+      <c r="BK5" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL5" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM5" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN5" s="3">
+        <v>0</v>
+      </c>
+      <c r="BP5" t="s">
         <v>121</v>
       </c>
-      <c r="BO5" t="s">
+      <c r="BQ5" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="6" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>90</v>
       </c>
@@ -3274,13 +3303,23 @@
       <c r="BJ6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="BK6" s="3"/>
-      <c r="BL6" s="3"/>
-      <c r="BN6" t="s">
+      <c r="BK6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="BL6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="BN6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP6" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="7" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>57</v>
       </c>
@@ -3467,18 +3506,28 @@
       <c r="BJ7" s="3">
         <v>8783</v>
       </c>
-      <c r="BK7" s="3"/>
-      <c r="BL7" s="3"/>
+      <c r="BK7" s="3">
+        <v>8783</v>
+      </c>
+      <c r="BL7" s="3">
+        <v>24</v>
+      </c>
+      <c r="BM7" s="3">
+        <v>24</v>
+      </c>
       <c r="BN7" s="3">
-        <f>BG10*BN9/100+BG9*BN11/100</f>
+        <v>24</v>
+      </c>
+      <c r="BP7" s="3">
+        <f>BG10*BP9/100+BG9*BP11/100</f>
         <v>13532045.806827499</v>
       </c>
-      <c r="BO7" s="3">
-        <f>BH10*BO9/100+BH9*BO11/100</f>
+      <c r="BQ7" s="3">
+        <f>BH10*BQ9/100+BH9*BQ11/100</f>
         <v>4543046.5541842831</v>
       </c>
     </row>
-    <row r="8" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>93</v>
       </c>
@@ -3609,13 +3658,23 @@
       <c r="BJ8" s="3">
         <v>1</v>
       </c>
-      <c r="BK8" s="3"/>
-      <c r="BL8" s="3"/>
-      <c r="BN8" t="s">
+      <c r="BK8" s="3">
+        <v>1</v>
+      </c>
+      <c r="BL8" s="3">
+        <v>365</v>
+      </c>
+      <c r="BM8" s="3">
+        <v>365</v>
+      </c>
+      <c r="BN8" s="3">
+        <v>365</v>
+      </c>
+      <c r="BP8" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="9" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>81</v>
       </c>
@@ -3802,18 +3861,28 @@
       <c r="BJ9" s="3">
         <v>20</v>
       </c>
-      <c r="BK9" s="3"/>
-      <c r="BL9" s="3"/>
-      <c r="BN9" s="14">
+      <c r="BK9" s="3">
+        <v>20</v>
+      </c>
+      <c r="BL9" s="3">
+        <v>20.000000000003102</v>
+      </c>
+      <c r="BM9" s="3">
+        <v>20.000000000003102</v>
+      </c>
+      <c r="BN9" s="3">
+        <v>20.000000000003102</v>
+      </c>
+      <c r="BP9" s="14">
         <f>BG25-BH25</f>
         <v>13732381.696135998</v>
       </c>
-      <c r="BO9" s="14">
+      <c r="BQ9" s="14">
         <f>BF25-BE25</f>
         <v>4567672.5717809796</v>
       </c>
     </row>
-    <row r="10" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>82</v>
       </c>
@@ -4000,13 +4069,23 @@
       <c r="BJ10" s="3">
         <v>20</v>
       </c>
-      <c r="BK10" s="3"/>
-      <c r="BL10" s="3"/>
-      <c r="BN10" t="s">
+      <c r="BK10" s="3">
+        <v>20</v>
+      </c>
+      <c r="BL10" s="3">
+        <v>80.000000000012406</v>
+      </c>
+      <c r="BM10" s="3">
+        <v>80.000000000012406</v>
+      </c>
+      <c r="BN10" s="3">
+        <v>80.000000000012406</v>
+      </c>
+      <c r="BP10" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="11" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>64</v>
       </c>
@@ -4193,20 +4272,30 @@
       <c r="BJ11" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="BK11" s="3"/>
-      <c r="BL11" s="3"/>
-      <c r="BN11" s="14">
+      <c r="BK11" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="BL11" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="BM11" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="BN11" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="BP11" s="14">
         <f>BG26-BH26</f>
         <v>12730702.249583006</v>
       </c>
-      <c r="BO11" s="14">
+      <c r="BQ11" s="14">
         <f>BF26-BE26</f>
         <v>4444542.4837939739</v>
       </c>
     </row>
-    <row r="12" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -4268,19 +4357,29 @@
       <c r="BG12" s="3"/>
       <c r="BH12" s="3"/>
       <c r="BI12" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="BJ12" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="BK12" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="BL12" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="BM12" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="BN12" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="BP12" s="14"/>
+      <c r="BQ12" s="14"/>
+    </row>
+    <row r="13" spans="1:69" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>137</v>
-      </c>
-      <c r="BJ12" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="BK12" s="3"/>
-      <c r="BL12" s="3"/>
-      <c r="BN12" s="14"/>
-      <c r="BO12" s="14"/>
-    </row>
-    <row r="13" spans="1:67" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>138</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -4347,12 +4446,22 @@
       <c r="BJ13" s="3">
         <v>1000</v>
       </c>
-      <c r="BK13" s="3"/>
-      <c r="BL13" s="3"/>
-      <c r="BN13" s="14"/>
-      <c r="BO13" s="14"/>
-    </row>
-    <row r="14" spans="1:67" x14ac:dyDescent="0.25">
+      <c r="BK13" s="3">
+        <v>1000</v>
+      </c>
+      <c r="BL13" s="3">
+        <v>1000</v>
+      </c>
+      <c r="BM13" s="3">
+        <v>1000</v>
+      </c>
+      <c r="BN13" s="3">
+        <v>1000</v>
+      </c>
+      <c r="BP13" s="14"/>
+      <c r="BQ13" s="14"/>
+    </row>
+    <row r="14" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -4537,15 +4646,25 @@
         <v>85</v>
       </c>
       <c r="BJ14" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="BK14" s="3"/>
-      <c r="BL14" s="3"/>
-      <c r="BN14" t="s">
+        <v>138</v>
+      </c>
+      <c r="BK14" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="BL14" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="BM14" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="BN14" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="BP14" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="15" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>65</v>
       </c>
@@ -4732,18 +4851,28 @@
       <c r="BJ15" s="3">
         <v>0</v>
       </c>
-      <c r="BK15" s="3"/>
-      <c r="BL15" s="3"/>
-      <c r="BN15" s="14">
+      <c r="BK15" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL15" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM15" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN15" s="3">
+        <v>0</v>
+      </c>
+      <c r="BP15" s="14">
         <f>BF29-BG29</f>
         <v>38523714.222420037</v>
       </c>
-      <c r="BO15" s="14">
+      <c r="BQ15" s="14">
         <f>BF29-BE29</f>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>9</v>
       </c>
@@ -4810,8 +4939,10 @@
       <c r="BJ16" s="3"/>
       <c r="BK16" s="3"/>
       <c r="BL16" s="3"/>
-    </row>
-    <row r="17" spans="1:67" x14ac:dyDescent="0.25">
+      <c r="BM16" s="3"/>
+      <c r="BN16" s="3"/>
+    </row>
+    <row r="17" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>67</v>
       </c>
@@ -4998,13 +5129,23 @@
       <c r="BJ17" s="5">
         <v>-502069865.02486098</v>
       </c>
-      <c r="BK17" s="5"/>
-      <c r="BL17" s="5"/>
-      <c r="BN17" s="14" t="s">
+      <c r="BK17" s="5">
+        <v>-606622189.14133501</v>
+      </c>
+      <c r="BL17" s="5">
+        <v>-423622435.56663299</v>
+      </c>
+      <c r="BM17" s="5">
+        <v>-525293340.18129599</v>
+      </c>
+      <c r="BN17" s="5">
+        <v>-607684781.88519204</v>
+      </c>
+      <c r="BP17" s="14" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="18" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>66</v>
       </c>
@@ -5191,18 +5332,28 @@
       <c r="BJ18" s="3">
         <v>428.86366796493502</v>
       </c>
-      <c r="BK18" s="3"/>
-      <c r="BL18" s="3"/>
-      <c r="BN18" s="14">
-        <f>BN7</f>
+      <c r="BK18" s="13">
+        <v>11910.0523951053</v>
+      </c>
+      <c r="BL18" s="3">
+        <v>784.941906929016</v>
+      </c>
+      <c r="BM18" s="3">
+        <v>469.51246690750099</v>
+      </c>
+      <c r="BN18" s="3">
+        <v>3738.2014219760799</v>
+      </c>
+      <c r="BP18" s="14">
+        <f>BP7</f>
         <v>13532045.806827499</v>
       </c>
-      <c r="BO18" s="14">
-        <f>BO7</f>
+      <c r="BQ18" s="14">
+        <f>BQ7</f>
         <v>4543046.5541842831</v>
       </c>
     </row>
-    <row r="19" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>80</v>
       </c>
@@ -5389,11 +5540,21 @@
       <c r="BJ19" s="3">
         <v>9.0225550635375701E-13</v>
       </c>
-      <c r="BK19" s="3"/>
-      <c r="BL19" s="3"/>
-      <c r="BN19" s="3"/>
-    </row>
-    <row r="20" spans="1:67" x14ac:dyDescent="0.25">
+      <c r="BK19" s="3">
+        <v>9.0427404752907003E-4</v>
+      </c>
+      <c r="BL19" s="3">
+        <v>1.2211326181060301E-4</v>
+      </c>
+      <c r="BM19" s="3">
+        <v>9.7508422984112792E-6</v>
+      </c>
+      <c r="BN19" s="3">
+        <v>8.1318162268899895E-4</v>
+      </c>
+      <c r="BP19" s="3"/>
+    </row>
+    <row r="20" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>83</v>
       </c>
@@ -5580,16 +5741,26 @@
       <c r="BJ20" s="3">
         <v>0</v>
       </c>
-      <c r="BK20" s="3"/>
-      <c r="BL20" s="3"/>
-      <c r="BN20" s="3" t="s">
+      <c r="BK20" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL20" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM20" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN20" s="3">
+        <v>0</v>
+      </c>
+      <c r="BP20" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="BO20" t="s">
+      <c r="BQ20" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="21" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>97</v>
       </c>
@@ -5776,18 +5947,28 @@
       <c r="BJ21" s="3">
         <v>79.360228286980799</v>
       </c>
-      <c r="BK21" s="3"/>
-      <c r="BL21" s="3"/>
-      <c r="BN21" s="14">
+      <c r="BK21" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL21" s="3">
+        <v>136.309150960653</v>
+      </c>
+      <c r="BM21" s="3">
+        <v>115.391295741608</v>
+      </c>
+      <c r="BN21" s="3">
+        <v>0</v>
+      </c>
+      <c r="BP21" s="14">
         <f>'250718_investment'!L5</f>
         <v>180.68099999996281</v>
       </c>
-      <c r="BO21" s="3">
-        <f>BN15/(BN18-BO18)</f>
+      <c r="BQ21" s="3">
+        <f>BP15/(BP18-BQ18)</f>
         <v>4.2856510652275484</v>
       </c>
     </row>
-    <row r="22" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>98</v>
       </c>
@@ -5974,10 +6155,20 @@
       <c r="BJ22" s="3">
         <v>150.00000000000099</v>
       </c>
-      <c r="BK22" s="3"/>
-      <c r="BL22" s="3"/>
-    </row>
-    <row r="23" spans="1:67" x14ac:dyDescent="0.25">
+      <c r="BK22" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL22" s="3">
+        <v>150.00000000000199</v>
+      </c>
+      <c r="BM22" s="3">
+        <v>150.00000000000099</v>
+      </c>
+      <c r="BN22" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>99</v>
       </c>
@@ -6164,13 +6355,23 @@
       <c r="BJ23" s="3">
         <v>68.578081151739397</v>
       </c>
-      <c r="BK23" s="3"/>
-      <c r="BL23" s="3"/>
-      <c r="BN23" t="s">
+      <c r="BK23" s="3">
+        <v>3.2919992086239298</v>
+      </c>
+      <c r="BL23" s="3">
+        <v>100.173950233754</v>
+      </c>
+      <c r="BM23" s="3">
+        <v>95.019791232856306</v>
+      </c>
+      <c r="BN23" s="3">
+        <v>6.2946653740599796</v>
+      </c>
+      <c r="BP23" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="24" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>100</v>
       </c>
@@ -6357,14 +6558,24 @@
       <c r="BJ24" s="3">
         <v>150.00000000000099</v>
       </c>
-      <c r="BK24" s="3"/>
-      <c r="BL24" s="3"/>
-      <c r="BN24" s="5">
-        <f>(BN18-BO18)/BN21/1000</f>
+      <c r="BK24" s="3">
+        <v>7.0472548814924503</v>
+      </c>
+      <c r="BL24" s="3">
+        <v>150.00000000000199</v>
+      </c>
+      <c r="BM24" s="3">
+        <v>150.00000000000099</v>
+      </c>
+      <c r="BN24" s="3">
+        <v>8.7448226815953607</v>
+      </c>
+      <c r="BP24" s="5">
+        <f>(BP18-BQ18)/BP21/1000</f>
         <v>49.750661401282187</v>
       </c>
     </row>
-    <row r="25" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>68</v>
       </c>
@@ -6551,10 +6762,20 @@
       <c r="BJ25" s="3">
         <v>222505239.304602</v>
       </c>
-      <c r="BK25" s="3"/>
-      <c r="BL25" s="3"/>
-    </row>
-    <row r="26" spans="1:67" x14ac:dyDescent="0.25">
+      <c r="BK25" s="3">
+        <v>331027758.79087698</v>
+      </c>
+      <c r="BL25" s="3">
+        <v>132416238.484796</v>
+      </c>
+      <c r="BM25" s="3">
+        <v>245536194.188411</v>
+      </c>
+      <c r="BN25" s="3">
+        <v>331464587.11163098</v>
+      </c>
+    </row>
+    <row r="26" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>69</v>
       </c>
@@ -6741,13 +6962,23 @@
       <c r="BJ26" s="3">
         <v>234060243.661291</v>
       </c>
-      <c r="BK26" s="3"/>
-      <c r="BL26" s="3"/>
-      <c r="BN26" t="s">
+      <c r="BK26" s="3">
+        <v>324129883.19314897</v>
+      </c>
+      <c r="BL26" s="3">
+        <v>203091040.53803399</v>
+      </c>
+      <c r="BM26" s="3">
+        <v>259924674.949826</v>
+      </c>
+      <c r="BN26" s="3">
+        <v>329263368.95488399</v>
+      </c>
+      <c r="BP26" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="27" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>71</v>
       </c>
@@ -6934,14 +7165,24 @@
       <c r="BJ27" s="3">
         <v>0</v>
       </c>
-      <c r="BK27" s="3"/>
-      <c r="BL27" s="3"/>
-      <c r="BN27" s="15">
-        <f>BN24/8</f>
+      <c r="BK27" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL27" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM27" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN27" s="3">
+        <v>0</v>
+      </c>
+      <c r="BP27" s="15">
+        <f>BP24/8</f>
         <v>6.2188326751602734</v>
       </c>
     </row>
-    <row r="28" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>70</v>
       </c>
@@ -7128,10 +7369,20 @@
       <c r="BJ28" s="3">
         <v>0</v>
       </c>
-      <c r="BK28" s="3"/>
-      <c r="BL28" s="3"/>
-    </row>
-    <row r="29" spans="1:67" x14ac:dyDescent="0.25">
+      <c r="BK28" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL28" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM28" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN28" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>72</v>
       </c>
@@ -7318,13 +7569,23 @@
       <c r="BJ29" s="3">
         <v>277253624.84891802</v>
       </c>
-      <c r="BK29" s="3"/>
-      <c r="BL29" s="3"/>
-      <c r="BN29" t="s">
+      <c r="BK29" s="3">
+        <v>276974005.47001302</v>
+      </c>
+      <c r="BL29" s="3">
+        <v>277071236.67118299</v>
+      </c>
+      <c r="BM29" s="3">
+        <v>276879449.84059697</v>
+      </c>
+      <c r="BN29" s="3">
+        <v>276660438.404908</v>
+      </c>
+      <c r="BP29" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="30" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>73</v>
       </c>
@@ -7391,12 +7652,14 @@
       <c r="BJ30" s="3"/>
       <c r="BK30" s="3"/>
       <c r="BL30" s="3"/>
-      <c r="BN30" s="15">
-        <f>BN27*20</f>
+      <c r="BM30" s="3"/>
+      <c r="BN30" s="3"/>
+      <c r="BP30" s="15">
+        <f>BP27*20</f>
         <v>124.37665350320546</v>
       </c>
     </row>
-    <row r="31" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>2</v>
       </c>
@@ -7583,10 +7846,20 @@
       <c r="BJ31" s="3">
         <v>0</v>
       </c>
-      <c r="BK31" s="3"/>
-      <c r="BL31" s="3"/>
-    </row>
-    <row r="32" spans="1:67" x14ac:dyDescent="0.25">
+      <c r="BK31" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL31" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM31" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN31" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>0</v>
       </c>
@@ -7773,13 +8046,23 @@
       <c r="BJ32" s="3">
         <v>120</v>
       </c>
-      <c r="BK32" s="3"/>
-      <c r="BL32" s="3"/>
-      <c r="BN32" t="s">
+      <c r="BK32" s="3">
+        <v>120</v>
+      </c>
+      <c r="BL32" s="3">
+        <v>120</v>
+      </c>
+      <c r="BM32" s="3">
+        <v>120</v>
+      </c>
+      <c r="BN32" s="3">
+        <v>120</v>
+      </c>
+      <c r="BP32" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="33" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>1</v>
       </c>
@@ -7966,14 +8249,24 @@
       <c r="BJ33" s="3">
         <v>480</v>
       </c>
-      <c r="BK33" s="3"/>
-      <c r="BL33" s="3"/>
-      <c r="BN33" s="14">
+      <c r="BK33" s="3">
+        <v>200.380621095148</v>
+      </c>
+      <c r="BL33" s="3">
+        <v>297.61182226493798</v>
+      </c>
+      <c r="BM33" s="3">
+        <v>141.45337170994901</v>
+      </c>
+      <c r="BN33" s="3">
+        <v>20.423198173646899</v>
+      </c>
+      <c r="BP33" s="14">
         <f>BG41</f>
         <v>49494802.774962798</v>
       </c>
     </row>
-    <row r="34" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>15</v>
       </c>
@@ -8040,8 +8333,10 @@
       <c r="BJ34" s="3"/>
       <c r="BK34" s="3"/>
       <c r="BL34" s="3"/>
-    </row>
-    <row r="35" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="BM34" s="3"/>
+      <c r="BN34" s="3"/>
+    </row>
+    <row r="35" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>2</v>
       </c>
@@ -8228,13 +8523,23 @@
       <c r="BJ35" s="3">
         <v>0</v>
       </c>
-      <c r="BK35" s="3"/>
-      <c r="BL35" s="3"/>
-      <c r="BN35" t="s">
+      <c r="BK35" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL35" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM35" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN35" s="3">
+        <v>0</v>
+      </c>
+      <c r="BP35" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="36" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>0</v>
       </c>
@@ -8421,14 +8726,24 @@
       <c r="BJ36" s="3">
         <v>120</v>
       </c>
-      <c r="BK36" s="3"/>
-      <c r="BL36" s="3"/>
-      <c r="BN36" s="14">
-        <f>BN15+BN7</f>
+      <c r="BK36" s="3">
+        <v>120</v>
+      </c>
+      <c r="BL36" s="3">
+        <v>120</v>
+      </c>
+      <c r="BM36" s="3">
+        <v>120</v>
+      </c>
+      <c r="BN36" s="3">
+        <v>120</v>
+      </c>
+      <c r="BP36" s="14">
+        <f>BP15+BP7</f>
         <v>52055760.029247537</v>
       </c>
     </row>
-    <row r="37" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>1</v>
       </c>
@@ -8615,10 +8930,20 @@
       <c r="BJ37" s="3">
         <v>624</v>
       </c>
-      <c r="BK37" s="3"/>
-      <c r="BL37" s="3"/>
-    </row>
-    <row r="38" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="BK37" s="3">
+        <v>344.380621095148</v>
+      </c>
+      <c r="BL37" s="3">
+        <v>441.61182226493798</v>
+      </c>
+      <c r="BM37" s="3">
+        <v>249.824991678424</v>
+      </c>
+      <c r="BN37" s="3">
+        <v>30.8135559896226</v>
+      </c>
+    </row>
+    <row r="38" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>74</v>
       </c>
@@ -8685,11 +9010,13 @@
       <c r="BJ38" s="3"/>
       <c r="BK38" s="3"/>
       <c r="BL38" s="3"/>
-      <c r="BN38" t="s">
+      <c r="BM38" s="3"/>
+      <c r="BN38" s="3"/>
+      <c r="BP38" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="39" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>2</v>
       </c>
@@ -8876,14 +9203,24 @@
       <c r="BJ39" s="3">
         <v>0</v>
       </c>
-      <c r="BK39" s="3"/>
-      <c r="BL39" s="3"/>
-      <c r="BN39" s="16">
-        <f>(BN18-BO18)/BN33</f>
+      <c r="BK39" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL39" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM39" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN39" s="3">
+        <v>0</v>
+      </c>
+      <c r="BP39" s="16">
+        <f>(BP18-BQ18)/BP33</f>
         <v>0.18161501306537883</v>
       </c>
     </row>
-    <row r="40" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>0</v>
       </c>
@@ -9070,10 +9407,20 @@
       <c r="BJ40" s="3">
         <v>276629624.84891802</v>
       </c>
-      <c r="BK40" s="3"/>
-      <c r="BL40" s="3"/>
-    </row>
-    <row r="41" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="BK40" s="3">
+        <v>276629624.84891802</v>
+      </c>
+      <c r="BL40" s="3">
+        <v>276629624.84891802</v>
+      </c>
+      <c r="BM40" s="3">
+        <v>276629624.84891802</v>
+      </c>
+      <c r="BN40" s="3">
+        <v>276629624.84891802</v>
+      </c>
+    </row>
+    <row r="41" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>1</v>
       </c>
@@ -9260,10 +9607,20 @@
       <c r="BJ41" s="3">
         <v>624000</v>
       </c>
-      <c r="BK41" s="3"/>
-      <c r="BL41" s="3"/>
-    </row>
-    <row r="42" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="BK41" s="3">
+        <v>344380.62109514797</v>
+      </c>
+      <c r="BL41" s="3">
+        <v>441611.82226493797</v>
+      </c>
+      <c r="BM41" s="3">
+        <v>249824.991678424</v>
+      </c>
+      <c r="BN41" s="3">
+        <v>30813.5559896226</v>
+      </c>
+    </row>
+    <row r="42" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
         <v>76</v>
       </c>
@@ -9330,8 +9687,10 @@
       <c r="BJ42" s="3"/>
       <c r="BK42" s="3"/>
       <c r="BL42" s="3"/>
-    </row>
-    <row r="43" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="BM42" s="3"/>
+      <c r="BN42" s="3"/>
+    </row>
+    <row r="43" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>45</v>
       </c>
@@ -9398,8 +9757,10 @@
       <c r="BJ43" s="3"/>
       <c r="BK43" s="3"/>
       <c r="BL43" s="3"/>
-    </row>
-    <row r="44" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="BM43" s="3"/>
+      <c r="BN43" s="3"/>
+    </row>
+    <row r="44" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>2</v>
       </c>
@@ -9586,10 +9947,20 @@
       <c r="BJ44" s="3">
         <v>0</v>
       </c>
-      <c r="BK44" s="3"/>
-      <c r="BL44" s="3"/>
-    </row>
-    <row r="45" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="BK44" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL44" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM44" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN44" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>0</v>
       </c>
@@ -9776,10 +10147,20 @@
       <c r="BJ45" s="3">
         <v>120</v>
       </c>
-      <c r="BK45" s="3"/>
-      <c r="BL45" s="3"/>
-    </row>
-    <row r="46" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="BK45" s="3">
+        <v>120</v>
+      </c>
+      <c r="BL45" s="3">
+        <v>120</v>
+      </c>
+      <c r="BM45" s="3">
+        <v>120</v>
+      </c>
+      <c r="BN45" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="46" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>1</v>
       </c>
@@ -9966,10 +10347,20 @@
       <c r="BJ46" s="3">
         <v>98.084000000000003</v>
       </c>
-      <c r="BK46" s="3"/>
-      <c r="BL46" s="3"/>
-    </row>
-    <row r="47" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="BK46" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL46" s="3">
+        <v>216.36322807017501</v>
+      </c>
+      <c r="BM46" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="BN46" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>75</v>
       </c>
@@ -10156,10 +10547,20 @@
       <c r="BJ47" s="3">
         <v>0</v>
       </c>
-      <c r="BK47" s="3"/>
-      <c r="BL47" s="3"/>
-    </row>
-    <row r="48" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="BK47" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL47" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM47" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN47" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>46</v>
       </c>
@@ -10226,8 +10627,10 @@
       <c r="BJ48" s="3"/>
       <c r="BK48" s="3"/>
       <c r="BL48" s="3"/>
-    </row>
-    <row r="49" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BM48" s="3"/>
+      <c r="BN48" s="3"/>
+    </row>
+    <row r="49" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>0</v>
       </c>
@@ -10414,10 +10817,20 @@
       <c r="BJ49" s="3">
         <v>0</v>
       </c>
-      <c r="BK49" s="3"/>
-      <c r="BL49" s="3"/>
-    </row>
-    <row r="50" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK49" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL49" s="3">
+        <v>120</v>
+      </c>
+      <c r="BM49" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN49" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>24</v>
       </c>
@@ -10604,10 +11017,20 @@
       <c r="BJ50" s="3">
         <v>98.084000000000003</v>
       </c>
-      <c r="BK50" s="3"/>
-      <c r="BL50" s="3"/>
-    </row>
-    <row r="51" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK50" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="BL50" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="BM50" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="BN50" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="51" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>1</v>
       </c>
@@ -10794,10 +11217,20 @@
       <c r="BJ51" s="3">
         <v>102.10268421052599</v>
       </c>
-      <c r="BK51" s="3"/>
-      <c r="BL51" s="3"/>
-    </row>
-    <row r="52" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK51" s="3">
+        <v>99.212263157894796</v>
+      </c>
+      <c r="BL51" s="3">
+        <v>102.10268421052599</v>
+      </c>
+      <c r="BM51" s="3">
+        <v>102.10268421052599</v>
+      </c>
+      <c r="BN51" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>23</v>
       </c>
@@ -10864,8 +11297,10 @@
       <c r="BJ52" s="3"/>
       <c r="BK52" s="3"/>
       <c r="BL52" s="3"/>
-    </row>
-    <row r="53" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BM52" s="3"/>
+      <c r="BN52" s="3"/>
+    </row>
+    <row r="53" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>2</v>
       </c>
@@ -11052,10 +11487,20 @@
       <c r="BJ53" s="3">
         <v>0</v>
       </c>
-      <c r="BK53" s="3"/>
-      <c r="BL53" s="3"/>
-    </row>
-    <row r="54" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK53" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL53" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM53" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN53" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>0</v>
       </c>
@@ -11242,10 +11687,20 @@
       <c r="BJ54" s="3">
         <v>8348098.97574641</v>
       </c>
-      <c r="BK54" s="3"/>
-      <c r="BL54" s="3"/>
-    </row>
-    <row r="55" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK54" s="3">
+        <v>7737357.5964027597</v>
+      </c>
+      <c r="BL54" s="3">
+        <v>14018677.077594901</v>
+      </c>
+      <c r="BM54" s="3">
+        <v>8303305.3775849203</v>
+      </c>
+      <c r="BN54" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+    </row>
+    <row r="55" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>1</v>
       </c>
@@ -11432,10 +11887,20 @@
       <c r="BJ55" s="3">
         <v>3649204.89405635</v>
       </c>
-      <c r="BK55" s="3"/>
-      <c r="BL55" s="3"/>
-    </row>
-    <row r="56" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK55" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL55" s="3">
+        <v>6912967.7710731504</v>
+      </c>
+      <c r="BM55" s="3">
+        <v>3489731.0450522099</v>
+      </c>
+      <c r="BN55" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>35</v>
       </c>
@@ -11622,10 +12087,20 @@
       <c r="BJ56" s="3">
         <v>0</v>
       </c>
-      <c r="BK56" s="3"/>
-      <c r="BL56" s="3"/>
-    </row>
-    <row r="57" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK56" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL56" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM56" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN56" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>22</v>
       </c>
@@ -11692,8 +12167,10 @@
       <c r="BJ57" s="3"/>
       <c r="BK57" s="3"/>
       <c r="BL57" s="3"/>
-    </row>
-    <row r="58" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BM57" s="3"/>
+      <c r="BN57" s="3"/>
+    </row>
+    <row r="58" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>0</v>
       </c>
@@ -11880,10 +12357,20 @@
       <c r="BJ58" s="3">
         <v>0</v>
       </c>
-      <c r="BK58" s="3"/>
-      <c r="BL58" s="3"/>
-    </row>
-    <row r="59" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK58" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL58" s="3">
+        <v>5094141.5947218696</v>
+      </c>
+      <c r="BM58" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN58" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>24</v>
       </c>
@@ -12070,10 +12557,20 @@
       <c r="BJ59" s="3">
         <v>7685861.4146331698</v>
       </c>
-      <c r="BK59" s="3"/>
-      <c r="BL59" s="3"/>
-    </row>
-    <row r="60" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK59" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+      <c r="BL59" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+      <c r="BM59" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+      <c r="BN59" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+    </row>
+    <row r="60" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>1</v>
       </c>
@@ -12260,10 +12757,20 @@
       <c r="BJ60" s="3">
         <v>4311442.4551709602</v>
       </c>
-      <c r="BK60" s="3"/>
-      <c r="BL60" s="3"/>
-    </row>
-    <row r="61" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK60" s="3">
+        <v>51496.181769622497</v>
+      </c>
+      <c r="BL60" s="3">
+        <v>8167495.0036304398</v>
+      </c>
+      <c r="BM60" s="3">
+        <v>4123028.1723211999</v>
+      </c>
+      <c r="BN60" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>27</v>
       </c>
@@ -12330,8 +12837,10 @@
       <c r="BJ61" s="3"/>
       <c r="BK61" s="3"/>
       <c r="BL61" s="3"/>
-    </row>
-    <row r="62" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BM61" s="3"/>
+      <c r="BN61" s="3"/>
+    </row>
+    <row r="62" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>2</v>
       </c>
@@ -12518,10 +13027,20 @@
       <c r="BJ62" s="3">
         <v>0</v>
       </c>
-      <c r="BK62" s="3"/>
-      <c r="BL62" s="3"/>
-    </row>
-    <row r="63" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK62" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL62" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM62" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN62" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>0</v>
       </c>
@@ -12708,10 +13227,20 @@
       <c r="BJ63" s="3">
         <v>222505239.304602</v>
       </c>
-      <c r="BK63" s="3"/>
-      <c r="BL63" s="3"/>
-    </row>
-    <row r="64" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK63" s="3">
+        <v>331027758.79087698</v>
+      </c>
+      <c r="BL63" s="3">
+        <v>452712446.33587801</v>
+      </c>
+      <c r="BM63" s="3">
+        <v>245536194.188411</v>
+      </c>
+      <c r="BN63" s="3">
+        <v>331464587.11163098</v>
+      </c>
+    </row>
+    <row r="64" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>1</v>
       </c>
@@ -12898,10 +13427,20 @@
       <c r="BJ64" s="3">
         <v>0</v>
       </c>
-      <c r="BK64" s="3"/>
-      <c r="BL64" s="3"/>
-    </row>
-    <row r="65" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK64" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL64" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM64" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN64" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>28</v>
       </c>
@@ -12968,8 +13507,10 @@
       <c r="BJ65" s="3"/>
       <c r="BK65" s="3"/>
       <c r="BL65" s="3"/>
-    </row>
-    <row r="66" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BM65" s="3"/>
+      <c r="BN65" s="3"/>
+    </row>
+    <row r="66" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>0</v>
       </c>
@@ -13156,10 +13697,20 @@
       <c r="BJ66" s="3">
         <v>0</v>
       </c>
-      <c r="BK66" s="3"/>
-      <c r="BL66" s="3"/>
-    </row>
-    <row r="67" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK66" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL66" s="3">
+        <v>320296207.85106802</v>
+      </c>
+      <c r="BM66" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN66" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>24</v>
       </c>
@@ -13346,10 +13897,20 @@
       <c r="BJ67" s="3">
         <v>0</v>
       </c>
-      <c r="BK67" s="3"/>
-      <c r="BL67" s="3"/>
-    </row>
-    <row r="68" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK67" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL67" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM67" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN67" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>1</v>
       </c>
@@ -13536,10 +14097,20 @@
       <c r="BJ68" s="3">
         <v>0</v>
       </c>
-      <c r="BK68" s="3"/>
-      <c r="BL68" s="3"/>
-    </row>
-    <row r="69" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK68" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL68" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM68" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN68" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A69" s="9" t="s">
         <v>77</v>
       </c>
@@ -13606,8 +14177,10 @@
       <c r="BJ69" s="3"/>
       <c r="BK69" s="3"/>
       <c r="BL69" s="3"/>
-    </row>
-    <row r="70" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BM69" s="3"/>
+      <c r="BN69" s="3"/>
+    </row>
+    <row r="70" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>45</v>
       </c>
@@ -13674,8 +14247,10 @@
       <c r="BJ70" s="3"/>
       <c r="BK70" s="3"/>
       <c r="BL70" s="3"/>
-    </row>
-    <row r="71" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BM70" s="3"/>
+      <c r="BN70" s="3"/>
+    </row>
+    <row r="71" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>2</v>
       </c>
@@ -13862,10 +14437,20 @@
       <c r="BJ71" s="3">
         <v>0</v>
       </c>
-      <c r="BK71" s="3"/>
-      <c r="BL71" s="3"/>
-    </row>
-    <row r="72" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK71" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL71" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM71" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN71" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>0</v>
       </c>
@@ -14052,10 +14637,20 @@
       <c r="BJ72" s="3">
         <v>80</v>
       </c>
-      <c r="BK72" s="3"/>
-      <c r="BL72" s="3"/>
-    </row>
-    <row r="73" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK72" s="3">
+        <v>65.810415091664197</v>
+      </c>
+      <c r="BL72" s="3">
+        <v>80</v>
+      </c>
+      <c r="BM72" s="3">
+        <v>80</v>
+      </c>
+      <c r="BN72" s="3">
+        <v>77.976804403882795</v>
+      </c>
+    </row>
+    <row r="73" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>1</v>
       </c>
@@ -14242,10 +14837,20 @@
       <c r="BJ73" s="3">
         <v>98.084000000000003</v>
       </c>
-      <c r="BK73" s="3"/>
-      <c r="BL73" s="3"/>
-    </row>
-    <row r="74" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK73" s="3">
+        <v>32.485621477995601</v>
+      </c>
+      <c r="BL73" s="3">
+        <v>172.921684210526</v>
+      </c>
+      <c r="BM73" s="3">
+        <v>94.105543859649103</v>
+      </c>
+      <c r="BN73" s="3">
+        <v>20.2601351596863</v>
+      </c>
+    </row>
+    <row r="74" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>75</v>
       </c>
@@ -14432,10 +15037,20 @@
       <c r="BJ74" s="3">
         <v>0</v>
       </c>
-      <c r="BK74" s="3"/>
-      <c r="BL74" s="3"/>
-    </row>
-    <row r="75" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK74" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL74" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM74" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN74" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>46</v>
       </c>
@@ -14502,8 +15117,10 @@
       <c r="BJ75" s="3"/>
       <c r="BK75" s="3"/>
       <c r="BL75" s="3"/>
-    </row>
-    <row r="76" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BM75" s="3"/>
+      <c r="BN75" s="3"/>
+    </row>
+    <row r="76" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>0</v>
       </c>
@@ -14690,10 +15307,20 @@
       <c r="BJ76" s="3">
         <v>0</v>
       </c>
-      <c r="BK76" s="3"/>
-      <c r="BL76" s="3"/>
-    </row>
-    <row r="77" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK76" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL76" s="3">
+        <v>80</v>
+      </c>
+      <c r="BM76" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN76" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>24</v>
       </c>
@@ -14880,10 +15507,20 @@
       <c r="BJ77" s="3">
         <v>98.084000000000003</v>
       </c>
-      <c r="BK77" s="3"/>
-      <c r="BL77" s="3"/>
-    </row>
-    <row r="78" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK77" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="BL77" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="BM77" s="3">
+        <v>98.084000000000003</v>
+      </c>
+      <c r="BN77" s="3">
+        <v>98.084000000000003</v>
+      </c>
+    </row>
+    <row r="78" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>1</v>
       </c>
@@ -15070,10 +15707,20 @@
       <c r="BJ78" s="3">
         <v>62.102684210526299</v>
       </c>
-      <c r="BK78" s="3"/>
-      <c r="BL78" s="3"/>
-    </row>
-    <row r="79" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK78" s="3">
+        <v>43.440380003944497</v>
+      </c>
+      <c r="BL78" s="3">
+        <v>66.556350877193196</v>
+      </c>
+      <c r="BM78" s="3">
+        <v>62.102684210526299</v>
+      </c>
+      <c r="BN78" s="3">
+        <v>33.417737113869002</v>
+      </c>
+    </row>
+    <row r="79" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>23</v>
       </c>
@@ -15140,8 +15787,10 @@
       <c r="BJ79" s="3"/>
       <c r="BK79" s="3"/>
       <c r="BL79" s="3"/>
-    </row>
-    <row r="80" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BM79" s="3"/>
+      <c r="BN79" s="3"/>
+    </row>
+    <row r="80" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>2</v>
       </c>
@@ -15328,10 +15977,20 @@
       <c r="BJ80" s="3">
         <v>0</v>
       </c>
-      <c r="BK80" s="3"/>
-      <c r="BL80" s="3"/>
-    </row>
-    <row r="81" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK80" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL80" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM80" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN80" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>0</v>
       </c>
@@ -15518,10 +16177,20 @@
       <c r="BJ81" s="3">
         <v>8227029.5159309097</v>
       </c>
-      <c r="BK81" s="3"/>
-      <c r="BL81" s="3"/>
-    </row>
-    <row r="82" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK81" s="3">
+        <v>7710700.2683432698</v>
+      </c>
+      <c r="BL81" s="3">
+        <v>11442406.393465901</v>
+      </c>
+      <c r="BM81" s="3">
+        <v>8174998.0465153297</v>
+      </c>
+      <c r="BN81" s="3">
+        <v>7675385.5236858204</v>
+      </c>
+    </row>
+    <row r="82" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>1</v>
       </c>
@@ -15708,10 +16377,20 @@
       <c r="BJ82" s="3">
         <v>2982061.72486516</v>
       </c>
-      <c r="BK82" s="3"/>
-      <c r="BL82" s="3"/>
-    </row>
-    <row r="83" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK82" s="3">
+        <v>132489.805127036</v>
+      </c>
+      <c r="BL82" s="3">
+        <v>4504377.0382893896</v>
+      </c>
+      <c r="BM82" s="3">
+        <v>2782704.18947108</v>
+      </c>
+      <c r="BN82" s="3">
+        <v>29631.016788748901</v>
+      </c>
+    </row>
+    <row r="83" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>35</v>
       </c>
@@ -15898,10 +16577,20 @@
       <c r="BJ83" s="3">
         <v>0</v>
       </c>
-      <c r="BK83" s="3"/>
-      <c r="BL83" s="3"/>
-    </row>
-    <row r="84" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK83" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL83" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM83" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN83" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>22</v>
       </c>
@@ -15968,8 +16657,10 @@
       <c r="BJ84" s="3"/>
       <c r="BK84" s="3"/>
       <c r="BL84" s="3"/>
-    </row>
-    <row r="85" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BM84" s="3"/>
+      <c r="BN84" s="3"/>
+    </row>
+    <row r="85" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>0</v>
       </c>
@@ -16156,10 +16847,20 @@
       <c r="BJ85" s="3">
         <v>0</v>
       </c>
-      <c r="BK85" s="3"/>
-      <c r="BL85" s="3"/>
-    </row>
-    <row r="86" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK85" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL85" s="3">
+        <v>2954968.6617214298</v>
+      </c>
+      <c r="BM85" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN85" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>24</v>
       </c>
@@ -16346,10 +17047,20 @@
       <c r="BJ86" s="3">
         <v>7685861.4146331698</v>
       </c>
-      <c r="BK86" s="3"/>
-      <c r="BL86" s="3"/>
-    </row>
-    <row r="87" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK86" s="3">
+        <v>7685861.4146331698</v>
+      </c>
+      <c r="BL86" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+      <c r="BM86" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+      <c r="BN86" s="3">
+        <v>7670008.2503171796</v>
+      </c>
+    </row>
+    <row r="87" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>1</v>
       </c>
@@ -16536,10 +17247,20 @@
       <c r="BJ87" s="3">
         <v>3523229.82616458</v>
       </c>
-      <c r="BK87" s="3"/>
-      <c r="BL87" s="3"/>
-    </row>
-    <row r="88" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK87" s="3">
+        <v>157328.658836071</v>
+      </c>
+      <c r="BL87" s="3">
+        <v>5321806.5197182</v>
+      </c>
+      <c r="BM87" s="3">
+        <v>3287693.9856702201</v>
+      </c>
+      <c r="BN87" s="3">
+        <v>35008.290156839299</v>
+      </c>
+    </row>
+    <row r="88" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>27</v>
       </c>
@@ -16606,8 +17327,10 @@
       <c r="BJ88" s="3"/>
       <c r="BK88" s="3"/>
       <c r="BL88" s="3"/>
-    </row>
-    <row r="89" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BM88" s="3"/>
+      <c r="BN88" s="3"/>
+    </row>
+    <row r="89" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>2</v>
       </c>
@@ -16794,10 +17517,20 @@
       <c r="BJ89" s="3">
         <v>0</v>
       </c>
-      <c r="BK89" s="3"/>
-      <c r="BL89" s="3"/>
-    </row>
-    <row r="90" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK89" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL89" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM89" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN89" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>0</v>
       </c>
@@ -16984,10 +17717,20 @@
       <c r="BJ90" s="3">
         <v>234060243.661291</v>
       </c>
-      <c r="BK90" s="3"/>
-      <c r="BL90" s="3"/>
-    </row>
-    <row r="91" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK90" s="3">
+        <v>324129883.19314897</v>
+      </c>
+      <c r="BL90" s="3">
+        <v>387158870.48873401</v>
+      </c>
+      <c r="BM90" s="3">
+        <v>259924674.949826</v>
+      </c>
+      <c r="BN90" s="3">
+        <v>329263368.95488399</v>
+      </c>
+    </row>
+    <row r="91" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>1</v>
       </c>
@@ -17174,10 +17917,20 @@
       <c r="BJ91" s="3">
         <v>0</v>
       </c>
-      <c r="BK91" s="3"/>
-      <c r="BL91" s="3"/>
-    </row>
-    <row r="92" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK91" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL91" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM91" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN91" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>28</v>
       </c>
@@ -17244,8 +17997,10 @@
       <c r="BJ92" s="3"/>
       <c r="BK92" s="3"/>
       <c r="BL92" s="3"/>
-    </row>
-    <row r="93" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BM92" s="3"/>
+      <c r="BN92" s="3"/>
+    </row>
+    <row r="93" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>0</v>
       </c>
@@ -17432,10 +18187,20 @@
       <c r="BJ93" s="3">
         <v>0</v>
       </c>
-      <c r="BK93" s="3"/>
-      <c r="BL93" s="3"/>
-    </row>
-    <row r="94" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK93" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL93" s="3">
+        <v>184067829.950708</v>
+      </c>
+      <c r="BM93" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN93" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>24</v>
       </c>
@@ -17622,10 +18387,20 @@
       <c r="BJ94" s="3">
         <v>0</v>
       </c>
-      <c r="BK94" s="3"/>
-      <c r="BL94" s="3"/>
-    </row>
-    <row r="95" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK94" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL94" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM94" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN94" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>1</v>
       </c>
@@ -17812,10 +18587,20 @@
       <c r="BJ95" s="3">
         <v>0</v>
       </c>
-      <c r="BK95" s="3"/>
-      <c r="BL95" s="3"/>
-    </row>
-    <row r="96" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BK95" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL95" s="3">
+        <v>0</v>
+      </c>
+      <c r="BM95" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN95" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:66" x14ac:dyDescent="0.25">
       <c r="V96" s="3"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
setup for final experiments
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\Desktop\ongoing_projects\MVS\dev\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E35223AB-168D-4735-A344-6BA0BE81B79D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A938B698-BE97-4332-B1F4-77580A5E4802}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Experiments" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="147">
   <si>
     <t>Grid</t>
   </si>
@@ -500,6 +500,9 @@
   <si>
     <t>year</t>
   </si>
+  <si>
+    <t>Market</t>
+  </si>
 </sst>
 </file>
 
@@ -508,7 +511,7 @@
   <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -611,7 +614,7 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Bad" xfId="3" builtinId="27"/>
@@ -5111,8 +5114,8 @@
       <c r="AX17" s="5">
         <v>76036916539.554596</v>
       </c>
-      <c r="AY17" s="5">
-        <v>75805109783.920593</v>
+      <c r="AY17" s="5" t="s">
+        <v>146</v>
       </c>
       <c r="AZ17" s="5">
         <v>76059504933.349899</v>

</xml_diff>